<commit_message>
chore: update jigmu quotation template
</commit_message>
<xml_diff>
--- a/직무고시 견적서 양식.xlsx
+++ b/직무고시 견적서 양식.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Master\Documents\Antigravity program\직무고시 견적서\wkace-quotation-jigmu\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3B3A08E-9F77-458A-8572-EC5D854EE00D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72A1324C-9F9E-4C2A-8FB5-4815B3EA4723}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1704,6 +1704,60 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="41" fontId="14" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="14" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="14" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="14" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="14" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="14" fillId="0" borderId="24" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="14" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="14" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="14" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="14" fillId="0" borderId="29" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="14" fillId="0" borderId="31" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="14" fillId="0" borderId="30" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1713,6 +1767,249 @@
     <xf numFmtId="0" fontId="8" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="29" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="31" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="30" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="27" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="23" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="24" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="25" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="28" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="26" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="14" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="8" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="8" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="8" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="14" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="14" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="14" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="14" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="14" fillId="0" borderId="24" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="14" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="14" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="14" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="8" fillId="0" borderId="35" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="8" fillId="0" borderId="40" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="8" fillId="0" borderId="41" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
     <xf numFmtId="176" fontId="8" fillId="0" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
@@ -1740,239 +2037,209 @@
     <xf numFmtId="176" fontId="8" fillId="0" borderId="26" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="41" fontId="14" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="14" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="7" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="7" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="7" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="41" fontId="14" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="41" fontId="14" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="41" fontId="14" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="20" fillId="5" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="10" fillId="3" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="41" fontId="14" fillId="0" borderId="24" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="10" fillId="3" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="41" fontId="14" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="14" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="14" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="14" fillId="0" borderId="29" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="14" fillId="0" borderId="31" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="14" fillId="0" borderId="30" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="29" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="31" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="30" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="27" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="23" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="24" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="25" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="28" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="26" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="14" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="8" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="8" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="8" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="14" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="14" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="14" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="14" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="14" fillId="0" borderId="24" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="14" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="14" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="14" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="5" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="39" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1983,277 +2250,10 @@
     <xf numFmtId="0" fontId="21" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="8" fillId="0" borderId="35" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="8" fillId="0" borderId="40" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="8" fillId="0" borderId="41" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
     <xf numFmtId="0" fontId="19" fillId="6" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="6" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="5" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="5" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="5" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="7" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="7" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="7" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="9" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="20" fillId="5" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="10" fillId="3" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="10" fillId="3" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="5" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="39" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2892,33 +2892,33 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:40" s="1" customFormat="1" ht="54">
-      <c r="A1" s="239" t="s">
+      <c r="A1" s="241" t="s">
         <v>130</v>
       </c>
-      <c r="B1" s="239"/>
-      <c r="C1" s="239"/>
-      <c r="D1" s="239"/>
-      <c r="E1" s="239"/>
-      <c r="F1" s="239"/>
-      <c r="G1" s="239"/>
-      <c r="H1" s="239"/>
-      <c r="I1" s="239"/>
-      <c r="J1" s="239"/>
-      <c r="K1" s="239"/>
-      <c r="L1" s="239"/>
-      <c r="M1" s="239"/>
-      <c r="N1" s="239"/>
-      <c r="O1" s="239"/>
-      <c r="P1" s="239"/>
-      <c r="Q1" s="239"/>
-      <c r="R1" s="239"/>
-      <c r="S1" s="239"/>
-      <c r="T1" s="239"/>
-      <c r="U1" s="239"/>
-      <c r="V1" s="239"/>
-      <c r="W1" s="239"/>
-      <c r="X1" s="239"/>
-      <c r="Y1" s="239"/>
+      <c r="B1" s="241"/>
+      <c r="C1" s="241"/>
+      <c r="D1" s="241"/>
+      <c r="E1" s="241"/>
+      <c r="F1" s="241"/>
+      <c r="G1" s="241"/>
+      <c r="H1" s="241"/>
+      <c r="I1" s="241"/>
+      <c r="J1" s="241"/>
+      <c r="K1" s="241"/>
+      <c r="L1" s="241"/>
+      <c r="M1" s="241"/>
+      <c r="N1" s="241"/>
+      <c r="O1" s="241"/>
+      <c r="P1" s="241"/>
+      <c r="Q1" s="241"/>
+      <c r="R1" s="241"/>
+      <c r="S1" s="241"/>
+      <c r="T1" s="241"/>
+      <c r="U1" s="241"/>
+      <c r="V1" s="241"/>
+      <c r="W1" s="241"/>
+      <c r="X1" s="241"/>
+      <c r="Y1" s="241"/>
       <c r="AB1" s="2"/>
       <c r="AC1" s="3"/>
       <c r="AD1" s="3"/>
@@ -2973,33 +2973,33 @@
       <c r="AN2" s="3"/>
     </row>
     <row r="3" spans="1:40" s="1" customFormat="1" ht="26.25">
-      <c r="A3" s="240" t="s">
+      <c r="A3" s="242" t="s">
         <v>59</v>
       </c>
-      <c r="B3" s="240"/>
-      <c r="C3" s="240"/>
-      <c r="D3" s="240"/>
-      <c r="E3" s="240"/>
-      <c r="F3" s="240"/>
-      <c r="G3" s="240"/>
-      <c r="H3" s="240"/>
-      <c r="I3" s="240"/>
-      <c r="J3" s="240"/>
-      <c r="K3" s="240"/>
-      <c r="L3" s="240"/>
-      <c r="M3" s="240"/>
-      <c r="N3" s="240"/>
-      <c r="O3" s="240"/>
-      <c r="P3" s="240"/>
-      <c r="Q3" s="240"/>
-      <c r="R3" s="240"/>
-      <c r="S3" s="240"/>
-      <c r="T3" s="240"/>
-      <c r="U3" s="240"/>
-      <c r="V3" s="240"/>
-      <c r="W3" s="240"/>
-      <c r="X3" s="240"/>
-      <c r="Y3" s="240"/>
+      <c r="B3" s="242"/>
+      <c r="C3" s="242"/>
+      <c r="D3" s="242"/>
+      <c r="E3" s="242"/>
+      <c r="F3" s="242"/>
+      <c r="G3" s="242"/>
+      <c r="H3" s="242"/>
+      <c r="I3" s="242"/>
+      <c r="J3" s="242"/>
+      <c r="K3" s="242"/>
+      <c r="L3" s="242"/>
+      <c r="M3" s="242"/>
+      <c r="N3" s="242"/>
+      <c r="O3" s="242"/>
+      <c r="P3" s="242"/>
+      <c r="Q3" s="242"/>
+      <c r="R3" s="242"/>
+      <c r="S3" s="242"/>
+      <c r="T3" s="242"/>
+      <c r="U3" s="242"/>
+      <c r="V3" s="242"/>
+      <c r="W3" s="242"/>
+      <c r="X3" s="242"/>
+      <c r="Y3" s="242"/>
       <c r="AB3" s="2"/>
       <c r="AC3" s="3"/>
       <c r="AD3" s="3"/>
@@ -3099,38 +3099,38 @@
         <v>96</v>
       </c>
       <c r="B6" s="8"/>
-      <c r="C6" s="241">
+      <c r="C6" s="243">
         <f ca="1">TODAY()</f>
-        <v>46136</v>
-      </c>
-      <c r="D6" s="241"/>
-      <c r="E6" s="241"/>
-      <c r="F6" s="241"/>
+        <v>46142</v>
+      </c>
+      <c r="D6" s="243"/>
+      <c r="E6" s="243"/>
+      <c r="F6" s="243"/>
       <c r="G6" s="8"/>
       <c r="H6" s="8"/>
       <c r="I6" s="8"/>
       <c r="J6" s="9"/>
-      <c r="K6" s="232" t="s">
+      <c r="K6" s="230" t="s">
         <v>1</v>
       </c>
-      <c r="L6" s="223" t="s">
+      <c r="L6" s="222" t="s">
         <v>2</v>
       </c>
-      <c r="M6" s="224"/>
-      <c r="N6" s="225"/>
-      <c r="O6" s="247" t="s">
+      <c r="M6" s="223"/>
+      <c r="N6" s="224"/>
+      <c r="O6" s="249" t="s">
         <v>18</v>
       </c>
-      <c r="P6" s="248"/>
-      <c r="Q6" s="248"/>
-      <c r="R6" s="248"/>
-      <c r="S6" s="248"/>
-      <c r="T6" s="248"/>
-      <c r="U6" s="248"/>
-      <c r="V6" s="248"/>
-      <c r="W6" s="248"/>
-      <c r="X6" s="248"/>
-      <c r="Y6" s="249"/>
+      <c r="P6" s="250"/>
+      <c r="Q6" s="250"/>
+      <c r="R6" s="250"/>
+      <c r="S6" s="250"/>
+      <c r="T6" s="250"/>
+      <c r="U6" s="250"/>
+      <c r="V6" s="250"/>
+      <c r="W6" s="250"/>
+      <c r="X6" s="250"/>
+      <c r="Y6" s="251"/>
       <c r="AB6" s="2"/>
       <c r="AC6" s="3"/>
       <c r="AD6" s="3"/>
@@ -3160,29 +3160,29 @@
       <c r="H7" s="8"/>
       <c r="I7" s="8"/>
       <c r="J7" s="9"/>
-      <c r="K7" s="233"/>
-      <c r="L7" s="231" t="s">
+      <c r="K7" s="231"/>
+      <c r="L7" s="229" t="s">
         <v>22</v>
       </c>
-      <c r="M7" s="197"/>
-      <c r="N7" s="198"/>
-      <c r="O7" s="202" t="s">
+      <c r="M7" s="192"/>
+      <c r="N7" s="193"/>
+      <c r="O7" s="197" t="s">
         <v>17</v>
       </c>
-      <c r="P7" s="203"/>
-      <c r="Q7" s="203"/>
-      <c r="R7" s="203"/>
-      <c r="S7" s="230" t="s">
+      <c r="P7" s="198"/>
+      <c r="Q7" s="198"/>
+      <c r="R7" s="198"/>
+      <c r="S7" s="228" t="s">
         <v>25</v>
       </c>
-      <c r="T7" s="197"/>
-      <c r="U7" s="198"/>
-      <c r="V7" s="202" t="s">
+      <c r="T7" s="192"/>
+      <c r="U7" s="193"/>
+      <c r="V7" s="197" t="s">
         <v>20</v>
       </c>
-      <c r="W7" s="203"/>
-      <c r="X7" s="203"/>
-      <c r="Y7" s="229"/>
+      <c r="W7" s="198"/>
+      <c r="X7" s="198"/>
+      <c r="Y7" s="221"/>
       <c r="AB7" s="2"/>
       <c r="AC7" s="2"/>
       <c r="AD7" s="2"/>
@@ -3199,25 +3199,25 @@
       <c r="H8" s="11"/>
       <c r="I8" s="11"/>
       <c r="J8" s="12"/>
-      <c r="K8" s="233"/>
-      <c r="L8" s="231" t="s">
+      <c r="K8" s="231"/>
+      <c r="L8" s="229" t="s">
         <v>21</v>
       </c>
-      <c r="M8" s="197"/>
-      <c r="N8" s="198"/>
-      <c r="O8" s="202" t="s">
+      <c r="M8" s="192"/>
+      <c r="N8" s="193"/>
+      <c r="O8" s="197" t="s">
         <v>129</v>
       </c>
-      <c r="P8" s="203"/>
-      <c r="Q8" s="203"/>
-      <c r="R8" s="203"/>
-      <c r="S8" s="203"/>
-      <c r="T8" s="203"/>
-      <c r="U8" s="203"/>
-      <c r="V8" s="203"/>
-      <c r="W8" s="203"/>
-      <c r="X8" s="203"/>
-      <c r="Y8" s="229"/>
+      <c r="P8" s="198"/>
+      <c r="Q8" s="198"/>
+      <c r="R8" s="198"/>
+      <c r="S8" s="198"/>
+      <c r="T8" s="198"/>
+      <c r="U8" s="198"/>
+      <c r="V8" s="198"/>
+      <c r="W8" s="198"/>
+      <c r="X8" s="198"/>
+      <c r="Y8" s="221"/>
       <c r="AA8" s="2"/>
       <c r="AB8" s="2"/>
       <c r="AC8" s="2"/>
@@ -3237,29 +3237,29 @@
       <c r="H9" s="10"/>
       <c r="I9" s="8"/>
       <c r="J9" s="10"/>
-      <c r="K9" s="233"/>
-      <c r="L9" s="231" t="s">
+      <c r="K9" s="231"/>
+      <c r="L9" s="229" t="s">
         <v>23</v>
       </c>
-      <c r="M9" s="197"/>
-      <c r="N9" s="198"/>
-      <c r="O9" s="202" t="s">
+      <c r="M9" s="192"/>
+      <c r="N9" s="193"/>
+      <c r="O9" s="197" t="s">
         <v>9</v>
       </c>
-      <c r="P9" s="203"/>
-      <c r="Q9" s="203"/>
-      <c r="R9" s="203"/>
-      <c r="S9" s="196" t="s">
+      <c r="P9" s="198"/>
+      <c r="Q9" s="198"/>
+      <c r="R9" s="198"/>
+      <c r="S9" s="191" t="s">
         <v>26</v>
       </c>
-      <c r="T9" s="197"/>
-      <c r="U9" s="198"/>
-      <c r="V9" s="206" t="s">
+      <c r="T9" s="192"/>
+      <c r="U9" s="193"/>
+      <c r="V9" s="201" t="s">
         <v>31</v>
       </c>
-      <c r="W9" s="207"/>
-      <c r="X9" s="207"/>
-      <c r="Y9" s="208"/>
+      <c r="W9" s="202"/>
+      <c r="X9" s="202"/>
+      <c r="Y9" s="203"/>
       <c r="AB9" s="2"/>
       <c r="AC9" s="2"/>
       <c r="AD9" s="2"/>
@@ -3278,29 +3278,29 @@
       <c r="H10" s="10"/>
       <c r="I10" s="8"/>
       <c r="J10" s="9"/>
-      <c r="K10" s="234"/>
-      <c r="L10" s="244" t="s">
+      <c r="K10" s="232"/>
+      <c r="L10" s="246" t="s">
         <v>24</v>
       </c>
-      <c r="M10" s="245"/>
-      <c r="N10" s="246"/>
-      <c r="O10" s="204" t="s">
+      <c r="M10" s="247"/>
+      <c r="N10" s="248"/>
+      <c r="O10" s="199" t="s">
         <v>77</v>
       </c>
-      <c r="P10" s="205"/>
-      <c r="Q10" s="205"/>
-      <c r="R10" s="205"/>
-      <c r="S10" s="199" t="s">
+      <c r="P10" s="200"/>
+      <c r="Q10" s="200"/>
+      <c r="R10" s="200"/>
+      <c r="S10" s="194" t="s">
         <v>64</v>
       </c>
-      <c r="T10" s="200"/>
-      <c r="U10" s="201"/>
-      <c r="V10" s="204" t="s">
+      <c r="T10" s="195"/>
+      <c r="U10" s="196"/>
+      <c r="V10" s="199" t="s">
         <v>78</v>
       </c>
-      <c r="W10" s="205"/>
-      <c r="X10" s="205"/>
-      <c r="Y10" s="209"/>
+      <c r="W10" s="200"/>
+      <c r="X10" s="200"/>
+      <c r="Y10" s="204"/>
       <c r="AB10" s="2"/>
       <c r="AC10" s="2"/>
       <c r="AD10" s="2"/>
@@ -3351,10 +3351,10 @@
       <c r="E12" s="15"/>
       <c r="F12" s="15"/>
       <c r="G12" s="15"/>
-      <c r="H12" s="132"/>
-      <c r="I12" s="132"/>
-      <c r="J12" s="132"/>
-      <c r="K12" s="132"/>
+      <c r="H12" s="126"/>
+      <c r="I12" s="126"/>
+      <c r="J12" s="126"/>
+      <c r="K12" s="126"/>
       <c r="L12" s="15"/>
       <c r="M12" s="16"/>
       <c r="N12" s="14" t="s">
@@ -3412,10 +3412,10 @@
         <v>106</v>
       </c>
       <c r="Q13" s="3"/>
-      <c r="R13" s="243" t="s">
+      <c r="R13" s="245" t="s">
         <v>120</v>
       </c>
-      <c r="S13" s="243"/>
+      <c r="S13" s="245"/>
       <c r="T13" s="23" t="s">
         <v>121</v>
       </c>
@@ -3467,10 +3467,10 @@
         <v>107</v>
       </c>
       <c r="Q14" s="10"/>
-      <c r="R14" s="242" t="s">
+      <c r="R14" s="244" t="s">
         <v>123</v>
       </c>
-      <c r="S14" s="242"/>
+      <c r="S14" s="244"/>
       <c r="T14" s="23" t="s">
         <v>121</v>
       </c>
@@ -3514,10 +3514,10 @@
         <v>108</v>
       </c>
       <c r="Q15" s="10"/>
-      <c r="R15" s="242" t="s">
+      <c r="R15" s="244" t="s">
         <v>123</v>
       </c>
-      <c r="S15" s="242"/>
+      <c r="S15" s="244"/>
       <c r="T15" s="23" t="s">
         <v>121</v>
       </c>
@@ -3569,10 +3569,10 @@
         <v>109</v>
       </c>
       <c r="Q16" s="10"/>
-      <c r="R16" s="242" t="s">
+      <c r="R16" s="244" t="s">
         <v>123</v>
       </c>
-      <c r="S16" s="242"/>
+      <c r="S16" s="244"/>
       <c r="T16" s="23" t="s">
         <v>121</v>
       </c>
@@ -3589,21 +3589,21 @@
       <c r="AE16" s="39"/>
     </row>
     <row r="17" spans="1:34" s="1" customFormat="1" ht="20.100000000000001" customHeight="1" thickBot="1">
-      <c r="A17" s="226" t="s">
+      <c r="A17" s="225" t="s">
         <v>79</v>
       </c>
-      <c r="B17" s="227"/>
-      <c r="C17" s="227"/>
-      <c r="D17" s="227"/>
-      <c r="E17" s="227"/>
-      <c r="F17" s="227"/>
-      <c r="G17" s="227"/>
-      <c r="H17" s="227"/>
-      <c r="I17" s="227"/>
-      <c r="J17" s="227"/>
-      <c r="K17" s="227"/>
-      <c r="L17" s="227"/>
-      <c r="M17" s="228"/>
+      <c r="B17" s="226"/>
+      <c r="C17" s="226"/>
+      <c r="D17" s="226"/>
+      <c r="E17" s="226"/>
+      <c r="F17" s="226"/>
+      <c r="G17" s="226"/>
+      <c r="H17" s="226"/>
+      <c r="I17" s="226"/>
+      <c r="J17" s="226"/>
+      <c r="K17" s="226"/>
+      <c r="L17" s="226"/>
+      <c r="M17" s="227"/>
       <c r="N17" s="40"/>
       <c r="O17" s="41" t="s">
         <v>127</v>
@@ -3634,44 +3634,44 @@
       </c>
     </row>
     <row r="18" spans="1:34" s="45" customFormat="1" ht="39.950000000000003" customHeight="1">
-      <c r="A18" s="210" t="s">
+      <c r="A18" s="205" t="s">
         <v>69</v>
       </c>
-      <c r="B18" s="211"/>
-      <c r="C18" s="211"/>
-      <c r="D18" s="211"/>
-      <c r="E18" s="211"/>
-      <c r="F18" s="211"/>
-      <c r="G18" s="211"/>
-      <c r="H18" s="211"/>
-      <c r="I18" s="212"/>
-      <c r="J18" s="236" t="s">
+      <c r="B18" s="206"/>
+      <c r="C18" s="206"/>
+      <c r="D18" s="206"/>
+      <c r="E18" s="206"/>
+      <c r="F18" s="206"/>
+      <c r="G18" s="206"/>
+      <c r="H18" s="206"/>
+      <c r="I18" s="207"/>
+      <c r="J18" s="238" t="s">
         <v>0</v>
       </c>
-      <c r="K18" s="237"/>
-      <c r="L18" s="237"/>
-      <c r="M18" s="238">
+      <c r="K18" s="239"/>
+      <c r="L18" s="239"/>
+      <c r="M18" s="240">
         <f>U41</f>
         <v>1600000</v>
       </c>
-      <c r="N18" s="238"/>
-      <c r="O18" s="238"/>
-      <c r="P18" s="238"/>
-      <c r="Q18" s="238"/>
+      <c r="N18" s="240"/>
+      <c r="O18" s="240"/>
+      <c r="P18" s="240"/>
+      <c r="Q18" s="240"/>
       <c r="R18" s="43" t="s">
         <v>28</v>
       </c>
       <c r="S18" s="43" t="s">
         <v>55</v>
       </c>
-      <c r="T18" s="235">
+      <c r="T18" s="237">
         <f>U41</f>
         <v>1600000</v>
       </c>
-      <c r="U18" s="235"/>
-      <c r="V18" s="235"/>
-      <c r="W18" s="235"/>
-      <c r="X18" s="235"/>
+      <c r="U18" s="237"/>
+      <c r="V18" s="237"/>
+      <c r="W18" s="237"/>
+      <c r="X18" s="237"/>
       <c r="Y18" s="44" t="s">
         <v>54</v>
       </c>
@@ -3689,41 +3689,41 @@
       </c>
     </row>
     <row r="19" spans="1:34" s="1" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A19" s="131" t="s">
+      <c r="A19" s="125" t="s">
         <v>16</v>
       </c>
-      <c r="B19" s="132"/>
-      <c r="C19" s="132"/>
-      <c r="D19" s="132"/>
-      <c r="E19" s="132"/>
-      <c r="F19" s="132"/>
-      <c r="G19" s="132"/>
-      <c r="H19" s="132"/>
-      <c r="I19" s="133"/>
-      <c r="J19" s="98" t="s">
+      <c r="B19" s="126"/>
+      <c r="C19" s="126"/>
+      <c r="D19" s="126"/>
+      <c r="E19" s="126"/>
+      <c r="F19" s="126"/>
+      <c r="G19" s="126"/>
+      <c r="H19" s="126"/>
+      <c r="I19" s="127"/>
+      <c r="J19" s="104" t="s">
         <v>60</v>
       </c>
-      <c r="K19" s="99"/>
-      <c r="L19" s="99"/>
-      <c r="M19" s="99"/>
-      <c r="N19" s="100"/>
-      <c r="O19" s="125" t="s">
+      <c r="K19" s="105"/>
+      <c r="L19" s="105"/>
+      <c r="M19" s="105"/>
+      <c r="N19" s="106"/>
+      <c r="O19" s="119" t="s">
         <v>62</v>
       </c>
-      <c r="P19" s="126"/>
-      <c r="Q19" s="127"/>
-      <c r="R19" s="131" t="s">
+      <c r="P19" s="120"/>
+      <c r="Q19" s="121"/>
+      <c r="R19" s="125" t="s">
         <v>43</v>
       </c>
-      <c r="S19" s="132"/>
-      <c r="T19" s="132"/>
-      <c r="U19" s="132"/>
-      <c r="V19" s="133"/>
-      <c r="W19" s="131" t="s">
+      <c r="S19" s="126"/>
+      <c r="T19" s="126"/>
+      <c r="U19" s="126"/>
+      <c r="V19" s="127"/>
+      <c r="W19" s="125" t="s">
         <v>42</v>
       </c>
-      <c r="X19" s="132"/>
-      <c r="Y19" s="133"/>
+      <c r="X19" s="126"/>
+      <c r="Y19" s="127"/>
       <c r="AB19" s="31" t="s">
         <v>85</v>
       </c>
@@ -3738,15 +3738,15 @@
       </c>
     </row>
     <row r="20" spans="1:34" s="1" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A20" s="134"/>
-      <c r="B20" s="135"/>
-      <c r="C20" s="135"/>
-      <c r="D20" s="135"/>
-      <c r="E20" s="135"/>
-      <c r="F20" s="135"/>
-      <c r="G20" s="135"/>
-      <c r="H20" s="135"/>
-      <c r="I20" s="136"/>
+      <c r="A20" s="128"/>
+      <c r="B20" s="129"/>
+      <c r="C20" s="129"/>
+      <c r="D20" s="129"/>
+      <c r="E20" s="129"/>
+      <c r="F20" s="129"/>
+      <c r="G20" s="129"/>
+      <c r="H20" s="129"/>
+      <c r="I20" s="130"/>
       <c r="J20" s="46" t="s">
         <v>27</v>
       </c>
@@ -3762,17 +3762,17 @@
       <c r="N20" s="49" t="s">
         <v>58</v>
       </c>
-      <c r="O20" s="128"/>
-      <c r="P20" s="129"/>
-      <c r="Q20" s="130"/>
-      <c r="R20" s="134"/>
-      <c r="S20" s="135"/>
-      <c r="T20" s="135"/>
-      <c r="U20" s="135"/>
-      <c r="V20" s="136"/>
-      <c r="W20" s="134"/>
-      <c r="X20" s="135"/>
-      <c r="Y20" s="136"/>
+      <c r="O20" s="122"/>
+      <c r="P20" s="123"/>
+      <c r="Q20" s="124"/>
+      <c r="R20" s="128"/>
+      <c r="S20" s="129"/>
+      <c r="T20" s="129"/>
+      <c r="U20" s="129"/>
+      <c r="V20" s="130"/>
+      <c r="W20" s="128"/>
+      <c r="X20" s="129"/>
+      <c r="Y20" s="130"/>
       <c r="AB20" s="31" t="s">
         <v>85</v>
       </c>
@@ -3787,42 +3787,42 @@
       </c>
     </row>
     <row r="21" spans="1:34" s="1" customFormat="1" ht="20.100000000000001" customHeight="1" thickBot="1">
-      <c r="A21" s="77" t="s">
+      <c r="A21" s="95" t="s">
         <v>61</v>
       </c>
-      <c r="B21" s="78"/>
-      <c r="C21" s="78"/>
-      <c r="D21" s="78"/>
-      <c r="E21" s="78"/>
-      <c r="F21" s="78"/>
-      <c r="G21" s="78"/>
-      <c r="H21" s="78"/>
-      <c r="I21" s="79"/>
-      <c r="J21" s="110" t="s">
+      <c r="B21" s="96"/>
+      <c r="C21" s="96"/>
+      <c r="D21" s="96"/>
+      <c r="E21" s="96"/>
+      <c r="F21" s="96"/>
+      <c r="G21" s="96"/>
+      <c r="H21" s="96"/>
+      <c r="I21" s="97"/>
+      <c r="J21" s="101" t="s">
         <v>33</v>
       </c>
-      <c r="K21" s="111"/>
-      <c r="L21" s="111"/>
-      <c r="M21" s="111"/>
-      <c r="N21" s="112"/>
-      <c r="O21" s="113" t="s">
+      <c r="K21" s="102"/>
+      <c r="L21" s="102"/>
+      <c r="M21" s="102"/>
+      <c r="N21" s="103"/>
+      <c r="O21" s="107" t="s">
         <v>30</v>
       </c>
-      <c r="P21" s="114"/>
-      <c r="Q21" s="115"/>
-      <c r="R21" s="156">
+      <c r="P21" s="108"/>
+      <c r="Q21" s="109"/>
+      <c r="R21" s="150">
         <f>150000*8</f>
         <v>1200000</v>
       </c>
-      <c r="S21" s="157"/>
-      <c r="T21" s="157"/>
-      <c r="U21" s="157"/>
-      <c r="V21" s="158"/>
-      <c r="W21" s="104" t="s">
+      <c r="S21" s="151"/>
+      <c r="T21" s="151"/>
+      <c r="U21" s="151"/>
+      <c r="V21" s="152"/>
+      <c r="W21" s="92" t="s">
         <v>126</v>
       </c>
-      <c r="X21" s="105"/>
-      <c r="Y21" s="106"/>
+      <c r="X21" s="93"/>
+      <c r="Y21" s="94"/>
       <c r="AB21" s="50" t="s">
         <v>85</v>
       </c>
@@ -3837,37 +3837,37 @@
       </c>
     </row>
     <row r="22" spans="1:34" s="1" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A22" s="77" t="s">
+      <c r="A22" s="95" t="s">
         <v>45</v>
       </c>
-      <c r="B22" s="78"/>
-      <c r="C22" s="78"/>
-      <c r="D22" s="78"/>
-      <c r="E22" s="78"/>
-      <c r="F22" s="78"/>
-      <c r="G22" s="78"/>
-      <c r="H22" s="78"/>
-      <c r="I22" s="79"/>
-      <c r="J22" s="110"/>
-      <c r="K22" s="111"/>
-      <c r="L22" s="111"/>
-      <c r="M22" s="111"/>
-      <c r="N22" s="112"/>
-      <c r="O22" s="116" t="s">
+      <c r="B22" s="96"/>
+      <c r="C22" s="96"/>
+      <c r="D22" s="96"/>
+      <c r="E22" s="96"/>
+      <c r="F22" s="96"/>
+      <c r="G22" s="96"/>
+      <c r="H22" s="96"/>
+      <c r="I22" s="97"/>
+      <c r="J22" s="101"/>
+      <c r="K22" s="102"/>
+      <c r="L22" s="102"/>
+      <c r="M22" s="102"/>
+      <c r="N22" s="103"/>
+      <c r="O22" s="110" t="s">
         <v>10</v>
       </c>
-      <c r="P22" s="117"/>
-      <c r="Q22" s="118"/>
-      <c r="R22" s="137">
+      <c r="P22" s="111"/>
+      <c r="Q22" s="112"/>
+      <c r="R22" s="131">
         <v>200000</v>
       </c>
-      <c r="S22" s="138"/>
-      <c r="T22" s="138"/>
-      <c r="U22" s="138"/>
-      <c r="V22" s="139"/>
-      <c r="W22" s="89"/>
-      <c r="X22" s="159"/>
-      <c r="Y22" s="160"/>
+      <c r="S22" s="132"/>
+      <c r="T22" s="132"/>
+      <c r="U22" s="132"/>
+      <c r="V22" s="133"/>
+      <c r="W22" s="77"/>
+      <c r="X22" s="153"/>
+      <c r="Y22" s="154"/>
       <c r="AB22" s="19" t="s">
         <v>80</v>
       </c>
@@ -3880,24 +3880,24 @@
       <c r="AE22" s="21" t="s">
         <v>56</v>
       </c>
-      <c r="AF22" s="89" t="s">
+      <c r="AF22" s="77" t="s">
         <v>95</v>
       </c>
-      <c r="AG22" s="90"/>
-      <c r="AH22" s="91"/>
+      <c r="AG22" s="78"/>
+      <c r="AH22" s="79"/>
     </row>
     <row r="23" spans="1:34" s="1" customFormat="1" ht="20.100000000000001" customHeight="1">
       <c r="A23" s="53"/>
-      <c r="B23" s="256" t="s">
+      <c r="B23" s="254" t="s">
         <v>94</v>
       </c>
-      <c r="C23" s="256"/>
-      <c r="D23" s="256"/>
-      <c r="E23" s="256"/>
-      <c r="F23" s="256"/>
-      <c r="G23" s="256"/>
-      <c r="H23" s="256"/>
-      <c r="I23" s="257"/>
+      <c r="C23" s="254"/>
+      <c r="D23" s="254"/>
+      <c r="E23" s="254"/>
+      <c r="F23" s="254"/>
+      <c r="G23" s="254"/>
+      <c r="H23" s="254"/>
+      <c r="I23" s="255"/>
       <c r="J23" s="54"/>
       <c r="K23" s="54" t="s">
         <v>40</v>
@@ -3911,17 +3911,17 @@
       <c r="N23" s="54" t="s">
         <v>40</v>
       </c>
-      <c r="O23" s="119"/>
-      <c r="P23" s="120"/>
-      <c r="Q23" s="121"/>
-      <c r="R23" s="140"/>
-      <c r="S23" s="141"/>
-      <c r="T23" s="141"/>
-      <c r="U23" s="141"/>
-      <c r="V23" s="142"/>
-      <c r="W23" s="161"/>
-      <c r="X23" s="162"/>
-      <c r="Y23" s="163"/>
+      <c r="O23" s="113"/>
+      <c r="P23" s="114"/>
+      <c r="Q23" s="115"/>
+      <c r="R23" s="134"/>
+      <c r="S23" s="135"/>
+      <c r="T23" s="135"/>
+      <c r="U23" s="135"/>
+      <c r="V23" s="136"/>
+      <c r="W23" s="155"/>
+      <c r="X23" s="156"/>
+      <c r="Y23" s="157"/>
       <c r="AB23" s="31" t="s">
         <v>80</v>
       </c>
@@ -3934,22 +3934,22 @@
       <c r="AE23" s="32" t="s">
         <v>57</v>
       </c>
-      <c r="AF23" s="92"/>
-      <c r="AG23" s="93"/>
-      <c r="AH23" s="94"/>
+      <c r="AF23" s="80"/>
+      <c r="AG23" s="81"/>
+      <c r="AH23" s="82"/>
     </row>
     <row r="24" spans="1:34" s="1" customFormat="1" ht="20.100000000000001" customHeight="1">
       <c r="A24" s="53"/>
-      <c r="B24" s="256" t="s">
+      <c r="B24" s="254" t="s">
         <v>44</v>
       </c>
-      <c r="C24" s="256"/>
-      <c r="D24" s="256"/>
-      <c r="E24" s="256"/>
-      <c r="F24" s="256"/>
-      <c r="G24" s="256"/>
-      <c r="H24" s="256"/>
-      <c r="I24" s="257"/>
+      <c r="C24" s="254"/>
+      <c r="D24" s="254"/>
+      <c r="E24" s="254"/>
+      <c r="F24" s="254"/>
+      <c r="G24" s="254"/>
+      <c r="H24" s="254"/>
+      <c r="I24" s="255"/>
       <c r="J24" s="54"/>
       <c r="K24" s="54"/>
       <c r="L24" s="54"/>
@@ -3957,17 +3957,17 @@
       <c r="N24" s="54" t="s">
         <v>40</v>
       </c>
-      <c r="O24" s="119"/>
-      <c r="P24" s="120"/>
-      <c r="Q24" s="121"/>
-      <c r="R24" s="140"/>
-      <c r="S24" s="141"/>
-      <c r="T24" s="141"/>
-      <c r="U24" s="141"/>
-      <c r="V24" s="142"/>
-      <c r="W24" s="161"/>
-      <c r="X24" s="162"/>
-      <c r="Y24" s="163"/>
+      <c r="O24" s="113"/>
+      <c r="P24" s="114"/>
+      <c r="Q24" s="115"/>
+      <c r="R24" s="134"/>
+      <c r="S24" s="135"/>
+      <c r="T24" s="135"/>
+      <c r="U24" s="135"/>
+      <c r="V24" s="136"/>
+      <c r="W24" s="155"/>
+      <c r="X24" s="156"/>
+      <c r="Y24" s="157"/>
       <c r="AB24" s="31" t="s">
         <v>80</v>
       </c>
@@ -3980,22 +3980,22 @@
       <c r="AE24" s="39" t="s">
         <v>56</v>
       </c>
-      <c r="AF24" s="92"/>
-      <c r="AG24" s="93"/>
-      <c r="AH24" s="94"/>
+      <c r="AF24" s="80"/>
+      <c r="AG24" s="81"/>
+      <c r="AH24" s="82"/>
     </row>
     <row r="25" spans="1:34" s="1" customFormat="1" ht="20.100000000000001" customHeight="1" thickBot="1">
       <c r="A25" s="53"/>
-      <c r="B25" s="256" t="s">
+      <c r="B25" s="254" t="s">
         <v>3</v>
       </c>
-      <c r="C25" s="256"/>
-      <c r="D25" s="256"/>
-      <c r="E25" s="256"/>
-      <c r="F25" s="256"/>
-      <c r="G25" s="256"/>
-      <c r="H25" s="256"/>
-      <c r="I25" s="257"/>
+      <c r="C25" s="254"/>
+      <c r="D25" s="254"/>
+      <c r="E25" s="254"/>
+      <c r="F25" s="254"/>
+      <c r="G25" s="254"/>
+      <c r="H25" s="254"/>
+      <c r="I25" s="255"/>
       <c r="J25" s="54"/>
       <c r="K25" s="54"/>
       <c r="L25" s="54" t="s">
@@ -4005,17 +4005,17 @@
       <c r="N25" s="54" t="s">
         <v>40</v>
       </c>
-      <c r="O25" s="122"/>
-      <c r="P25" s="123"/>
-      <c r="Q25" s="124"/>
-      <c r="R25" s="143"/>
-      <c r="S25" s="144"/>
-      <c r="T25" s="144"/>
-      <c r="U25" s="144"/>
-      <c r="V25" s="145"/>
-      <c r="W25" s="164"/>
-      <c r="X25" s="165"/>
-      <c r="Y25" s="166"/>
+      <c r="O25" s="116"/>
+      <c r="P25" s="117"/>
+      <c r="Q25" s="118"/>
+      <c r="R25" s="137"/>
+      <c r="S25" s="138"/>
+      <c r="T25" s="138"/>
+      <c r="U25" s="138"/>
+      <c r="V25" s="139"/>
+      <c r="W25" s="158"/>
+      <c r="X25" s="159"/>
+      <c r="Y25" s="160"/>
       <c r="AB25" s="50" t="s">
         <v>80</v>
       </c>
@@ -4028,44 +4028,44 @@
       <c r="AE25" s="52" t="s">
         <v>58</v>
       </c>
-      <c r="AF25" s="95"/>
-      <c r="AG25" s="96"/>
-      <c r="AH25" s="97"/>
+      <c r="AF25" s="83"/>
+      <c r="AG25" s="84"/>
+      <c r="AH25" s="85"/>
     </row>
     <row r="26" spans="1:34" s="1" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A26" s="77" t="s">
+      <c r="A26" s="95" t="s">
         <v>46</v>
       </c>
-      <c r="B26" s="78"/>
-      <c r="C26" s="78"/>
-      <c r="D26" s="78"/>
-      <c r="E26" s="78"/>
-      <c r="F26" s="78"/>
-      <c r="G26" s="78"/>
-      <c r="H26" s="78"/>
-      <c r="I26" s="79"/>
+      <c r="B26" s="96"/>
+      <c r="C26" s="96"/>
+      <c r="D26" s="96"/>
+      <c r="E26" s="96"/>
+      <c r="F26" s="96"/>
+      <c r="G26" s="96"/>
+      <c r="H26" s="96"/>
+      <c r="I26" s="97"/>
       <c r="J26" s="55"/>
       <c r="K26" s="56"/>
       <c r="L26" s="56"/>
       <c r="M26" s="56"/>
       <c r="N26" s="57"/>
-      <c r="O26" s="116" t="s">
+      <c r="O26" s="110" t="s">
         <v>11</v>
       </c>
-      <c r="P26" s="117"/>
-      <c r="Q26" s="118"/>
-      <c r="R26" s="137">
+      <c r="P26" s="111"/>
+      <c r="Q26" s="112"/>
+      <c r="R26" s="131">
         <v>200000</v>
       </c>
-      <c r="S26" s="138"/>
-      <c r="T26" s="138"/>
-      <c r="U26" s="138"/>
-      <c r="V26" s="139"/>
-      <c r="W26" s="89" t="s">
+      <c r="S26" s="132"/>
+      <c r="T26" s="132"/>
+      <c r="U26" s="132"/>
+      <c r="V26" s="133"/>
+      <c r="W26" s="77" t="s">
         <v>75</v>
       </c>
-      <c r="X26" s="90"/>
-      <c r="Y26" s="91"/>
+      <c r="X26" s="78"/>
+      <c r="Y26" s="79"/>
       <c r="AB26" s="19" t="s">
         <v>85</v>
       </c>
@@ -4081,16 +4081,16 @@
     </row>
     <row r="27" spans="1:34" s="1" customFormat="1" ht="20.100000000000001" customHeight="1">
       <c r="A27" s="53"/>
-      <c r="B27" s="256" t="s">
+      <c r="B27" s="254" t="s">
         <v>76</v>
       </c>
-      <c r="C27" s="256"/>
-      <c r="D27" s="256"/>
-      <c r="E27" s="256"/>
-      <c r="F27" s="256"/>
-      <c r="G27" s="256"/>
-      <c r="H27" s="256"/>
-      <c r="I27" s="257"/>
+      <c r="C27" s="254"/>
+      <c r="D27" s="254"/>
+      <c r="E27" s="254"/>
+      <c r="F27" s="254"/>
+      <c r="G27" s="254"/>
+      <c r="H27" s="254"/>
+      <c r="I27" s="255"/>
       <c r="J27" s="54"/>
       <c r="K27" s="54"/>
       <c r="L27" s="54"/>
@@ -4098,17 +4098,17 @@
       <c r="N27" s="54" t="s">
         <v>40</v>
       </c>
-      <c r="O27" s="119"/>
-      <c r="P27" s="120"/>
-      <c r="Q27" s="121"/>
-      <c r="R27" s="140"/>
-      <c r="S27" s="141"/>
-      <c r="T27" s="141"/>
-      <c r="U27" s="141"/>
-      <c r="V27" s="142"/>
-      <c r="W27" s="92"/>
-      <c r="X27" s="93"/>
-      <c r="Y27" s="94"/>
+      <c r="O27" s="113"/>
+      <c r="P27" s="114"/>
+      <c r="Q27" s="115"/>
+      <c r="R27" s="134"/>
+      <c r="S27" s="135"/>
+      <c r="T27" s="135"/>
+      <c r="U27" s="135"/>
+      <c r="V27" s="136"/>
+      <c r="W27" s="80"/>
+      <c r="X27" s="81"/>
+      <c r="Y27" s="82"/>
       <c r="AB27" s="31" t="s">
         <v>85</v>
       </c>
@@ -4124,16 +4124,16 @@
     </row>
     <row r="28" spans="1:34" s="1" customFormat="1" ht="20.100000000000001" customHeight="1">
       <c r="A28" s="53"/>
-      <c r="B28" s="256" t="s">
+      <c r="B28" s="254" t="s">
         <v>3</v>
       </c>
-      <c r="C28" s="256"/>
-      <c r="D28" s="256"/>
-      <c r="E28" s="256"/>
-      <c r="F28" s="256"/>
-      <c r="G28" s="256"/>
-      <c r="H28" s="256"/>
-      <c r="I28" s="257"/>
+      <c r="C28" s="254"/>
+      <c r="D28" s="254"/>
+      <c r="E28" s="254"/>
+      <c r="F28" s="254"/>
+      <c r="G28" s="254"/>
+      <c r="H28" s="254"/>
+      <c r="I28" s="255"/>
       <c r="J28" s="54"/>
       <c r="K28" s="54"/>
       <c r="L28" s="54"/>
@@ -4141,17 +4141,17 @@
       <c r="N28" s="54" t="s">
         <v>40</v>
       </c>
-      <c r="O28" s="119"/>
-      <c r="P28" s="120"/>
-      <c r="Q28" s="121"/>
-      <c r="R28" s="140"/>
-      <c r="S28" s="141"/>
-      <c r="T28" s="141"/>
-      <c r="U28" s="141"/>
-      <c r="V28" s="142"/>
-      <c r="W28" s="92"/>
-      <c r="X28" s="93"/>
-      <c r="Y28" s="94"/>
+      <c r="O28" s="113"/>
+      <c r="P28" s="114"/>
+      <c r="Q28" s="115"/>
+      <c r="R28" s="134"/>
+      <c r="S28" s="135"/>
+      <c r="T28" s="135"/>
+      <c r="U28" s="135"/>
+      <c r="V28" s="136"/>
+      <c r="W28" s="80"/>
+      <c r="X28" s="81"/>
+      <c r="Y28" s="82"/>
       <c r="AB28" s="31" t="s">
         <v>85</v>
       </c>
@@ -4166,35 +4166,35 @@
       </c>
     </row>
     <row r="29" spans="1:34" s="1" customFormat="1" ht="20.100000000000001" customHeight="1" thickBot="1">
-      <c r="A29" s="77" t="s">
+      <c r="A29" s="95" t="s">
         <v>47</v>
       </c>
-      <c r="B29" s="78"/>
-      <c r="C29" s="78"/>
-      <c r="D29" s="78"/>
-      <c r="E29" s="78"/>
-      <c r="F29" s="78"/>
-      <c r="G29" s="78"/>
-      <c r="H29" s="78"/>
-      <c r="I29" s="79"/>
+      <c r="B29" s="96"/>
+      <c r="C29" s="96"/>
+      <c r="D29" s="96"/>
+      <c r="E29" s="96"/>
+      <c r="F29" s="96"/>
+      <c r="G29" s="96"/>
+      <c r="H29" s="96"/>
+      <c r="I29" s="97"/>
       <c r="J29" s="55"/>
       <c r="K29" s="56"/>
       <c r="L29" s="56"/>
       <c r="M29" s="56"/>
       <c r="N29" s="57"/>
-      <c r="O29" s="116" t="s">
+      <c r="O29" s="110" t="s">
         <v>12</v>
       </c>
-      <c r="P29" s="117"/>
-      <c r="Q29" s="118"/>
-      <c r="R29" s="140"/>
-      <c r="S29" s="141"/>
-      <c r="T29" s="141"/>
-      <c r="U29" s="141"/>
-      <c r="V29" s="142"/>
-      <c r="W29" s="92"/>
-      <c r="X29" s="93"/>
-      <c r="Y29" s="94"/>
+      <c r="P29" s="111"/>
+      <c r="Q29" s="112"/>
+      <c r="R29" s="134"/>
+      <c r="S29" s="135"/>
+      <c r="T29" s="135"/>
+      <c r="U29" s="135"/>
+      <c r="V29" s="136"/>
+      <c r="W29" s="80"/>
+      <c r="X29" s="81"/>
+      <c r="Y29" s="82"/>
       <c r="AB29" s="50" t="s">
         <v>85</v>
       </c>
@@ -4210,16 +4210,16 @@
     </row>
     <row r="30" spans="1:34" s="1" customFormat="1" ht="20.100000000000001" customHeight="1">
       <c r="A30" s="58"/>
-      <c r="B30" s="256" t="s">
+      <c r="B30" s="254" t="s">
         <v>76</v>
       </c>
-      <c r="C30" s="256"/>
-      <c r="D30" s="256"/>
-      <c r="E30" s="256"/>
-      <c r="F30" s="256"/>
-      <c r="G30" s="256"/>
-      <c r="H30" s="256"/>
-      <c r="I30" s="257"/>
+      <c r="C30" s="254"/>
+      <c r="D30" s="254"/>
+      <c r="E30" s="254"/>
+      <c r="F30" s="254"/>
+      <c r="G30" s="254"/>
+      <c r="H30" s="254"/>
+      <c r="I30" s="255"/>
       <c r="J30" s="59"/>
       <c r="K30" s="59"/>
       <c r="L30" s="59"/>
@@ -4227,17 +4227,17 @@
       <c r="N30" s="54" t="s">
         <v>40</v>
       </c>
-      <c r="O30" s="119"/>
-      <c r="P30" s="120"/>
-      <c r="Q30" s="121"/>
-      <c r="R30" s="140"/>
-      <c r="S30" s="141"/>
-      <c r="T30" s="141"/>
-      <c r="U30" s="141"/>
-      <c r="V30" s="142"/>
-      <c r="W30" s="92"/>
-      <c r="X30" s="93"/>
-      <c r="Y30" s="94"/>
+      <c r="O30" s="113"/>
+      <c r="P30" s="114"/>
+      <c r="Q30" s="115"/>
+      <c r="R30" s="134"/>
+      <c r="S30" s="135"/>
+      <c r="T30" s="135"/>
+      <c r="U30" s="135"/>
+      <c r="V30" s="136"/>
+      <c r="W30" s="80"/>
+      <c r="X30" s="81"/>
+      <c r="Y30" s="82"/>
       <c r="AB30" s="2" t="s">
         <v>91</v>
       </c>
@@ -4246,35 +4246,35 @@
       <c r="AE30" s="2"/>
     </row>
     <row r="31" spans="1:34" s="1" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A31" s="77" t="s">
+      <c r="A31" s="95" t="s">
         <v>48</v>
       </c>
-      <c r="B31" s="78"/>
-      <c r="C31" s="78"/>
-      <c r="D31" s="78"/>
-      <c r="E31" s="78"/>
-      <c r="F31" s="78"/>
-      <c r="G31" s="78"/>
-      <c r="H31" s="78"/>
-      <c r="I31" s="79"/>
+      <c r="B31" s="96"/>
+      <c r="C31" s="96"/>
+      <c r="D31" s="96"/>
+      <c r="E31" s="96"/>
+      <c r="F31" s="96"/>
+      <c r="G31" s="96"/>
+      <c r="H31" s="96"/>
+      <c r="I31" s="97"/>
       <c r="J31" s="55"/>
       <c r="K31" s="56"/>
       <c r="L31" s="56"/>
       <c r="M31" s="56"/>
       <c r="N31" s="57"/>
-      <c r="O31" s="101" t="s">
+      <c r="O31" s="89" t="s">
         <v>13</v>
       </c>
-      <c r="P31" s="102"/>
-      <c r="Q31" s="103"/>
-      <c r="R31" s="143"/>
-      <c r="S31" s="144"/>
-      <c r="T31" s="144"/>
-      <c r="U31" s="144"/>
-      <c r="V31" s="145"/>
-      <c r="W31" s="95"/>
-      <c r="X31" s="96"/>
-      <c r="Y31" s="97"/>
+      <c r="P31" s="90"/>
+      <c r="Q31" s="91"/>
+      <c r="R31" s="137"/>
+      <c r="S31" s="138"/>
+      <c r="T31" s="138"/>
+      <c r="U31" s="138"/>
+      <c r="V31" s="139"/>
+      <c r="W31" s="83"/>
+      <c r="X31" s="84"/>
+      <c r="Y31" s="85"/>
       <c r="AB31" s="2" t="s">
         <v>92</v>
       </c>
@@ -4285,19 +4285,19 @@
       <c r="AE31" s="2"/>
     </row>
     <row r="32" spans="1:34" s="1" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A32" s="214" t="s">
+      <c r="A32" s="212" t="s">
         <v>49</v>
       </c>
-      <c r="B32" s="215"/>
-      <c r="C32" s="216"/>
-      <c r="D32" s="258" t="s">
+      <c r="B32" s="213"/>
+      <c r="C32" s="214"/>
+      <c r="D32" s="86" t="s">
         <v>4</v>
       </c>
-      <c r="E32" s="259"/>
-      <c r="F32" s="259"/>
-      <c r="G32" s="259"/>
-      <c r="H32" s="259"/>
-      <c r="I32" s="260"/>
+      <c r="E32" s="87"/>
+      <c r="F32" s="87"/>
+      <c r="G32" s="87"/>
+      <c r="H32" s="87"/>
+      <c r="I32" s="88"/>
       <c r="J32" s="60"/>
       <c r="K32" s="54"/>
       <c r="L32" s="54"/>
@@ -4305,38 +4305,38 @@
       <c r="N32" s="54" t="s">
         <v>40</v>
       </c>
-      <c r="O32" s="116" t="s">
+      <c r="O32" s="110" t="s">
         <v>19</v>
       </c>
-      <c r="P32" s="117"/>
-      <c r="Q32" s="118"/>
-      <c r="R32" s="146">
+      <c r="P32" s="111"/>
+      <c r="Q32" s="112"/>
+      <c r="R32" s="140">
         <v>200000</v>
       </c>
-      <c r="S32" s="147"/>
-      <c r="T32" s="147"/>
-      <c r="U32" s="147"/>
-      <c r="V32" s="148"/>
-      <c r="W32" s="155"/>
-      <c r="X32" s="90"/>
-      <c r="Y32" s="91"/>
+      <c r="S32" s="141"/>
+      <c r="T32" s="141"/>
+      <c r="U32" s="141"/>
+      <c r="V32" s="142"/>
+      <c r="W32" s="149"/>
+      <c r="X32" s="78"/>
+      <c r="Y32" s="79"/>
       <c r="AB32" s="2"/>
       <c r="AC32" s="2"/>
       <c r="AD32" s="2"/>
       <c r="AE32" s="2"/>
     </row>
     <row r="33" spans="1:31" s="1" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A33" s="217"/>
-      <c r="B33" s="218"/>
-      <c r="C33" s="219"/>
-      <c r="D33" s="258" t="s">
+      <c r="A33" s="215"/>
+      <c r="B33" s="216"/>
+      <c r="C33" s="217"/>
+      <c r="D33" s="86" t="s">
         <v>5</v>
       </c>
-      <c r="E33" s="259"/>
-      <c r="F33" s="259"/>
-      <c r="G33" s="259"/>
-      <c r="H33" s="259"/>
-      <c r="I33" s="260"/>
+      <c r="E33" s="87"/>
+      <c r="F33" s="87"/>
+      <c r="G33" s="87"/>
+      <c r="H33" s="87"/>
+      <c r="I33" s="88"/>
       <c r="J33" s="60"/>
       <c r="K33" s="54"/>
       <c r="L33" s="54"/>
@@ -4344,34 +4344,34 @@
       <c r="N33" s="54" t="s">
         <v>40</v>
       </c>
-      <c r="O33" s="119"/>
-      <c r="P33" s="120"/>
-      <c r="Q33" s="121"/>
-      <c r="R33" s="149"/>
-      <c r="S33" s="150"/>
-      <c r="T33" s="150"/>
-      <c r="U33" s="150"/>
-      <c r="V33" s="151"/>
-      <c r="W33" s="92"/>
-      <c r="X33" s="93"/>
-      <c r="Y33" s="94"/>
+      <c r="O33" s="113"/>
+      <c r="P33" s="114"/>
+      <c r="Q33" s="115"/>
+      <c r="R33" s="143"/>
+      <c r="S33" s="144"/>
+      <c r="T33" s="144"/>
+      <c r="U33" s="144"/>
+      <c r="V33" s="145"/>
+      <c r="W33" s="80"/>
+      <c r="X33" s="81"/>
+      <c r="Y33" s="82"/>
       <c r="AB33" s="2"/>
       <c r="AC33" s="2"/>
       <c r="AD33" s="2"/>
       <c r="AE33" s="2"/>
     </row>
     <row r="34" spans="1:31" s="1" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A34" s="220"/>
-      <c r="B34" s="221"/>
-      <c r="C34" s="222"/>
-      <c r="D34" s="258" t="s">
+      <c r="A34" s="218"/>
+      <c r="B34" s="219"/>
+      <c r="C34" s="220"/>
+      <c r="D34" s="86" t="s">
         <v>6</v>
       </c>
-      <c r="E34" s="259"/>
-      <c r="F34" s="259"/>
-      <c r="G34" s="259"/>
-      <c r="H34" s="259"/>
-      <c r="I34" s="260"/>
+      <c r="E34" s="87"/>
+      <c r="F34" s="87"/>
+      <c r="G34" s="87"/>
+      <c r="H34" s="87"/>
+      <c r="I34" s="88"/>
       <c r="J34" s="60"/>
       <c r="K34" s="54" t="s">
         <v>40</v>
@@ -4385,34 +4385,34 @@
       <c r="N34" s="54" t="s">
         <v>40</v>
       </c>
-      <c r="O34" s="122"/>
-      <c r="P34" s="123"/>
-      <c r="Q34" s="124"/>
-      <c r="R34" s="152"/>
-      <c r="S34" s="153"/>
-      <c r="T34" s="153"/>
-      <c r="U34" s="153"/>
-      <c r="V34" s="154"/>
-      <c r="W34" s="95"/>
-      <c r="X34" s="96"/>
-      <c r="Y34" s="97"/>
+      <c r="O34" s="116"/>
+      <c r="P34" s="117"/>
+      <c r="Q34" s="118"/>
+      <c r="R34" s="146"/>
+      <c r="S34" s="147"/>
+      <c r="T34" s="147"/>
+      <c r="U34" s="147"/>
+      <c r="V34" s="148"/>
+      <c r="W34" s="83"/>
+      <c r="X34" s="84"/>
+      <c r="Y34" s="85"/>
       <c r="AB34" s="2"/>
       <c r="AC34" s="2"/>
       <c r="AD34" s="2"/>
       <c r="AE34" s="2"/>
     </row>
     <row r="35" spans="1:31" s="1" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A35" s="77" t="s">
+      <c r="A35" s="95" t="s">
         <v>50</v>
       </c>
-      <c r="B35" s="78"/>
-      <c r="C35" s="78"/>
-      <c r="D35" s="78"/>
-      <c r="E35" s="78"/>
-      <c r="F35" s="78"/>
-      <c r="G35" s="78"/>
-      <c r="H35" s="78"/>
-      <c r="I35" s="79"/>
+      <c r="B35" s="96"/>
+      <c r="C35" s="96"/>
+      <c r="D35" s="96"/>
+      <c r="E35" s="96"/>
+      <c r="F35" s="96"/>
+      <c r="G35" s="96"/>
+      <c r="H35" s="96"/>
+      <c r="I35" s="97"/>
       <c r="J35" s="54"/>
       <c r="K35" s="54" t="s">
         <v>40</v>
@@ -4426,38 +4426,38 @@
       <c r="N35" s="54" t="s">
         <v>40</v>
       </c>
-      <c r="O35" s="101" t="s">
+      <c r="O35" s="89" t="s">
         <v>41</v>
       </c>
-      <c r="P35" s="102"/>
-      <c r="Q35" s="103"/>
-      <c r="R35" s="107">
+      <c r="P35" s="90"/>
+      <c r="Q35" s="91"/>
+      <c r="R35" s="98">
         <v>600000</v>
       </c>
-      <c r="S35" s="108"/>
-      <c r="T35" s="108"/>
-      <c r="U35" s="108"/>
-      <c r="V35" s="109"/>
-      <c r="W35" s="104"/>
-      <c r="X35" s="105"/>
-      <c r="Y35" s="106"/>
+      <c r="S35" s="99"/>
+      <c r="T35" s="99"/>
+      <c r="U35" s="99"/>
+      <c r="V35" s="100"/>
+      <c r="W35" s="92"/>
+      <c r="X35" s="93"/>
+      <c r="Y35" s="94"/>
       <c r="AB35" s="2"/>
       <c r="AC35" s="2"/>
       <c r="AD35" s="2"/>
       <c r="AE35" s="2"/>
     </row>
     <row r="36" spans="1:31" s="1" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A36" s="77" t="s">
+      <c r="A36" s="95" t="s">
         <v>51</v>
       </c>
-      <c r="B36" s="78"/>
-      <c r="C36" s="78"/>
-      <c r="D36" s="78"/>
-      <c r="E36" s="78"/>
-      <c r="F36" s="78"/>
-      <c r="G36" s="78"/>
-      <c r="H36" s="78"/>
-      <c r="I36" s="79"/>
+      <c r="B36" s="96"/>
+      <c r="C36" s="96"/>
+      <c r="D36" s="96"/>
+      <c r="E36" s="96"/>
+      <c r="F36" s="96"/>
+      <c r="G36" s="96"/>
+      <c r="H36" s="96"/>
+      <c r="I36" s="97"/>
       <c r="J36" s="54"/>
       <c r="K36" s="54"/>
       <c r="L36" s="54"/>
@@ -4465,38 +4465,38 @@
       <c r="N36" s="54" t="s">
         <v>40</v>
       </c>
-      <c r="O36" s="101" t="s">
+      <c r="O36" s="89" t="s">
         <v>14</v>
       </c>
-      <c r="P36" s="102"/>
-      <c r="Q36" s="103"/>
-      <c r="R36" s="107">
+      <c r="P36" s="90"/>
+      <c r="Q36" s="91"/>
+      <c r="R36" s="98">
         <v>300000</v>
       </c>
-      <c r="S36" s="108"/>
-      <c r="T36" s="108"/>
-      <c r="U36" s="108"/>
-      <c r="V36" s="109"/>
-      <c r="W36" s="104"/>
-      <c r="X36" s="105"/>
-      <c r="Y36" s="106"/>
+      <c r="S36" s="99"/>
+      <c r="T36" s="99"/>
+      <c r="U36" s="99"/>
+      <c r="V36" s="100"/>
+      <c r="W36" s="92"/>
+      <c r="X36" s="93"/>
+      <c r="Y36" s="94"/>
       <c r="AB36" s="2"/>
       <c r="AC36" s="2"/>
       <c r="AD36" s="2"/>
       <c r="AE36" s="2"/>
     </row>
     <row r="37" spans="1:31" s="1" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A37" s="181" t="s">
+      <c r="A37" s="164" t="s">
         <v>52</v>
       </c>
-      <c r="B37" s="182"/>
-      <c r="C37" s="182"/>
-      <c r="D37" s="182"/>
-      <c r="E37" s="182"/>
-      <c r="F37" s="182"/>
-      <c r="G37" s="182"/>
-      <c r="H37" s="182"/>
-      <c r="I37" s="183"/>
+      <c r="B37" s="165"/>
+      <c r="C37" s="165"/>
+      <c r="D37" s="165"/>
+      <c r="E37" s="165"/>
+      <c r="F37" s="165"/>
+      <c r="G37" s="165"/>
+      <c r="H37" s="165"/>
+      <c r="I37" s="166"/>
       <c r="J37" s="60"/>
       <c r="K37" s="54" t="s">
         <v>40</v>
@@ -4510,38 +4510,38 @@
       <c r="N37" s="54" t="s">
         <v>40</v>
       </c>
-      <c r="O37" s="113"/>
-      <c r="P37" s="114"/>
-      <c r="Q37" s="115"/>
-      <c r="R37" s="107">
+      <c r="O37" s="107"/>
+      <c r="P37" s="108"/>
+      <c r="Q37" s="109"/>
+      <c r="R37" s="98">
         <v>100000</v>
       </c>
-      <c r="S37" s="108"/>
-      <c r="T37" s="108"/>
-      <c r="U37" s="108"/>
-      <c r="V37" s="109"/>
-      <c r="W37" s="104"/>
-      <c r="X37" s="105"/>
-      <c r="Y37" s="106"/>
+      <c r="S37" s="99"/>
+      <c r="T37" s="99"/>
+      <c r="U37" s="99"/>
+      <c r="V37" s="100"/>
+      <c r="W37" s="92"/>
+      <c r="X37" s="93"/>
+      <c r="Y37" s="94"/>
       <c r="AB37" s="2"/>
       <c r="AC37" s="2"/>
       <c r="AD37" s="2"/>
       <c r="AE37" s="2"/>
     </row>
     <row r="38" spans="1:31" s="1" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A38" s="184" t="s">
+      <c r="A38" s="167" t="s">
         <v>63</v>
       </c>
-      <c r="B38" s="185"/>
-      <c r="C38" s="186"/>
-      <c r="D38" s="258" t="s">
+      <c r="B38" s="168"/>
+      <c r="C38" s="169"/>
+      <c r="D38" s="86" t="s">
         <v>72</v>
       </c>
-      <c r="E38" s="259"/>
-      <c r="F38" s="259"/>
-      <c r="G38" s="259"/>
-      <c r="H38" s="259"/>
-      <c r="I38" s="260"/>
+      <c r="E38" s="87"/>
+      <c r="F38" s="87"/>
+      <c r="G38" s="87"/>
+      <c r="H38" s="87"/>
+      <c r="I38" s="88"/>
       <c r="J38" s="60"/>
       <c r="K38" s="54"/>
       <c r="L38" s="54"/>
@@ -4549,69 +4549,69 @@
       <c r="N38" s="54" t="s">
         <v>40</v>
       </c>
-      <c r="O38" s="116" t="s">
+      <c r="O38" s="110" t="s">
         <v>15</v>
       </c>
-      <c r="P38" s="117"/>
-      <c r="Q38" s="118"/>
-      <c r="R38" s="173"/>
-      <c r="S38" s="173"/>
-      <c r="T38" s="173"/>
-      <c r="U38" s="173"/>
-      <c r="V38" s="173"/>
-      <c r="W38" s="80"/>
-      <c r="X38" s="81"/>
-      <c r="Y38" s="82"/>
+      <c r="P38" s="111"/>
+      <c r="Q38" s="112"/>
+      <c r="R38" s="176"/>
+      <c r="S38" s="176"/>
+      <c r="T38" s="176"/>
+      <c r="U38" s="176"/>
+      <c r="V38" s="176"/>
+      <c r="W38" s="179"/>
+      <c r="X38" s="180"/>
+      <c r="Y38" s="181"/>
       <c r="AB38" s="2"/>
       <c r="AC38" s="2"/>
       <c r="AD38" s="2"/>
       <c r="AE38" s="2"/>
     </row>
     <row r="39" spans="1:31" s="1" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A39" s="187"/>
-      <c r="B39" s="188"/>
-      <c r="C39" s="189"/>
-      <c r="D39" s="258" t="s">
+      <c r="A39" s="170"/>
+      <c r="B39" s="171"/>
+      <c r="C39" s="172"/>
+      <c r="D39" s="86" t="s">
         <v>73</v>
       </c>
-      <c r="E39" s="259"/>
-      <c r="F39" s="259"/>
-      <c r="G39" s="259"/>
-      <c r="H39" s="259"/>
-      <c r="I39" s="260"/>
+      <c r="E39" s="87"/>
+      <c r="F39" s="87"/>
+      <c r="G39" s="87"/>
+      <c r="H39" s="87"/>
+      <c r="I39" s="88"/>
       <c r="J39" s="60"/>
       <c r="K39" s="54"/>
       <c r="L39" s="54"/>
       <c r="M39" s="54"/>
       <c r="N39" s="54"/>
-      <c r="O39" s="119"/>
-      <c r="P39" s="120"/>
-      <c r="Q39" s="121"/>
-      <c r="R39" s="174"/>
-      <c r="S39" s="174"/>
-      <c r="T39" s="174"/>
-      <c r="U39" s="174"/>
-      <c r="V39" s="174"/>
-      <c r="W39" s="83"/>
-      <c r="X39" s="84"/>
-      <c r="Y39" s="85"/>
+      <c r="O39" s="113"/>
+      <c r="P39" s="114"/>
+      <c r="Q39" s="115"/>
+      <c r="R39" s="177"/>
+      <c r="S39" s="177"/>
+      <c r="T39" s="177"/>
+      <c r="U39" s="177"/>
+      <c r="V39" s="177"/>
+      <c r="W39" s="182"/>
+      <c r="X39" s="183"/>
+      <c r="Y39" s="184"/>
       <c r="AB39" s="2"/>
       <c r="AC39" s="2"/>
       <c r="AD39" s="2"/>
       <c r="AE39" s="2"/>
     </row>
     <row r="40" spans="1:31" s="1" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A40" s="190"/>
-      <c r="B40" s="191"/>
-      <c r="C40" s="192"/>
-      <c r="D40" s="258" t="s">
+      <c r="A40" s="173"/>
+      <c r="B40" s="174"/>
+      <c r="C40" s="175"/>
+      <c r="D40" s="86" t="s">
         <v>3</v>
       </c>
-      <c r="E40" s="259"/>
-      <c r="F40" s="259"/>
-      <c r="G40" s="259"/>
-      <c r="H40" s="259"/>
-      <c r="I40" s="260"/>
+      <c r="E40" s="87"/>
+      <c r="F40" s="87"/>
+      <c r="G40" s="87"/>
+      <c r="H40" s="87"/>
+      <c r="I40" s="88"/>
       <c r="J40" s="60"/>
       <c r="K40" s="54"/>
       <c r="L40" s="54"/>
@@ -4619,75 +4619,75 @@
       <c r="N40" s="54" t="s">
         <v>40</v>
       </c>
-      <c r="O40" s="122"/>
-      <c r="P40" s="123"/>
-      <c r="Q40" s="124"/>
-      <c r="R40" s="175"/>
-      <c r="S40" s="175"/>
-      <c r="T40" s="175"/>
-      <c r="U40" s="175"/>
-      <c r="V40" s="175"/>
-      <c r="W40" s="86"/>
-      <c r="X40" s="87"/>
-      <c r="Y40" s="88"/>
+      <c r="O40" s="116"/>
+      <c r="P40" s="117"/>
+      <c r="Q40" s="118"/>
+      <c r="R40" s="178"/>
+      <c r="S40" s="178"/>
+      <c r="T40" s="178"/>
+      <c r="U40" s="178"/>
+      <c r="V40" s="178"/>
+      <c r="W40" s="185"/>
+      <c r="X40" s="186"/>
+      <c r="Y40" s="187"/>
       <c r="AB40" s="2"/>
       <c r="AC40" s="2"/>
       <c r="AD40" s="2"/>
       <c r="AE40" s="2"/>
     </row>
     <row r="41" spans="1:31" s="1" customFormat="1" ht="30" customHeight="1">
-      <c r="A41" s="176" t="s">
+      <c r="A41" s="259" t="s">
         <v>39</v>
       </c>
-      <c r="B41" s="177"/>
-      <c r="C41" s="177"/>
-      <c r="D41" s="177"/>
-      <c r="E41" s="177"/>
-      <c r="F41" s="177"/>
-      <c r="G41" s="177"/>
-      <c r="H41" s="177"/>
-      <c r="I41" s="177"/>
-      <c r="J41" s="177"/>
-      <c r="K41" s="177"/>
-      <c r="L41" s="177"/>
-      <c r="M41" s="177"/>
-      <c r="N41" s="178" t="s">
+      <c r="B41" s="260"/>
+      <c r="C41" s="260"/>
+      <c r="D41" s="260"/>
+      <c r="E41" s="260"/>
+      <c r="F41" s="260"/>
+      <c r="G41" s="260"/>
+      <c r="H41" s="260"/>
+      <c r="I41" s="260"/>
+      <c r="J41" s="260"/>
+      <c r="K41" s="260"/>
+      <c r="L41" s="260"/>
+      <c r="M41" s="260"/>
+      <c r="N41" s="161" t="s">
         <v>53</v>
       </c>
-      <c r="O41" s="179"/>
-      <c r="P41" s="179"/>
-      <c r="Q41" s="179"/>
-      <c r="R41" s="179"/>
-      <c r="S41" s="179"/>
-      <c r="T41" s="180"/>
-      <c r="U41" s="213">
+      <c r="O41" s="162"/>
+      <c r="P41" s="162"/>
+      <c r="Q41" s="162"/>
+      <c r="R41" s="162"/>
+      <c r="S41" s="162"/>
+      <c r="T41" s="163"/>
+      <c r="U41" s="211">
         <f>SUM(R22:V40)</f>
         <v>1600000</v>
       </c>
-      <c r="V41" s="179"/>
-      <c r="W41" s="179"/>
-      <c r="X41" s="179"/>
-      <c r="Y41" s="180"/>
+      <c r="V41" s="162"/>
+      <c r="W41" s="162"/>
+      <c r="X41" s="162"/>
+      <c r="Y41" s="163"/>
       <c r="AB41" s="2"/>
       <c r="AC41" s="2"/>
       <c r="AD41" s="2"/>
       <c r="AE41" s="2"/>
     </row>
     <row r="42" spans="1:31" s="13" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A42" s="167" t="s">
+      <c r="A42" s="256" t="s">
         <v>34</v>
       </c>
-      <c r="B42" s="168"/>
-      <c r="C42" s="168"/>
-      <c r="D42" s="168"/>
-      <c r="E42" s="168"/>
-      <c r="F42" s="168"/>
-      <c r="G42" s="168"/>
-      <c r="H42" s="168"/>
-      <c r="I42" s="168"/>
-      <c r="J42" s="168"/>
-      <c r="K42" s="168"/>
-      <c r="L42" s="169"/>
+      <c r="B42" s="257"/>
+      <c r="C42" s="257"/>
+      <c r="D42" s="257"/>
+      <c r="E42" s="257"/>
+      <c r="F42" s="257"/>
+      <c r="G42" s="257"/>
+      <c r="H42" s="257"/>
+      <c r="I42" s="257"/>
+      <c r="J42" s="257"/>
+      <c r="K42" s="257"/>
+      <c r="L42" s="258"/>
       <c r="M42" s="61" t="s">
         <v>35</v>
       </c>
@@ -4709,20 +4709,20 @@
       <c r="AE42" s="64"/>
     </row>
     <row r="43" spans="1:31" s="13" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A43" s="170" t="s">
+      <c r="A43" s="208" t="s">
         <v>36</v>
       </c>
-      <c r="B43" s="171"/>
-      <c r="C43" s="171"/>
-      <c r="D43" s="171"/>
-      <c r="E43" s="171"/>
-      <c r="F43" s="171"/>
-      <c r="G43" s="171"/>
-      <c r="H43" s="171"/>
-      <c r="I43" s="171"/>
-      <c r="J43" s="171"/>
-      <c r="K43" s="171"/>
-      <c r="L43" s="172"/>
+      <c r="B43" s="209"/>
+      <c r="C43" s="209"/>
+      <c r="D43" s="209"/>
+      <c r="E43" s="209"/>
+      <c r="F43" s="209"/>
+      <c r="G43" s="209"/>
+      <c r="H43" s="209"/>
+      <c r="I43" s="209"/>
+      <c r="J43" s="209"/>
+      <c r="K43" s="209"/>
+      <c r="L43" s="210"/>
       <c r="M43" s="65" t="s">
         <v>65</v>
       </c>
@@ -4733,20 +4733,20 @@
       <c r="AE43" s="64"/>
     </row>
     <row r="44" spans="1:31" s="13" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A44" s="170" t="s">
+      <c r="A44" s="208" t="s">
         <v>37</v>
       </c>
-      <c r="B44" s="171"/>
-      <c r="C44" s="171"/>
-      <c r="D44" s="171"/>
-      <c r="E44" s="171"/>
-      <c r="F44" s="171"/>
-      <c r="G44" s="171"/>
-      <c r="H44" s="171"/>
-      <c r="I44" s="171"/>
-      <c r="J44" s="171"/>
-      <c r="K44" s="171"/>
-      <c r="L44" s="172"/>
+      <c r="B44" s="209"/>
+      <c r="C44" s="209"/>
+      <c r="D44" s="209"/>
+      <c r="E44" s="209"/>
+      <c r="F44" s="209"/>
+      <c r="G44" s="209"/>
+      <c r="H44" s="209"/>
+      <c r="I44" s="209"/>
+      <c r="J44" s="209"/>
+      <c r="K44" s="209"/>
+      <c r="L44" s="210"/>
       <c r="M44" s="66" t="s">
         <v>118</v>
       </c>
@@ -4768,20 +4768,20 @@
       <c r="AE44" s="64"/>
     </row>
     <row r="45" spans="1:31" s="13" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A45" s="170" t="s">
+      <c r="A45" s="208" t="s">
         <v>32</v>
       </c>
-      <c r="B45" s="171"/>
-      <c r="C45" s="171"/>
-      <c r="D45" s="171"/>
-      <c r="E45" s="171"/>
-      <c r="F45" s="171"/>
-      <c r="G45" s="171"/>
-      <c r="H45" s="171"/>
-      <c r="I45" s="171"/>
-      <c r="J45" s="171"/>
-      <c r="K45" s="171"/>
-      <c r="L45" s="172"/>
+      <c r="B45" s="209"/>
+      <c r="C45" s="209"/>
+      <c r="D45" s="209"/>
+      <c r="E45" s="209"/>
+      <c r="F45" s="209"/>
+      <c r="G45" s="209"/>
+      <c r="H45" s="209"/>
+      <c r="I45" s="209"/>
+      <c r="J45" s="209"/>
+      <c r="K45" s="209"/>
+      <c r="L45" s="210"/>
       <c r="M45" s="69" t="s">
         <v>117</v>
       </c>
@@ -4830,17 +4830,17 @@
       <c r="A47" s="74" t="s">
         <v>111</v>
       </c>
-      <c r="D47" s="171" t="s">
+      <c r="D47" s="209" t="s">
         <v>114</v>
       </c>
-      <c r="E47" s="171"/>
-      <c r="F47" s="171"/>
-      <c r="G47" s="171"/>
-      <c r="H47" s="171"/>
-      <c r="I47" s="171"/>
-      <c r="J47" s="171"/>
-      <c r="K47" s="171"/>
-      <c r="L47" s="172"/>
+      <c r="E47" s="209"/>
+      <c r="F47" s="209"/>
+      <c r="G47" s="209"/>
+      <c r="H47" s="209"/>
+      <c r="I47" s="209"/>
+      <c r="J47" s="209"/>
+      <c r="K47" s="209"/>
+      <c r="L47" s="210"/>
       <c r="M47" s="65" t="s">
         <v>74</v>
       </c>
@@ -4854,17 +4854,17 @@
       <c r="A48" s="74" t="s">
         <v>110</v>
       </c>
-      <c r="D48" s="171" t="s">
+      <c r="D48" s="209" t="s">
         <v>78</v>
       </c>
-      <c r="E48" s="171"/>
-      <c r="F48" s="171"/>
-      <c r="G48" s="171"/>
-      <c r="H48" s="171"/>
-      <c r="I48" s="171"/>
-      <c r="J48" s="171"/>
-      <c r="K48" s="171"/>
-      <c r="L48" s="172"/>
+      <c r="E48" s="209"/>
+      <c r="F48" s="209"/>
+      <c r="G48" s="209"/>
+      <c r="H48" s="209"/>
+      <c r="I48" s="209"/>
+      <c r="J48" s="209"/>
+      <c r="K48" s="209"/>
+      <c r="L48" s="210"/>
       <c r="M48" s="65" t="s">
         <v>67</v>
       </c>
@@ -4878,17 +4878,17 @@
       <c r="A49" s="74" t="s">
         <v>112</v>
       </c>
-      <c r="D49" s="250" t="s">
+      <c r="D49" s="252" t="s">
         <v>115</v>
       </c>
-      <c r="E49" s="250"/>
-      <c r="F49" s="250"/>
-      <c r="G49" s="250"/>
-      <c r="H49" s="250"/>
-      <c r="I49" s="250"/>
-      <c r="J49" s="250"/>
-      <c r="K49" s="250"/>
-      <c r="L49" s="251"/>
+      <c r="E49" s="252"/>
+      <c r="F49" s="252"/>
+      <c r="G49" s="252"/>
+      <c r="H49" s="252"/>
+      <c r="I49" s="252"/>
+      <c r="J49" s="252"/>
+      <c r="K49" s="252"/>
+      <c r="L49" s="253"/>
       <c r="M49" s="65" t="s">
         <v>68</v>
       </c>
@@ -4902,17 +4902,17 @@
       <c r="A50" s="74" t="s">
         <v>113</v>
       </c>
-      <c r="D50" s="252" t="s">
+      <c r="D50" s="233" t="s">
         <v>116</v>
       </c>
-      <c r="E50" s="252"/>
-      <c r="F50" s="252"/>
-      <c r="G50" s="252"/>
-      <c r="H50" s="252"/>
-      <c r="I50" s="252"/>
-      <c r="J50" s="252"/>
-      <c r="K50" s="252"/>
-      <c r="L50" s="253"/>
+      <c r="E50" s="233"/>
+      <c r="F50" s="233"/>
+      <c r="G50" s="233"/>
+      <c r="H50" s="233"/>
+      <c r="I50" s="233"/>
+      <c r="J50" s="233"/>
+      <c r="K50" s="233"/>
+      <c r="L50" s="234"/>
       <c r="M50" s="65" t="s">
         <v>119</v>
       </c>
@@ -4924,15 +4924,15 @@
     </row>
     <row r="51" spans="1:31" s="13" customFormat="1" ht="20.100000000000001" customHeight="1">
       <c r="A51" s="74"/>
-      <c r="D51" s="254"/>
-      <c r="E51" s="254"/>
-      <c r="F51" s="254"/>
-      <c r="G51" s="254"/>
-      <c r="H51" s="254"/>
-      <c r="I51" s="254"/>
-      <c r="J51" s="254"/>
-      <c r="K51" s="254"/>
-      <c r="L51" s="255"/>
+      <c r="D51" s="235"/>
+      <c r="E51" s="235"/>
+      <c r="F51" s="235"/>
+      <c r="G51" s="235"/>
+      <c r="H51" s="235"/>
+      <c r="I51" s="235"/>
+      <c r="J51" s="235"/>
+      <c r="K51" s="235"/>
+      <c r="L51" s="236"/>
       <c r="M51" s="65" t="s">
         <v>124</v>
       </c>
@@ -4943,33 +4943,33 @@
       <c r="AE51" s="64"/>
     </row>
     <row r="52" spans="1:31" s="1" customFormat="1" ht="35.25" customHeight="1">
-      <c r="A52" s="193" t="s">
+      <c r="A52" s="188" t="s">
         <v>70</v>
       </c>
-      <c r="B52" s="194"/>
-      <c r="C52" s="194"/>
-      <c r="D52" s="194"/>
-      <c r="E52" s="194"/>
-      <c r="F52" s="194"/>
-      <c r="G52" s="194"/>
-      <c r="H52" s="194"/>
-      <c r="I52" s="194"/>
-      <c r="J52" s="194"/>
-      <c r="K52" s="194"/>
-      <c r="L52" s="194"/>
-      <c r="M52" s="194"/>
-      <c r="N52" s="194"/>
-      <c r="O52" s="194"/>
-      <c r="P52" s="194"/>
-      <c r="Q52" s="194"/>
-      <c r="R52" s="194"/>
-      <c r="S52" s="194"/>
-      <c r="T52" s="194"/>
-      <c r="U52" s="194"/>
-      <c r="V52" s="194"/>
-      <c r="W52" s="194"/>
-      <c r="X52" s="194"/>
-      <c r="Y52" s="195"/>
+      <c r="B52" s="189"/>
+      <c r="C52" s="189"/>
+      <c r="D52" s="189"/>
+      <c r="E52" s="189"/>
+      <c r="F52" s="189"/>
+      <c r="G52" s="189"/>
+      <c r="H52" s="189"/>
+      <c r="I52" s="189"/>
+      <c r="J52" s="189"/>
+      <c r="K52" s="189"/>
+      <c r="L52" s="189"/>
+      <c r="M52" s="189"/>
+      <c r="N52" s="189"/>
+      <c r="O52" s="189"/>
+      <c r="P52" s="189"/>
+      <c r="Q52" s="189"/>
+      <c r="R52" s="189"/>
+      <c r="S52" s="189"/>
+      <c r="T52" s="189"/>
+      <c r="U52" s="189"/>
+      <c r="V52" s="189"/>
+      <c r="W52" s="189"/>
+      <c r="X52" s="189"/>
+      <c r="Y52" s="190"/>
       <c r="AB52" s="2"/>
       <c r="AC52" s="2"/>
       <c r="AD52" s="2"/>
@@ -5017,6 +5017,11 @@
     <mergeCell ref="B27:I27"/>
     <mergeCell ref="B28:I28"/>
     <mergeCell ref="B30:I30"/>
+    <mergeCell ref="A42:L42"/>
+    <mergeCell ref="A43:L43"/>
+    <mergeCell ref="A44:L44"/>
+    <mergeCell ref="A41:M41"/>
+    <mergeCell ref="A29:I29"/>
     <mergeCell ref="D50:L51"/>
     <mergeCell ref="T18:X18"/>
     <mergeCell ref="J18:L18"/>
@@ -5058,21 +5063,15 @@
     <mergeCell ref="U41:Y41"/>
     <mergeCell ref="A31:I31"/>
     <mergeCell ref="A32:C34"/>
-    <mergeCell ref="A42:L42"/>
-    <mergeCell ref="A43:L43"/>
-    <mergeCell ref="A44:L44"/>
-    <mergeCell ref="R36:V36"/>
-    <mergeCell ref="W36:Y36"/>
-    <mergeCell ref="R37:V37"/>
-    <mergeCell ref="W37:Y37"/>
-    <mergeCell ref="D38:I38"/>
-    <mergeCell ref="R38:V40"/>
-    <mergeCell ref="A41:M41"/>
     <mergeCell ref="N41:T41"/>
     <mergeCell ref="A36:I36"/>
     <mergeCell ref="O38:Q40"/>
     <mergeCell ref="A37:I37"/>
     <mergeCell ref="A38:C40"/>
+    <mergeCell ref="R36:V36"/>
+    <mergeCell ref="R37:V37"/>
+    <mergeCell ref="D38:I38"/>
+    <mergeCell ref="R38:V40"/>
     <mergeCell ref="W19:Y20"/>
     <mergeCell ref="R26:V31"/>
     <mergeCell ref="W26:Y31"/>
@@ -5095,8 +5094,6 @@
     <mergeCell ref="O19:Q20"/>
     <mergeCell ref="O21:Q21"/>
     <mergeCell ref="O22:Q25"/>
-    <mergeCell ref="A29:I29"/>
-    <mergeCell ref="W38:Y40"/>
     <mergeCell ref="AF22:AH25"/>
     <mergeCell ref="D39:I39"/>
     <mergeCell ref="D40:I40"/>
@@ -5107,13 +5104,16 @@
     <mergeCell ref="D32:I32"/>
     <mergeCell ref="D33:I33"/>
     <mergeCell ref="D34:I34"/>
+    <mergeCell ref="W36:Y36"/>
+    <mergeCell ref="W37:Y37"/>
+    <mergeCell ref="W38:Y40"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="D49" r:id="rId1" xr:uid="{D4EC795B-C12B-4860-8B0F-9363B51335B3}"/>
   </hyperlinks>
-  <printOptions horizontalCentered="1" verticalCentered="1"/>
-  <pageMargins left="0.31496062992125984" right="0.23622047244094491" top="0.51181102362204722" bottom="0.26" header="0" footer="0"/>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.23622047244094491" right="0.23622047244094491" top="0.51181102362204722" bottom="0.27559055118110237" header="0" footer="0"/>
   <pageSetup paperSize="9" scale="65" orientation="portrait" horizontalDpi="4294967293" verticalDpi="4294967293" r:id="rId2"/>
   <headerFooter alignWithMargins="0"/>
   <drawing r:id="rId3"/>

</xml_diff>

<commit_message>
chore: adjust quotation template row heights
</commit_message>
<xml_diff>
--- a/직무고시 견적서 양식.xlsx
+++ b/직무고시 견적서 양식.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Master\Documents\Antigravity program\직무고시 견적서\wkace-quotation-jigmu\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72A1324C-9F9E-4C2A-8FB5-4815B3EA4723}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF7345FA-979D-4589-BDBF-77833413C4BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1704,6 +1704,369 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="5" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="39" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="10" fillId="3" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="10" fillId="3" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="7" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="7" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="7" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="20" fillId="5" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="29" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="31" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="30" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="27" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="23" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="24" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="25" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="28" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="26" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
     <xf numFmtId="41" fontId="14" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
@@ -1731,23 +2094,35 @@
     <xf numFmtId="41" fontId="14" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="14" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="41" fontId="14" fillId="0" borderId="29" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
@@ -1758,23 +2133,29 @@
     <xf numFmtId="41" fontId="14" fillId="0" borderId="30" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="29" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="31" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="30" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    <xf numFmtId="41" fontId="14" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="14" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="14" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="14" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="14" fillId="0" borderId="24" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="14" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="14" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="14" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="4" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1794,6 +2175,15 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1801,33 +2191,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1848,168 +2211,6 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="27" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="23" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="24" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="25" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="28" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="26" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="14" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="8" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="8" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="8" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="14" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="14" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="14" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="14" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="14" fillId="0" borderId="24" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="14" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="14" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="14" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="5" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="5" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="5" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="8" fillId="0" borderId="35" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="8" fillId="0" borderId="40" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="8" fillId="0" borderId="41" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
     <xf numFmtId="176" fontId="8" fillId="0" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
@@ -2037,224 +2238,23 @@
     <xf numFmtId="176" fontId="8" fillId="0" borderId="26" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="7" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="7" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="7" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="9" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="20" fillId="5" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="10" fillId="3" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="10" fillId="3" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="5" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="39" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="35" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="40" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="41" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -2892,33 +2892,33 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:40" s="1" customFormat="1" ht="54">
-      <c r="A1" s="241" t="s">
+      <c r="A1" s="100" t="s">
         <v>130</v>
       </c>
-      <c r="B1" s="241"/>
-      <c r="C1" s="241"/>
-      <c r="D1" s="241"/>
-      <c r="E1" s="241"/>
-      <c r="F1" s="241"/>
-      <c r="G1" s="241"/>
-      <c r="H1" s="241"/>
-      <c r="I1" s="241"/>
-      <c r="J1" s="241"/>
-      <c r="K1" s="241"/>
-      <c r="L1" s="241"/>
-      <c r="M1" s="241"/>
-      <c r="N1" s="241"/>
-      <c r="O1" s="241"/>
-      <c r="P1" s="241"/>
-      <c r="Q1" s="241"/>
-      <c r="R1" s="241"/>
-      <c r="S1" s="241"/>
-      <c r="T1" s="241"/>
-      <c r="U1" s="241"/>
-      <c r="V1" s="241"/>
-      <c r="W1" s="241"/>
-      <c r="X1" s="241"/>
-      <c r="Y1" s="241"/>
+      <c r="B1" s="100"/>
+      <c r="C1" s="100"/>
+      <c r="D1" s="100"/>
+      <c r="E1" s="100"/>
+      <c r="F1" s="100"/>
+      <c r="G1" s="100"/>
+      <c r="H1" s="100"/>
+      <c r="I1" s="100"/>
+      <c r="J1" s="100"/>
+      <c r="K1" s="100"/>
+      <c r="L1" s="100"/>
+      <c r="M1" s="100"/>
+      <c r="N1" s="100"/>
+      <c r="O1" s="100"/>
+      <c r="P1" s="100"/>
+      <c r="Q1" s="100"/>
+      <c r="R1" s="100"/>
+      <c r="S1" s="100"/>
+      <c r="T1" s="100"/>
+      <c r="U1" s="100"/>
+      <c r="V1" s="100"/>
+      <c r="W1" s="100"/>
+      <c r="X1" s="100"/>
+      <c r="Y1" s="100"/>
       <c r="AB1" s="2"/>
       <c r="AC1" s="3"/>
       <c r="AD1" s="3"/>
@@ -2973,33 +2973,33 @@
       <c r="AN2" s="3"/>
     </row>
     <row r="3" spans="1:40" s="1" customFormat="1" ht="26.25">
-      <c r="A3" s="242" t="s">
+      <c r="A3" s="101" t="s">
         <v>59</v>
       </c>
-      <c r="B3" s="242"/>
-      <c r="C3" s="242"/>
-      <c r="D3" s="242"/>
-      <c r="E3" s="242"/>
-      <c r="F3" s="242"/>
-      <c r="G3" s="242"/>
-      <c r="H3" s="242"/>
-      <c r="I3" s="242"/>
-      <c r="J3" s="242"/>
-      <c r="K3" s="242"/>
-      <c r="L3" s="242"/>
-      <c r="M3" s="242"/>
-      <c r="N3" s="242"/>
-      <c r="O3" s="242"/>
-      <c r="P3" s="242"/>
-      <c r="Q3" s="242"/>
-      <c r="R3" s="242"/>
-      <c r="S3" s="242"/>
-      <c r="T3" s="242"/>
-      <c r="U3" s="242"/>
-      <c r="V3" s="242"/>
-      <c r="W3" s="242"/>
-      <c r="X3" s="242"/>
-      <c r="Y3" s="242"/>
+      <c r="B3" s="101"/>
+      <c r="C3" s="101"/>
+      <c r="D3" s="101"/>
+      <c r="E3" s="101"/>
+      <c r="F3" s="101"/>
+      <c r="G3" s="101"/>
+      <c r="H3" s="101"/>
+      <c r="I3" s="101"/>
+      <c r="J3" s="101"/>
+      <c r="K3" s="101"/>
+      <c r="L3" s="101"/>
+      <c r="M3" s="101"/>
+      <c r="N3" s="101"/>
+      <c r="O3" s="101"/>
+      <c r="P3" s="101"/>
+      <c r="Q3" s="101"/>
+      <c r="R3" s="101"/>
+      <c r="S3" s="101"/>
+      <c r="T3" s="101"/>
+      <c r="U3" s="101"/>
+      <c r="V3" s="101"/>
+      <c r="W3" s="101"/>
+      <c r="X3" s="101"/>
+      <c r="Y3" s="101"/>
       <c r="AB3" s="2"/>
       <c r="AC3" s="3"/>
       <c r="AD3" s="3"/>
@@ -3099,38 +3099,38 @@
         <v>96</v>
       </c>
       <c r="B6" s="8"/>
-      <c r="C6" s="243">
+      <c r="C6" s="102">
         <f ca="1">TODAY()</f>
-        <v>46142</v>
-      </c>
-      <c r="D6" s="243"/>
-      <c r="E6" s="243"/>
-      <c r="F6" s="243"/>
+        <v>46148</v>
+      </c>
+      <c r="D6" s="102"/>
+      <c r="E6" s="102"/>
+      <c r="F6" s="102"/>
       <c r="G6" s="8"/>
       <c r="H6" s="8"/>
       <c r="I6" s="8"/>
       <c r="J6" s="9"/>
-      <c r="K6" s="230" t="s">
+      <c r="K6" s="125" t="s">
         <v>1</v>
       </c>
-      <c r="L6" s="222" t="s">
+      <c r="L6" s="118" t="s">
         <v>2</v>
       </c>
-      <c r="M6" s="223"/>
-      <c r="N6" s="224"/>
-      <c r="O6" s="249" t="s">
+      <c r="M6" s="119"/>
+      <c r="N6" s="120"/>
+      <c r="O6" s="112" t="s">
         <v>18</v>
       </c>
-      <c r="P6" s="250"/>
-      <c r="Q6" s="250"/>
-      <c r="R6" s="250"/>
-      <c r="S6" s="250"/>
-      <c r="T6" s="250"/>
-      <c r="U6" s="250"/>
-      <c r="V6" s="250"/>
-      <c r="W6" s="250"/>
-      <c r="X6" s="250"/>
-      <c r="Y6" s="251"/>
+      <c r="P6" s="113"/>
+      <c r="Q6" s="113"/>
+      <c r="R6" s="113"/>
+      <c r="S6" s="113"/>
+      <c r="T6" s="113"/>
+      <c r="U6" s="113"/>
+      <c r="V6" s="113"/>
+      <c r="W6" s="113"/>
+      <c r="X6" s="113"/>
+      <c r="Y6" s="114"/>
       <c r="AB6" s="2"/>
       <c r="AC6" s="3"/>
       <c r="AD6" s="3"/>
@@ -3160,29 +3160,29 @@
       <c r="H7" s="8"/>
       <c r="I7" s="8"/>
       <c r="J7" s="9"/>
-      <c r="K7" s="231"/>
-      <c r="L7" s="229" t="s">
+      <c r="K7" s="126"/>
+      <c r="L7" s="104" t="s">
         <v>22</v>
       </c>
-      <c r="M7" s="192"/>
-      <c r="N7" s="193"/>
-      <c r="O7" s="197" t="s">
+      <c r="M7" s="105"/>
+      <c r="N7" s="106"/>
+      <c r="O7" s="115" t="s">
         <v>17</v>
       </c>
-      <c r="P7" s="198"/>
-      <c r="Q7" s="198"/>
-      <c r="R7" s="198"/>
-      <c r="S7" s="228" t="s">
+      <c r="P7" s="116"/>
+      <c r="Q7" s="116"/>
+      <c r="R7" s="116"/>
+      <c r="S7" s="124" t="s">
         <v>25</v>
       </c>
-      <c r="T7" s="192"/>
-      <c r="U7" s="193"/>
-      <c r="V7" s="197" t="s">
+      <c r="T7" s="105"/>
+      <c r="U7" s="106"/>
+      <c r="V7" s="115" t="s">
         <v>20</v>
       </c>
-      <c r="W7" s="198"/>
-      <c r="X7" s="198"/>
-      <c r="Y7" s="221"/>
+      <c r="W7" s="116"/>
+      <c r="X7" s="116"/>
+      <c r="Y7" s="117"/>
       <c r="AB7" s="2"/>
       <c r="AC7" s="2"/>
       <c r="AD7" s="2"/>
@@ -3199,25 +3199,25 @@
       <c r="H8" s="11"/>
       <c r="I8" s="11"/>
       <c r="J8" s="12"/>
-      <c r="K8" s="231"/>
-      <c r="L8" s="229" t="s">
+      <c r="K8" s="126"/>
+      <c r="L8" s="104" t="s">
         <v>21</v>
       </c>
-      <c r="M8" s="192"/>
-      <c r="N8" s="193"/>
-      <c r="O8" s="197" t="s">
+      <c r="M8" s="105"/>
+      <c r="N8" s="106"/>
+      <c r="O8" s="115" t="s">
         <v>129</v>
       </c>
-      <c r="P8" s="198"/>
-      <c r="Q8" s="198"/>
-      <c r="R8" s="198"/>
-      <c r="S8" s="198"/>
-      <c r="T8" s="198"/>
-      <c r="U8" s="198"/>
-      <c r="V8" s="198"/>
-      <c r="W8" s="198"/>
-      <c r="X8" s="198"/>
-      <c r="Y8" s="221"/>
+      <c r="P8" s="116"/>
+      <c r="Q8" s="116"/>
+      <c r="R8" s="116"/>
+      <c r="S8" s="116"/>
+      <c r="T8" s="116"/>
+      <c r="U8" s="116"/>
+      <c r="V8" s="116"/>
+      <c r="W8" s="116"/>
+      <c r="X8" s="116"/>
+      <c r="Y8" s="117"/>
       <c r="AA8" s="2"/>
       <c r="AB8" s="2"/>
       <c r="AC8" s="2"/>
@@ -3237,29 +3237,29 @@
       <c r="H9" s="10"/>
       <c r="I9" s="8"/>
       <c r="J9" s="10"/>
-      <c r="K9" s="231"/>
-      <c r="L9" s="229" t="s">
+      <c r="K9" s="126"/>
+      <c r="L9" s="104" t="s">
         <v>23</v>
       </c>
-      <c r="M9" s="192"/>
-      <c r="N9" s="193"/>
-      <c r="O9" s="197" t="s">
+      <c r="M9" s="105"/>
+      <c r="N9" s="106"/>
+      <c r="O9" s="115" t="s">
         <v>9</v>
       </c>
-      <c r="P9" s="198"/>
-      <c r="Q9" s="198"/>
-      <c r="R9" s="198"/>
-      <c r="S9" s="191" t="s">
+      <c r="P9" s="116"/>
+      <c r="Q9" s="116"/>
+      <c r="R9" s="116"/>
+      <c r="S9" s="136" t="s">
         <v>26</v>
       </c>
-      <c r="T9" s="192"/>
-      <c r="U9" s="193"/>
-      <c r="V9" s="201" t="s">
+      <c r="T9" s="105"/>
+      <c r="U9" s="106"/>
+      <c r="V9" s="142" t="s">
         <v>31</v>
       </c>
-      <c r="W9" s="202"/>
-      <c r="X9" s="202"/>
-      <c r="Y9" s="203"/>
+      <c r="W9" s="143"/>
+      <c r="X9" s="143"/>
+      <c r="Y9" s="144"/>
       <c r="AB9" s="2"/>
       <c r="AC9" s="2"/>
       <c r="AD9" s="2"/>
@@ -3278,29 +3278,29 @@
       <c r="H10" s="10"/>
       <c r="I10" s="8"/>
       <c r="J10" s="9"/>
-      <c r="K10" s="232"/>
-      <c r="L10" s="246" t="s">
+      <c r="K10" s="127"/>
+      <c r="L10" s="109" t="s">
         <v>24</v>
       </c>
-      <c r="M10" s="247"/>
-      <c r="N10" s="248"/>
-      <c r="O10" s="199" t="s">
+      <c r="M10" s="110"/>
+      <c r="N10" s="111"/>
+      <c r="O10" s="140" t="s">
         <v>77</v>
       </c>
-      <c r="P10" s="200"/>
-      <c r="Q10" s="200"/>
-      <c r="R10" s="200"/>
-      <c r="S10" s="194" t="s">
+      <c r="P10" s="141"/>
+      <c r="Q10" s="141"/>
+      <c r="R10" s="141"/>
+      <c r="S10" s="137" t="s">
         <v>64</v>
       </c>
-      <c r="T10" s="195"/>
-      <c r="U10" s="196"/>
-      <c r="V10" s="199" t="s">
+      <c r="T10" s="138"/>
+      <c r="U10" s="139"/>
+      <c r="V10" s="140" t="s">
         <v>78</v>
       </c>
-      <c r="W10" s="200"/>
-      <c r="X10" s="200"/>
-      <c r="Y10" s="204"/>
+      <c r="W10" s="141"/>
+      <c r="X10" s="141"/>
+      <c r="Y10" s="145"/>
       <c r="AB10" s="2"/>
       <c r="AC10" s="2"/>
       <c r="AD10" s="2"/>
@@ -3351,10 +3351,10 @@
       <c r="E12" s="15"/>
       <c r="F12" s="15"/>
       <c r="G12" s="15"/>
-      <c r="H12" s="126"/>
-      <c r="I12" s="126"/>
-      <c r="J12" s="126"/>
-      <c r="K12" s="126"/>
+      <c r="H12" s="103"/>
+      <c r="I12" s="103"/>
+      <c r="J12" s="103"/>
+      <c r="K12" s="103"/>
       <c r="L12" s="15"/>
       <c r="M12" s="16"/>
       <c r="N12" s="14" t="s">
@@ -3412,10 +3412,10 @@
         <v>106</v>
       </c>
       <c r="Q13" s="3"/>
-      <c r="R13" s="245" t="s">
+      <c r="R13" s="108" t="s">
         <v>120</v>
       </c>
-      <c r="S13" s="245"/>
+      <c r="S13" s="108"/>
       <c r="T13" s="23" t="s">
         <v>121</v>
       </c>
@@ -3467,10 +3467,10 @@
         <v>107</v>
       </c>
       <c r="Q14" s="10"/>
-      <c r="R14" s="244" t="s">
+      <c r="R14" s="107" t="s">
         <v>123</v>
       </c>
-      <c r="S14" s="244"/>
+      <c r="S14" s="107"/>
       <c r="T14" s="23" t="s">
         <v>121</v>
       </c>
@@ -3514,10 +3514,10 @@
         <v>108</v>
       </c>
       <c r="Q15" s="10"/>
-      <c r="R15" s="244" t="s">
+      <c r="R15" s="107" t="s">
         <v>123</v>
       </c>
-      <c r="S15" s="244"/>
+      <c r="S15" s="107"/>
       <c r="T15" s="23" t="s">
         <v>121</v>
       </c>
@@ -3569,10 +3569,10 @@
         <v>109</v>
       </c>
       <c r="Q16" s="10"/>
-      <c r="R16" s="244" t="s">
+      <c r="R16" s="107" t="s">
         <v>123</v>
       </c>
-      <c r="S16" s="244"/>
+      <c r="S16" s="107"/>
       <c r="T16" s="23" t="s">
         <v>121</v>
       </c>
@@ -3589,21 +3589,21 @@
       <c r="AE16" s="39"/>
     </row>
     <row r="17" spans="1:34" s="1" customFormat="1" ht="20.100000000000001" customHeight="1" thickBot="1">
-      <c r="A17" s="225" t="s">
+      <c r="A17" s="121" t="s">
         <v>79</v>
       </c>
-      <c r="B17" s="226"/>
-      <c r="C17" s="226"/>
-      <c r="D17" s="226"/>
-      <c r="E17" s="226"/>
-      <c r="F17" s="226"/>
-      <c r="G17" s="226"/>
-      <c r="H17" s="226"/>
-      <c r="I17" s="226"/>
-      <c r="J17" s="226"/>
-      <c r="K17" s="226"/>
-      <c r="L17" s="226"/>
-      <c r="M17" s="227"/>
+      <c r="B17" s="122"/>
+      <c r="C17" s="122"/>
+      <c r="D17" s="122"/>
+      <c r="E17" s="122"/>
+      <c r="F17" s="122"/>
+      <c r="G17" s="122"/>
+      <c r="H17" s="122"/>
+      <c r="I17" s="122"/>
+      <c r="J17" s="122"/>
+      <c r="K17" s="122"/>
+      <c r="L17" s="122"/>
+      <c r="M17" s="123"/>
       <c r="N17" s="40"/>
       <c r="O17" s="41" t="s">
         <v>127</v>
@@ -3634,44 +3634,44 @@
       </c>
     </row>
     <row r="18" spans="1:34" s="45" customFormat="1" ht="39.950000000000003" customHeight="1">
-      <c r="A18" s="205" t="s">
+      <c r="A18" s="146" t="s">
         <v>69</v>
       </c>
-      <c r="B18" s="206"/>
-      <c r="C18" s="206"/>
-      <c r="D18" s="206"/>
-      <c r="E18" s="206"/>
-      <c r="F18" s="206"/>
-      <c r="G18" s="206"/>
-      <c r="H18" s="206"/>
-      <c r="I18" s="207"/>
-      <c r="J18" s="238" t="s">
+      <c r="B18" s="147"/>
+      <c r="C18" s="147"/>
+      <c r="D18" s="147"/>
+      <c r="E18" s="147"/>
+      <c r="F18" s="147"/>
+      <c r="G18" s="147"/>
+      <c r="H18" s="147"/>
+      <c r="I18" s="148"/>
+      <c r="J18" s="97" t="s">
         <v>0</v>
       </c>
-      <c r="K18" s="239"/>
-      <c r="L18" s="239"/>
-      <c r="M18" s="240">
+      <c r="K18" s="98"/>
+      <c r="L18" s="98"/>
+      <c r="M18" s="99">
         <f>U41</f>
         <v>1600000</v>
       </c>
-      <c r="N18" s="240"/>
-      <c r="O18" s="240"/>
-      <c r="P18" s="240"/>
-      <c r="Q18" s="240"/>
+      <c r="N18" s="99"/>
+      <c r="O18" s="99"/>
+      <c r="P18" s="99"/>
+      <c r="Q18" s="99"/>
       <c r="R18" s="43" t="s">
         <v>28</v>
       </c>
       <c r="S18" s="43" t="s">
         <v>55</v>
       </c>
-      <c r="T18" s="237">
+      <c r="T18" s="96">
         <f>U41</f>
         <v>1600000</v>
       </c>
-      <c r="U18" s="237"/>
-      <c r="V18" s="237"/>
-      <c r="W18" s="237"/>
-      <c r="X18" s="237"/>
+      <c r="U18" s="96"/>
+      <c r="V18" s="96"/>
+      <c r="W18" s="96"/>
+      <c r="X18" s="96"/>
       <c r="Y18" s="44" t="s">
         <v>54</v>
       </c>
@@ -3689,41 +3689,41 @@
       </c>
     </row>
     <row r="19" spans="1:34" s="1" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A19" s="125" t="s">
+      <c r="A19" s="128" t="s">
         <v>16</v>
       </c>
-      <c r="B19" s="126"/>
-      <c r="C19" s="126"/>
-      <c r="D19" s="126"/>
-      <c r="E19" s="126"/>
-      <c r="F19" s="126"/>
-      <c r="G19" s="126"/>
-      <c r="H19" s="126"/>
-      <c r="I19" s="127"/>
-      <c r="J19" s="104" t="s">
+      <c r="B19" s="103"/>
+      <c r="C19" s="103"/>
+      <c r="D19" s="103"/>
+      <c r="E19" s="103"/>
+      <c r="F19" s="103"/>
+      <c r="G19" s="103"/>
+      <c r="H19" s="103"/>
+      <c r="I19" s="129"/>
+      <c r="J19" s="231" t="s">
         <v>60</v>
       </c>
-      <c r="K19" s="105"/>
-      <c r="L19" s="105"/>
-      <c r="M19" s="105"/>
-      <c r="N19" s="106"/>
-      <c r="O19" s="119" t="s">
+      <c r="K19" s="232"/>
+      <c r="L19" s="232"/>
+      <c r="M19" s="232"/>
+      <c r="N19" s="233"/>
+      <c r="O19" s="240" t="s">
         <v>62</v>
       </c>
-      <c r="P19" s="120"/>
-      <c r="Q19" s="121"/>
-      <c r="R19" s="125" t="s">
+      <c r="P19" s="241"/>
+      <c r="Q19" s="242"/>
+      <c r="R19" s="128" t="s">
         <v>43</v>
       </c>
-      <c r="S19" s="126"/>
-      <c r="T19" s="126"/>
-      <c r="U19" s="126"/>
-      <c r="V19" s="127"/>
-      <c r="W19" s="125" t="s">
+      <c r="S19" s="103"/>
+      <c r="T19" s="103"/>
+      <c r="U19" s="103"/>
+      <c r="V19" s="129"/>
+      <c r="W19" s="128" t="s">
         <v>42</v>
       </c>
-      <c r="X19" s="126"/>
-      <c r="Y19" s="127"/>
+      <c r="X19" s="103"/>
+      <c r="Y19" s="129"/>
       <c r="AB19" s="31" t="s">
         <v>85</v>
       </c>
@@ -3738,15 +3738,15 @@
       </c>
     </row>
     <row r="20" spans="1:34" s="1" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A20" s="128"/>
-      <c r="B20" s="129"/>
-      <c r="C20" s="129"/>
-      <c r="D20" s="129"/>
-      <c r="E20" s="129"/>
-      <c r="F20" s="129"/>
-      <c r="G20" s="129"/>
-      <c r="H20" s="129"/>
-      <c r="I20" s="130"/>
+      <c r="A20" s="130"/>
+      <c r="B20" s="131"/>
+      <c r="C20" s="131"/>
+      <c r="D20" s="131"/>
+      <c r="E20" s="131"/>
+      <c r="F20" s="131"/>
+      <c r="G20" s="131"/>
+      <c r="H20" s="131"/>
+      <c r="I20" s="132"/>
       <c r="J20" s="46" t="s">
         <v>27</v>
       </c>
@@ -3762,17 +3762,17 @@
       <c r="N20" s="49" t="s">
         <v>58</v>
       </c>
-      <c r="O20" s="122"/>
-      <c r="P20" s="123"/>
-      <c r="Q20" s="124"/>
-      <c r="R20" s="128"/>
-      <c r="S20" s="129"/>
-      <c r="T20" s="129"/>
-      <c r="U20" s="129"/>
-      <c r="V20" s="130"/>
-      <c r="W20" s="128"/>
-      <c r="X20" s="129"/>
-      <c r="Y20" s="130"/>
+      <c r="O20" s="243"/>
+      <c r="P20" s="244"/>
+      <c r="Q20" s="245"/>
+      <c r="R20" s="130"/>
+      <c r="S20" s="131"/>
+      <c r="T20" s="131"/>
+      <c r="U20" s="131"/>
+      <c r="V20" s="132"/>
+      <c r="W20" s="130"/>
+      <c r="X20" s="131"/>
+      <c r="Y20" s="132"/>
       <c r="AB20" s="31" t="s">
         <v>85</v>
       </c>
@@ -3786,43 +3786,43 @@
         <v>56</v>
       </c>
     </row>
-    <row r="21" spans="1:34" s="1" customFormat="1" ht="20.100000000000001" customHeight="1" thickBot="1">
-      <c r="A21" s="95" t="s">
+    <row r="21" spans="1:34" s="1" customFormat="1" ht="31.5" customHeight="1" thickBot="1">
+      <c r="A21" s="89" t="s">
         <v>61</v>
       </c>
-      <c r="B21" s="96"/>
-      <c r="C21" s="96"/>
-      <c r="D21" s="96"/>
-      <c r="E21" s="96"/>
-      <c r="F21" s="96"/>
-      <c r="G21" s="96"/>
-      <c r="H21" s="96"/>
-      <c r="I21" s="97"/>
-      <c r="J21" s="101" t="s">
+      <c r="B21" s="90"/>
+      <c r="C21" s="90"/>
+      <c r="D21" s="90"/>
+      <c r="E21" s="90"/>
+      <c r="F21" s="90"/>
+      <c r="G21" s="90"/>
+      <c r="H21" s="90"/>
+      <c r="I21" s="91"/>
+      <c r="J21" s="228" t="s">
         <v>33</v>
       </c>
-      <c r="K21" s="102"/>
-      <c r="L21" s="102"/>
-      <c r="M21" s="102"/>
-      <c r="N21" s="103"/>
-      <c r="O21" s="107" t="s">
+      <c r="K21" s="229"/>
+      <c r="L21" s="229"/>
+      <c r="M21" s="229"/>
+      <c r="N21" s="230"/>
+      <c r="O21" s="237" t="s">
         <v>30</v>
       </c>
-      <c r="P21" s="108"/>
-      <c r="Q21" s="109"/>
-      <c r="R21" s="150">
+      <c r="P21" s="238"/>
+      <c r="Q21" s="239"/>
+      <c r="R21" s="255">
         <f>150000*8</f>
         <v>1200000</v>
       </c>
-      <c r="S21" s="151"/>
-      <c r="T21" s="151"/>
-      <c r="U21" s="151"/>
-      <c r="V21" s="152"/>
-      <c r="W21" s="92" t="s">
+      <c r="S21" s="256"/>
+      <c r="T21" s="256"/>
+      <c r="U21" s="256"/>
+      <c r="V21" s="257"/>
+      <c r="W21" s="217" t="s">
         <v>126</v>
       </c>
-      <c r="X21" s="93"/>
-      <c r="Y21" s="94"/>
+      <c r="X21" s="218"/>
+      <c r="Y21" s="219"/>
       <c r="AB21" s="50" t="s">
         <v>85</v>
       </c>
@@ -3836,38 +3836,38 @@
         <v>86</v>
       </c>
     </row>
-    <row r="22" spans="1:34" s="1" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A22" s="95" t="s">
+    <row r="22" spans="1:34" s="1" customFormat="1" ht="31.5" customHeight="1">
+      <c r="A22" s="89" t="s">
         <v>45</v>
       </c>
-      <c r="B22" s="96"/>
-      <c r="C22" s="96"/>
-      <c r="D22" s="96"/>
-      <c r="E22" s="96"/>
-      <c r="F22" s="96"/>
-      <c r="G22" s="96"/>
-      <c r="H22" s="96"/>
-      <c r="I22" s="97"/>
-      <c r="J22" s="101"/>
-      <c r="K22" s="102"/>
-      <c r="L22" s="102"/>
-      <c r="M22" s="102"/>
-      <c r="N22" s="103"/>
-      <c r="O22" s="110" t="s">
+      <c r="B22" s="90"/>
+      <c r="C22" s="90"/>
+      <c r="D22" s="90"/>
+      <c r="E22" s="90"/>
+      <c r="F22" s="90"/>
+      <c r="G22" s="90"/>
+      <c r="H22" s="90"/>
+      <c r="I22" s="91"/>
+      <c r="J22" s="228"/>
+      <c r="K22" s="229"/>
+      <c r="L22" s="229"/>
+      <c r="M22" s="229"/>
+      <c r="N22" s="230"/>
+      <c r="O22" s="162" t="s">
         <v>10</v>
       </c>
-      <c r="P22" s="111"/>
-      <c r="Q22" s="112"/>
-      <c r="R22" s="131">
+      <c r="P22" s="163"/>
+      <c r="Q22" s="164"/>
+      <c r="R22" s="189">
         <v>200000</v>
       </c>
-      <c r="S22" s="132"/>
-      <c r="T22" s="132"/>
-      <c r="U22" s="132"/>
-      <c r="V22" s="133"/>
-      <c r="W22" s="77"/>
-      <c r="X22" s="153"/>
-      <c r="Y22" s="154"/>
+      <c r="S22" s="190"/>
+      <c r="T22" s="190"/>
+      <c r="U22" s="190"/>
+      <c r="V22" s="191"/>
+      <c r="W22" s="198"/>
+      <c r="X22" s="220"/>
+      <c r="Y22" s="221"/>
       <c r="AB22" s="19" t="s">
         <v>80</v>
       </c>
@@ -3880,24 +3880,24 @@
       <c r="AE22" s="21" t="s">
         <v>56</v>
       </c>
-      <c r="AF22" s="77" t="s">
+      <c r="AF22" s="198" t="s">
         <v>95</v>
       </c>
-      <c r="AG22" s="78"/>
-      <c r="AH22" s="79"/>
-    </row>
-    <row r="23" spans="1:34" s="1" customFormat="1" ht="20.100000000000001" customHeight="1">
+      <c r="AG22" s="199"/>
+      <c r="AH22" s="200"/>
+    </row>
+    <row r="23" spans="1:34" s="1" customFormat="1" ht="31.5" customHeight="1">
       <c r="A23" s="53"/>
-      <c r="B23" s="254" t="s">
+      <c r="B23" s="81" t="s">
         <v>94</v>
       </c>
-      <c r="C23" s="254"/>
-      <c r="D23" s="254"/>
-      <c r="E23" s="254"/>
-      <c r="F23" s="254"/>
-      <c r="G23" s="254"/>
-      <c r="H23" s="254"/>
-      <c r="I23" s="255"/>
+      <c r="C23" s="81"/>
+      <c r="D23" s="81"/>
+      <c r="E23" s="81"/>
+      <c r="F23" s="81"/>
+      <c r="G23" s="81"/>
+      <c r="H23" s="81"/>
+      <c r="I23" s="82"/>
       <c r="J23" s="54"/>
       <c r="K23" s="54" t="s">
         <v>40</v>
@@ -3911,17 +3911,17 @@
       <c r="N23" s="54" t="s">
         <v>40</v>
       </c>
-      <c r="O23" s="113"/>
-      <c r="P23" s="114"/>
-      <c r="Q23" s="115"/>
-      <c r="R23" s="134"/>
-      <c r="S23" s="135"/>
-      <c r="T23" s="135"/>
-      <c r="U23" s="135"/>
-      <c r="V23" s="136"/>
-      <c r="W23" s="155"/>
-      <c r="X23" s="156"/>
-      <c r="Y23" s="157"/>
+      <c r="O23" s="165"/>
+      <c r="P23" s="166"/>
+      <c r="Q23" s="167"/>
+      <c r="R23" s="192"/>
+      <c r="S23" s="193"/>
+      <c r="T23" s="193"/>
+      <c r="U23" s="193"/>
+      <c r="V23" s="194"/>
+      <c r="W23" s="222"/>
+      <c r="X23" s="223"/>
+      <c r="Y23" s="224"/>
       <c r="AB23" s="31" t="s">
         <v>80</v>
       </c>
@@ -3934,22 +3934,22 @@
       <c r="AE23" s="32" t="s">
         <v>57</v>
       </c>
-      <c r="AF23" s="80"/>
-      <c r="AG23" s="81"/>
-      <c r="AH23" s="82"/>
-    </row>
-    <row r="24" spans="1:34" s="1" customFormat="1" ht="20.100000000000001" customHeight="1">
+      <c r="AF23" s="201"/>
+      <c r="AG23" s="202"/>
+      <c r="AH23" s="203"/>
+    </row>
+    <row r="24" spans="1:34" s="1" customFormat="1" ht="31.5" customHeight="1">
       <c r="A24" s="53"/>
-      <c r="B24" s="254" t="s">
+      <c r="B24" s="81" t="s">
         <v>44</v>
       </c>
-      <c r="C24" s="254"/>
-      <c r="D24" s="254"/>
-      <c r="E24" s="254"/>
-      <c r="F24" s="254"/>
-      <c r="G24" s="254"/>
-      <c r="H24" s="254"/>
-      <c r="I24" s="255"/>
+      <c r="C24" s="81"/>
+      <c r="D24" s="81"/>
+      <c r="E24" s="81"/>
+      <c r="F24" s="81"/>
+      <c r="G24" s="81"/>
+      <c r="H24" s="81"/>
+      <c r="I24" s="82"/>
       <c r="J24" s="54"/>
       <c r="K24" s="54"/>
       <c r="L24" s="54"/>
@@ -3957,17 +3957,17 @@
       <c r="N24" s="54" t="s">
         <v>40</v>
       </c>
-      <c r="O24" s="113"/>
-      <c r="P24" s="114"/>
-      <c r="Q24" s="115"/>
-      <c r="R24" s="134"/>
-      <c r="S24" s="135"/>
-      <c r="T24" s="135"/>
-      <c r="U24" s="135"/>
-      <c r="V24" s="136"/>
-      <c r="W24" s="155"/>
-      <c r="X24" s="156"/>
-      <c r="Y24" s="157"/>
+      <c r="O24" s="165"/>
+      <c r="P24" s="166"/>
+      <c r="Q24" s="167"/>
+      <c r="R24" s="192"/>
+      <c r="S24" s="193"/>
+      <c r="T24" s="193"/>
+      <c r="U24" s="193"/>
+      <c r="V24" s="194"/>
+      <c r="W24" s="222"/>
+      <c r="X24" s="223"/>
+      <c r="Y24" s="224"/>
       <c r="AB24" s="31" t="s">
         <v>80</v>
       </c>
@@ -3980,22 +3980,22 @@
       <c r="AE24" s="39" t="s">
         <v>56</v>
       </c>
-      <c r="AF24" s="80"/>
-      <c r="AG24" s="81"/>
-      <c r="AH24" s="82"/>
-    </row>
-    <row r="25" spans="1:34" s="1" customFormat="1" ht="20.100000000000001" customHeight="1" thickBot="1">
+      <c r="AF24" s="201"/>
+      <c r="AG24" s="202"/>
+      <c r="AH24" s="203"/>
+    </row>
+    <row r="25" spans="1:34" s="1" customFormat="1" ht="31.5" customHeight="1" thickBot="1">
       <c r="A25" s="53"/>
-      <c r="B25" s="254" t="s">
+      <c r="B25" s="81" t="s">
         <v>3</v>
       </c>
-      <c r="C25" s="254"/>
-      <c r="D25" s="254"/>
-      <c r="E25" s="254"/>
-      <c r="F25" s="254"/>
-      <c r="G25" s="254"/>
-      <c r="H25" s="254"/>
-      <c r="I25" s="255"/>
+      <c r="C25" s="81"/>
+      <c r="D25" s="81"/>
+      <c r="E25" s="81"/>
+      <c r="F25" s="81"/>
+      <c r="G25" s="81"/>
+      <c r="H25" s="81"/>
+      <c r="I25" s="82"/>
       <c r="J25" s="54"/>
       <c r="K25" s="54"/>
       <c r="L25" s="54" t="s">
@@ -4005,17 +4005,17 @@
       <c r="N25" s="54" t="s">
         <v>40</v>
       </c>
-      <c r="O25" s="116"/>
-      <c r="P25" s="117"/>
-      <c r="Q25" s="118"/>
-      <c r="R25" s="137"/>
-      <c r="S25" s="138"/>
-      <c r="T25" s="138"/>
-      <c r="U25" s="138"/>
-      <c r="V25" s="139"/>
-      <c r="W25" s="158"/>
-      <c r="X25" s="159"/>
-      <c r="Y25" s="160"/>
+      <c r="O25" s="168"/>
+      <c r="P25" s="169"/>
+      <c r="Q25" s="170"/>
+      <c r="R25" s="195"/>
+      <c r="S25" s="196"/>
+      <c r="T25" s="196"/>
+      <c r="U25" s="196"/>
+      <c r="V25" s="197"/>
+      <c r="W25" s="225"/>
+      <c r="X25" s="226"/>
+      <c r="Y25" s="227"/>
       <c r="AB25" s="50" t="s">
         <v>80</v>
       </c>
@@ -4028,44 +4028,44 @@
       <c r="AE25" s="52" t="s">
         <v>58</v>
       </c>
-      <c r="AF25" s="83"/>
-      <c r="AG25" s="84"/>
-      <c r="AH25" s="85"/>
-    </row>
-    <row r="26" spans="1:34" s="1" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A26" s="95" t="s">
+      <c r="AF25" s="204"/>
+      <c r="AG25" s="205"/>
+      <c r="AH25" s="206"/>
+    </row>
+    <row r="26" spans="1:34" s="1" customFormat="1" ht="31.5" customHeight="1">
+      <c r="A26" s="89" t="s">
         <v>46</v>
       </c>
-      <c r="B26" s="96"/>
-      <c r="C26" s="96"/>
-      <c r="D26" s="96"/>
-      <c r="E26" s="96"/>
-      <c r="F26" s="96"/>
-      <c r="G26" s="96"/>
-      <c r="H26" s="96"/>
-      <c r="I26" s="97"/>
+      <c r="B26" s="90"/>
+      <c r="C26" s="90"/>
+      <c r="D26" s="90"/>
+      <c r="E26" s="90"/>
+      <c r="F26" s="90"/>
+      <c r="G26" s="90"/>
+      <c r="H26" s="90"/>
+      <c r="I26" s="91"/>
       <c r="J26" s="55"/>
       <c r="K26" s="56"/>
       <c r="L26" s="56"/>
       <c r="M26" s="56"/>
       <c r="N26" s="57"/>
-      <c r="O26" s="110" t="s">
+      <c r="O26" s="162" t="s">
         <v>11</v>
       </c>
-      <c r="P26" s="111"/>
-      <c r="Q26" s="112"/>
-      <c r="R26" s="131">
+      <c r="P26" s="163"/>
+      <c r="Q26" s="164"/>
+      <c r="R26" s="189">
         <v>200000</v>
       </c>
-      <c r="S26" s="132"/>
-      <c r="T26" s="132"/>
-      <c r="U26" s="132"/>
-      <c r="V26" s="133"/>
-      <c r="W26" s="77" t="s">
+      <c r="S26" s="190"/>
+      <c r="T26" s="190"/>
+      <c r="U26" s="190"/>
+      <c r="V26" s="191"/>
+      <c r="W26" s="198" t="s">
         <v>75</v>
       </c>
-      <c r="X26" s="78"/>
-      <c r="Y26" s="79"/>
+      <c r="X26" s="199"/>
+      <c r="Y26" s="200"/>
       <c r="AB26" s="19" t="s">
         <v>85</v>
       </c>
@@ -4079,18 +4079,18 @@
         <v>56</v>
       </c>
     </row>
-    <row r="27" spans="1:34" s="1" customFormat="1" ht="20.100000000000001" customHeight="1">
+    <row r="27" spans="1:34" s="1" customFormat="1" ht="31.5" customHeight="1">
       <c r="A27" s="53"/>
-      <c r="B27" s="254" t="s">
+      <c r="B27" s="81" t="s">
         <v>76</v>
       </c>
-      <c r="C27" s="254"/>
-      <c r="D27" s="254"/>
-      <c r="E27" s="254"/>
-      <c r="F27" s="254"/>
-      <c r="G27" s="254"/>
-      <c r="H27" s="254"/>
-      <c r="I27" s="255"/>
+      <c r="C27" s="81"/>
+      <c r="D27" s="81"/>
+      <c r="E27" s="81"/>
+      <c r="F27" s="81"/>
+      <c r="G27" s="81"/>
+      <c r="H27" s="81"/>
+      <c r="I27" s="82"/>
       <c r="J27" s="54"/>
       <c r="K27" s="54"/>
       <c r="L27" s="54"/>
@@ -4098,17 +4098,17 @@
       <c r="N27" s="54" t="s">
         <v>40</v>
       </c>
-      <c r="O27" s="113"/>
-      <c r="P27" s="114"/>
-      <c r="Q27" s="115"/>
-      <c r="R27" s="134"/>
-      <c r="S27" s="135"/>
-      <c r="T27" s="135"/>
-      <c r="U27" s="135"/>
-      <c r="V27" s="136"/>
-      <c r="W27" s="80"/>
-      <c r="X27" s="81"/>
-      <c r="Y27" s="82"/>
+      <c r="O27" s="165"/>
+      <c r="P27" s="166"/>
+      <c r="Q27" s="167"/>
+      <c r="R27" s="192"/>
+      <c r="S27" s="193"/>
+      <c r="T27" s="193"/>
+      <c r="U27" s="193"/>
+      <c r="V27" s="194"/>
+      <c r="W27" s="201"/>
+      <c r="X27" s="202"/>
+      <c r="Y27" s="203"/>
       <c r="AB27" s="31" t="s">
         <v>85</v>
       </c>
@@ -4122,18 +4122,18 @@
         <v>57</v>
       </c>
     </row>
-    <row r="28" spans="1:34" s="1" customFormat="1" ht="20.100000000000001" customHeight="1">
+    <row r="28" spans="1:34" s="1" customFormat="1" ht="31.5" customHeight="1">
       <c r="A28" s="53"/>
-      <c r="B28" s="254" t="s">
+      <c r="B28" s="81" t="s">
         <v>3</v>
       </c>
-      <c r="C28" s="254"/>
-      <c r="D28" s="254"/>
-      <c r="E28" s="254"/>
-      <c r="F28" s="254"/>
-      <c r="G28" s="254"/>
-      <c r="H28" s="254"/>
-      <c r="I28" s="255"/>
+      <c r="C28" s="81"/>
+      <c r="D28" s="81"/>
+      <c r="E28" s="81"/>
+      <c r="F28" s="81"/>
+      <c r="G28" s="81"/>
+      <c r="H28" s="81"/>
+      <c r="I28" s="82"/>
       <c r="J28" s="54"/>
       <c r="K28" s="54"/>
       <c r="L28" s="54"/>
@@ -4141,17 +4141,17 @@
       <c r="N28" s="54" t="s">
         <v>40</v>
       </c>
-      <c r="O28" s="113"/>
-      <c r="P28" s="114"/>
-      <c r="Q28" s="115"/>
-      <c r="R28" s="134"/>
-      <c r="S28" s="135"/>
-      <c r="T28" s="135"/>
-      <c r="U28" s="135"/>
-      <c r="V28" s="136"/>
-      <c r="W28" s="80"/>
-      <c r="X28" s="81"/>
-      <c r="Y28" s="82"/>
+      <c r="O28" s="165"/>
+      <c r="P28" s="166"/>
+      <c r="Q28" s="167"/>
+      <c r="R28" s="192"/>
+      <c r="S28" s="193"/>
+      <c r="T28" s="193"/>
+      <c r="U28" s="193"/>
+      <c r="V28" s="194"/>
+      <c r="W28" s="201"/>
+      <c r="X28" s="202"/>
+      <c r="Y28" s="203"/>
       <c r="AB28" s="31" t="s">
         <v>85</v>
       </c>
@@ -4165,36 +4165,36 @@
         <v>56</v>
       </c>
     </row>
-    <row r="29" spans="1:34" s="1" customFormat="1" ht="20.100000000000001" customHeight="1" thickBot="1">
-      <c r="A29" s="95" t="s">
+    <row r="29" spans="1:34" s="1" customFormat="1" ht="31.5" customHeight="1" thickBot="1">
+      <c r="A29" s="89" t="s">
         <v>47</v>
       </c>
-      <c r="B29" s="96"/>
-      <c r="C29" s="96"/>
-      <c r="D29" s="96"/>
-      <c r="E29" s="96"/>
-      <c r="F29" s="96"/>
-      <c r="G29" s="96"/>
-      <c r="H29" s="96"/>
-      <c r="I29" s="97"/>
+      <c r="B29" s="90"/>
+      <c r="C29" s="90"/>
+      <c r="D29" s="90"/>
+      <c r="E29" s="90"/>
+      <c r="F29" s="90"/>
+      <c r="G29" s="90"/>
+      <c r="H29" s="90"/>
+      <c r="I29" s="91"/>
       <c r="J29" s="55"/>
       <c r="K29" s="56"/>
       <c r="L29" s="56"/>
       <c r="M29" s="56"/>
       <c r="N29" s="57"/>
-      <c r="O29" s="110" t="s">
+      <c r="O29" s="162" t="s">
         <v>12</v>
       </c>
-      <c r="P29" s="111"/>
-      <c r="Q29" s="112"/>
-      <c r="R29" s="134"/>
-      <c r="S29" s="135"/>
-      <c r="T29" s="135"/>
-      <c r="U29" s="135"/>
-      <c r="V29" s="136"/>
-      <c r="W29" s="80"/>
-      <c r="X29" s="81"/>
-      <c r="Y29" s="82"/>
+      <c r="P29" s="163"/>
+      <c r="Q29" s="164"/>
+      <c r="R29" s="192"/>
+      <c r="S29" s="193"/>
+      <c r="T29" s="193"/>
+      <c r="U29" s="193"/>
+      <c r="V29" s="194"/>
+      <c r="W29" s="201"/>
+      <c r="X29" s="202"/>
+      <c r="Y29" s="203"/>
       <c r="AB29" s="50" t="s">
         <v>85</v>
       </c>
@@ -4208,18 +4208,18 @@
         <v>86</v>
       </c>
     </row>
-    <row r="30" spans="1:34" s="1" customFormat="1" ht="20.100000000000001" customHeight="1">
+    <row r="30" spans="1:34" s="1" customFormat="1" ht="31.5" customHeight="1">
       <c r="A30" s="58"/>
-      <c r="B30" s="254" t="s">
+      <c r="B30" s="81" t="s">
         <v>76</v>
       </c>
-      <c r="C30" s="254"/>
-      <c r="D30" s="254"/>
-      <c r="E30" s="254"/>
-      <c r="F30" s="254"/>
-      <c r="G30" s="254"/>
-      <c r="H30" s="254"/>
-      <c r="I30" s="255"/>
+      <c r="C30" s="81"/>
+      <c r="D30" s="81"/>
+      <c r="E30" s="81"/>
+      <c r="F30" s="81"/>
+      <c r="G30" s="81"/>
+      <c r="H30" s="81"/>
+      <c r="I30" s="82"/>
       <c r="J30" s="59"/>
       <c r="K30" s="59"/>
       <c r="L30" s="59"/>
@@ -4227,17 +4227,17 @@
       <c r="N30" s="54" t="s">
         <v>40</v>
       </c>
-      <c r="O30" s="113"/>
-      <c r="P30" s="114"/>
-      <c r="Q30" s="115"/>
-      <c r="R30" s="134"/>
-      <c r="S30" s="135"/>
-      <c r="T30" s="135"/>
-      <c r="U30" s="135"/>
-      <c r="V30" s="136"/>
-      <c r="W30" s="80"/>
-      <c r="X30" s="81"/>
-      <c r="Y30" s="82"/>
+      <c r="O30" s="165"/>
+      <c r="P30" s="166"/>
+      <c r="Q30" s="167"/>
+      <c r="R30" s="192"/>
+      <c r="S30" s="193"/>
+      <c r="T30" s="193"/>
+      <c r="U30" s="193"/>
+      <c r="V30" s="194"/>
+      <c r="W30" s="201"/>
+      <c r="X30" s="202"/>
+      <c r="Y30" s="203"/>
       <c r="AB30" s="2" t="s">
         <v>91</v>
       </c>
@@ -4245,36 +4245,36 @@
       <c r="AD30" s="2"/>
       <c r="AE30" s="2"/>
     </row>
-    <row r="31" spans="1:34" s="1" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A31" s="95" t="s">
+    <row r="31" spans="1:34" s="1" customFormat="1" ht="31.5" customHeight="1">
+      <c r="A31" s="89" t="s">
         <v>48</v>
       </c>
-      <c r="B31" s="96"/>
-      <c r="C31" s="96"/>
-      <c r="D31" s="96"/>
-      <c r="E31" s="96"/>
-      <c r="F31" s="96"/>
-      <c r="G31" s="96"/>
-      <c r="H31" s="96"/>
-      <c r="I31" s="97"/>
+      <c r="B31" s="90"/>
+      <c r="C31" s="90"/>
+      <c r="D31" s="90"/>
+      <c r="E31" s="90"/>
+      <c r="F31" s="90"/>
+      <c r="G31" s="90"/>
+      <c r="H31" s="90"/>
+      <c r="I31" s="91"/>
       <c r="J31" s="55"/>
       <c r="K31" s="56"/>
       <c r="L31" s="56"/>
       <c r="M31" s="56"/>
       <c r="N31" s="57"/>
-      <c r="O31" s="89" t="s">
+      <c r="O31" s="234" t="s">
         <v>13</v>
       </c>
-      <c r="P31" s="90"/>
-      <c r="Q31" s="91"/>
-      <c r="R31" s="137"/>
-      <c r="S31" s="138"/>
-      <c r="T31" s="138"/>
-      <c r="U31" s="138"/>
-      <c r="V31" s="139"/>
-      <c r="W31" s="83"/>
-      <c r="X31" s="84"/>
-      <c r="Y31" s="85"/>
+      <c r="P31" s="235"/>
+      <c r="Q31" s="236"/>
+      <c r="R31" s="195"/>
+      <c r="S31" s="196"/>
+      <c r="T31" s="196"/>
+      <c r="U31" s="196"/>
+      <c r="V31" s="197"/>
+      <c r="W31" s="204"/>
+      <c r="X31" s="205"/>
+      <c r="Y31" s="206"/>
       <c r="AB31" s="2" t="s">
         <v>92</v>
       </c>
@@ -4284,20 +4284,20 @@
       <c r="AD31" s="2"/>
       <c r="AE31" s="2"/>
     </row>
-    <row r="32" spans="1:34" s="1" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A32" s="212" t="s">
+    <row r="32" spans="1:34" s="1" customFormat="1" ht="31.5" customHeight="1">
+      <c r="A32" s="152" t="s">
         <v>49</v>
       </c>
-      <c r="B32" s="213"/>
-      <c r="C32" s="214"/>
-      <c r="D32" s="86" t="s">
+      <c r="B32" s="153"/>
+      <c r="C32" s="154"/>
+      <c r="D32" s="186" t="s">
         <v>4</v>
       </c>
-      <c r="E32" s="87"/>
-      <c r="F32" s="87"/>
-      <c r="G32" s="87"/>
-      <c r="H32" s="87"/>
-      <c r="I32" s="88"/>
+      <c r="E32" s="187"/>
+      <c r="F32" s="187"/>
+      <c r="G32" s="187"/>
+      <c r="H32" s="187"/>
+      <c r="I32" s="188"/>
       <c r="J32" s="60"/>
       <c r="K32" s="54"/>
       <c r="L32" s="54"/>
@@ -4305,38 +4305,38 @@
       <c r="N32" s="54" t="s">
         <v>40</v>
       </c>
-      <c r="O32" s="110" t="s">
+      <c r="O32" s="162" t="s">
         <v>19</v>
       </c>
-      <c r="P32" s="111"/>
-      <c r="Q32" s="112"/>
-      <c r="R32" s="140">
+      <c r="P32" s="163"/>
+      <c r="Q32" s="164"/>
+      <c r="R32" s="207">
         <v>200000</v>
       </c>
-      <c r="S32" s="141"/>
-      <c r="T32" s="141"/>
-      <c r="U32" s="141"/>
-      <c r="V32" s="142"/>
-      <c r="W32" s="149"/>
-      <c r="X32" s="78"/>
-      <c r="Y32" s="79"/>
+      <c r="S32" s="208"/>
+      <c r="T32" s="208"/>
+      <c r="U32" s="208"/>
+      <c r="V32" s="209"/>
+      <c r="W32" s="216"/>
+      <c r="X32" s="199"/>
+      <c r="Y32" s="200"/>
       <c r="AB32" s="2"/>
       <c r="AC32" s="2"/>
       <c r="AD32" s="2"/>
       <c r="AE32" s="2"/>
     </row>
-    <row r="33" spans="1:31" s="1" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A33" s="215"/>
-      <c r="B33" s="216"/>
-      <c r="C33" s="217"/>
-      <c r="D33" s="86" t="s">
+    <row r="33" spans="1:31" s="1" customFormat="1" ht="31.5" customHeight="1">
+      <c r="A33" s="155"/>
+      <c r="B33" s="156"/>
+      <c r="C33" s="157"/>
+      <c r="D33" s="186" t="s">
         <v>5</v>
       </c>
-      <c r="E33" s="87"/>
-      <c r="F33" s="87"/>
-      <c r="G33" s="87"/>
-      <c r="H33" s="87"/>
-      <c r="I33" s="88"/>
+      <c r="E33" s="187"/>
+      <c r="F33" s="187"/>
+      <c r="G33" s="187"/>
+      <c r="H33" s="187"/>
+      <c r="I33" s="188"/>
       <c r="J33" s="60"/>
       <c r="K33" s="54"/>
       <c r="L33" s="54"/>
@@ -4344,34 +4344,34 @@
       <c r="N33" s="54" t="s">
         <v>40</v>
       </c>
-      <c r="O33" s="113"/>
-      <c r="P33" s="114"/>
-      <c r="Q33" s="115"/>
-      <c r="R33" s="143"/>
-      <c r="S33" s="144"/>
-      <c r="T33" s="144"/>
-      <c r="U33" s="144"/>
-      <c r="V33" s="145"/>
-      <c r="W33" s="80"/>
-      <c r="X33" s="81"/>
-      <c r="Y33" s="82"/>
+      <c r="O33" s="165"/>
+      <c r="P33" s="166"/>
+      <c r="Q33" s="167"/>
+      <c r="R33" s="210"/>
+      <c r="S33" s="211"/>
+      <c r="T33" s="211"/>
+      <c r="U33" s="211"/>
+      <c r="V33" s="212"/>
+      <c r="W33" s="201"/>
+      <c r="X33" s="202"/>
+      <c r="Y33" s="203"/>
       <c r="AB33" s="2"/>
       <c r="AC33" s="2"/>
       <c r="AD33" s="2"/>
       <c r="AE33" s="2"/>
     </row>
-    <row r="34" spans="1:31" s="1" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A34" s="218"/>
-      <c r="B34" s="219"/>
-      <c r="C34" s="220"/>
-      <c r="D34" s="86" t="s">
+    <row r="34" spans="1:31" s="1" customFormat="1" ht="31.5" customHeight="1">
+      <c r="A34" s="158"/>
+      <c r="B34" s="159"/>
+      <c r="C34" s="160"/>
+      <c r="D34" s="186" t="s">
         <v>6</v>
       </c>
-      <c r="E34" s="87"/>
-      <c r="F34" s="87"/>
-      <c r="G34" s="87"/>
-      <c r="H34" s="87"/>
-      <c r="I34" s="88"/>
+      <c r="E34" s="187"/>
+      <c r="F34" s="187"/>
+      <c r="G34" s="187"/>
+      <c r="H34" s="187"/>
+      <c r="I34" s="188"/>
       <c r="J34" s="60"/>
       <c r="K34" s="54" t="s">
         <v>40</v>
@@ -4385,34 +4385,34 @@
       <c r="N34" s="54" t="s">
         <v>40</v>
       </c>
-      <c r="O34" s="116"/>
-      <c r="P34" s="117"/>
-      <c r="Q34" s="118"/>
-      <c r="R34" s="146"/>
-      <c r="S34" s="147"/>
-      <c r="T34" s="147"/>
-      <c r="U34" s="147"/>
-      <c r="V34" s="148"/>
-      <c r="W34" s="83"/>
-      <c r="X34" s="84"/>
-      <c r="Y34" s="85"/>
+      <c r="O34" s="168"/>
+      <c r="P34" s="169"/>
+      <c r="Q34" s="170"/>
+      <c r="R34" s="213"/>
+      <c r="S34" s="214"/>
+      <c r="T34" s="214"/>
+      <c r="U34" s="214"/>
+      <c r="V34" s="215"/>
+      <c r="W34" s="204"/>
+      <c r="X34" s="205"/>
+      <c r="Y34" s="206"/>
       <c r="AB34" s="2"/>
       <c r="AC34" s="2"/>
       <c r="AD34" s="2"/>
       <c r="AE34" s="2"/>
     </row>
-    <row r="35" spans="1:31" s="1" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A35" s="95" t="s">
+    <row r="35" spans="1:31" s="1" customFormat="1" ht="31.5" customHeight="1">
+      <c r="A35" s="89" t="s">
         <v>50</v>
       </c>
-      <c r="B35" s="96"/>
-      <c r="C35" s="96"/>
-      <c r="D35" s="96"/>
-      <c r="E35" s="96"/>
-      <c r="F35" s="96"/>
-      <c r="G35" s="96"/>
-      <c r="H35" s="96"/>
-      <c r="I35" s="97"/>
+      <c r="B35" s="90"/>
+      <c r="C35" s="90"/>
+      <c r="D35" s="90"/>
+      <c r="E35" s="90"/>
+      <c r="F35" s="90"/>
+      <c r="G35" s="90"/>
+      <c r="H35" s="90"/>
+      <c r="I35" s="91"/>
       <c r="J35" s="54"/>
       <c r="K35" s="54" t="s">
         <v>40</v>
@@ -4426,38 +4426,38 @@
       <c r="N35" s="54" t="s">
         <v>40</v>
       </c>
-      <c r="O35" s="89" t="s">
+      <c r="O35" s="234" t="s">
         <v>41</v>
       </c>
-      <c r="P35" s="90"/>
-      <c r="Q35" s="91"/>
-      <c r="R35" s="98">
+      <c r="P35" s="235"/>
+      <c r="Q35" s="236"/>
+      <c r="R35" s="183">
         <v>600000</v>
       </c>
-      <c r="S35" s="99"/>
-      <c r="T35" s="99"/>
-      <c r="U35" s="99"/>
-      <c r="V35" s="100"/>
-      <c r="W35" s="92"/>
-      <c r="X35" s="93"/>
-      <c r="Y35" s="94"/>
+      <c r="S35" s="184"/>
+      <c r="T35" s="184"/>
+      <c r="U35" s="184"/>
+      <c r="V35" s="185"/>
+      <c r="W35" s="217"/>
+      <c r="X35" s="218"/>
+      <c r="Y35" s="219"/>
       <c r="AB35" s="2"/>
       <c r="AC35" s="2"/>
       <c r="AD35" s="2"/>
       <c r="AE35" s="2"/>
     </row>
-    <row r="36" spans="1:31" s="1" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A36" s="95" t="s">
+    <row r="36" spans="1:31" s="1" customFormat="1" ht="31.5" customHeight="1">
+      <c r="A36" s="89" t="s">
         <v>51</v>
       </c>
-      <c r="B36" s="96"/>
-      <c r="C36" s="96"/>
-      <c r="D36" s="96"/>
-      <c r="E36" s="96"/>
-      <c r="F36" s="96"/>
-      <c r="G36" s="96"/>
-      <c r="H36" s="96"/>
-      <c r="I36" s="97"/>
+      <c r="B36" s="90"/>
+      <c r="C36" s="90"/>
+      <c r="D36" s="90"/>
+      <c r="E36" s="90"/>
+      <c r="F36" s="90"/>
+      <c r="G36" s="90"/>
+      <c r="H36" s="90"/>
+      <c r="I36" s="91"/>
       <c r="J36" s="54"/>
       <c r="K36" s="54"/>
       <c r="L36" s="54"/>
@@ -4465,38 +4465,38 @@
       <c r="N36" s="54" t="s">
         <v>40</v>
       </c>
-      <c r="O36" s="89" t="s">
+      <c r="O36" s="234" t="s">
         <v>14</v>
       </c>
-      <c r="P36" s="90"/>
-      <c r="Q36" s="91"/>
-      <c r="R36" s="98">
+      <c r="P36" s="235"/>
+      <c r="Q36" s="236"/>
+      <c r="R36" s="183">
         <v>300000</v>
       </c>
-      <c r="S36" s="99"/>
-      <c r="T36" s="99"/>
-      <c r="U36" s="99"/>
-      <c r="V36" s="100"/>
-      <c r="W36" s="92"/>
-      <c r="X36" s="93"/>
-      <c r="Y36" s="94"/>
+      <c r="S36" s="184"/>
+      <c r="T36" s="184"/>
+      <c r="U36" s="184"/>
+      <c r="V36" s="185"/>
+      <c r="W36" s="217"/>
+      <c r="X36" s="218"/>
+      <c r="Y36" s="219"/>
       <c r="AB36" s="2"/>
       <c r="AC36" s="2"/>
       <c r="AD36" s="2"/>
       <c r="AE36" s="2"/>
     </row>
-    <row r="37" spans="1:31" s="1" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A37" s="164" t="s">
+    <row r="37" spans="1:31" s="1" customFormat="1" ht="31.5" customHeight="1">
+      <c r="A37" s="171" t="s">
         <v>52</v>
       </c>
-      <c r="B37" s="165"/>
-      <c r="C37" s="165"/>
-      <c r="D37" s="165"/>
-      <c r="E37" s="165"/>
-      <c r="F37" s="165"/>
-      <c r="G37" s="165"/>
-      <c r="H37" s="165"/>
-      <c r="I37" s="166"/>
+      <c r="B37" s="172"/>
+      <c r="C37" s="172"/>
+      <c r="D37" s="172"/>
+      <c r="E37" s="172"/>
+      <c r="F37" s="172"/>
+      <c r="G37" s="172"/>
+      <c r="H37" s="172"/>
+      <c r="I37" s="173"/>
       <c r="J37" s="60"/>
       <c r="K37" s="54" t="s">
         <v>40</v>
@@ -4510,38 +4510,38 @@
       <c r="N37" s="54" t="s">
         <v>40</v>
       </c>
-      <c r="O37" s="107"/>
-      <c r="P37" s="108"/>
-      <c r="Q37" s="109"/>
-      <c r="R37" s="98">
+      <c r="O37" s="237"/>
+      <c r="P37" s="238"/>
+      <c r="Q37" s="239"/>
+      <c r="R37" s="183">
         <v>100000</v>
       </c>
-      <c r="S37" s="99"/>
-      <c r="T37" s="99"/>
-      <c r="U37" s="99"/>
-      <c r="V37" s="100"/>
-      <c r="W37" s="92"/>
-      <c r="X37" s="93"/>
-      <c r="Y37" s="94"/>
+      <c r="S37" s="184"/>
+      <c r="T37" s="184"/>
+      <c r="U37" s="184"/>
+      <c r="V37" s="185"/>
+      <c r="W37" s="217"/>
+      <c r="X37" s="218"/>
+      <c r="Y37" s="219"/>
       <c r="AB37" s="2"/>
       <c r="AC37" s="2"/>
       <c r="AD37" s="2"/>
       <c r="AE37" s="2"/>
     </row>
-    <row r="38" spans="1:31" s="1" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A38" s="167" t="s">
+    <row r="38" spans="1:31" s="1" customFormat="1" ht="31.5" customHeight="1">
+      <c r="A38" s="174" t="s">
         <v>63</v>
       </c>
-      <c r="B38" s="168"/>
-      <c r="C38" s="169"/>
-      <c r="D38" s="86" t="s">
+      <c r="B38" s="175"/>
+      <c r="C38" s="176"/>
+      <c r="D38" s="186" t="s">
         <v>72</v>
       </c>
-      <c r="E38" s="87"/>
-      <c r="F38" s="87"/>
-      <c r="G38" s="87"/>
-      <c r="H38" s="87"/>
-      <c r="I38" s="88"/>
+      <c r="E38" s="187"/>
+      <c r="F38" s="187"/>
+      <c r="G38" s="187"/>
+      <c r="H38" s="187"/>
+      <c r="I38" s="188"/>
       <c r="J38" s="60"/>
       <c r="K38" s="54"/>
       <c r="L38" s="54"/>
@@ -4549,69 +4549,69 @@
       <c r="N38" s="54" t="s">
         <v>40</v>
       </c>
-      <c r="O38" s="110" t="s">
+      <c r="O38" s="162" t="s">
         <v>15</v>
       </c>
-      <c r="P38" s="111"/>
-      <c r="Q38" s="112"/>
-      <c r="R38" s="176"/>
-      <c r="S38" s="176"/>
-      <c r="T38" s="176"/>
-      <c r="U38" s="176"/>
-      <c r="V38" s="176"/>
-      <c r="W38" s="179"/>
-      <c r="X38" s="180"/>
-      <c r="Y38" s="181"/>
+      <c r="P38" s="163"/>
+      <c r="Q38" s="164"/>
+      <c r="R38" s="258"/>
+      <c r="S38" s="258"/>
+      <c r="T38" s="258"/>
+      <c r="U38" s="258"/>
+      <c r="V38" s="258"/>
+      <c r="W38" s="246"/>
+      <c r="X38" s="247"/>
+      <c r="Y38" s="248"/>
       <c r="AB38" s="2"/>
       <c r="AC38" s="2"/>
       <c r="AD38" s="2"/>
       <c r="AE38" s="2"/>
     </row>
-    <row r="39" spans="1:31" s="1" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A39" s="170"/>
-      <c r="B39" s="171"/>
-      <c r="C39" s="172"/>
-      <c r="D39" s="86" t="s">
+    <row r="39" spans="1:31" s="1" customFormat="1" ht="31.5" customHeight="1">
+      <c r="A39" s="177"/>
+      <c r="B39" s="178"/>
+      <c r="C39" s="179"/>
+      <c r="D39" s="186" t="s">
         <v>73</v>
       </c>
-      <c r="E39" s="87"/>
-      <c r="F39" s="87"/>
-      <c r="G39" s="87"/>
-      <c r="H39" s="87"/>
-      <c r="I39" s="88"/>
+      <c r="E39" s="187"/>
+      <c r="F39" s="187"/>
+      <c r="G39" s="187"/>
+      <c r="H39" s="187"/>
+      <c r="I39" s="188"/>
       <c r="J39" s="60"/>
       <c r="K39" s="54"/>
       <c r="L39" s="54"/>
       <c r="M39" s="54"/>
       <c r="N39" s="54"/>
-      <c r="O39" s="113"/>
-      <c r="P39" s="114"/>
-      <c r="Q39" s="115"/>
-      <c r="R39" s="177"/>
-      <c r="S39" s="177"/>
-      <c r="T39" s="177"/>
-      <c r="U39" s="177"/>
-      <c r="V39" s="177"/>
-      <c r="W39" s="182"/>
-      <c r="X39" s="183"/>
-      <c r="Y39" s="184"/>
+      <c r="O39" s="165"/>
+      <c r="P39" s="166"/>
+      <c r="Q39" s="167"/>
+      <c r="R39" s="259"/>
+      <c r="S39" s="259"/>
+      <c r="T39" s="259"/>
+      <c r="U39" s="259"/>
+      <c r="V39" s="259"/>
+      <c r="W39" s="249"/>
+      <c r="X39" s="250"/>
+      <c r="Y39" s="251"/>
       <c r="AB39" s="2"/>
       <c r="AC39" s="2"/>
       <c r="AD39" s="2"/>
       <c r="AE39" s="2"/>
     </row>
-    <row r="40" spans="1:31" s="1" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A40" s="173"/>
-      <c r="B40" s="174"/>
-      <c r="C40" s="175"/>
-      <c r="D40" s="86" t="s">
+    <row r="40" spans="1:31" s="1" customFormat="1" ht="31.5" customHeight="1">
+      <c r="A40" s="180"/>
+      <c r="B40" s="181"/>
+      <c r="C40" s="182"/>
+      <c r="D40" s="186" t="s">
         <v>3</v>
       </c>
-      <c r="E40" s="87"/>
-      <c r="F40" s="87"/>
-      <c r="G40" s="87"/>
-      <c r="H40" s="87"/>
-      <c r="I40" s="88"/>
+      <c r="E40" s="187"/>
+      <c r="F40" s="187"/>
+      <c r="G40" s="187"/>
+      <c r="H40" s="187"/>
+      <c r="I40" s="188"/>
       <c r="J40" s="60"/>
       <c r="K40" s="54"/>
       <c r="L40" s="54"/>
@@ -4619,75 +4619,75 @@
       <c r="N40" s="54" t="s">
         <v>40</v>
       </c>
-      <c r="O40" s="116"/>
-      <c r="P40" s="117"/>
-      <c r="Q40" s="118"/>
-      <c r="R40" s="178"/>
-      <c r="S40" s="178"/>
-      <c r="T40" s="178"/>
-      <c r="U40" s="178"/>
-      <c r="V40" s="178"/>
-      <c r="W40" s="185"/>
-      <c r="X40" s="186"/>
-      <c r="Y40" s="187"/>
+      <c r="O40" s="168"/>
+      <c r="P40" s="169"/>
+      <c r="Q40" s="170"/>
+      <c r="R40" s="260"/>
+      <c r="S40" s="260"/>
+      <c r="T40" s="260"/>
+      <c r="U40" s="260"/>
+      <c r="V40" s="260"/>
+      <c r="W40" s="252"/>
+      <c r="X40" s="253"/>
+      <c r="Y40" s="254"/>
       <c r="AB40" s="2"/>
       <c r="AC40" s="2"/>
       <c r="AD40" s="2"/>
       <c r="AE40" s="2"/>
     </row>
     <row r="41" spans="1:31" s="1" customFormat="1" ht="30" customHeight="1">
-      <c r="A41" s="259" t="s">
+      <c r="A41" s="87" t="s">
         <v>39</v>
       </c>
-      <c r="B41" s="260"/>
-      <c r="C41" s="260"/>
-      <c r="D41" s="260"/>
-      <c r="E41" s="260"/>
-      <c r="F41" s="260"/>
-      <c r="G41" s="260"/>
-      <c r="H41" s="260"/>
-      <c r="I41" s="260"/>
-      <c r="J41" s="260"/>
-      <c r="K41" s="260"/>
-      <c r="L41" s="260"/>
-      <c r="M41" s="260"/>
+      <c r="B41" s="88"/>
+      <c r="C41" s="88"/>
+      <c r="D41" s="88"/>
+      <c r="E41" s="88"/>
+      <c r="F41" s="88"/>
+      <c r="G41" s="88"/>
+      <c r="H41" s="88"/>
+      <c r="I41" s="88"/>
+      <c r="J41" s="88"/>
+      <c r="K41" s="88"/>
+      <c r="L41" s="88"/>
+      <c r="M41" s="88"/>
       <c r="N41" s="161" t="s">
         <v>53</v>
       </c>
-      <c r="O41" s="162"/>
-      <c r="P41" s="162"/>
-      <c r="Q41" s="162"/>
-      <c r="R41" s="162"/>
-      <c r="S41" s="162"/>
-      <c r="T41" s="163"/>
-      <c r="U41" s="211">
+      <c r="O41" s="150"/>
+      <c r="P41" s="150"/>
+      <c r="Q41" s="150"/>
+      <c r="R41" s="150"/>
+      <c r="S41" s="150"/>
+      <c r="T41" s="151"/>
+      <c r="U41" s="149">
         <f>SUM(R22:V40)</f>
         <v>1600000</v>
       </c>
-      <c r="V41" s="162"/>
-      <c r="W41" s="162"/>
-      <c r="X41" s="162"/>
-      <c r="Y41" s="163"/>
+      <c r="V41" s="150"/>
+      <c r="W41" s="150"/>
+      <c r="X41" s="150"/>
+      <c r="Y41" s="151"/>
       <c r="AB41" s="2"/>
       <c r="AC41" s="2"/>
       <c r="AD41" s="2"/>
       <c r="AE41" s="2"/>
     </row>
     <row r="42" spans="1:31" s="13" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A42" s="256" t="s">
+      <c r="A42" s="83" t="s">
         <v>34</v>
       </c>
-      <c r="B42" s="257"/>
-      <c r="C42" s="257"/>
-      <c r="D42" s="257"/>
-      <c r="E42" s="257"/>
-      <c r="F42" s="257"/>
-      <c r="G42" s="257"/>
-      <c r="H42" s="257"/>
-      <c r="I42" s="257"/>
-      <c r="J42" s="257"/>
-      <c r="K42" s="257"/>
-      <c r="L42" s="258"/>
+      <c r="B42" s="84"/>
+      <c r="C42" s="84"/>
+      <c r="D42" s="84"/>
+      <c r="E42" s="84"/>
+      <c r="F42" s="84"/>
+      <c r="G42" s="84"/>
+      <c r="H42" s="84"/>
+      <c r="I42" s="84"/>
+      <c r="J42" s="84"/>
+      <c r="K42" s="84"/>
+      <c r="L42" s="85"/>
       <c r="M42" s="61" t="s">
         <v>35</v>
       </c>
@@ -4709,20 +4709,20 @@
       <c r="AE42" s="64"/>
     </row>
     <row r="43" spans="1:31" s="13" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A43" s="208" t="s">
+      <c r="A43" s="86" t="s">
         <v>36</v>
       </c>
-      <c r="B43" s="209"/>
-      <c r="C43" s="209"/>
-      <c r="D43" s="209"/>
-      <c r="E43" s="209"/>
-      <c r="F43" s="209"/>
-      <c r="G43" s="209"/>
-      <c r="H43" s="209"/>
-      <c r="I43" s="209"/>
-      <c r="J43" s="209"/>
-      <c r="K43" s="209"/>
-      <c r="L43" s="210"/>
+      <c r="B43" s="79"/>
+      <c r="C43" s="79"/>
+      <c r="D43" s="79"/>
+      <c r="E43" s="79"/>
+      <c r="F43" s="79"/>
+      <c r="G43" s="79"/>
+      <c r="H43" s="79"/>
+      <c r="I43" s="79"/>
+      <c r="J43" s="79"/>
+      <c r="K43" s="79"/>
+      <c r="L43" s="80"/>
       <c r="M43" s="65" t="s">
         <v>65</v>
       </c>
@@ -4733,20 +4733,20 @@
       <c r="AE43" s="64"/>
     </row>
     <row r="44" spans="1:31" s="13" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A44" s="208" t="s">
+      <c r="A44" s="86" t="s">
         <v>37</v>
       </c>
-      <c r="B44" s="209"/>
-      <c r="C44" s="209"/>
-      <c r="D44" s="209"/>
-      <c r="E44" s="209"/>
-      <c r="F44" s="209"/>
-      <c r="G44" s="209"/>
-      <c r="H44" s="209"/>
-      <c r="I44" s="209"/>
-      <c r="J44" s="209"/>
-      <c r="K44" s="209"/>
-      <c r="L44" s="210"/>
+      <c r="B44" s="79"/>
+      <c r="C44" s="79"/>
+      <c r="D44" s="79"/>
+      <c r="E44" s="79"/>
+      <c r="F44" s="79"/>
+      <c r="G44" s="79"/>
+      <c r="H44" s="79"/>
+      <c r="I44" s="79"/>
+      <c r="J44" s="79"/>
+      <c r="K44" s="79"/>
+      <c r="L44" s="80"/>
       <c r="M44" s="66" t="s">
         <v>118</v>
       </c>
@@ -4768,20 +4768,20 @@
       <c r="AE44" s="64"/>
     </row>
     <row r="45" spans="1:31" s="13" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A45" s="208" t="s">
+      <c r="A45" s="86" t="s">
         <v>32</v>
       </c>
-      <c r="B45" s="209"/>
-      <c r="C45" s="209"/>
-      <c r="D45" s="209"/>
-      <c r="E45" s="209"/>
-      <c r="F45" s="209"/>
-      <c r="G45" s="209"/>
-      <c r="H45" s="209"/>
-      <c r="I45" s="209"/>
-      <c r="J45" s="209"/>
-      <c r="K45" s="209"/>
-      <c r="L45" s="210"/>
+      <c r="B45" s="79"/>
+      <c r="C45" s="79"/>
+      <c r="D45" s="79"/>
+      <c r="E45" s="79"/>
+      <c r="F45" s="79"/>
+      <c r="G45" s="79"/>
+      <c r="H45" s="79"/>
+      <c r="I45" s="79"/>
+      <c r="J45" s="79"/>
+      <c r="K45" s="79"/>
+      <c r="L45" s="80"/>
       <c r="M45" s="69" t="s">
         <v>117</v>
       </c>
@@ -4830,17 +4830,17 @@
       <c r="A47" s="74" t="s">
         <v>111</v>
       </c>
-      <c r="D47" s="209" t="s">
+      <c r="D47" s="79" t="s">
         <v>114</v>
       </c>
-      <c r="E47" s="209"/>
-      <c r="F47" s="209"/>
-      <c r="G47" s="209"/>
-      <c r="H47" s="209"/>
-      <c r="I47" s="209"/>
-      <c r="J47" s="209"/>
-      <c r="K47" s="209"/>
-      <c r="L47" s="210"/>
+      <c r="E47" s="79"/>
+      <c r="F47" s="79"/>
+      <c r="G47" s="79"/>
+      <c r="H47" s="79"/>
+      <c r="I47" s="79"/>
+      <c r="J47" s="79"/>
+      <c r="K47" s="79"/>
+      <c r="L47" s="80"/>
       <c r="M47" s="65" t="s">
         <v>74</v>
       </c>
@@ -4854,17 +4854,17 @@
       <c r="A48" s="74" t="s">
         <v>110</v>
       </c>
-      <c r="D48" s="209" t="s">
+      <c r="D48" s="79" t="s">
         <v>78</v>
       </c>
-      <c r="E48" s="209"/>
-      <c r="F48" s="209"/>
-      <c r="G48" s="209"/>
-      <c r="H48" s="209"/>
-      <c r="I48" s="209"/>
-      <c r="J48" s="209"/>
-      <c r="K48" s="209"/>
-      <c r="L48" s="210"/>
+      <c r="E48" s="79"/>
+      <c r="F48" s="79"/>
+      <c r="G48" s="79"/>
+      <c r="H48" s="79"/>
+      <c r="I48" s="79"/>
+      <c r="J48" s="79"/>
+      <c r="K48" s="79"/>
+      <c r="L48" s="80"/>
       <c r="M48" s="65" t="s">
         <v>67</v>
       </c>
@@ -4878,17 +4878,17 @@
       <c r="A49" s="74" t="s">
         <v>112</v>
       </c>
-      <c r="D49" s="252" t="s">
+      <c r="D49" s="77" t="s">
         <v>115</v>
       </c>
-      <c r="E49" s="252"/>
-      <c r="F49" s="252"/>
-      <c r="G49" s="252"/>
-      <c r="H49" s="252"/>
-      <c r="I49" s="252"/>
-      <c r="J49" s="252"/>
-      <c r="K49" s="252"/>
-      <c r="L49" s="253"/>
+      <c r="E49" s="77"/>
+      <c r="F49" s="77"/>
+      <c r="G49" s="77"/>
+      <c r="H49" s="77"/>
+      <c r="I49" s="77"/>
+      <c r="J49" s="77"/>
+      <c r="K49" s="77"/>
+      <c r="L49" s="78"/>
       <c r="M49" s="65" t="s">
         <v>68</v>
       </c>
@@ -4902,17 +4902,17 @@
       <c r="A50" s="74" t="s">
         <v>113</v>
       </c>
-      <c r="D50" s="233" t="s">
+      <c r="D50" s="92" t="s">
         <v>116</v>
       </c>
-      <c r="E50" s="233"/>
-      <c r="F50" s="233"/>
-      <c r="G50" s="233"/>
-      <c r="H50" s="233"/>
-      <c r="I50" s="233"/>
-      <c r="J50" s="233"/>
-      <c r="K50" s="233"/>
-      <c r="L50" s="234"/>
+      <c r="E50" s="92"/>
+      <c r="F50" s="92"/>
+      <c r="G50" s="92"/>
+      <c r="H50" s="92"/>
+      <c r="I50" s="92"/>
+      <c r="J50" s="92"/>
+      <c r="K50" s="92"/>
+      <c r="L50" s="93"/>
       <c r="M50" s="65" t="s">
         <v>119</v>
       </c>
@@ -4924,15 +4924,15 @@
     </row>
     <row r="51" spans="1:31" s="13" customFormat="1" ht="20.100000000000001" customHeight="1">
       <c r="A51" s="74"/>
-      <c r="D51" s="235"/>
-      <c r="E51" s="235"/>
-      <c r="F51" s="235"/>
-      <c r="G51" s="235"/>
-      <c r="H51" s="235"/>
-      <c r="I51" s="235"/>
-      <c r="J51" s="235"/>
-      <c r="K51" s="235"/>
-      <c r="L51" s="236"/>
+      <c r="D51" s="94"/>
+      <c r="E51" s="94"/>
+      <c r="F51" s="94"/>
+      <c r="G51" s="94"/>
+      <c r="H51" s="94"/>
+      <c r="I51" s="94"/>
+      <c r="J51" s="94"/>
+      <c r="K51" s="94"/>
+      <c r="L51" s="95"/>
       <c r="M51" s="65" t="s">
         <v>124</v>
       </c>
@@ -4943,33 +4943,33 @@
       <c r="AE51" s="64"/>
     </row>
     <row r="52" spans="1:31" s="1" customFormat="1" ht="35.25" customHeight="1">
-      <c r="A52" s="188" t="s">
+      <c r="A52" s="133" t="s">
         <v>70</v>
       </c>
-      <c r="B52" s="189"/>
-      <c r="C52" s="189"/>
-      <c r="D52" s="189"/>
-      <c r="E52" s="189"/>
-      <c r="F52" s="189"/>
-      <c r="G52" s="189"/>
-      <c r="H52" s="189"/>
-      <c r="I52" s="189"/>
-      <c r="J52" s="189"/>
-      <c r="K52" s="189"/>
-      <c r="L52" s="189"/>
-      <c r="M52" s="189"/>
-      <c r="N52" s="189"/>
-      <c r="O52" s="189"/>
-      <c r="P52" s="189"/>
-      <c r="Q52" s="189"/>
-      <c r="R52" s="189"/>
-      <c r="S52" s="189"/>
-      <c r="T52" s="189"/>
-      <c r="U52" s="189"/>
-      <c r="V52" s="189"/>
-      <c r="W52" s="189"/>
-      <c r="X52" s="189"/>
-      <c r="Y52" s="190"/>
+      <c r="B52" s="134"/>
+      <c r="C52" s="134"/>
+      <c r="D52" s="134"/>
+      <c r="E52" s="134"/>
+      <c r="F52" s="134"/>
+      <c r="G52" s="134"/>
+      <c r="H52" s="134"/>
+      <c r="I52" s="134"/>
+      <c r="J52" s="134"/>
+      <c r="K52" s="134"/>
+      <c r="L52" s="134"/>
+      <c r="M52" s="134"/>
+      <c r="N52" s="134"/>
+      <c r="O52" s="134"/>
+      <c r="P52" s="134"/>
+      <c r="Q52" s="134"/>
+      <c r="R52" s="134"/>
+      <c r="S52" s="134"/>
+      <c r="T52" s="134"/>
+      <c r="U52" s="134"/>
+      <c r="V52" s="134"/>
+      <c r="W52" s="134"/>
+      <c r="X52" s="134"/>
+      <c r="Y52" s="135"/>
       <c r="AB52" s="2"/>
       <c r="AC52" s="2"/>
       <c r="AD52" s="2"/>
@@ -5008,20 +5008,75 @@
     </row>
   </sheetData>
   <mergeCells count="99">
-    <mergeCell ref="D49:L49"/>
-    <mergeCell ref="D48:L48"/>
-    <mergeCell ref="D47:L47"/>
-    <mergeCell ref="B23:I23"/>
-    <mergeCell ref="B24:I24"/>
-    <mergeCell ref="B25:I25"/>
-    <mergeCell ref="B27:I27"/>
-    <mergeCell ref="B28:I28"/>
-    <mergeCell ref="B30:I30"/>
-    <mergeCell ref="A42:L42"/>
-    <mergeCell ref="A43:L43"/>
-    <mergeCell ref="A44:L44"/>
-    <mergeCell ref="A41:M41"/>
-    <mergeCell ref="A29:I29"/>
+    <mergeCell ref="AF22:AH25"/>
+    <mergeCell ref="D39:I39"/>
+    <mergeCell ref="D40:I40"/>
+    <mergeCell ref="O35:Q35"/>
+    <mergeCell ref="W35:Y35"/>
+    <mergeCell ref="A35:I35"/>
+    <mergeCell ref="R35:V35"/>
+    <mergeCell ref="D32:I32"/>
+    <mergeCell ref="D33:I33"/>
+    <mergeCell ref="D34:I34"/>
+    <mergeCell ref="W36:Y36"/>
+    <mergeCell ref="W37:Y37"/>
+    <mergeCell ref="W38:Y40"/>
+    <mergeCell ref="J21:N21"/>
+    <mergeCell ref="J22:N22"/>
+    <mergeCell ref="J19:N19"/>
+    <mergeCell ref="O36:Q36"/>
+    <mergeCell ref="O37:Q37"/>
+    <mergeCell ref="O32:Q34"/>
+    <mergeCell ref="O26:Q28"/>
+    <mergeCell ref="O29:Q30"/>
+    <mergeCell ref="O31:Q31"/>
+    <mergeCell ref="O19:Q20"/>
+    <mergeCell ref="O21:Q21"/>
+    <mergeCell ref="O22:Q25"/>
+    <mergeCell ref="W19:Y20"/>
+    <mergeCell ref="R26:V31"/>
+    <mergeCell ref="W26:Y31"/>
+    <mergeCell ref="R32:V34"/>
+    <mergeCell ref="W32:Y34"/>
+    <mergeCell ref="R19:V20"/>
+    <mergeCell ref="R21:V21"/>
+    <mergeCell ref="W21:Y21"/>
+    <mergeCell ref="R22:V25"/>
+    <mergeCell ref="W22:Y25"/>
+    <mergeCell ref="N41:T41"/>
+    <mergeCell ref="A36:I36"/>
+    <mergeCell ref="O38:Q40"/>
+    <mergeCell ref="A37:I37"/>
+    <mergeCell ref="A38:C40"/>
+    <mergeCell ref="R36:V36"/>
+    <mergeCell ref="R37:V37"/>
+    <mergeCell ref="D38:I38"/>
+    <mergeCell ref="R38:V40"/>
+    <mergeCell ref="A19:I20"/>
+    <mergeCell ref="A52:Y52"/>
+    <mergeCell ref="S9:U9"/>
+    <mergeCell ref="S10:U10"/>
+    <mergeCell ref="O9:R9"/>
+    <mergeCell ref="O10:R10"/>
+    <mergeCell ref="V9:Y9"/>
+    <mergeCell ref="V10:Y10"/>
+    <mergeCell ref="A21:I21"/>
+    <mergeCell ref="A22:I22"/>
+    <mergeCell ref="A18:I18"/>
+    <mergeCell ref="A26:I26"/>
+    <mergeCell ref="A45:L45"/>
+    <mergeCell ref="U41:Y41"/>
+    <mergeCell ref="A31:I31"/>
+    <mergeCell ref="A32:C34"/>
+    <mergeCell ref="V7:Y7"/>
+    <mergeCell ref="L6:N6"/>
+    <mergeCell ref="A17:M17"/>
+    <mergeCell ref="O8:Y8"/>
+    <mergeCell ref="O7:R7"/>
+    <mergeCell ref="S7:U7"/>
+    <mergeCell ref="L7:N7"/>
+    <mergeCell ref="L8:N8"/>
+    <mergeCell ref="K6:K10"/>
     <mergeCell ref="D50:L51"/>
     <mergeCell ref="T18:X18"/>
     <mergeCell ref="J18:L18"/>
@@ -5038,75 +5093,20 @@
     <mergeCell ref="R15:S15"/>
     <mergeCell ref="L10:N10"/>
     <mergeCell ref="O6:Y6"/>
-    <mergeCell ref="V7:Y7"/>
-    <mergeCell ref="L6:N6"/>
-    <mergeCell ref="A17:M17"/>
-    <mergeCell ref="O8:Y8"/>
-    <mergeCell ref="O7:R7"/>
-    <mergeCell ref="S7:U7"/>
-    <mergeCell ref="L7:N7"/>
-    <mergeCell ref="L8:N8"/>
-    <mergeCell ref="K6:K10"/>
-    <mergeCell ref="A19:I20"/>
-    <mergeCell ref="A52:Y52"/>
-    <mergeCell ref="S9:U9"/>
-    <mergeCell ref="S10:U10"/>
-    <mergeCell ref="O9:R9"/>
-    <mergeCell ref="O10:R10"/>
-    <mergeCell ref="V9:Y9"/>
-    <mergeCell ref="V10:Y10"/>
-    <mergeCell ref="A21:I21"/>
-    <mergeCell ref="A22:I22"/>
-    <mergeCell ref="A18:I18"/>
-    <mergeCell ref="A26:I26"/>
-    <mergeCell ref="A45:L45"/>
-    <mergeCell ref="U41:Y41"/>
-    <mergeCell ref="A31:I31"/>
-    <mergeCell ref="A32:C34"/>
-    <mergeCell ref="N41:T41"/>
-    <mergeCell ref="A36:I36"/>
-    <mergeCell ref="O38:Q40"/>
-    <mergeCell ref="A37:I37"/>
-    <mergeCell ref="A38:C40"/>
-    <mergeCell ref="R36:V36"/>
-    <mergeCell ref="R37:V37"/>
-    <mergeCell ref="D38:I38"/>
-    <mergeCell ref="R38:V40"/>
-    <mergeCell ref="W19:Y20"/>
-    <mergeCell ref="R26:V31"/>
-    <mergeCell ref="W26:Y31"/>
-    <mergeCell ref="R32:V34"/>
-    <mergeCell ref="W32:Y34"/>
-    <mergeCell ref="R19:V20"/>
-    <mergeCell ref="R21:V21"/>
-    <mergeCell ref="W21:Y21"/>
-    <mergeCell ref="R22:V25"/>
-    <mergeCell ref="W22:Y25"/>
-    <mergeCell ref="J21:N21"/>
-    <mergeCell ref="J22:N22"/>
-    <mergeCell ref="J19:N19"/>
-    <mergeCell ref="O36:Q36"/>
-    <mergeCell ref="O37:Q37"/>
-    <mergeCell ref="O32:Q34"/>
-    <mergeCell ref="O26:Q28"/>
-    <mergeCell ref="O29:Q30"/>
-    <mergeCell ref="O31:Q31"/>
-    <mergeCell ref="O19:Q20"/>
-    <mergeCell ref="O21:Q21"/>
-    <mergeCell ref="O22:Q25"/>
-    <mergeCell ref="AF22:AH25"/>
-    <mergeCell ref="D39:I39"/>
-    <mergeCell ref="D40:I40"/>
-    <mergeCell ref="O35:Q35"/>
-    <mergeCell ref="W35:Y35"/>
-    <mergeCell ref="A35:I35"/>
-    <mergeCell ref="R35:V35"/>
-    <mergeCell ref="D32:I32"/>
-    <mergeCell ref="D33:I33"/>
-    <mergeCell ref="D34:I34"/>
-    <mergeCell ref="W36:Y36"/>
-    <mergeCell ref="W37:Y37"/>
-    <mergeCell ref="W38:Y40"/>
+    <mergeCell ref="D49:L49"/>
+    <mergeCell ref="D48:L48"/>
+    <mergeCell ref="D47:L47"/>
+    <mergeCell ref="B23:I23"/>
+    <mergeCell ref="B24:I24"/>
+    <mergeCell ref="B25:I25"/>
+    <mergeCell ref="B27:I27"/>
+    <mergeCell ref="B28:I28"/>
+    <mergeCell ref="B30:I30"/>
+    <mergeCell ref="A42:L42"/>
+    <mergeCell ref="A43:L43"/>
+    <mergeCell ref="A44:L44"/>
+    <mergeCell ref="A41:M41"/>
+    <mergeCell ref="A29:I29"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <hyperlinks>
@@ -5114,7 +5114,7 @@
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.23622047244094491" right="0.23622047244094491" top="0.51181102362204722" bottom="0.27559055118110237" header="0" footer="0"/>
-  <pageSetup paperSize="9" scale="65" orientation="portrait" horizontalDpi="4294967293" verticalDpi="4294967293" r:id="rId2"/>
+  <pageSetup paperSize="9" scale="55" orientation="portrait" horizontalDpi="4294967293" verticalDpi="4294967293" r:id="rId2"/>
   <headerFooter alignWithMargins="0"/>
   <drawing r:id="rId3"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update template certification text
</commit_message>
<xml_diff>
--- a/직무고시 견적서 양식.xlsx
+++ b/직무고시 견적서 양식.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Master\Documents\Antigravity program\직무고시 견적서\wkace-quotation-jigmu\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF7345FA-979D-4589-BDBF-77833413C4BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE15C472-61A3-41A7-8179-B5BC07E96A17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="견적서" sheetId="1" r:id="rId1"/>
@@ -268,10 +268,6 @@
   </si>
   <si>
     <t>연차</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>(산업자원부 인정 엔지니어링 사업자 신고 제 E-05-00586호)</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
@@ -590,6 +586,36 @@
     <t>점검범위 :</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
+  <si>
+    <r>
+      <t xml:space="preserve">(전기설비 </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="18"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="major"/>
+      </rPr>
+      <t>종합 시험자</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="18"/>
+        <color indexed="8"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="major"/>
+      </rPr>
+      <t xml:space="preserve"> 인증 2026-C1-0040호)</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
@@ -602,7 +628,7 @@
     <numFmt numFmtId="178" formatCode="0&quot;회&quot;"/>
     <numFmt numFmtId="179" formatCode="yyyy&quot;년&quot;\ m&quot;월&quot;\ d&quot;일&quot;;@"/>
   </numFmts>
-  <fonts count="26">
+  <fonts count="27">
     <font>
       <sz val="11"/>
       <name val="굴림체"/>
@@ -815,6 +841,15 @@
     <font>
       <sz val="10"/>
       <color indexed="8"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
+      <scheme val="major"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="1"/>
       <name val="맑은 고딕"/>
       <family val="3"/>
       <charset val="129"/>
@@ -2040,6 +2075,15 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="35" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="40" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="41" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
     <xf numFmtId="176" fontId="13" fillId="0" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
     </xf>
@@ -2124,6 +2168,15 @@
     <xf numFmtId="41" fontId="14" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
     <xf numFmtId="41" fontId="14" fillId="0" borderId="29" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
@@ -2237,24 +2290,6 @@
     </xf>
     <xf numFmtId="176" fontId="8" fillId="0" borderId="26" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="35" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="40" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="41" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -2893,7 +2928,7 @@
   <sheetData>
     <row r="1" spans="1:40" s="1" customFormat="1" ht="54">
       <c r="A1" s="100" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B1" s="100"/>
       <c r="C1" s="100"/>
@@ -2974,7 +3009,7 @@
     </row>
     <row r="3" spans="1:40" s="1" customFormat="1" ht="26.25">
       <c r="A3" s="101" t="s">
-        <v>59</v>
+        <v>134</v>
       </c>
       <c r="B3" s="101"/>
       <c r="C3" s="101"/>
@@ -3096,7 +3131,7 @@
     </row>
     <row r="6" spans="1:40" s="1" customFormat="1" ht="20.100000000000001" customHeight="1">
       <c r="A6" s="8" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B6" s="8"/>
       <c r="C6" s="102">
@@ -3147,11 +3182,11 @@
     </row>
     <row r="7" spans="1:40" s="1" customFormat="1" ht="20.100000000000001" customHeight="1">
       <c r="A7" s="10" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B7" s="8"/>
       <c r="C7" s="8" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D7" s="8"/>
       <c r="E7" s="8"/>
@@ -3206,7 +3241,7 @@
       <c r="M8" s="105"/>
       <c r="N8" s="106"/>
       <c r="O8" s="115" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="P8" s="116"/>
       <c r="Q8" s="116"/>
@@ -3285,18 +3320,18 @@
       <c r="M10" s="110"/>
       <c r="N10" s="111"/>
       <c r="O10" s="140" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="P10" s="141"/>
       <c r="Q10" s="141"/>
       <c r="R10" s="141"/>
       <c r="S10" s="137" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="T10" s="138"/>
       <c r="U10" s="139"/>
       <c r="V10" s="140" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="W10" s="141"/>
       <c r="X10" s="141"/>
@@ -3333,17 +3368,17 @@
       <c r="X11" s="2"/>
       <c r="Y11" s="2"/>
       <c r="AB11" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="AC11" s="2" t="s">
         <v>87</v>
-      </c>
-      <c r="AC11" s="2" t="s">
-        <v>88</v>
       </c>
       <c r="AD11" s="2"/>
       <c r="AE11" s="2"/>
     </row>
     <row r="12" spans="1:40" s="1" customFormat="1" ht="20.100000000000001" customHeight="1">
       <c r="A12" s="14" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B12" s="15"/>
       <c r="C12" s="15"/>
@@ -3358,7 +3393,7 @@
       <c r="L12" s="15"/>
       <c r="M12" s="16"/>
       <c r="N12" s="14" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="O12" s="17"/>
       <c r="P12" s="17"/>
@@ -3372,13 +3407,13 @@
       <c r="X12" s="17"/>
       <c r="Y12" s="18"/>
       <c r="AB12" s="19" t="s">
+        <v>79</v>
+      </c>
+      <c r="AC12" s="20" t="s">
+        <v>88</v>
+      </c>
+      <c r="AD12" s="20" t="s">
         <v>80</v>
-      </c>
-      <c r="AC12" s="20" t="s">
-        <v>89</v>
-      </c>
-      <c r="AD12" s="20" t="s">
-        <v>81</v>
       </c>
       <c r="AE12" s="21" t="s">
         <v>56</v>
@@ -3387,14 +3422,14 @@
     <row r="13" spans="1:40" s="30" customFormat="1" ht="20.100000000000001" customHeight="1">
       <c r="A13" s="22"/>
       <c r="B13" s="23" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D13" s="24"/>
       <c r="E13" s="10" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F13" s="10"/>
       <c r="G13" s="10"/>
@@ -3406,34 +3441,34 @@
       <c r="M13" s="28"/>
       <c r="N13" s="22"/>
       <c r="O13" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="P13" s="10" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="Q13" s="3"/>
       <c r="R13" s="108" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="S13" s="108"/>
       <c r="T13" s="23" t="s">
+        <v>120</v>
+      </c>
+      <c r="U13" s="10" t="s">
         <v>121</v>
-      </c>
-      <c r="U13" s="10" t="s">
-        <v>122</v>
       </c>
       <c r="V13" s="3"/>
       <c r="W13" s="3"/>
       <c r="X13" s="3"/>
       <c r="Y13" s="29"/>
       <c r="AB13" s="31" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="AC13" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="AD13" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AE13" s="32" t="s">
         <v>57</v>
@@ -3445,11 +3480,11 @@
         <v>29</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D14" s="24"/>
       <c r="E14" s="10" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F14" s="10"/>
       <c r="G14" s="10"/>
@@ -3464,18 +3499,18 @@
         <v>29</v>
       </c>
       <c r="P14" s="10" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="Q14" s="10"/>
       <c r="R14" s="107" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="S14" s="107"/>
       <c r="T14" s="23" t="s">
+        <v>120</v>
+      </c>
+      <c r="U14" s="10" t="s">
         <v>121</v>
-      </c>
-      <c r="U14" s="10" t="s">
-        <v>122</v>
       </c>
       <c r="V14" s="10"/>
       <c r="W14" s="10"/>
@@ -3489,14 +3524,14 @@
     <row r="15" spans="1:40" s="1" customFormat="1" ht="20.100000000000001" customHeight="1">
       <c r="A15" s="35"/>
       <c r="B15" s="23" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C15" s="36" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D15" s="10"/>
       <c r="E15" s="37" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F15" s="37"/>
       <c r="G15" s="10"/>
@@ -3508,34 +3543,34 @@
       <c r="M15" s="38"/>
       <c r="N15" s="33"/>
       <c r="O15" s="10" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="P15" s="10" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="Q15" s="10"/>
       <c r="R15" s="107" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="S15" s="107"/>
       <c r="T15" s="23" t="s">
+        <v>120</v>
+      </c>
+      <c r="U15" s="10" t="s">
         <v>121</v>
-      </c>
-      <c r="U15" s="10" t="s">
-        <v>122</v>
       </c>
       <c r="V15" s="10"/>
       <c r="W15" s="10"/>
       <c r="X15" s="10"/>
       <c r="Y15" s="34"/>
       <c r="AB15" s="31" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="AC15" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="AD15" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="AE15" s="39" t="s">
         <v>56</v>
@@ -3544,14 +3579,14 @@
     <row r="16" spans="1:40" s="1" customFormat="1" ht="20.100000000000001" customHeight="1">
       <c r="A16" s="35"/>
       <c r="B16" s="23" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C16" s="36" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D16" s="10"/>
       <c r="E16" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F16" s="37"/>
       <c r="G16" s="10"/>
@@ -3563,21 +3598,21 @@
       <c r="M16" s="38"/>
       <c r="N16" s="33"/>
       <c r="O16" s="10" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="P16" s="10" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="Q16" s="10"/>
       <c r="R16" s="107" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="S16" s="107"/>
       <c r="T16" s="23" t="s">
+        <v>120</v>
+      </c>
+      <c r="U16" s="10" t="s">
         <v>121</v>
-      </c>
-      <c r="U16" s="10" t="s">
-        <v>122</v>
       </c>
       <c r="V16" s="10"/>
       <c r="W16" s="10"/>
@@ -3590,7 +3625,7 @@
     </row>
     <row r="17" spans="1:34" s="1" customFormat="1" ht="20.100000000000001" customHeight="1" thickBot="1">
       <c r="A17" s="121" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B17" s="122"/>
       <c r="C17" s="122"/>
@@ -3606,10 +3641,10 @@
       <c r="M17" s="123"/>
       <c r="N17" s="40"/>
       <c r="O17" s="41" t="s">
+        <v>126</v>
+      </c>
+      <c r="P17" s="41" t="s">
         <v>127</v>
-      </c>
-      <c r="P17" s="41" t="s">
-        <v>128</v>
       </c>
       <c r="Q17" s="41"/>
       <c r="R17" s="41"/>
@@ -3621,13 +3656,13 @@
       <c r="X17" s="41"/>
       <c r="Y17" s="42"/>
       <c r="AB17" s="31" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="AC17" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="AD17" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="AE17" s="39" t="s">
         <v>58</v>
@@ -3635,7 +3670,7 @@
     </row>
     <row r="18" spans="1:34" s="45" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A18" s="146" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B18" s="147"/>
       <c r="C18" s="147"/>
@@ -3676,13 +3711,13 @@
         <v>54</v>
       </c>
       <c r="AB18" s="19" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="AC18" s="20" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="AD18" s="20" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="AE18" s="21" t="s">
         <v>56</v>
@@ -3700,18 +3735,18 @@
       <c r="G19" s="103"/>
       <c r="H19" s="103"/>
       <c r="I19" s="129"/>
-      <c r="J19" s="231" t="s">
-        <v>60</v>
-      </c>
-      <c r="K19" s="232"/>
-      <c r="L19" s="232"/>
-      <c r="M19" s="232"/>
-      <c r="N19" s="233"/>
-      <c r="O19" s="240" t="s">
-        <v>62</v>
-      </c>
-      <c r="P19" s="241"/>
-      <c r="Q19" s="242"/>
+      <c r="J19" s="237" t="s">
+        <v>59</v>
+      </c>
+      <c r="K19" s="238"/>
+      <c r="L19" s="238"/>
+      <c r="M19" s="238"/>
+      <c r="N19" s="239"/>
+      <c r="O19" s="246" t="s">
+        <v>61</v>
+      </c>
+      <c r="P19" s="247"/>
+      <c r="Q19" s="248"/>
       <c r="R19" s="128" t="s">
         <v>43</v>
       </c>
@@ -3725,13 +3760,13 @@
       <c r="X19" s="103"/>
       <c r="Y19" s="129"/>
       <c r="AB19" s="31" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="AC19" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="AD19" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AE19" s="32" t="s">
         <v>57</v>
@@ -3762,9 +3797,9 @@
       <c r="N20" s="49" t="s">
         <v>58</v>
       </c>
-      <c r="O20" s="243"/>
-      <c r="P20" s="244"/>
-      <c r="Q20" s="245"/>
+      <c r="O20" s="249"/>
+      <c r="P20" s="250"/>
+      <c r="Q20" s="251"/>
       <c r="R20" s="130"/>
       <c r="S20" s="131"/>
       <c r="T20" s="131"/>
@@ -3774,13 +3809,13 @@
       <c r="X20" s="131"/>
       <c r="Y20" s="132"/>
       <c r="AB20" s="31" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="AC20" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="AD20" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="AE20" s="39" t="s">
         <v>56</v>
@@ -3788,7 +3823,7 @@
     </row>
     <row r="21" spans="1:34" s="1" customFormat="1" ht="31.5" customHeight="1" thickBot="1">
       <c r="A21" s="89" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B21" s="90"/>
       <c r="C21" s="90"/>
@@ -3798,42 +3833,42 @@
       <c r="G21" s="90"/>
       <c r="H21" s="90"/>
       <c r="I21" s="91"/>
-      <c r="J21" s="228" t="s">
+      <c r="J21" s="234" t="s">
         <v>33</v>
       </c>
-      <c r="K21" s="229"/>
-      <c r="L21" s="229"/>
-      <c r="M21" s="229"/>
-      <c r="N21" s="230"/>
-      <c r="O21" s="237" t="s">
+      <c r="K21" s="235"/>
+      <c r="L21" s="235"/>
+      <c r="M21" s="235"/>
+      <c r="N21" s="236"/>
+      <c r="O21" s="243" t="s">
         <v>30</v>
       </c>
-      <c r="P21" s="238"/>
-      <c r="Q21" s="239"/>
-      <c r="R21" s="255">
+      <c r="P21" s="244"/>
+      <c r="Q21" s="245"/>
+      <c r="R21" s="220">
         <f>150000*8</f>
         <v>1200000</v>
       </c>
-      <c r="S21" s="256"/>
-      <c r="T21" s="256"/>
-      <c r="U21" s="256"/>
-      <c r="V21" s="257"/>
-      <c r="W21" s="217" t="s">
-        <v>126</v>
-      </c>
-      <c r="X21" s="218"/>
-      <c r="Y21" s="219"/>
+      <c r="S21" s="221"/>
+      <c r="T21" s="221"/>
+      <c r="U21" s="221"/>
+      <c r="V21" s="222"/>
+      <c r="W21" s="223" t="s">
+        <v>125</v>
+      </c>
+      <c r="X21" s="224"/>
+      <c r="Y21" s="225"/>
       <c r="AB21" s="50" t="s">
+        <v>84</v>
+      </c>
+      <c r="AC21" s="51" t="s">
+        <v>88</v>
+      </c>
+      <c r="AD21" s="51" t="s">
+        <v>83</v>
+      </c>
+      <c r="AE21" s="52" t="s">
         <v>85</v>
-      </c>
-      <c r="AC21" s="51" t="s">
-        <v>89</v>
-      </c>
-      <c r="AD21" s="51" t="s">
-        <v>84</v>
-      </c>
-      <c r="AE21" s="52" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="22" spans="1:34" s="1" customFormat="1" ht="31.5" customHeight="1">
@@ -3848,48 +3883,48 @@
       <c r="G22" s="90"/>
       <c r="H22" s="90"/>
       <c r="I22" s="91"/>
-      <c r="J22" s="228"/>
-      <c r="K22" s="229"/>
-      <c r="L22" s="229"/>
-      <c r="M22" s="229"/>
-      <c r="N22" s="230"/>
+      <c r="J22" s="234"/>
+      <c r="K22" s="235"/>
+      <c r="L22" s="235"/>
+      <c r="M22" s="235"/>
+      <c r="N22" s="236"/>
       <c r="O22" s="162" t="s">
         <v>10</v>
       </c>
       <c r="P22" s="163"/>
       <c r="Q22" s="164"/>
-      <c r="R22" s="189">
+      <c r="R22" s="192">
         <v>200000</v>
       </c>
-      <c r="S22" s="190"/>
-      <c r="T22" s="190"/>
-      <c r="U22" s="190"/>
-      <c r="V22" s="191"/>
-      <c r="W22" s="198"/>
-      <c r="X22" s="220"/>
-      <c r="Y22" s="221"/>
+      <c r="S22" s="193"/>
+      <c r="T22" s="193"/>
+      <c r="U22" s="193"/>
+      <c r="V22" s="194"/>
+      <c r="W22" s="201"/>
+      <c r="X22" s="226"/>
+      <c r="Y22" s="227"/>
       <c r="AB22" s="19" t="s">
+        <v>79</v>
+      </c>
+      <c r="AC22" s="20" t="s">
+        <v>89</v>
+      </c>
+      <c r="AD22" s="20" t="s">
         <v>80</v>
-      </c>
-      <c r="AC22" s="20" t="s">
-        <v>90</v>
-      </c>
-      <c r="AD22" s="20" t="s">
-        <v>81</v>
       </c>
       <c r="AE22" s="21" t="s">
         <v>56</v>
       </c>
-      <c r="AF22" s="198" t="s">
-        <v>95</v>
-      </c>
-      <c r="AG22" s="199"/>
-      <c r="AH22" s="200"/>
+      <c r="AF22" s="201" t="s">
+        <v>94</v>
+      </c>
+      <c r="AG22" s="202"/>
+      <c r="AH22" s="203"/>
     </row>
     <row r="23" spans="1:34" s="1" customFormat="1" ht="31.5" customHeight="1">
       <c r="A23" s="53"/>
       <c r="B23" s="81" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C23" s="81"/>
       <c r="D23" s="81"/>
@@ -3914,29 +3949,29 @@
       <c r="O23" s="165"/>
       <c r="P23" s="166"/>
       <c r="Q23" s="167"/>
-      <c r="R23" s="192"/>
-      <c r="S23" s="193"/>
-      <c r="T23" s="193"/>
-      <c r="U23" s="193"/>
-      <c r="V23" s="194"/>
-      <c r="W23" s="222"/>
-      <c r="X23" s="223"/>
-      <c r="Y23" s="224"/>
+      <c r="R23" s="195"/>
+      <c r="S23" s="196"/>
+      <c r="T23" s="196"/>
+      <c r="U23" s="196"/>
+      <c r="V23" s="197"/>
+      <c r="W23" s="228"/>
+      <c r="X23" s="229"/>
+      <c r="Y23" s="230"/>
       <c r="AB23" s="31" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="AC23" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="AD23" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AE23" s="32" t="s">
         <v>57</v>
       </c>
-      <c r="AF23" s="201"/>
-      <c r="AG23" s="202"/>
-      <c r="AH23" s="203"/>
+      <c r="AF23" s="204"/>
+      <c r="AG23" s="205"/>
+      <c r="AH23" s="206"/>
     </row>
     <row r="24" spans="1:34" s="1" customFormat="1" ht="31.5" customHeight="1">
       <c r="A24" s="53"/>
@@ -3960,29 +3995,29 @@
       <c r="O24" s="165"/>
       <c r="P24" s="166"/>
       <c r="Q24" s="167"/>
-      <c r="R24" s="192"/>
-      <c r="S24" s="193"/>
-      <c r="T24" s="193"/>
-      <c r="U24" s="193"/>
-      <c r="V24" s="194"/>
-      <c r="W24" s="222"/>
-      <c r="X24" s="223"/>
-      <c r="Y24" s="224"/>
+      <c r="R24" s="195"/>
+      <c r="S24" s="196"/>
+      <c r="T24" s="196"/>
+      <c r="U24" s="196"/>
+      <c r="V24" s="197"/>
+      <c r="W24" s="228"/>
+      <c r="X24" s="229"/>
+      <c r="Y24" s="230"/>
       <c r="AB24" s="31" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="AC24" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="AD24" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="AE24" s="39" t="s">
         <v>56</v>
       </c>
-      <c r="AF24" s="201"/>
-      <c r="AG24" s="202"/>
-      <c r="AH24" s="203"/>
+      <c r="AF24" s="204"/>
+      <c r="AG24" s="205"/>
+      <c r="AH24" s="206"/>
     </row>
     <row r="25" spans="1:34" s="1" customFormat="1" ht="31.5" customHeight="1" thickBot="1">
       <c r="A25" s="53"/>
@@ -4008,29 +4043,29 @@
       <c r="O25" s="168"/>
       <c r="P25" s="169"/>
       <c r="Q25" s="170"/>
-      <c r="R25" s="195"/>
-      <c r="S25" s="196"/>
-      <c r="T25" s="196"/>
-      <c r="U25" s="196"/>
-      <c r="V25" s="197"/>
-      <c r="W25" s="225"/>
-      <c r="X25" s="226"/>
-      <c r="Y25" s="227"/>
+      <c r="R25" s="198"/>
+      <c r="S25" s="199"/>
+      <c r="T25" s="199"/>
+      <c r="U25" s="199"/>
+      <c r="V25" s="200"/>
+      <c r="W25" s="231"/>
+      <c r="X25" s="232"/>
+      <c r="Y25" s="233"/>
       <c r="AB25" s="50" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="AC25" s="51" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="AD25" s="51" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="AE25" s="52" t="s">
         <v>58</v>
       </c>
-      <c r="AF25" s="204"/>
-      <c r="AG25" s="205"/>
-      <c r="AH25" s="206"/>
+      <c r="AF25" s="207"/>
+      <c r="AG25" s="208"/>
+      <c r="AH25" s="209"/>
     </row>
     <row r="26" spans="1:34" s="1" customFormat="1" ht="31.5" customHeight="1">
       <c r="A26" s="89" t="s">
@@ -4054,26 +4089,26 @@
       </c>
       <c r="P26" s="163"/>
       <c r="Q26" s="164"/>
-      <c r="R26" s="189">
+      <c r="R26" s="192">
         <v>200000</v>
       </c>
-      <c r="S26" s="190"/>
-      <c r="T26" s="190"/>
-      <c r="U26" s="190"/>
-      <c r="V26" s="191"/>
-      <c r="W26" s="198" t="s">
-        <v>75</v>
-      </c>
-      <c r="X26" s="199"/>
-      <c r="Y26" s="200"/>
+      <c r="S26" s="193"/>
+      <c r="T26" s="193"/>
+      <c r="U26" s="193"/>
+      <c r="V26" s="194"/>
+      <c r="W26" s="201" t="s">
+        <v>74</v>
+      </c>
+      <c r="X26" s="202"/>
+      <c r="Y26" s="203"/>
       <c r="AB26" s="19" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="AC26" s="20" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="AD26" s="20" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="AE26" s="21" t="s">
         <v>56</v>
@@ -4082,7 +4117,7 @@
     <row r="27" spans="1:34" s="1" customFormat="1" ht="31.5" customHeight="1">
       <c r="A27" s="53"/>
       <c r="B27" s="81" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C27" s="81"/>
       <c r="D27" s="81"/>
@@ -4101,22 +4136,22 @@
       <c r="O27" s="165"/>
       <c r="P27" s="166"/>
       <c r="Q27" s="167"/>
-      <c r="R27" s="192"/>
-      <c r="S27" s="193"/>
-      <c r="T27" s="193"/>
-      <c r="U27" s="193"/>
-      <c r="V27" s="194"/>
-      <c r="W27" s="201"/>
-      <c r="X27" s="202"/>
-      <c r="Y27" s="203"/>
+      <c r="R27" s="195"/>
+      <c r="S27" s="196"/>
+      <c r="T27" s="196"/>
+      <c r="U27" s="196"/>
+      <c r="V27" s="197"/>
+      <c r="W27" s="204"/>
+      <c r="X27" s="205"/>
+      <c r="Y27" s="206"/>
       <c r="AB27" s="31" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="AC27" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="AD27" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AE27" s="32" t="s">
         <v>57</v>
@@ -4144,22 +4179,22 @@
       <c r="O28" s="165"/>
       <c r="P28" s="166"/>
       <c r="Q28" s="167"/>
-      <c r="R28" s="192"/>
-      <c r="S28" s="193"/>
-      <c r="T28" s="193"/>
-      <c r="U28" s="193"/>
-      <c r="V28" s="194"/>
-      <c r="W28" s="201"/>
-      <c r="X28" s="202"/>
-      <c r="Y28" s="203"/>
+      <c r="R28" s="195"/>
+      <c r="S28" s="196"/>
+      <c r="T28" s="196"/>
+      <c r="U28" s="196"/>
+      <c r="V28" s="197"/>
+      <c r="W28" s="204"/>
+      <c r="X28" s="205"/>
+      <c r="Y28" s="206"/>
       <c r="AB28" s="31" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="AC28" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="AD28" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="AE28" s="39" t="s">
         <v>56</v>
@@ -4187,31 +4222,31 @@
       </c>
       <c r="P29" s="163"/>
       <c r="Q29" s="164"/>
-      <c r="R29" s="192"/>
-      <c r="S29" s="193"/>
-      <c r="T29" s="193"/>
-      <c r="U29" s="193"/>
-      <c r="V29" s="194"/>
-      <c r="W29" s="201"/>
-      <c r="X29" s="202"/>
-      <c r="Y29" s="203"/>
+      <c r="R29" s="195"/>
+      <c r="S29" s="196"/>
+      <c r="T29" s="196"/>
+      <c r="U29" s="196"/>
+      <c r="V29" s="197"/>
+      <c r="W29" s="204"/>
+      <c r="X29" s="205"/>
+      <c r="Y29" s="206"/>
       <c r="AB29" s="50" t="s">
+        <v>84</v>
+      </c>
+      <c r="AC29" s="51" t="s">
+        <v>89</v>
+      </c>
+      <c r="AD29" s="51" t="s">
+        <v>83</v>
+      </c>
+      <c r="AE29" s="52" t="s">
         <v>85</v>
-      </c>
-      <c r="AC29" s="51" t="s">
-        <v>90</v>
-      </c>
-      <c r="AD29" s="51" t="s">
-        <v>84</v>
-      </c>
-      <c r="AE29" s="52" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="30" spans="1:34" s="1" customFormat="1" ht="31.5" customHeight="1">
       <c r="A30" s="58"/>
       <c r="B30" s="81" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C30" s="81"/>
       <c r="D30" s="81"/>
@@ -4230,16 +4265,16 @@
       <c r="O30" s="165"/>
       <c r="P30" s="166"/>
       <c r="Q30" s="167"/>
-      <c r="R30" s="192"/>
-      <c r="S30" s="193"/>
-      <c r="T30" s="193"/>
-      <c r="U30" s="193"/>
-      <c r="V30" s="194"/>
-      <c r="W30" s="201"/>
-      <c r="X30" s="202"/>
-      <c r="Y30" s="203"/>
+      <c r="R30" s="195"/>
+      <c r="S30" s="196"/>
+      <c r="T30" s="196"/>
+      <c r="U30" s="196"/>
+      <c r="V30" s="197"/>
+      <c r="W30" s="204"/>
+      <c r="X30" s="205"/>
+      <c r="Y30" s="206"/>
       <c r="AB30" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="AC30" s="2"/>
       <c r="AD30" s="2"/>
@@ -4262,24 +4297,24 @@
       <c r="L31" s="56"/>
       <c r="M31" s="56"/>
       <c r="N31" s="57"/>
-      <c r="O31" s="234" t="s">
+      <c r="O31" s="240" t="s">
         <v>13</v>
       </c>
-      <c r="P31" s="235"/>
-      <c r="Q31" s="236"/>
-      <c r="R31" s="195"/>
-      <c r="S31" s="196"/>
-      <c r="T31" s="196"/>
-      <c r="U31" s="196"/>
-      <c r="V31" s="197"/>
-      <c r="W31" s="204"/>
-      <c r="X31" s="205"/>
-      <c r="Y31" s="206"/>
+      <c r="P31" s="241"/>
+      <c r="Q31" s="242"/>
+      <c r="R31" s="198"/>
+      <c r="S31" s="199"/>
+      <c r="T31" s="199"/>
+      <c r="U31" s="199"/>
+      <c r="V31" s="200"/>
+      <c r="W31" s="207"/>
+      <c r="X31" s="208"/>
+      <c r="Y31" s="209"/>
       <c r="AB31" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="AC31" s="2" t="s">
         <v>92</v>
-      </c>
-      <c r="AC31" s="2" t="s">
-        <v>93</v>
       </c>
       <c r="AD31" s="2"/>
       <c r="AE31" s="2"/>
@@ -4310,16 +4345,16 @@
       </c>
       <c r="P32" s="163"/>
       <c r="Q32" s="164"/>
-      <c r="R32" s="207">
+      <c r="R32" s="210">
         <v>200000</v>
       </c>
-      <c r="S32" s="208"/>
-      <c r="T32" s="208"/>
-      <c r="U32" s="208"/>
-      <c r="V32" s="209"/>
-      <c r="W32" s="216"/>
-      <c r="X32" s="199"/>
-      <c r="Y32" s="200"/>
+      <c r="S32" s="211"/>
+      <c r="T32" s="211"/>
+      <c r="U32" s="211"/>
+      <c r="V32" s="212"/>
+      <c r="W32" s="219"/>
+      <c r="X32" s="202"/>
+      <c r="Y32" s="203"/>
       <c r="AB32" s="2"/>
       <c r="AC32" s="2"/>
       <c r="AD32" s="2"/>
@@ -4347,14 +4382,14 @@
       <c r="O33" s="165"/>
       <c r="P33" s="166"/>
       <c r="Q33" s="167"/>
-      <c r="R33" s="210"/>
-      <c r="S33" s="211"/>
-      <c r="T33" s="211"/>
-      <c r="U33" s="211"/>
-      <c r="V33" s="212"/>
-      <c r="W33" s="201"/>
-      <c r="X33" s="202"/>
-      <c r="Y33" s="203"/>
+      <c r="R33" s="213"/>
+      <c r="S33" s="214"/>
+      <c r="T33" s="214"/>
+      <c r="U33" s="214"/>
+      <c r="V33" s="215"/>
+      <c r="W33" s="204"/>
+      <c r="X33" s="205"/>
+      <c r="Y33" s="206"/>
       <c r="AB33" s="2"/>
       <c r="AC33" s="2"/>
       <c r="AD33" s="2"/>
@@ -4388,14 +4423,14 @@
       <c r="O34" s="168"/>
       <c r="P34" s="169"/>
       <c r="Q34" s="170"/>
-      <c r="R34" s="213"/>
-      <c r="S34" s="214"/>
-      <c r="T34" s="214"/>
-      <c r="U34" s="214"/>
-      <c r="V34" s="215"/>
-      <c r="W34" s="204"/>
-      <c r="X34" s="205"/>
-      <c r="Y34" s="206"/>
+      <c r="R34" s="216"/>
+      <c r="S34" s="217"/>
+      <c r="T34" s="217"/>
+      <c r="U34" s="217"/>
+      <c r="V34" s="218"/>
+      <c r="W34" s="207"/>
+      <c r="X34" s="208"/>
+      <c r="Y34" s="209"/>
       <c r="AB34" s="2"/>
       <c r="AC34" s="2"/>
       <c r="AD34" s="2"/>
@@ -4426,11 +4461,11 @@
       <c r="N35" s="54" t="s">
         <v>40</v>
       </c>
-      <c r="O35" s="234" t="s">
+      <c r="O35" s="240" t="s">
         <v>41</v>
       </c>
-      <c r="P35" s="235"/>
-      <c r="Q35" s="236"/>
+      <c r="P35" s="241"/>
+      <c r="Q35" s="242"/>
       <c r="R35" s="183">
         <v>600000</v>
       </c>
@@ -4438,9 +4473,9 @@
       <c r="T35" s="184"/>
       <c r="U35" s="184"/>
       <c r="V35" s="185"/>
-      <c r="W35" s="217"/>
-      <c r="X35" s="218"/>
-      <c r="Y35" s="219"/>
+      <c r="W35" s="223"/>
+      <c r="X35" s="224"/>
+      <c r="Y35" s="225"/>
       <c r="AB35" s="2"/>
       <c r="AC35" s="2"/>
       <c r="AD35" s="2"/>
@@ -4465,11 +4500,11 @@
       <c r="N36" s="54" t="s">
         <v>40</v>
       </c>
-      <c r="O36" s="234" t="s">
+      <c r="O36" s="240" t="s">
         <v>14</v>
       </c>
-      <c r="P36" s="235"/>
-      <c r="Q36" s="236"/>
+      <c r="P36" s="241"/>
+      <c r="Q36" s="242"/>
       <c r="R36" s="183">
         <v>300000</v>
       </c>
@@ -4477,9 +4512,9 @@
       <c r="T36" s="184"/>
       <c r="U36" s="184"/>
       <c r="V36" s="185"/>
-      <c r="W36" s="217"/>
-      <c r="X36" s="218"/>
-      <c r="Y36" s="219"/>
+      <c r="W36" s="223"/>
+      <c r="X36" s="224"/>
+      <c r="Y36" s="225"/>
       <c r="AB36" s="2"/>
       <c r="AC36" s="2"/>
       <c r="AD36" s="2"/>
@@ -4510,9 +4545,9 @@
       <c r="N37" s="54" t="s">
         <v>40</v>
       </c>
-      <c r="O37" s="237"/>
-      <c r="P37" s="238"/>
-      <c r="Q37" s="239"/>
+      <c r="O37" s="243"/>
+      <c r="P37" s="244"/>
+      <c r="Q37" s="245"/>
       <c r="R37" s="183">
         <v>100000</v>
       </c>
@@ -4520,9 +4555,9 @@
       <c r="T37" s="184"/>
       <c r="U37" s="184"/>
       <c r="V37" s="185"/>
-      <c r="W37" s="217"/>
-      <c r="X37" s="218"/>
-      <c r="Y37" s="219"/>
+      <c r="W37" s="223"/>
+      <c r="X37" s="224"/>
+      <c r="Y37" s="225"/>
       <c r="AB37" s="2"/>
       <c r="AC37" s="2"/>
       <c r="AD37" s="2"/>
@@ -4530,12 +4565,12 @@
     </row>
     <row r="38" spans="1:31" s="1" customFormat="1" ht="31.5" customHeight="1">
       <c r="A38" s="174" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B38" s="175"/>
       <c r="C38" s="176"/>
       <c r="D38" s="186" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E38" s="187"/>
       <c r="F38" s="187"/>
@@ -4554,14 +4589,14 @@
       </c>
       <c r="P38" s="163"/>
       <c r="Q38" s="164"/>
-      <c r="R38" s="258"/>
-      <c r="S38" s="258"/>
-      <c r="T38" s="258"/>
-      <c r="U38" s="258"/>
-      <c r="V38" s="258"/>
-      <c r="W38" s="246"/>
-      <c r="X38" s="247"/>
-      <c r="Y38" s="248"/>
+      <c r="R38" s="189"/>
+      <c r="S38" s="189"/>
+      <c r="T38" s="189"/>
+      <c r="U38" s="189"/>
+      <c r="V38" s="189"/>
+      <c r="W38" s="252"/>
+      <c r="X38" s="253"/>
+      <c r="Y38" s="254"/>
       <c r="AB38" s="2"/>
       <c r="AC38" s="2"/>
       <c r="AD38" s="2"/>
@@ -4572,7 +4607,7 @@
       <c r="B39" s="178"/>
       <c r="C39" s="179"/>
       <c r="D39" s="186" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E39" s="187"/>
       <c r="F39" s="187"/>
@@ -4587,14 +4622,14 @@
       <c r="O39" s="165"/>
       <c r="P39" s="166"/>
       <c r="Q39" s="167"/>
-      <c r="R39" s="259"/>
-      <c r="S39" s="259"/>
-      <c r="T39" s="259"/>
-      <c r="U39" s="259"/>
-      <c r="V39" s="259"/>
-      <c r="W39" s="249"/>
-      <c r="X39" s="250"/>
-      <c r="Y39" s="251"/>
+      <c r="R39" s="190"/>
+      <c r="S39" s="190"/>
+      <c r="T39" s="190"/>
+      <c r="U39" s="190"/>
+      <c r="V39" s="190"/>
+      <c r="W39" s="255"/>
+      <c r="X39" s="256"/>
+      <c r="Y39" s="257"/>
       <c r="AB39" s="2"/>
       <c r="AC39" s="2"/>
       <c r="AD39" s="2"/>
@@ -4622,14 +4657,14 @@
       <c r="O40" s="168"/>
       <c r="P40" s="169"/>
       <c r="Q40" s="170"/>
-      <c r="R40" s="260"/>
-      <c r="S40" s="260"/>
-      <c r="T40" s="260"/>
-      <c r="U40" s="260"/>
-      <c r="V40" s="260"/>
-      <c r="W40" s="252"/>
-      <c r="X40" s="253"/>
-      <c r="Y40" s="254"/>
+      <c r="R40" s="191"/>
+      <c r="S40" s="191"/>
+      <c r="T40" s="191"/>
+      <c r="U40" s="191"/>
+      <c r="V40" s="191"/>
+      <c r="W40" s="258"/>
+      <c r="X40" s="259"/>
+      <c r="Y40" s="260"/>
       <c r="AB40" s="2"/>
       <c r="AC40" s="2"/>
       <c r="AD40" s="2"/>
@@ -4724,7 +4759,7 @@
       <c r="K43" s="79"/>
       <c r="L43" s="80"/>
       <c r="M43" s="65" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="Y43" s="38"/>
       <c r="AB43" s="64"/>
@@ -4748,7 +4783,7 @@
       <c r="K44" s="79"/>
       <c r="L44" s="80"/>
       <c r="M44" s="66" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="N44" s="67"/>
       <c r="O44" s="67"/>
@@ -4783,7 +4818,7 @@
       <c r="K45" s="79"/>
       <c r="L45" s="80"/>
       <c r="M45" s="69" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="N45" s="70"/>
       <c r="O45" s="70"/>
@@ -4818,7 +4853,7 @@
       <c r="K46" s="73"/>
       <c r="L46" s="73"/>
       <c r="M46" s="65" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="Y46" s="38"/>
       <c r="AB46" s="64"/>
@@ -4828,10 +4863,10 @@
     </row>
     <row r="47" spans="1:31" s="13" customFormat="1" ht="20.100000000000001" customHeight="1">
       <c r="A47" s="74" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D47" s="79" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E47" s="79"/>
       <c r="F47" s="79"/>
@@ -4842,7 +4877,7 @@
       <c r="K47" s="79"/>
       <c r="L47" s="80"/>
       <c r="M47" s="65" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="Y47" s="38"/>
       <c r="AB47" s="64"/>
@@ -4852,10 +4887,10 @@
     </row>
     <row r="48" spans="1:31" s="13" customFormat="1" ht="20.100000000000001" customHeight="1">
       <c r="A48" s="74" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D48" s="79" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E48" s="79"/>
       <c r="F48" s="79"/>
@@ -4866,7 +4901,7 @@
       <c r="K48" s="79"/>
       <c r="L48" s="80"/>
       <c r="M48" s="65" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="Y48" s="38"/>
       <c r="AB48" s="64"/>
@@ -4876,10 +4911,10 @@
     </row>
     <row r="49" spans="1:31" s="13" customFormat="1" ht="20.100000000000001" customHeight="1">
       <c r="A49" s="74" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D49" s="77" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E49" s="77"/>
       <c r="F49" s="77"/>
@@ -4890,7 +4925,7 @@
       <c r="K49" s="77"/>
       <c r="L49" s="78"/>
       <c r="M49" s="65" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="Y49" s="38"/>
       <c r="AB49" s="64"/>
@@ -4900,10 +4935,10 @@
     </row>
     <row r="50" spans="1:31" s="13" customFormat="1" ht="20.100000000000001" customHeight="1">
       <c r="A50" s="74" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D50" s="92" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E50" s="92"/>
       <c r="F50" s="92"/>
@@ -4914,7 +4949,7 @@
       <c r="K50" s="92"/>
       <c r="L50" s="93"/>
       <c r="M50" s="65" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="Y50" s="38"/>
       <c r="AB50" s="64"/>
@@ -4934,7 +4969,7 @@
       <c r="K51" s="94"/>
       <c r="L51" s="95"/>
       <c r="M51" s="65" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="Y51" s="38"/>
       <c r="AB51" s="64"/>
@@ -4944,7 +4979,7 @@
     </row>
     <row r="52" spans="1:31" s="1" customFormat="1" ht="35.25" customHeight="1">
       <c r="A52" s="133" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B52" s="134"/>
       <c r="C52" s="134"/>

</xml_diff>

<commit_message>
chore: normalize template certification text font
</commit_message>
<xml_diff>
--- a/직무고시 견적서 양식.xlsx
+++ b/직무고시 견적서 양식.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Master\Documents\Antigravity program\직무고시 견적서\wkace-quotation-jigmu\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE15C472-61A3-41A7-8179-B5BC07E96A17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC5DAEDB-37A8-4C37-B1B4-304E989502A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="견적서" sheetId="1" r:id="rId1"/>
@@ -587,33 +587,7 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">(전기설비 </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="18"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="major"/>
-      </rPr>
-      <t>종합 시험자</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="18"/>
-        <color indexed="8"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="major"/>
-      </rPr>
-      <t xml:space="preserve"> 인증 2026-C1-0040호)</t>
-    </r>
+    <t>(전기설비 종합 시험자 인증 2026-C1-0040호)</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -628,7 +602,7 @@
     <numFmt numFmtId="178" formatCode="0&quot;회&quot;"/>
     <numFmt numFmtId="179" formatCode="yyyy&quot;년&quot;\ m&quot;월&quot;\ d&quot;일&quot;;@"/>
   </numFmts>
-  <fonts count="27">
+  <fonts count="26">
     <font>
       <sz val="11"/>
       <name val="굴림체"/>
@@ -841,15 +815,6 @@
     <font>
       <sz val="10"/>
       <color indexed="8"/>
-      <name val="맑은 고딕"/>
-      <family val="3"/>
-      <charset val="129"/>
-      <scheme val="major"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="1"/>
       <name val="맑은 고딕"/>
       <family val="3"/>
       <charset val="129"/>
@@ -1739,18 +1704,537 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="41" fontId="14" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="14" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="14" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="14" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="14" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="14" fillId="0" borderId="24" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="14" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="14" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="14" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="14" fillId="0" borderId="29" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="14" fillId="0" borderId="31" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="14" fillId="0" borderId="30" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="29" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="31" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="30" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="8" fillId="0" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="8" fillId="0" borderId="27" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="8" fillId="0" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="8" fillId="0" borderId="23" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="8" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="8" fillId="0" borderId="24" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="8" fillId="0" borderId="25" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="8" fillId="0" borderId="28" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="8" fillId="0" borderId="26" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="27" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="23" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="24" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="25" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="28" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="26" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="14" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="14" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="14" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="14" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="14" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="14" fillId="0" borderId="24" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="14" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="14" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="14" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="35" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="40" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="41" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="7" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="7" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="7" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="20" fillId="5" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="10" fillId="3" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="10" fillId="3" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="5" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="39" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1766,530 +2250,11 @@
     <xf numFmtId="0" fontId="21" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="19" fillId="6" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="6" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="10" fillId="3" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="10" fillId="3" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="7" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="7" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="7" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="9" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="20" fillId="5" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="5" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="5" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="5" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="29" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="31" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="30" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="35" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="40" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="41" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="27" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="23" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="24" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="25" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="28" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="26" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="14" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="14" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="14" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="14" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="14" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="14" fillId="0" borderId="24" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="14" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="14" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="14" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="14" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="14" fillId="0" borderId="29" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="14" fillId="0" borderId="31" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="14" fillId="0" borderId="30" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="14" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="14" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="14" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="14" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="14" fillId="0" borderId="24" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="14" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="14" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="14" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="8" fillId="0" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="8" fillId="0" borderId="27" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="8" fillId="0" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="8" fillId="0" borderId="23" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="8" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="8" fillId="0" borderId="24" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="8" fillId="0" borderId="25" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="8" fillId="0" borderId="28" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="8" fillId="0" borderId="26" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -2927,33 +2892,33 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:40" s="1" customFormat="1" ht="54">
-      <c r="A1" s="100" t="s">
+      <c r="A1" s="241" t="s">
         <v>129</v>
       </c>
-      <c r="B1" s="100"/>
-      <c r="C1" s="100"/>
-      <c r="D1" s="100"/>
-      <c r="E1" s="100"/>
-      <c r="F1" s="100"/>
-      <c r="G1" s="100"/>
-      <c r="H1" s="100"/>
-      <c r="I1" s="100"/>
-      <c r="J1" s="100"/>
-      <c r="K1" s="100"/>
-      <c r="L1" s="100"/>
-      <c r="M1" s="100"/>
-      <c r="N1" s="100"/>
-      <c r="O1" s="100"/>
-      <c r="P1" s="100"/>
-      <c r="Q1" s="100"/>
-      <c r="R1" s="100"/>
-      <c r="S1" s="100"/>
-      <c r="T1" s="100"/>
-      <c r="U1" s="100"/>
-      <c r="V1" s="100"/>
-      <c r="W1" s="100"/>
-      <c r="X1" s="100"/>
-      <c r="Y1" s="100"/>
+      <c r="B1" s="241"/>
+      <c r="C1" s="241"/>
+      <c r="D1" s="241"/>
+      <c r="E1" s="241"/>
+      <c r="F1" s="241"/>
+      <c r="G1" s="241"/>
+      <c r="H1" s="241"/>
+      <c r="I1" s="241"/>
+      <c r="J1" s="241"/>
+      <c r="K1" s="241"/>
+      <c r="L1" s="241"/>
+      <c r="M1" s="241"/>
+      <c r="N1" s="241"/>
+      <c r="O1" s="241"/>
+      <c r="P1" s="241"/>
+      <c r="Q1" s="241"/>
+      <c r="R1" s="241"/>
+      <c r="S1" s="241"/>
+      <c r="T1" s="241"/>
+      <c r="U1" s="241"/>
+      <c r="V1" s="241"/>
+      <c r="W1" s="241"/>
+      <c r="X1" s="241"/>
+      <c r="Y1" s="241"/>
       <c r="AB1" s="2"/>
       <c r="AC1" s="3"/>
       <c r="AD1" s="3"/>
@@ -3008,33 +2973,33 @@
       <c r="AN2" s="3"/>
     </row>
     <row r="3" spans="1:40" s="1" customFormat="1" ht="26.25">
-      <c r="A3" s="101" t="s">
+      <c r="A3" s="242" t="s">
         <v>134</v>
       </c>
-      <c r="B3" s="101"/>
-      <c r="C3" s="101"/>
-      <c r="D3" s="101"/>
-      <c r="E3" s="101"/>
-      <c r="F3" s="101"/>
-      <c r="G3" s="101"/>
-      <c r="H3" s="101"/>
-      <c r="I3" s="101"/>
-      <c r="J3" s="101"/>
-      <c r="K3" s="101"/>
-      <c r="L3" s="101"/>
-      <c r="M3" s="101"/>
-      <c r="N3" s="101"/>
-      <c r="O3" s="101"/>
-      <c r="P3" s="101"/>
-      <c r="Q3" s="101"/>
-      <c r="R3" s="101"/>
-      <c r="S3" s="101"/>
-      <c r="T3" s="101"/>
-      <c r="U3" s="101"/>
-      <c r="V3" s="101"/>
-      <c r="W3" s="101"/>
-      <c r="X3" s="101"/>
-      <c r="Y3" s="101"/>
+      <c r="B3" s="242"/>
+      <c r="C3" s="242"/>
+      <c r="D3" s="242"/>
+      <c r="E3" s="242"/>
+      <c r="F3" s="242"/>
+      <c r="G3" s="242"/>
+      <c r="H3" s="242"/>
+      <c r="I3" s="242"/>
+      <c r="J3" s="242"/>
+      <c r="K3" s="242"/>
+      <c r="L3" s="242"/>
+      <c r="M3" s="242"/>
+      <c r="N3" s="242"/>
+      <c r="O3" s="242"/>
+      <c r="P3" s="242"/>
+      <c r="Q3" s="242"/>
+      <c r="R3" s="242"/>
+      <c r="S3" s="242"/>
+      <c r="T3" s="242"/>
+      <c r="U3" s="242"/>
+      <c r="V3" s="242"/>
+      <c r="W3" s="242"/>
+      <c r="X3" s="242"/>
+      <c r="Y3" s="242"/>
       <c r="AB3" s="2"/>
       <c r="AC3" s="3"/>
       <c r="AD3" s="3"/>
@@ -3134,38 +3099,38 @@
         <v>95</v>
       </c>
       <c r="B6" s="8"/>
-      <c r="C6" s="102">
+      <c r="C6" s="243">
         <f ca="1">TODAY()</f>
         <v>46148</v>
       </c>
-      <c r="D6" s="102"/>
-      <c r="E6" s="102"/>
-      <c r="F6" s="102"/>
+      <c r="D6" s="243"/>
+      <c r="E6" s="243"/>
+      <c r="F6" s="243"/>
       <c r="G6" s="8"/>
       <c r="H6" s="8"/>
       <c r="I6" s="8"/>
       <c r="J6" s="9"/>
-      <c r="K6" s="125" t="s">
+      <c r="K6" s="230" t="s">
         <v>1</v>
       </c>
-      <c r="L6" s="118" t="s">
+      <c r="L6" s="222" t="s">
         <v>2</v>
       </c>
-      <c r="M6" s="119"/>
-      <c r="N6" s="120"/>
-      <c r="O6" s="112" t="s">
+      <c r="M6" s="223"/>
+      <c r="N6" s="224"/>
+      <c r="O6" s="249" t="s">
         <v>18</v>
       </c>
-      <c r="P6" s="113"/>
-      <c r="Q6" s="113"/>
-      <c r="R6" s="113"/>
-      <c r="S6" s="113"/>
-      <c r="T6" s="113"/>
-      <c r="U6" s="113"/>
-      <c r="V6" s="113"/>
-      <c r="W6" s="113"/>
-      <c r="X6" s="113"/>
-      <c r="Y6" s="114"/>
+      <c r="P6" s="250"/>
+      <c r="Q6" s="250"/>
+      <c r="R6" s="250"/>
+      <c r="S6" s="250"/>
+      <c r="T6" s="250"/>
+      <c r="U6" s="250"/>
+      <c r="V6" s="250"/>
+      <c r="W6" s="250"/>
+      <c r="X6" s="250"/>
+      <c r="Y6" s="251"/>
       <c r="AB6" s="2"/>
       <c r="AC6" s="3"/>
       <c r="AD6" s="3"/>
@@ -3195,29 +3160,29 @@
       <c r="H7" s="8"/>
       <c r="I7" s="8"/>
       <c r="J7" s="9"/>
-      <c r="K7" s="126"/>
-      <c r="L7" s="104" t="s">
+      <c r="K7" s="231"/>
+      <c r="L7" s="229" t="s">
         <v>22</v>
       </c>
-      <c r="M7" s="105"/>
-      <c r="N7" s="106"/>
-      <c r="O7" s="115" t="s">
+      <c r="M7" s="192"/>
+      <c r="N7" s="193"/>
+      <c r="O7" s="197" t="s">
         <v>17</v>
       </c>
-      <c r="P7" s="116"/>
-      <c r="Q7" s="116"/>
-      <c r="R7" s="116"/>
-      <c r="S7" s="124" t="s">
+      <c r="P7" s="198"/>
+      <c r="Q7" s="198"/>
+      <c r="R7" s="198"/>
+      <c r="S7" s="228" t="s">
         <v>25</v>
       </c>
-      <c r="T7" s="105"/>
-      <c r="U7" s="106"/>
-      <c r="V7" s="115" t="s">
+      <c r="T7" s="192"/>
+      <c r="U7" s="193"/>
+      <c r="V7" s="197" t="s">
         <v>20</v>
       </c>
-      <c r="W7" s="116"/>
-      <c r="X7" s="116"/>
-      <c r="Y7" s="117"/>
+      <c r="W7" s="198"/>
+      <c r="X7" s="198"/>
+      <c r="Y7" s="221"/>
       <c r="AB7" s="2"/>
       <c r="AC7" s="2"/>
       <c r="AD7" s="2"/>
@@ -3234,25 +3199,25 @@
       <c r="H8" s="11"/>
       <c r="I8" s="11"/>
       <c r="J8" s="12"/>
-      <c r="K8" s="126"/>
-      <c r="L8" s="104" t="s">
+      <c r="K8" s="231"/>
+      <c r="L8" s="229" t="s">
         <v>21</v>
       </c>
-      <c r="M8" s="105"/>
-      <c r="N8" s="106"/>
-      <c r="O8" s="115" t="s">
+      <c r="M8" s="192"/>
+      <c r="N8" s="193"/>
+      <c r="O8" s="197" t="s">
         <v>128</v>
       </c>
-      <c r="P8" s="116"/>
-      <c r="Q8" s="116"/>
-      <c r="R8" s="116"/>
-      <c r="S8" s="116"/>
-      <c r="T8" s="116"/>
-      <c r="U8" s="116"/>
-      <c r="V8" s="116"/>
-      <c r="W8" s="116"/>
-      <c r="X8" s="116"/>
-      <c r="Y8" s="117"/>
+      <c r="P8" s="198"/>
+      <c r="Q8" s="198"/>
+      <c r="R8" s="198"/>
+      <c r="S8" s="198"/>
+      <c r="T8" s="198"/>
+      <c r="U8" s="198"/>
+      <c r="V8" s="198"/>
+      <c r="W8" s="198"/>
+      <c r="X8" s="198"/>
+      <c r="Y8" s="221"/>
       <c r="AA8" s="2"/>
       <c r="AB8" s="2"/>
       <c r="AC8" s="2"/>
@@ -3272,29 +3237,29 @@
       <c r="H9" s="10"/>
       <c r="I9" s="8"/>
       <c r="J9" s="10"/>
-      <c r="K9" s="126"/>
-      <c r="L9" s="104" t="s">
+      <c r="K9" s="231"/>
+      <c r="L9" s="229" t="s">
         <v>23</v>
       </c>
-      <c r="M9" s="105"/>
-      <c r="N9" s="106"/>
-      <c r="O9" s="115" t="s">
+      <c r="M9" s="192"/>
+      <c r="N9" s="193"/>
+      <c r="O9" s="197" t="s">
         <v>9</v>
       </c>
-      <c r="P9" s="116"/>
-      <c r="Q9" s="116"/>
-      <c r="R9" s="116"/>
-      <c r="S9" s="136" t="s">
+      <c r="P9" s="198"/>
+      <c r="Q9" s="198"/>
+      <c r="R9" s="198"/>
+      <c r="S9" s="191" t="s">
         <v>26</v>
       </c>
-      <c r="T9" s="105"/>
-      <c r="U9" s="106"/>
-      <c r="V9" s="142" t="s">
+      <c r="T9" s="192"/>
+      <c r="U9" s="193"/>
+      <c r="V9" s="201" t="s">
         <v>31</v>
       </c>
-      <c r="W9" s="143"/>
-      <c r="X9" s="143"/>
-      <c r="Y9" s="144"/>
+      <c r="W9" s="202"/>
+      <c r="X9" s="202"/>
+      <c r="Y9" s="203"/>
       <c r="AB9" s="2"/>
       <c r="AC9" s="2"/>
       <c r="AD9" s="2"/>
@@ -3313,29 +3278,29 @@
       <c r="H10" s="10"/>
       <c r="I10" s="8"/>
       <c r="J10" s="9"/>
-      <c r="K10" s="127"/>
-      <c r="L10" s="109" t="s">
+      <c r="K10" s="232"/>
+      <c r="L10" s="246" t="s">
         <v>24</v>
       </c>
-      <c r="M10" s="110"/>
-      <c r="N10" s="111"/>
-      <c r="O10" s="140" t="s">
+      <c r="M10" s="247"/>
+      <c r="N10" s="248"/>
+      <c r="O10" s="199" t="s">
         <v>76</v>
       </c>
-      <c r="P10" s="141"/>
-      <c r="Q10" s="141"/>
-      <c r="R10" s="141"/>
-      <c r="S10" s="137" t="s">
+      <c r="P10" s="200"/>
+      <c r="Q10" s="200"/>
+      <c r="R10" s="200"/>
+      <c r="S10" s="194" t="s">
         <v>63</v>
       </c>
-      <c r="T10" s="138"/>
-      <c r="U10" s="139"/>
-      <c r="V10" s="140" t="s">
+      <c r="T10" s="195"/>
+      <c r="U10" s="196"/>
+      <c r="V10" s="199" t="s">
         <v>77</v>
       </c>
-      <c r="W10" s="141"/>
-      <c r="X10" s="141"/>
-      <c r="Y10" s="145"/>
+      <c r="W10" s="200"/>
+      <c r="X10" s="200"/>
+      <c r="Y10" s="204"/>
       <c r="AB10" s="2"/>
       <c r="AC10" s="2"/>
       <c r="AD10" s="2"/>
@@ -3386,10 +3351,10 @@
       <c r="E12" s="15"/>
       <c r="F12" s="15"/>
       <c r="G12" s="15"/>
-      <c r="H12" s="103"/>
-      <c r="I12" s="103"/>
-      <c r="J12" s="103"/>
-      <c r="K12" s="103"/>
+      <c r="H12" s="135"/>
+      <c r="I12" s="135"/>
+      <c r="J12" s="135"/>
+      <c r="K12" s="135"/>
       <c r="L12" s="15"/>
       <c r="M12" s="16"/>
       <c r="N12" s="14" t="s">
@@ -3447,10 +3412,10 @@
         <v>105</v>
       </c>
       <c r="Q13" s="3"/>
-      <c r="R13" s="108" t="s">
+      <c r="R13" s="245" t="s">
         <v>119</v>
       </c>
-      <c r="S13" s="108"/>
+      <c r="S13" s="245"/>
       <c r="T13" s="23" t="s">
         <v>120</v>
       </c>
@@ -3502,10 +3467,10 @@
         <v>106</v>
       </c>
       <c r="Q14" s="10"/>
-      <c r="R14" s="107" t="s">
+      <c r="R14" s="244" t="s">
         <v>122</v>
       </c>
-      <c r="S14" s="107"/>
+      <c r="S14" s="244"/>
       <c r="T14" s="23" t="s">
         <v>120</v>
       </c>
@@ -3549,10 +3514,10 @@
         <v>107</v>
       </c>
       <c r="Q15" s="10"/>
-      <c r="R15" s="107" t="s">
+      <c r="R15" s="244" t="s">
         <v>122</v>
       </c>
-      <c r="S15" s="107"/>
+      <c r="S15" s="244"/>
       <c r="T15" s="23" t="s">
         <v>120</v>
       </c>
@@ -3604,10 +3569,10 @@
         <v>108</v>
       </c>
       <c r="Q16" s="10"/>
-      <c r="R16" s="107" t="s">
+      <c r="R16" s="244" t="s">
         <v>122</v>
       </c>
-      <c r="S16" s="107"/>
+      <c r="S16" s="244"/>
       <c r="T16" s="23" t="s">
         <v>120</v>
       </c>
@@ -3624,21 +3589,21 @@
       <c r="AE16" s="39"/>
     </row>
     <row r="17" spans="1:34" s="1" customFormat="1" ht="20.100000000000001" customHeight="1" thickBot="1">
-      <c r="A17" s="121" t="s">
+      <c r="A17" s="225" t="s">
         <v>78</v>
       </c>
-      <c r="B17" s="122"/>
-      <c r="C17" s="122"/>
-      <c r="D17" s="122"/>
-      <c r="E17" s="122"/>
-      <c r="F17" s="122"/>
-      <c r="G17" s="122"/>
-      <c r="H17" s="122"/>
-      <c r="I17" s="122"/>
-      <c r="J17" s="122"/>
-      <c r="K17" s="122"/>
-      <c r="L17" s="122"/>
-      <c r="M17" s="123"/>
+      <c r="B17" s="226"/>
+      <c r="C17" s="226"/>
+      <c r="D17" s="226"/>
+      <c r="E17" s="226"/>
+      <c r="F17" s="226"/>
+      <c r="G17" s="226"/>
+      <c r="H17" s="226"/>
+      <c r="I17" s="226"/>
+      <c r="J17" s="226"/>
+      <c r="K17" s="226"/>
+      <c r="L17" s="226"/>
+      <c r="M17" s="227"/>
       <c r="N17" s="40"/>
       <c r="O17" s="41" t="s">
         <v>126</v>
@@ -3669,44 +3634,44 @@
       </c>
     </row>
     <row r="18" spans="1:34" s="45" customFormat="1" ht="39.950000000000003" customHeight="1">
-      <c r="A18" s="146" t="s">
+      <c r="A18" s="205" t="s">
         <v>68</v>
       </c>
-      <c r="B18" s="147"/>
-      <c r="C18" s="147"/>
-      <c r="D18" s="147"/>
-      <c r="E18" s="147"/>
-      <c r="F18" s="147"/>
-      <c r="G18" s="147"/>
-      <c r="H18" s="147"/>
-      <c r="I18" s="148"/>
-      <c r="J18" s="97" t="s">
+      <c r="B18" s="206"/>
+      <c r="C18" s="206"/>
+      <c r="D18" s="206"/>
+      <c r="E18" s="206"/>
+      <c r="F18" s="206"/>
+      <c r="G18" s="206"/>
+      <c r="H18" s="206"/>
+      <c r="I18" s="207"/>
+      <c r="J18" s="238" t="s">
         <v>0</v>
       </c>
-      <c r="K18" s="98"/>
-      <c r="L18" s="98"/>
-      <c r="M18" s="99">
+      <c r="K18" s="239"/>
+      <c r="L18" s="239"/>
+      <c r="M18" s="240">
         <f>U41</f>
         <v>1600000</v>
       </c>
-      <c r="N18" s="99"/>
-      <c r="O18" s="99"/>
-      <c r="P18" s="99"/>
-      <c r="Q18" s="99"/>
+      <c r="N18" s="240"/>
+      <c r="O18" s="240"/>
+      <c r="P18" s="240"/>
+      <c r="Q18" s="240"/>
       <c r="R18" s="43" t="s">
         <v>28</v>
       </c>
       <c r="S18" s="43" t="s">
         <v>55</v>
       </c>
-      <c r="T18" s="96">
+      <c r="T18" s="237">
         <f>U41</f>
         <v>1600000</v>
       </c>
-      <c r="U18" s="96"/>
-      <c r="V18" s="96"/>
-      <c r="W18" s="96"/>
-      <c r="X18" s="96"/>
+      <c r="U18" s="237"/>
+      <c r="V18" s="237"/>
+      <c r="W18" s="237"/>
+      <c r="X18" s="237"/>
       <c r="Y18" s="44" t="s">
         <v>54</v>
       </c>
@@ -3724,41 +3689,41 @@
       </c>
     </row>
     <row r="19" spans="1:34" s="1" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A19" s="128" t="s">
+      <c r="A19" s="134" t="s">
         <v>16</v>
       </c>
-      <c r="B19" s="103"/>
-      <c r="C19" s="103"/>
-      <c r="D19" s="103"/>
-      <c r="E19" s="103"/>
-      <c r="F19" s="103"/>
-      <c r="G19" s="103"/>
-      <c r="H19" s="103"/>
-      <c r="I19" s="129"/>
-      <c r="J19" s="237" t="s">
+      <c r="B19" s="135"/>
+      <c r="C19" s="135"/>
+      <c r="D19" s="135"/>
+      <c r="E19" s="135"/>
+      <c r="F19" s="135"/>
+      <c r="G19" s="135"/>
+      <c r="H19" s="135"/>
+      <c r="I19" s="136"/>
+      <c r="J19" s="113" t="s">
         <v>59</v>
       </c>
-      <c r="K19" s="238"/>
-      <c r="L19" s="238"/>
-      <c r="M19" s="238"/>
-      <c r="N19" s="239"/>
-      <c r="O19" s="246" t="s">
+      <c r="K19" s="114"/>
+      <c r="L19" s="114"/>
+      <c r="M19" s="114"/>
+      <c r="N19" s="115"/>
+      <c r="O19" s="128" t="s">
         <v>61</v>
       </c>
-      <c r="P19" s="247"/>
-      <c r="Q19" s="248"/>
-      <c r="R19" s="128" t="s">
+      <c r="P19" s="129"/>
+      <c r="Q19" s="130"/>
+      <c r="R19" s="134" t="s">
         <v>43</v>
       </c>
-      <c r="S19" s="103"/>
-      <c r="T19" s="103"/>
-      <c r="U19" s="103"/>
-      <c r="V19" s="129"/>
-      <c r="W19" s="128" t="s">
+      <c r="S19" s="135"/>
+      <c r="T19" s="135"/>
+      <c r="U19" s="135"/>
+      <c r="V19" s="136"/>
+      <c r="W19" s="134" t="s">
         <v>42</v>
       </c>
-      <c r="X19" s="103"/>
-      <c r="Y19" s="129"/>
+      <c r="X19" s="135"/>
+      <c r="Y19" s="136"/>
       <c r="AB19" s="31" t="s">
         <v>84</v>
       </c>
@@ -3773,15 +3738,15 @@
       </c>
     </row>
     <row r="20" spans="1:34" s="1" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A20" s="130"/>
-      <c r="B20" s="131"/>
-      <c r="C20" s="131"/>
-      <c r="D20" s="131"/>
-      <c r="E20" s="131"/>
-      <c r="F20" s="131"/>
-      <c r="G20" s="131"/>
-      <c r="H20" s="131"/>
-      <c r="I20" s="132"/>
+      <c r="A20" s="137"/>
+      <c r="B20" s="138"/>
+      <c r="C20" s="138"/>
+      <c r="D20" s="138"/>
+      <c r="E20" s="138"/>
+      <c r="F20" s="138"/>
+      <c r="G20" s="138"/>
+      <c r="H20" s="138"/>
+      <c r="I20" s="139"/>
       <c r="J20" s="46" t="s">
         <v>27</v>
       </c>
@@ -3797,17 +3762,17 @@
       <c r="N20" s="49" t="s">
         <v>58</v>
       </c>
-      <c r="O20" s="249"/>
-      <c r="P20" s="250"/>
-      <c r="Q20" s="251"/>
-      <c r="R20" s="130"/>
-      <c r="S20" s="131"/>
-      <c r="T20" s="131"/>
-      <c r="U20" s="131"/>
-      <c r="V20" s="132"/>
-      <c r="W20" s="130"/>
-      <c r="X20" s="131"/>
-      <c r="Y20" s="132"/>
+      <c r="O20" s="131"/>
+      <c r="P20" s="132"/>
+      <c r="Q20" s="133"/>
+      <c r="R20" s="137"/>
+      <c r="S20" s="138"/>
+      <c r="T20" s="138"/>
+      <c r="U20" s="138"/>
+      <c r="V20" s="139"/>
+      <c r="W20" s="137"/>
+      <c r="X20" s="138"/>
+      <c r="Y20" s="139"/>
       <c r="AB20" s="31" t="s">
         <v>84</v>
       </c>
@@ -3822,42 +3787,42 @@
       </c>
     </row>
     <row r="21" spans="1:34" s="1" customFormat="1" ht="31.5" customHeight="1" thickBot="1">
-      <c r="A21" s="89" t="s">
+      <c r="A21" s="95" t="s">
         <v>60</v>
       </c>
-      <c r="B21" s="90"/>
-      <c r="C21" s="90"/>
-      <c r="D21" s="90"/>
-      <c r="E21" s="90"/>
-      <c r="F21" s="90"/>
-      <c r="G21" s="90"/>
-      <c r="H21" s="90"/>
-      <c r="I21" s="91"/>
-      <c r="J21" s="234" t="s">
+      <c r="B21" s="96"/>
+      <c r="C21" s="96"/>
+      <c r="D21" s="96"/>
+      <c r="E21" s="96"/>
+      <c r="F21" s="96"/>
+      <c r="G21" s="96"/>
+      <c r="H21" s="96"/>
+      <c r="I21" s="97"/>
+      <c r="J21" s="110" t="s">
         <v>33</v>
       </c>
-      <c r="K21" s="235"/>
-      <c r="L21" s="235"/>
-      <c r="M21" s="235"/>
-      <c r="N21" s="236"/>
-      <c r="O21" s="243" t="s">
+      <c r="K21" s="111"/>
+      <c r="L21" s="111"/>
+      <c r="M21" s="111"/>
+      <c r="N21" s="112"/>
+      <c r="O21" s="116" t="s">
         <v>30</v>
       </c>
-      <c r="P21" s="244"/>
-      <c r="Q21" s="245"/>
-      <c r="R21" s="220">
+      <c r="P21" s="117"/>
+      <c r="Q21" s="118"/>
+      <c r="R21" s="159">
         <f>150000*8</f>
         <v>1200000</v>
       </c>
-      <c r="S21" s="221"/>
-      <c r="T21" s="221"/>
-      <c r="U21" s="221"/>
-      <c r="V21" s="222"/>
-      <c r="W21" s="223" t="s">
+      <c r="S21" s="160"/>
+      <c r="T21" s="160"/>
+      <c r="U21" s="160"/>
+      <c r="V21" s="161"/>
+      <c r="W21" s="92" t="s">
         <v>125</v>
       </c>
-      <c r="X21" s="224"/>
-      <c r="Y21" s="225"/>
+      <c r="X21" s="93"/>
+      <c r="Y21" s="94"/>
       <c r="AB21" s="50" t="s">
         <v>84</v>
       </c>
@@ -3872,37 +3837,37 @@
       </c>
     </row>
     <row r="22" spans="1:34" s="1" customFormat="1" ht="31.5" customHeight="1">
-      <c r="A22" s="89" t="s">
+      <c r="A22" s="95" t="s">
         <v>45</v>
       </c>
-      <c r="B22" s="90"/>
-      <c r="C22" s="90"/>
-      <c r="D22" s="90"/>
-      <c r="E22" s="90"/>
-      <c r="F22" s="90"/>
-      <c r="G22" s="90"/>
-      <c r="H22" s="90"/>
-      <c r="I22" s="91"/>
-      <c r="J22" s="234"/>
-      <c r="K22" s="235"/>
-      <c r="L22" s="235"/>
-      <c r="M22" s="235"/>
-      <c r="N22" s="236"/>
-      <c r="O22" s="162" t="s">
+      <c r="B22" s="96"/>
+      <c r="C22" s="96"/>
+      <c r="D22" s="96"/>
+      <c r="E22" s="96"/>
+      <c r="F22" s="96"/>
+      <c r="G22" s="96"/>
+      <c r="H22" s="96"/>
+      <c r="I22" s="97"/>
+      <c r="J22" s="110"/>
+      <c r="K22" s="111"/>
+      <c r="L22" s="111"/>
+      <c r="M22" s="111"/>
+      <c r="N22" s="112"/>
+      <c r="O22" s="119" t="s">
         <v>10</v>
       </c>
-      <c r="P22" s="163"/>
-      <c r="Q22" s="164"/>
-      <c r="R22" s="192">
+      <c r="P22" s="120"/>
+      <c r="Q22" s="121"/>
+      <c r="R22" s="140">
         <v>200000</v>
       </c>
-      <c r="S22" s="193"/>
-      <c r="T22" s="193"/>
-      <c r="U22" s="193"/>
-      <c r="V22" s="194"/>
-      <c r="W22" s="201"/>
-      <c r="X22" s="226"/>
-      <c r="Y22" s="227"/>
+      <c r="S22" s="141"/>
+      <c r="T22" s="141"/>
+      <c r="U22" s="141"/>
+      <c r="V22" s="142"/>
+      <c r="W22" s="77"/>
+      <c r="X22" s="162"/>
+      <c r="Y22" s="163"/>
       <c r="AB22" s="19" t="s">
         <v>79</v>
       </c>
@@ -3915,24 +3880,24 @@
       <c r="AE22" s="21" t="s">
         <v>56</v>
       </c>
-      <c r="AF22" s="201" t="s">
+      <c r="AF22" s="77" t="s">
         <v>94</v>
       </c>
-      <c r="AG22" s="202"/>
-      <c r="AH22" s="203"/>
+      <c r="AG22" s="78"/>
+      <c r="AH22" s="79"/>
     </row>
     <row r="23" spans="1:34" s="1" customFormat="1" ht="31.5" customHeight="1">
       <c r="A23" s="53"/>
-      <c r="B23" s="81" t="s">
+      <c r="B23" s="254" t="s">
         <v>93</v>
       </c>
-      <c r="C23" s="81"/>
-      <c r="D23" s="81"/>
-      <c r="E23" s="81"/>
-      <c r="F23" s="81"/>
-      <c r="G23" s="81"/>
-      <c r="H23" s="81"/>
-      <c r="I23" s="82"/>
+      <c r="C23" s="254"/>
+      <c r="D23" s="254"/>
+      <c r="E23" s="254"/>
+      <c r="F23" s="254"/>
+      <c r="G23" s="254"/>
+      <c r="H23" s="254"/>
+      <c r="I23" s="255"/>
       <c r="J23" s="54"/>
       <c r="K23" s="54" t="s">
         <v>40</v>
@@ -3946,17 +3911,17 @@
       <c r="N23" s="54" t="s">
         <v>40</v>
       </c>
-      <c r="O23" s="165"/>
-      <c r="P23" s="166"/>
-      <c r="Q23" s="167"/>
-      <c r="R23" s="195"/>
-      <c r="S23" s="196"/>
-      <c r="T23" s="196"/>
-      <c r="U23" s="196"/>
-      <c r="V23" s="197"/>
-      <c r="W23" s="228"/>
-      <c r="X23" s="229"/>
-      <c r="Y23" s="230"/>
+      <c r="O23" s="122"/>
+      <c r="P23" s="123"/>
+      <c r="Q23" s="124"/>
+      <c r="R23" s="143"/>
+      <c r="S23" s="144"/>
+      <c r="T23" s="144"/>
+      <c r="U23" s="144"/>
+      <c r="V23" s="145"/>
+      <c r="W23" s="164"/>
+      <c r="X23" s="165"/>
+      <c r="Y23" s="166"/>
       <c r="AB23" s="31" t="s">
         <v>79</v>
       </c>
@@ -3969,22 +3934,22 @@
       <c r="AE23" s="32" t="s">
         <v>57</v>
       </c>
-      <c r="AF23" s="204"/>
-      <c r="AG23" s="205"/>
-      <c r="AH23" s="206"/>
+      <c r="AF23" s="80"/>
+      <c r="AG23" s="81"/>
+      <c r="AH23" s="82"/>
     </row>
     <row r="24" spans="1:34" s="1" customFormat="1" ht="31.5" customHeight="1">
       <c r="A24" s="53"/>
-      <c r="B24" s="81" t="s">
+      <c r="B24" s="254" t="s">
         <v>44</v>
       </c>
-      <c r="C24" s="81"/>
-      <c r="D24" s="81"/>
-      <c r="E24" s="81"/>
-      <c r="F24" s="81"/>
-      <c r="G24" s="81"/>
-      <c r="H24" s="81"/>
-      <c r="I24" s="82"/>
+      <c r="C24" s="254"/>
+      <c r="D24" s="254"/>
+      <c r="E24" s="254"/>
+      <c r="F24" s="254"/>
+      <c r="G24" s="254"/>
+      <c r="H24" s="254"/>
+      <c r="I24" s="255"/>
       <c r="J24" s="54"/>
       <c r="K24" s="54"/>
       <c r="L24" s="54"/>
@@ -3992,17 +3957,17 @@
       <c r="N24" s="54" t="s">
         <v>40</v>
       </c>
-      <c r="O24" s="165"/>
-      <c r="P24" s="166"/>
-      <c r="Q24" s="167"/>
-      <c r="R24" s="195"/>
-      <c r="S24" s="196"/>
-      <c r="T24" s="196"/>
-      <c r="U24" s="196"/>
-      <c r="V24" s="197"/>
-      <c r="W24" s="228"/>
-      <c r="X24" s="229"/>
-      <c r="Y24" s="230"/>
+      <c r="O24" s="122"/>
+      <c r="P24" s="123"/>
+      <c r="Q24" s="124"/>
+      <c r="R24" s="143"/>
+      <c r="S24" s="144"/>
+      <c r="T24" s="144"/>
+      <c r="U24" s="144"/>
+      <c r="V24" s="145"/>
+      <c r="W24" s="164"/>
+      <c r="X24" s="165"/>
+      <c r="Y24" s="166"/>
       <c r="AB24" s="31" t="s">
         <v>79</v>
       </c>
@@ -4015,22 +3980,22 @@
       <c r="AE24" s="39" t="s">
         <v>56</v>
       </c>
-      <c r="AF24" s="204"/>
-      <c r="AG24" s="205"/>
-      <c r="AH24" s="206"/>
+      <c r="AF24" s="80"/>
+      <c r="AG24" s="81"/>
+      <c r="AH24" s="82"/>
     </row>
     <row r="25" spans="1:34" s="1" customFormat="1" ht="31.5" customHeight="1" thickBot="1">
       <c r="A25" s="53"/>
-      <c r="B25" s="81" t="s">
+      <c r="B25" s="254" t="s">
         <v>3</v>
       </c>
-      <c r="C25" s="81"/>
-      <c r="D25" s="81"/>
-      <c r="E25" s="81"/>
-      <c r="F25" s="81"/>
-      <c r="G25" s="81"/>
-      <c r="H25" s="81"/>
-      <c r="I25" s="82"/>
+      <c r="C25" s="254"/>
+      <c r="D25" s="254"/>
+      <c r="E25" s="254"/>
+      <c r="F25" s="254"/>
+      <c r="G25" s="254"/>
+      <c r="H25" s="254"/>
+      <c r="I25" s="255"/>
       <c r="J25" s="54"/>
       <c r="K25" s="54"/>
       <c r="L25" s="54" t="s">
@@ -4040,17 +4005,17 @@
       <c r="N25" s="54" t="s">
         <v>40</v>
       </c>
-      <c r="O25" s="168"/>
-      <c r="P25" s="169"/>
-      <c r="Q25" s="170"/>
-      <c r="R25" s="198"/>
-      <c r="S25" s="199"/>
-      <c r="T25" s="199"/>
-      <c r="U25" s="199"/>
-      <c r="V25" s="200"/>
-      <c r="W25" s="231"/>
-      <c r="X25" s="232"/>
-      <c r="Y25" s="233"/>
+      <c r="O25" s="125"/>
+      <c r="P25" s="126"/>
+      <c r="Q25" s="127"/>
+      <c r="R25" s="146"/>
+      <c r="S25" s="147"/>
+      <c r="T25" s="147"/>
+      <c r="U25" s="147"/>
+      <c r="V25" s="148"/>
+      <c r="W25" s="167"/>
+      <c r="X25" s="168"/>
+      <c r="Y25" s="169"/>
       <c r="AB25" s="50" t="s">
         <v>79</v>
       </c>
@@ -4063,44 +4028,44 @@
       <c r="AE25" s="52" t="s">
         <v>58</v>
       </c>
-      <c r="AF25" s="207"/>
-      <c r="AG25" s="208"/>
-      <c r="AH25" s="209"/>
+      <c r="AF25" s="83"/>
+      <c r="AG25" s="84"/>
+      <c r="AH25" s="85"/>
     </row>
     <row r="26" spans="1:34" s="1" customFormat="1" ht="31.5" customHeight="1">
-      <c r="A26" s="89" t="s">
+      <c r="A26" s="95" t="s">
         <v>46</v>
       </c>
-      <c r="B26" s="90"/>
-      <c r="C26" s="90"/>
-      <c r="D26" s="90"/>
-      <c r="E26" s="90"/>
-      <c r="F26" s="90"/>
-      <c r="G26" s="90"/>
-      <c r="H26" s="90"/>
-      <c r="I26" s="91"/>
+      <c r="B26" s="96"/>
+      <c r="C26" s="96"/>
+      <c r="D26" s="96"/>
+      <c r="E26" s="96"/>
+      <c r="F26" s="96"/>
+      <c r="G26" s="96"/>
+      <c r="H26" s="96"/>
+      <c r="I26" s="97"/>
       <c r="J26" s="55"/>
       <c r="K26" s="56"/>
       <c r="L26" s="56"/>
       <c r="M26" s="56"/>
       <c r="N26" s="57"/>
-      <c r="O26" s="162" t="s">
+      <c r="O26" s="119" t="s">
         <v>11</v>
       </c>
-      <c r="P26" s="163"/>
-      <c r="Q26" s="164"/>
-      <c r="R26" s="192">
+      <c r="P26" s="120"/>
+      <c r="Q26" s="121"/>
+      <c r="R26" s="140">
         <v>200000</v>
       </c>
-      <c r="S26" s="193"/>
-      <c r="T26" s="193"/>
-      <c r="U26" s="193"/>
-      <c r="V26" s="194"/>
-      <c r="W26" s="201" t="s">
+      <c r="S26" s="141"/>
+      <c r="T26" s="141"/>
+      <c r="U26" s="141"/>
+      <c r="V26" s="142"/>
+      <c r="W26" s="77" t="s">
         <v>74</v>
       </c>
-      <c r="X26" s="202"/>
-      <c r="Y26" s="203"/>
+      <c r="X26" s="78"/>
+      <c r="Y26" s="79"/>
       <c r="AB26" s="19" t="s">
         <v>84</v>
       </c>
@@ -4116,16 +4081,16 @@
     </row>
     <row r="27" spans="1:34" s="1" customFormat="1" ht="31.5" customHeight="1">
       <c r="A27" s="53"/>
-      <c r="B27" s="81" t="s">
+      <c r="B27" s="254" t="s">
         <v>75</v>
       </c>
-      <c r="C27" s="81"/>
-      <c r="D27" s="81"/>
-      <c r="E27" s="81"/>
-      <c r="F27" s="81"/>
-      <c r="G27" s="81"/>
-      <c r="H27" s="81"/>
-      <c r="I27" s="82"/>
+      <c r="C27" s="254"/>
+      <c r="D27" s="254"/>
+      <c r="E27" s="254"/>
+      <c r="F27" s="254"/>
+      <c r="G27" s="254"/>
+      <c r="H27" s="254"/>
+      <c r="I27" s="255"/>
       <c r="J27" s="54"/>
       <c r="K27" s="54"/>
       <c r="L27" s="54"/>
@@ -4133,17 +4098,17 @@
       <c r="N27" s="54" t="s">
         <v>40</v>
       </c>
-      <c r="O27" s="165"/>
-      <c r="P27" s="166"/>
-      <c r="Q27" s="167"/>
-      <c r="R27" s="195"/>
-      <c r="S27" s="196"/>
-      <c r="T27" s="196"/>
-      <c r="U27" s="196"/>
-      <c r="V27" s="197"/>
-      <c r="W27" s="204"/>
-      <c r="X27" s="205"/>
-      <c r="Y27" s="206"/>
+      <c r="O27" s="122"/>
+      <c r="P27" s="123"/>
+      <c r="Q27" s="124"/>
+      <c r="R27" s="143"/>
+      <c r="S27" s="144"/>
+      <c r="T27" s="144"/>
+      <c r="U27" s="144"/>
+      <c r="V27" s="145"/>
+      <c r="W27" s="80"/>
+      <c r="X27" s="81"/>
+      <c r="Y27" s="82"/>
       <c r="AB27" s="31" t="s">
         <v>84</v>
       </c>
@@ -4159,16 +4124,16 @@
     </row>
     <row r="28" spans="1:34" s="1" customFormat="1" ht="31.5" customHeight="1">
       <c r="A28" s="53"/>
-      <c r="B28" s="81" t="s">
+      <c r="B28" s="254" t="s">
         <v>3</v>
       </c>
-      <c r="C28" s="81"/>
-      <c r="D28" s="81"/>
-      <c r="E28" s="81"/>
-      <c r="F28" s="81"/>
-      <c r="G28" s="81"/>
-      <c r="H28" s="81"/>
-      <c r="I28" s="82"/>
+      <c r="C28" s="254"/>
+      <c r="D28" s="254"/>
+      <c r="E28" s="254"/>
+      <c r="F28" s="254"/>
+      <c r="G28" s="254"/>
+      <c r="H28" s="254"/>
+      <c r="I28" s="255"/>
       <c r="J28" s="54"/>
       <c r="K28" s="54"/>
       <c r="L28" s="54"/>
@@ -4176,17 +4141,17 @@
       <c r="N28" s="54" t="s">
         <v>40</v>
       </c>
-      <c r="O28" s="165"/>
-      <c r="P28" s="166"/>
-      <c r="Q28" s="167"/>
-      <c r="R28" s="195"/>
-      <c r="S28" s="196"/>
-      <c r="T28" s="196"/>
-      <c r="U28" s="196"/>
-      <c r="V28" s="197"/>
-      <c r="W28" s="204"/>
-      <c r="X28" s="205"/>
-      <c r="Y28" s="206"/>
+      <c r="O28" s="122"/>
+      <c r="P28" s="123"/>
+      <c r="Q28" s="124"/>
+      <c r="R28" s="143"/>
+      <c r="S28" s="144"/>
+      <c r="T28" s="144"/>
+      <c r="U28" s="144"/>
+      <c r="V28" s="145"/>
+      <c r="W28" s="80"/>
+      <c r="X28" s="81"/>
+      <c r="Y28" s="82"/>
       <c r="AB28" s="31" t="s">
         <v>84</v>
       </c>
@@ -4201,35 +4166,35 @@
       </c>
     </row>
     <row r="29" spans="1:34" s="1" customFormat="1" ht="31.5" customHeight="1" thickBot="1">
-      <c r="A29" s="89" t="s">
+      <c r="A29" s="95" t="s">
         <v>47</v>
       </c>
-      <c r="B29" s="90"/>
-      <c r="C29" s="90"/>
-      <c r="D29" s="90"/>
-      <c r="E29" s="90"/>
-      <c r="F29" s="90"/>
-      <c r="G29" s="90"/>
-      <c r="H29" s="90"/>
-      <c r="I29" s="91"/>
+      <c r="B29" s="96"/>
+      <c r="C29" s="96"/>
+      <c r="D29" s="96"/>
+      <c r="E29" s="96"/>
+      <c r="F29" s="96"/>
+      <c r="G29" s="96"/>
+      <c r="H29" s="96"/>
+      <c r="I29" s="97"/>
       <c r="J29" s="55"/>
       <c r="K29" s="56"/>
       <c r="L29" s="56"/>
       <c r="M29" s="56"/>
       <c r="N29" s="57"/>
-      <c r="O29" s="162" t="s">
+      <c r="O29" s="119" t="s">
         <v>12</v>
       </c>
-      <c r="P29" s="163"/>
-      <c r="Q29" s="164"/>
-      <c r="R29" s="195"/>
-      <c r="S29" s="196"/>
-      <c r="T29" s="196"/>
-      <c r="U29" s="196"/>
-      <c r="V29" s="197"/>
-      <c r="W29" s="204"/>
-      <c r="X29" s="205"/>
-      <c r="Y29" s="206"/>
+      <c r="P29" s="120"/>
+      <c r="Q29" s="121"/>
+      <c r="R29" s="143"/>
+      <c r="S29" s="144"/>
+      <c r="T29" s="144"/>
+      <c r="U29" s="144"/>
+      <c r="V29" s="145"/>
+      <c r="W29" s="80"/>
+      <c r="X29" s="81"/>
+      <c r="Y29" s="82"/>
       <c r="AB29" s="50" t="s">
         <v>84</v>
       </c>
@@ -4245,16 +4210,16 @@
     </row>
     <row r="30" spans="1:34" s="1" customFormat="1" ht="31.5" customHeight="1">
       <c r="A30" s="58"/>
-      <c r="B30" s="81" t="s">
+      <c r="B30" s="254" t="s">
         <v>75</v>
       </c>
-      <c r="C30" s="81"/>
-      <c r="D30" s="81"/>
-      <c r="E30" s="81"/>
-      <c r="F30" s="81"/>
-      <c r="G30" s="81"/>
-      <c r="H30" s="81"/>
-      <c r="I30" s="82"/>
+      <c r="C30" s="254"/>
+      <c r="D30" s="254"/>
+      <c r="E30" s="254"/>
+      <c r="F30" s="254"/>
+      <c r="G30" s="254"/>
+      <c r="H30" s="254"/>
+      <c r="I30" s="255"/>
       <c r="J30" s="59"/>
       <c r="K30" s="59"/>
       <c r="L30" s="59"/>
@@ -4262,17 +4227,17 @@
       <c r="N30" s="54" t="s">
         <v>40</v>
       </c>
-      <c r="O30" s="165"/>
-      <c r="P30" s="166"/>
-      <c r="Q30" s="167"/>
-      <c r="R30" s="195"/>
-      <c r="S30" s="196"/>
-      <c r="T30" s="196"/>
-      <c r="U30" s="196"/>
-      <c r="V30" s="197"/>
-      <c r="W30" s="204"/>
-      <c r="X30" s="205"/>
-      <c r="Y30" s="206"/>
+      <c r="O30" s="122"/>
+      <c r="P30" s="123"/>
+      <c r="Q30" s="124"/>
+      <c r="R30" s="143"/>
+      <c r="S30" s="144"/>
+      <c r="T30" s="144"/>
+      <c r="U30" s="144"/>
+      <c r="V30" s="145"/>
+      <c r="W30" s="80"/>
+      <c r="X30" s="81"/>
+      <c r="Y30" s="82"/>
       <c r="AB30" s="2" t="s">
         <v>90</v>
       </c>
@@ -4281,35 +4246,35 @@
       <c r="AE30" s="2"/>
     </row>
     <row r="31" spans="1:34" s="1" customFormat="1" ht="31.5" customHeight="1">
-      <c r="A31" s="89" t="s">
+      <c r="A31" s="95" t="s">
         <v>48</v>
       </c>
-      <c r="B31" s="90"/>
-      <c r="C31" s="90"/>
-      <c r="D31" s="90"/>
-      <c r="E31" s="90"/>
-      <c r="F31" s="90"/>
-      <c r="G31" s="90"/>
-      <c r="H31" s="90"/>
-      <c r="I31" s="91"/>
+      <c r="B31" s="96"/>
+      <c r="C31" s="96"/>
+      <c r="D31" s="96"/>
+      <c r="E31" s="96"/>
+      <c r="F31" s="96"/>
+      <c r="G31" s="96"/>
+      <c r="H31" s="96"/>
+      <c r="I31" s="97"/>
       <c r="J31" s="55"/>
       <c r="K31" s="56"/>
       <c r="L31" s="56"/>
       <c r="M31" s="56"/>
       <c r="N31" s="57"/>
-      <c r="O31" s="240" t="s">
+      <c r="O31" s="89" t="s">
         <v>13</v>
       </c>
-      <c r="P31" s="241"/>
-      <c r="Q31" s="242"/>
-      <c r="R31" s="198"/>
-      <c r="S31" s="199"/>
-      <c r="T31" s="199"/>
-      <c r="U31" s="199"/>
-      <c r="V31" s="200"/>
-      <c r="W31" s="207"/>
-      <c r="X31" s="208"/>
-      <c r="Y31" s="209"/>
+      <c r="P31" s="90"/>
+      <c r="Q31" s="91"/>
+      <c r="R31" s="146"/>
+      <c r="S31" s="147"/>
+      <c r="T31" s="147"/>
+      <c r="U31" s="147"/>
+      <c r="V31" s="148"/>
+      <c r="W31" s="83"/>
+      <c r="X31" s="84"/>
+      <c r="Y31" s="85"/>
       <c r="AB31" s="2" t="s">
         <v>91</v>
       </c>
@@ -4320,19 +4285,19 @@
       <c r="AE31" s="2"/>
     </row>
     <row r="32" spans="1:34" s="1" customFormat="1" ht="31.5" customHeight="1">
-      <c r="A32" s="152" t="s">
+      <c r="A32" s="212" t="s">
         <v>49</v>
       </c>
-      <c r="B32" s="153"/>
-      <c r="C32" s="154"/>
-      <c r="D32" s="186" t="s">
+      <c r="B32" s="213"/>
+      <c r="C32" s="214"/>
+      <c r="D32" s="86" t="s">
         <v>4</v>
       </c>
-      <c r="E32" s="187"/>
-      <c r="F32" s="187"/>
-      <c r="G32" s="187"/>
-      <c r="H32" s="187"/>
-      <c r="I32" s="188"/>
+      <c r="E32" s="87"/>
+      <c r="F32" s="87"/>
+      <c r="G32" s="87"/>
+      <c r="H32" s="87"/>
+      <c r="I32" s="88"/>
       <c r="J32" s="60"/>
       <c r="K32" s="54"/>
       <c r="L32" s="54"/>
@@ -4340,38 +4305,38 @@
       <c r="N32" s="54" t="s">
         <v>40</v>
       </c>
-      <c r="O32" s="162" t="s">
+      <c r="O32" s="119" t="s">
         <v>19</v>
       </c>
-      <c r="P32" s="163"/>
-      <c r="Q32" s="164"/>
-      <c r="R32" s="210">
+      <c r="P32" s="120"/>
+      <c r="Q32" s="121"/>
+      <c r="R32" s="149">
         <v>200000</v>
       </c>
-      <c r="S32" s="211"/>
-      <c r="T32" s="211"/>
-      <c r="U32" s="211"/>
-      <c r="V32" s="212"/>
-      <c r="W32" s="219"/>
-      <c r="X32" s="202"/>
-      <c r="Y32" s="203"/>
+      <c r="S32" s="150"/>
+      <c r="T32" s="150"/>
+      <c r="U32" s="150"/>
+      <c r="V32" s="151"/>
+      <c r="W32" s="158"/>
+      <c r="X32" s="78"/>
+      <c r="Y32" s="79"/>
       <c r="AB32" s="2"/>
       <c r="AC32" s="2"/>
       <c r="AD32" s="2"/>
       <c r="AE32" s="2"/>
     </row>
     <row r="33" spans="1:31" s="1" customFormat="1" ht="31.5" customHeight="1">
-      <c r="A33" s="155"/>
-      <c r="B33" s="156"/>
-      <c r="C33" s="157"/>
-      <c r="D33" s="186" t="s">
+      <c r="A33" s="215"/>
+      <c r="B33" s="216"/>
+      <c r="C33" s="217"/>
+      <c r="D33" s="86" t="s">
         <v>5</v>
       </c>
-      <c r="E33" s="187"/>
-      <c r="F33" s="187"/>
-      <c r="G33" s="187"/>
-      <c r="H33" s="187"/>
-      <c r="I33" s="188"/>
+      <c r="E33" s="87"/>
+      <c r="F33" s="87"/>
+      <c r="G33" s="87"/>
+      <c r="H33" s="87"/>
+      <c r="I33" s="88"/>
       <c r="J33" s="60"/>
       <c r="K33" s="54"/>
       <c r="L33" s="54"/>
@@ -4379,34 +4344,34 @@
       <c r="N33" s="54" t="s">
         <v>40</v>
       </c>
-      <c r="O33" s="165"/>
-      <c r="P33" s="166"/>
-      <c r="Q33" s="167"/>
-      <c r="R33" s="213"/>
-      <c r="S33" s="214"/>
-      <c r="T33" s="214"/>
-      <c r="U33" s="214"/>
-      <c r="V33" s="215"/>
-      <c r="W33" s="204"/>
-      <c r="X33" s="205"/>
-      <c r="Y33" s="206"/>
+      <c r="O33" s="122"/>
+      <c r="P33" s="123"/>
+      <c r="Q33" s="124"/>
+      <c r="R33" s="152"/>
+      <c r="S33" s="153"/>
+      <c r="T33" s="153"/>
+      <c r="U33" s="153"/>
+      <c r="V33" s="154"/>
+      <c r="W33" s="80"/>
+      <c r="X33" s="81"/>
+      <c r="Y33" s="82"/>
       <c r="AB33" s="2"/>
       <c r="AC33" s="2"/>
       <c r="AD33" s="2"/>
       <c r="AE33" s="2"/>
     </row>
     <row r="34" spans="1:31" s="1" customFormat="1" ht="31.5" customHeight="1">
-      <c r="A34" s="158"/>
-      <c r="B34" s="159"/>
-      <c r="C34" s="160"/>
-      <c r="D34" s="186" t="s">
+      <c r="A34" s="218"/>
+      <c r="B34" s="219"/>
+      <c r="C34" s="220"/>
+      <c r="D34" s="86" t="s">
         <v>6</v>
       </c>
-      <c r="E34" s="187"/>
-      <c r="F34" s="187"/>
-      <c r="G34" s="187"/>
-      <c r="H34" s="187"/>
-      <c r="I34" s="188"/>
+      <c r="E34" s="87"/>
+      <c r="F34" s="87"/>
+      <c r="G34" s="87"/>
+      <c r="H34" s="87"/>
+      <c r="I34" s="88"/>
       <c r="J34" s="60"/>
       <c r="K34" s="54" t="s">
         <v>40</v>
@@ -4420,34 +4385,34 @@
       <c r="N34" s="54" t="s">
         <v>40</v>
       </c>
-      <c r="O34" s="168"/>
-      <c r="P34" s="169"/>
-      <c r="Q34" s="170"/>
-      <c r="R34" s="216"/>
-      <c r="S34" s="217"/>
-      <c r="T34" s="217"/>
-      <c r="U34" s="217"/>
-      <c r="V34" s="218"/>
-      <c r="W34" s="207"/>
-      <c r="X34" s="208"/>
-      <c r="Y34" s="209"/>
+      <c r="O34" s="125"/>
+      <c r="P34" s="126"/>
+      <c r="Q34" s="127"/>
+      <c r="R34" s="155"/>
+      <c r="S34" s="156"/>
+      <c r="T34" s="156"/>
+      <c r="U34" s="156"/>
+      <c r="V34" s="157"/>
+      <c r="W34" s="83"/>
+      <c r="X34" s="84"/>
+      <c r="Y34" s="85"/>
       <c r="AB34" s="2"/>
       <c r="AC34" s="2"/>
       <c r="AD34" s="2"/>
       <c r="AE34" s="2"/>
     </row>
     <row r="35" spans="1:31" s="1" customFormat="1" ht="31.5" customHeight="1">
-      <c r="A35" s="89" t="s">
+      <c r="A35" s="95" t="s">
         <v>50</v>
       </c>
-      <c r="B35" s="90"/>
-      <c r="C35" s="90"/>
-      <c r="D35" s="90"/>
-      <c r="E35" s="90"/>
-      <c r="F35" s="90"/>
-      <c r="G35" s="90"/>
-      <c r="H35" s="90"/>
-      <c r="I35" s="91"/>
+      <c r="B35" s="96"/>
+      <c r="C35" s="96"/>
+      <c r="D35" s="96"/>
+      <c r="E35" s="96"/>
+      <c r="F35" s="96"/>
+      <c r="G35" s="96"/>
+      <c r="H35" s="96"/>
+      <c r="I35" s="97"/>
       <c r="J35" s="54"/>
       <c r="K35" s="54" t="s">
         <v>40</v>
@@ -4461,38 +4426,38 @@
       <c r="N35" s="54" t="s">
         <v>40</v>
       </c>
-      <c r="O35" s="240" t="s">
+      <c r="O35" s="89" t="s">
         <v>41</v>
       </c>
-      <c r="P35" s="241"/>
-      <c r="Q35" s="242"/>
-      <c r="R35" s="183">
+      <c r="P35" s="90"/>
+      <c r="Q35" s="91"/>
+      <c r="R35" s="98">
         <v>600000</v>
       </c>
-      <c r="S35" s="184"/>
-      <c r="T35" s="184"/>
-      <c r="U35" s="184"/>
-      <c r="V35" s="185"/>
-      <c r="W35" s="223"/>
-      <c r="X35" s="224"/>
-      <c r="Y35" s="225"/>
+      <c r="S35" s="99"/>
+      <c r="T35" s="99"/>
+      <c r="U35" s="99"/>
+      <c r="V35" s="100"/>
+      <c r="W35" s="92"/>
+      <c r="X35" s="93"/>
+      <c r="Y35" s="94"/>
       <c r="AB35" s="2"/>
       <c r="AC35" s="2"/>
       <c r="AD35" s="2"/>
       <c r="AE35" s="2"/>
     </row>
     <row r="36" spans="1:31" s="1" customFormat="1" ht="31.5" customHeight="1">
-      <c r="A36" s="89" t="s">
+      <c r="A36" s="95" t="s">
         <v>51</v>
       </c>
-      <c r="B36" s="90"/>
-      <c r="C36" s="90"/>
-      <c r="D36" s="90"/>
-      <c r="E36" s="90"/>
-      <c r="F36" s="90"/>
-      <c r="G36" s="90"/>
-      <c r="H36" s="90"/>
-      <c r="I36" s="91"/>
+      <c r="B36" s="96"/>
+      <c r="C36" s="96"/>
+      <c r="D36" s="96"/>
+      <c r="E36" s="96"/>
+      <c r="F36" s="96"/>
+      <c r="G36" s="96"/>
+      <c r="H36" s="96"/>
+      <c r="I36" s="97"/>
       <c r="J36" s="54"/>
       <c r="K36" s="54"/>
       <c r="L36" s="54"/>
@@ -4500,38 +4465,38 @@
       <c r="N36" s="54" t="s">
         <v>40</v>
       </c>
-      <c r="O36" s="240" t="s">
+      <c r="O36" s="89" t="s">
         <v>14</v>
       </c>
-      <c r="P36" s="241"/>
-      <c r="Q36" s="242"/>
-      <c r="R36" s="183">
+      <c r="P36" s="90"/>
+      <c r="Q36" s="91"/>
+      <c r="R36" s="98">
         <v>300000</v>
       </c>
-      <c r="S36" s="184"/>
-      <c r="T36" s="184"/>
-      <c r="U36" s="184"/>
-      <c r="V36" s="185"/>
-      <c r="W36" s="223"/>
-      <c r="X36" s="224"/>
-      <c r="Y36" s="225"/>
+      <c r="S36" s="99"/>
+      <c r="T36" s="99"/>
+      <c r="U36" s="99"/>
+      <c r="V36" s="100"/>
+      <c r="W36" s="92"/>
+      <c r="X36" s="93"/>
+      <c r="Y36" s="94"/>
       <c r="AB36" s="2"/>
       <c r="AC36" s="2"/>
       <c r="AD36" s="2"/>
       <c r="AE36" s="2"/>
     </row>
     <row r="37" spans="1:31" s="1" customFormat="1" ht="31.5" customHeight="1">
-      <c r="A37" s="171" t="s">
+      <c r="A37" s="173" t="s">
         <v>52</v>
       </c>
-      <c r="B37" s="172"/>
-      <c r="C37" s="172"/>
-      <c r="D37" s="172"/>
-      <c r="E37" s="172"/>
-      <c r="F37" s="172"/>
-      <c r="G37" s="172"/>
-      <c r="H37" s="172"/>
-      <c r="I37" s="173"/>
+      <c r="B37" s="174"/>
+      <c r="C37" s="174"/>
+      <c r="D37" s="174"/>
+      <c r="E37" s="174"/>
+      <c r="F37" s="174"/>
+      <c r="G37" s="174"/>
+      <c r="H37" s="174"/>
+      <c r="I37" s="175"/>
       <c r="J37" s="60"/>
       <c r="K37" s="54" t="s">
         <v>40</v>
@@ -4545,38 +4510,38 @@
       <c r="N37" s="54" t="s">
         <v>40</v>
       </c>
-      <c r="O37" s="243"/>
-      <c r="P37" s="244"/>
-      <c r="Q37" s="245"/>
-      <c r="R37" s="183">
+      <c r="O37" s="116"/>
+      <c r="P37" s="117"/>
+      <c r="Q37" s="118"/>
+      <c r="R37" s="98">
         <v>100000</v>
       </c>
-      <c r="S37" s="184"/>
-      <c r="T37" s="184"/>
-      <c r="U37" s="184"/>
-      <c r="V37" s="185"/>
-      <c r="W37" s="223"/>
-      <c r="X37" s="224"/>
-      <c r="Y37" s="225"/>
+      <c r="S37" s="99"/>
+      <c r="T37" s="99"/>
+      <c r="U37" s="99"/>
+      <c r="V37" s="100"/>
+      <c r="W37" s="92"/>
+      <c r="X37" s="93"/>
+      <c r="Y37" s="94"/>
       <c r="AB37" s="2"/>
       <c r="AC37" s="2"/>
       <c r="AD37" s="2"/>
       <c r="AE37" s="2"/>
     </row>
     <row r="38" spans="1:31" s="1" customFormat="1" ht="31.5" customHeight="1">
-      <c r="A38" s="174" t="s">
+      <c r="A38" s="176" t="s">
         <v>62</v>
       </c>
-      <c r="B38" s="175"/>
-      <c r="C38" s="176"/>
-      <c r="D38" s="186" t="s">
+      <c r="B38" s="177"/>
+      <c r="C38" s="178"/>
+      <c r="D38" s="86" t="s">
         <v>71</v>
       </c>
-      <c r="E38" s="187"/>
-      <c r="F38" s="187"/>
-      <c r="G38" s="187"/>
-      <c r="H38" s="187"/>
-      <c r="I38" s="188"/>
+      <c r="E38" s="87"/>
+      <c r="F38" s="87"/>
+      <c r="G38" s="87"/>
+      <c r="H38" s="87"/>
+      <c r="I38" s="88"/>
       <c r="J38" s="60"/>
       <c r="K38" s="54"/>
       <c r="L38" s="54"/>
@@ -4584,69 +4549,69 @@
       <c r="N38" s="54" t="s">
         <v>40</v>
       </c>
-      <c r="O38" s="162" t="s">
+      <c r="O38" s="119" t="s">
         <v>15</v>
       </c>
-      <c r="P38" s="163"/>
-      <c r="Q38" s="164"/>
-      <c r="R38" s="189"/>
-      <c r="S38" s="189"/>
-      <c r="T38" s="189"/>
-      <c r="U38" s="189"/>
-      <c r="V38" s="189"/>
-      <c r="W38" s="252"/>
-      <c r="X38" s="253"/>
-      <c r="Y38" s="254"/>
+      <c r="P38" s="120"/>
+      <c r="Q38" s="121"/>
+      <c r="R38" s="185"/>
+      <c r="S38" s="185"/>
+      <c r="T38" s="185"/>
+      <c r="U38" s="185"/>
+      <c r="V38" s="185"/>
+      <c r="W38" s="101"/>
+      <c r="X38" s="102"/>
+      <c r="Y38" s="103"/>
       <c r="AB38" s="2"/>
       <c r="AC38" s="2"/>
       <c r="AD38" s="2"/>
       <c r="AE38" s="2"/>
     </row>
     <row r="39" spans="1:31" s="1" customFormat="1" ht="31.5" customHeight="1">
-      <c r="A39" s="177"/>
-      <c r="B39" s="178"/>
-      <c r="C39" s="179"/>
-      <c r="D39" s="186" t="s">
+      <c r="A39" s="179"/>
+      <c r="B39" s="180"/>
+      <c r="C39" s="181"/>
+      <c r="D39" s="86" t="s">
         <v>72</v>
       </c>
-      <c r="E39" s="187"/>
-      <c r="F39" s="187"/>
-      <c r="G39" s="187"/>
-      <c r="H39" s="187"/>
-      <c r="I39" s="188"/>
+      <c r="E39" s="87"/>
+      <c r="F39" s="87"/>
+      <c r="G39" s="87"/>
+      <c r="H39" s="87"/>
+      <c r="I39" s="88"/>
       <c r="J39" s="60"/>
       <c r="K39" s="54"/>
       <c r="L39" s="54"/>
       <c r="M39" s="54"/>
       <c r="N39" s="54"/>
-      <c r="O39" s="165"/>
-      <c r="P39" s="166"/>
-      <c r="Q39" s="167"/>
-      <c r="R39" s="190"/>
-      <c r="S39" s="190"/>
-      <c r="T39" s="190"/>
-      <c r="U39" s="190"/>
-      <c r="V39" s="190"/>
-      <c r="W39" s="255"/>
-      <c r="X39" s="256"/>
-      <c r="Y39" s="257"/>
+      <c r="O39" s="122"/>
+      <c r="P39" s="123"/>
+      <c r="Q39" s="124"/>
+      <c r="R39" s="186"/>
+      <c r="S39" s="186"/>
+      <c r="T39" s="186"/>
+      <c r="U39" s="186"/>
+      <c r="V39" s="186"/>
+      <c r="W39" s="104"/>
+      <c r="X39" s="105"/>
+      <c r="Y39" s="106"/>
       <c r="AB39" s="2"/>
       <c r="AC39" s="2"/>
       <c r="AD39" s="2"/>
       <c r="AE39" s="2"/>
     </row>
     <row r="40" spans="1:31" s="1" customFormat="1" ht="31.5" customHeight="1">
-      <c r="A40" s="180"/>
-      <c r="B40" s="181"/>
-      <c r="C40" s="182"/>
-      <c r="D40" s="186" t="s">
+      <c r="A40" s="182"/>
+      <c r="B40" s="183"/>
+      <c r="C40" s="184"/>
+      <c r="D40" s="86" t="s">
         <v>3</v>
       </c>
-      <c r="E40" s="187"/>
-      <c r="F40" s="187"/>
-      <c r="G40" s="187"/>
-      <c r="H40" s="187"/>
-      <c r="I40" s="188"/>
+      <c r="E40" s="87"/>
+      <c r="F40" s="87"/>
+      <c r="G40" s="87"/>
+      <c r="H40" s="87"/>
+      <c r="I40" s="88"/>
       <c r="J40" s="60"/>
       <c r="K40" s="54"/>
       <c r="L40" s="54"/>
@@ -4654,75 +4619,75 @@
       <c r="N40" s="54" t="s">
         <v>40</v>
       </c>
-      <c r="O40" s="168"/>
-      <c r="P40" s="169"/>
-      <c r="Q40" s="170"/>
-      <c r="R40" s="191"/>
-      <c r="S40" s="191"/>
-      <c r="T40" s="191"/>
-      <c r="U40" s="191"/>
-      <c r="V40" s="191"/>
-      <c r="W40" s="258"/>
-      <c r="X40" s="259"/>
-      <c r="Y40" s="260"/>
+      <c r="O40" s="125"/>
+      <c r="P40" s="126"/>
+      <c r="Q40" s="127"/>
+      <c r="R40" s="187"/>
+      <c r="S40" s="187"/>
+      <c r="T40" s="187"/>
+      <c r="U40" s="187"/>
+      <c r="V40" s="187"/>
+      <c r="W40" s="107"/>
+      <c r="X40" s="108"/>
+      <c r="Y40" s="109"/>
       <c r="AB40" s="2"/>
       <c r="AC40" s="2"/>
       <c r="AD40" s="2"/>
       <c r="AE40" s="2"/>
     </row>
     <row r="41" spans="1:31" s="1" customFormat="1" ht="30" customHeight="1">
-      <c r="A41" s="87" t="s">
+      <c r="A41" s="259" t="s">
         <v>39</v>
       </c>
-      <c r="B41" s="88"/>
-      <c r="C41" s="88"/>
-      <c r="D41" s="88"/>
-      <c r="E41" s="88"/>
-      <c r="F41" s="88"/>
-      <c r="G41" s="88"/>
-      <c r="H41" s="88"/>
-      <c r="I41" s="88"/>
-      <c r="J41" s="88"/>
-      <c r="K41" s="88"/>
-      <c r="L41" s="88"/>
-      <c r="M41" s="88"/>
-      <c r="N41" s="161" t="s">
+      <c r="B41" s="260"/>
+      <c r="C41" s="260"/>
+      <c r="D41" s="260"/>
+      <c r="E41" s="260"/>
+      <c r="F41" s="260"/>
+      <c r="G41" s="260"/>
+      <c r="H41" s="260"/>
+      <c r="I41" s="260"/>
+      <c r="J41" s="260"/>
+      <c r="K41" s="260"/>
+      <c r="L41" s="260"/>
+      <c r="M41" s="260"/>
+      <c r="N41" s="170" t="s">
         <v>53</v>
       </c>
-      <c r="O41" s="150"/>
-      <c r="P41" s="150"/>
-      <c r="Q41" s="150"/>
-      <c r="R41" s="150"/>
-      <c r="S41" s="150"/>
-      <c r="T41" s="151"/>
-      <c r="U41" s="149">
+      <c r="O41" s="171"/>
+      <c r="P41" s="171"/>
+      <c r="Q41" s="171"/>
+      <c r="R41" s="171"/>
+      <c r="S41" s="171"/>
+      <c r="T41" s="172"/>
+      <c r="U41" s="211">
         <f>SUM(R22:V40)</f>
         <v>1600000</v>
       </c>
-      <c r="V41" s="150"/>
-      <c r="W41" s="150"/>
-      <c r="X41" s="150"/>
-      <c r="Y41" s="151"/>
+      <c r="V41" s="171"/>
+      <c r="W41" s="171"/>
+      <c r="X41" s="171"/>
+      <c r="Y41" s="172"/>
       <c r="AB41" s="2"/>
       <c r="AC41" s="2"/>
       <c r="AD41" s="2"/>
       <c r="AE41" s="2"/>
     </row>
     <row r="42" spans="1:31" s="13" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A42" s="83" t="s">
+      <c r="A42" s="256" t="s">
         <v>34</v>
       </c>
-      <c r="B42" s="84"/>
-      <c r="C42" s="84"/>
-      <c r="D42" s="84"/>
-      <c r="E42" s="84"/>
-      <c r="F42" s="84"/>
-      <c r="G42" s="84"/>
-      <c r="H42" s="84"/>
-      <c r="I42" s="84"/>
-      <c r="J42" s="84"/>
-      <c r="K42" s="84"/>
-      <c r="L42" s="85"/>
+      <c r="B42" s="257"/>
+      <c r="C42" s="257"/>
+      <c r="D42" s="257"/>
+      <c r="E42" s="257"/>
+      <c r="F42" s="257"/>
+      <c r="G42" s="257"/>
+      <c r="H42" s="257"/>
+      <c r="I42" s="257"/>
+      <c r="J42" s="257"/>
+      <c r="K42" s="257"/>
+      <c r="L42" s="258"/>
       <c r="M42" s="61" t="s">
         <v>35</v>
       </c>
@@ -4744,20 +4709,20 @@
       <c r="AE42" s="64"/>
     </row>
     <row r="43" spans="1:31" s="13" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A43" s="86" t="s">
+      <c r="A43" s="208" t="s">
         <v>36</v>
       </c>
-      <c r="B43" s="79"/>
-      <c r="C43" s="79"/>
-      <c r="D43" s="79"/>
-      <c r="E43" s="79"/>
-      <c r="F43" s="79"/>
-      <c r="G43" s="79"/>
-      <c r="H43" s="79"/>
-      <c r="I43" s="79"/>
-      <c r="J43" s="79"/>
-      <c r="K43" s="79"/>
-      <c r="L43" s="80"/>
+      <c r="B43" s="209"/>
+      <c r="C43" s="209"/>
+      <c r="D43" s="209"/>
+      <c r="E43" s="209"/>
+      <c r="F43" s="209"/>
+      <c r="G43" s="209"/>
+      <c r="H43" s="209"/>
+      <c r="I43" s="209"/>
+      <c r="J43" s="209"/>
+      <c r="K43" s="209"/>
+      <c r="L43" s="210"/>
       <c r="M43" s="65" t="s">
         <v>64</v>
       </c>
@@ -4768,20 +4733,20 @@
       <c r="AE43" s="64"/>
     </row>
     <row r="44" spans="1:31" s="13" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A44" s="86" t="s">
+      <c r="A44" s="208" t="s">
         <v>37</v>
       </c>
-      <c r="B44" s="79"/>
-      <c r="C44" s="79"/>
-      <c r="D44" s="79"/>
-      <c r="E44" s="79"/>
-      <c r="F44" s="79"/>
-      <c r="G44" s="79"/>
-      <c r="H44" s="79"/>
-      <c r="I44" s="79"/>
-      <c r="J44" s="79"/>
-      <c r="K44" s="79"/>
-      <c r="L44" s="80"/>
+      <c r="B44" s="209"/>
+      <c r="C44" s="209"/>
+      <c r="D44" s="209"/>
+      <c r="E44" s="209"/>
+      <c r="F44" s="209"/>
+      <c r="G44" s="209"/>
+      <c r="H44" s="209"/>
+      <c r="I44" s="209"/>
+      <c r="J44" s="209"/>
+      <c r="K44" s="209"/>
+      <c r="L44" s="210"/>
       <c r="M44" s="66" t="s">
         <v>117</v>
       </c>
@@ -4803,20 +4768,20 @@
       <c r="AE44" s="64"/>
     </row>
     <row r="45" spans="1:31" s="13" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A45" s="86" t="s">
+      <c r="A45" s="208" t="s">
         <v>32</v>
       </c>
-      <c r="B45" s="79"/>
-      <c r="C45" s="79"/>
-      <c r="D45" s="79"/>
-      <c r="E45" s="79"/>
-      <c r="F45" s="79"/>
-      <c r="G45" s="79"/>
-      <c r="H45" s="79"/>
-      <c r="I45" s="79"/>
-      <c r="J45" s="79"/>
-      <c r="K45" s="79"/>
-      <c r="L45" s="80"/>
+      <c r="B45" s="209"/>
+      <c r="C45" s="209"/>
+      <c r="D45" s="209"/>
+      <c r="E45" s="209"/>
+      <c r="F45" s="209"/>
+      <c r="G45" s="209"/>
+      <c r="H45" s="209"/>
+      <c r="I45" s="209"/>
+      <c r="J45" s="209"/>
+      <c r="K45" s="209"/>
+      <c r="L45" s="210"/>
       <c r="M45" s="69" t="s">
         <v>116</v>
       </c>
@@ -4865,17 +4830,17 @@
       <c r="A47" s="74" t="s">
         <v>110</v>
       </c>
-      <c r="D47" s="79" t="s">
+      <c r="D47" s="209" t="s">
         <v>113</v>
       </c>
-      <c r="E47" s="79"/>
-      <c r="F47" s="79"/>
-      <c r="G47" s="79"/>
-      <c r="H47" s="79"/>
-      <c r="I47" s="79"/>
-      <c r="J47" s="79"/>
-      <c r="K47" s="79"/>
-      <c r="L47" s="80"/>
+      <c r="E47" s="209"/>
+      <c r="F47" s="209"/>
+      <c r="G47" s="209"/>
+      <c r="H47" s="209"/>
+      <c r="I47" s="209"/>
+      <c r="J47" s="209"/>
+      <c r="K47" s="209"/>
+      <c r="L47" s="210"/>
       <c r="M47" s="65" t="s">
         <v>73</v>
       </c>
@@ -4889,17 +4854,17 @@
       <c r="A48" s="74" t="s">
         <v>109</v>
       </c>
-      <c r="D48" s="79" t="s">
+      <c r="D48" s="209" t="s">
         <v>77</v>
       </c>
-      <c r="E48" s="79"/>
-      <c r="F48" s="79"/>
-      <c r="G48" s="79"/>
-      <c r="H48" s="79"/>
-      <c r="I48" s="79"/>
-      <c r="J48" s="79"/>
-      <c r="K48" s="79"/>
-      <c r="L48" s="80"/>
+      <c r="E48" s="209"/>
+      <c r="F48" s="209"/>
+      <c r="G48" s="209"/>
+      <c r="H48" s="209"/>
+      <c r="I48" s="209"/>
+      <c r="J48" s="209"/>
+      <c r="K48" s="209"/>
+      <c r="L48" s="210"/>
       <c r="M48" s="65" t="s">
         <v>66</v>
       </c>
@@ -4913,17 +4878,17 @@
       <c r="A49" s="74" t="s">
         <v>111</v>
       </c>
-      <c r="D49" s="77" t="s">
+      <c r="D49" s="252" t="s">
         <v>114</v>
       </c>
-      <c r="E49" s="77"/>
-      <c r="F49" s="77"/>
-      <c r="G49" s="77"/>
-      <c r="H49" s="77"/>
-      <c r="I49" s="77"/>
-      <c r="J49" s="77"/>
-      <c r="K49" s="77"/>
-      <c r="L49" s="78"/>
+      <c r="E49" s="252"/>
+      <c r="F49" s="252"/>
+      <c r="G49" s="252"/>
+      <c r="H49" s="252"/>
+      <c r="I49" s="252"/>
+      <c r="J49" s="252"/>
+      <c r="K49" s="252"/>
+      <c r="L49" s="253"/>
       <c r="M49" s="65" t="s">
         <v>67</v>
       </c>
@@ -4937,17 +4902,17 @@
       <c r="A50" s="74" t="s">
         <v>112</v>
       </c>
-      <c r="D50" s="92" t="s">
+      <c r="D50" s="233" t="s">
         <v>115</v>
       </c>
-      <c r="E50" s="92"/>
-      <c r="F50" s="92"/>
-      <c r="G50" s="92"/>
-      <c r="H50" s="92"/>
-      <c r="I50" s="92"/>
-      <c r="J50" s="92"/>
-      <c r="K50" s="92"/>
-      <c r="L50" s="93"/>
+      <c r="E50" s="233"/>
+      <c r="F50" s="233"/>
+      <c r="G50" s="233"/>
+      <c r="H50" s="233"/>
+      <c r="I50" s="233"/>
+      <c r="J50" s="233"/>
+      <c r="K50" s="233"/>
+      <c r="L50" s="234"/>
       <c r="M50" s="65" t="s">
         <v>118</v>
       </c>
@@ -4959,15 +4924,15 @@
     </row>
     <row r="51" spans="1:31" s="13" customFormat="1" ht="20.100000000000001" customHeight="1">
       <c r="A51" s="74"/>
-      <c r="D51" s="94"/>
-      <c r="E51" s="94"/>
-      <c r="F51" s="94"/>
-      <c r="G51" s="94"/>
-      <c r="H51" s="94"/>
-      <c r="I51" s="94"/>
-      <c r="J51" s="94"/>
-      <c r="K51" s="94"/>
-      <c r="L51" s="95"/>
+      <c r="D51" s="235"/>
+      <c r="E51" s="235"/>
+      <c r="F51" s="235"/>
+      <c r="G51" s="235"/>
+      <c r="H51" s="235"/>
+      <c r="I51" s="235"/>
+      <c r="J51" s="235"/>
+      <c r="K51" s="235"/>
+      <c r="L51" s="236"/>
       <c r="M51" s="65" t="s">
         <v>123</v>
       </c>
@@ -4978,33 +4943,33 @@
       <c r="AE51" s="64"/>
     </row>
     <row r="52" spans="1:31" s="1" customFormat="1" ht="35.25" customHeight="1">
-      <c r="A52" s="133" t="s">
+      <c r="A52" s="188" t="s">
         <v>69</v>
       </c>
-      <c r="B52" s="134"/>
-      <c r="C52" s="134"/>
-      <c r="D52" s="134"/>
-      <c r="E52" s="134"/>
-      <c r="F52" s="134"/>
-      <c r="G52" s="134"/>
-      <c r="H52" s="134"/>
-      <c r="I52" s="134"/>
-      <c r="J52" s="134"/>
-      <c r="K52" s="134"/>
-      <c r="L52" s="134"/>
-      <c r="M52" s="134"/>
-      <c r="N52" s="134"/>
-      <c r="O52" s="134"/>
-      <c r="P52" s="134"/>
-      <c r="Q52" s="134"/>
-      <c r="R52" s="134"/>
-      <c r="S52" s="134"/>
-      <c r="T52" s="134"/>
-      <c r="U52" s="134"/>
-      <c r="V52" s="134"/>
-      <c r="W52" s="134"/>
-      <c r="X52" s="134"/>
-      <c r="Y52" s="135"/>
+      <c r="B52" s="189"/>
+      <c r="C52" s="189"/>
+      <c r="D52" s="189"/>
+      <c r="E52" s="189"/>
+      <c r="F52" s="189"/>
+      <c r="G52" s="189"/>
+      <c r="H52" s="189"/>
+      <c r="I52" s="189"/>
+      <c r="J52" s="189"/>
+      <c r="K52" s="189"/>
+      <c r="L52" s="189"/>
+      <c r="M52" s="189"/>
+      <c r="N52" s="189"/>
+      <c r="O52" s="189"/>
+      <c r="P52" s="189"/>
+      <c r="Q52" s="189"/>
+      <c r="R52" s="189"/>
+      <c r="S52" s="189"/>
+      <c r="T52" s="189"/>
+      <c r="U52" s="189"/>
+      <c r="V52" s="189"/>
+      <c r="W52" s="189"/>
+      <c r="X52" s="189"/>
+      <c r="Y52" s="190"/>
       <c r="AB52" s="2"/>
       <c r="AC52" s="2"/>
       <c r="AD52" s="2"/>
@@ -5043,50 +5008,45 @@
     </row>
   </sheetData>
   <mergeCells count="99">
-    <mergeCell ref="AF22:AH25"/>
-    <mergeCell ref="D39:I39"/>
-    <mergeCell ref="D40:I40"/>
-    <mergeCell ref="O35:Q35"/>
-    <mergeCell ref="W35:Y35"/>
-    <mergeCell ref="A35:I35"/>
-    <mergeCell ref="R35:V35"/>
-    <mergeCell ref="D32:I32"/>
-    <mergeCell ref="D33:I33"/>
-    <mergeCell ref="D34:I34"/>
-    <mergeCell ref="W36:Y36"/>
-    <mergeCell ref="W37:Y37"/>
-    <mergeCell ref="W38:Y40"/>
-    <mergeCell ref="J21:N21"/>
-    <mergeCell ref="J22:N22"/>
-    <mergeCell ref="J19:N19"/>
-    <mergeCell ref="O36:Q36"/>
-    <mergeCell ref="O37:Q37"/>
-    <mergeCell ref="O32:Q34"/>
-    <mergeCell ref="O26:Q28"/>
-    <mergeCell ref="O29:Q30"/>
-    <mergeCell ref="O31:Q31"/>
-    <mergeCell ref="O19:Q20"/>
-    <mergeCell ref="O21:Q21"/>
-    <mergeCell ref="O22:Q25"/>
-    <mergeCell ref="W19:Y20"/>
-    <mergeCell ref="R26:V31"/>
-    <mergeCell ref="W26:Y31"/>
-    <mergeCell ref="R32:V34"/>
-    <mergeCell ref="W32:Y34"/>
-    <mergeCell ref="R19:V20"/>
-    <mergeCell ref="R21:V21"/>
-    <mergeCell ref="W21:Y21"/>
-    <mergeCell ref="R22:V25"/>
-    <mergeCell ref="W22:Y25"/>
-    <mergeCell ref="N41:T41"/>
-    <mergeCell ref="A36:I36"/>
-    <mergeCell ref="O38:Q40"/>
-    <mergeCell ref="A37:I37"/>
-    <mergeCell ref="A38:C40"/>
-    <mergeCell ref="R36:V36"/>
-    <mergeCell ref="R37:V37"/>
-    <mergeCell ref="D38:I38"/>
-    <mergeCell ref="R38:V40"/>
+    <mergeCell ref="D49:L49"/>
+    <mergeCell ref="D48:L48"/>
+    <mergeCell ref="D47:L47"/>
+    <mergeCell ref="B23:I23"/>
+    <mergeCell ref="B24:I24"/>
+    <mergeCell ref="B25:I25"/>
+    <mergeCell ref="B27:I27"/>
+    <mergeCell ref="B28:I28"/>
+    <mergeCell ref="B30:I30"/>
+    <mergeCell ref="A42:L42"/>
+    <mergeCell ref="A43:L43"/>
+    <mergeCell ref="A44:L44"/>
+    <mergeCell ref="A41:M41"/>
+    <mergeCell ref="A29:I29"/>
+    <mergeCell ref="D50:L51"/>
+    <mergeCell ref="T18:X18"/>
+    <mergeCell ref="J18:L18"/>
+    <mergeCell ref="M18:Q18"/>
+    <mergeCell ref="A1:Y1"/>
+    <mergeCell ref="A3:Y3"/>
+    <mergeCell ref="C6:F6"/>
+    <mergeCell ref="H12:I12"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="L9:N9"/>
+    <mergeCell ref="R16:S16"/>
+    <mergeCell ref="R13:S13"/>
+    <mergeCell ref="R14:S14"/>
+    <mergeCell ref="R15:S15"/>
+    <mergeCell ref="L10:N10"/>
+    <mergeCell ref="O6:Y6"/>
+    <mergeCell ref="V7:Y7"/>
+    <mergeCell ref="L6:N6"/>
+    <mergeCell ref="A17:M17"/>
+    <mergeCell ref="O8:Y8"/>
+    <mergeCell ref="O7:R7"/>
+    <mergeCell ref="S7:U7"/>
+    <mergeCell ref="L7:N7"/>
+    <mergeCell ref="L8:N8"/>
+    <mergeCell ref="K6:K10"/>
     <mergeCell ref="A19:I20"/>
     <mergeCell ref="A52:Y52"/>
     <mergeCell ref="S9:U9"/>
@@ -5103,45 +5063,50 @@
     <mergeCell ref="U41:Y41"/>
     <mergeCell ref="A31:I31"/>
     <mergeCell ref="A32:C34"/>
-    <mergeCell ref="V7:Y7"/>
-    <mergeCell ref="L6:N6"/>
-    <mergeCell ref="A17:M17"/>
-    <mergeCell ref="O8:Y8"/>
-    <mergeCell ref="O7:R7"/>
-    <mergeCell ref="S7:U7"/>
-    <mergeCell ref="L7:N7"/>
-    <mergeCell ref="L8:N8"/>
-    <mergeCell ref="K6:K10"/>
-    <mergeCell ref="D50:L51"/>
-    <mergeCell ref="T18:X18"/>
-    <mergeCell ref="J18:L18"/>
-    <mergeCell ref="M18:Q18"/>
-    <mergeCell ref="A1:Y1"/>
-    <mergeCell ref="A3:Y3"/>
-    <mergeCell ref="C6:F6"/>
-    <mergeCell ref="H12:I12"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="L9:N9"/>
-    <mergeCell ref="R16:S16"/>
-    <mergeCell ref="R13:S13"/>
-    <mergeCell ref="R14:S14"/>
-    <mergeCell ref="R15:S15"/>
-    <mergeCell ref="L10:N10"/>
-    <mergeCell ref="O6:Y6"/>
-    <mergeCell ref="D49:L49"/>
-    <mergeCell ref="D48:L48"/>
-    <mergeCell ref="D47:L47"/>
-    <mergeCell ref="B23:I23"/>
-    <mergeCell ref="B24:I24"/>
-    <mergeCell ref="B25:I25"/>
-    <mergeCell ref="B27:I27"/>
-    <mergeCell ref="B28:I28"/>
-    <mergeCell ref="B30:I30"/>
-    <mergeCell ref="A42:L42"/>
-    <mergeCell ref="A43:L43"/>
-    <mergeCell ref="A44:L44"/>
-    <mergeCell ref="A41:M41"/>
-    <mergeCell ref="A29:I29"/>
+    <mergeCell ref="N41:T41"/>
+    <mergeCell ref="A36:I36"/>
+    <mergeCell ref="O38:Q40"/>
+    <mergeCell ref="A37:I37"/>
+    <mergeCell ref="A38:C40"/>
+    <mergeCell ref="R36:V36"/>
+    <mergeCell ref="R37:V37"/>
+    <mergeCell ref="D38:I38"/>
+    <mergeCell ref="R38:V40"/>
+    <mergeCell ref="W19:Y20"/>
+    <mergeCell ref="R26:V31"/>
+    <mergeCell ref="W26:Y31"/>
+    <mergeCell ref="R32:V34"/>
+    <mergeCell ref="W32:Y34"/>
+    <mergeCell ref="R19:V20"/>
+    <mergeCell ref="R21:V21"/>
+    <mergeCell ref="W21:Y21"/>
+    <mergeCell ref="R22:V25"/>
+    <mergeCell ref="W22:Y25"/>
+    <mergeCell ref="J21:N21"/>
+    <mergeCell ref="J22:N22"/>
+    <mergeCell ref="J19:N19"/>
+    <mergeCell ref="O36:Q36"/>
+    <mergeCell ref="O37:Q37"/>
+    <mergeCell ref="O32:Q34"/>
+    <mergeCell ref="O26:Q28"/>
+    <mergeCell ref="O29:Q30"/>
+    <mergeCell ref="O31:Q31"/>
+    <mergeCell ref="O19:Q20"/>
+    <mergeCell ref="O21:Q21"/>
+    <mergeCell ref="O22:Q25"/>
+    <mergeCell ref="AF22:AH25"/>
+    <mergeCell ref="D39:I39"/>
+    <mergeCell ref="D40:I40"/>
+    <mergeCell ref="O35:Q35"/>
+    <mergeCell ref="W35:Y35"/>
+    <mergeCell ref="A35:I35"/>
+    <mergeCell ref="R35:V35"/>
+    <mergeCell ref="D32:I32"/>
+    <mergeCell ref="D33:I33"/>
+    <mergeCell ref="D34:I34"/>
+    <mergeCell ref="W36:Y36"/>
+    <mergeCell ref="W37:Y37"/>
+    <mergeCell ref="W38:Y40"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <hyperlinks>

</xml_diff>

<commit_message>
chore: update quotation template font sizes
</commit_message>
<xml_diff>
--- a/직무고시 견적서 양식.xlsx
+++ b/직무고시 견적서 양식.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Master\Documents\Antigravity program\직무고시 견적서\wkace-quotation-jigmu\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC5DAEDB-37A8-4C37-B1B4-304E989502A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF4AF699-BE6F-4B95-B880-15F699676468}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="견적서" sheetId="1" r:id="rId1"/>
@@ -231,10 +231,6 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t xml:space="preserve"> 예비발전 설비</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t xml:space="preserve"> 열화상 적외선측정 진단</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -280,11 +276,6 @@
   </si>
   <si>
     <t>기록 서식</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t xml:space="preserve"> 태양광발전
- 설비</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
@@ -590,6 +581,16 @@
     <t>(전기설비 종합 시험자 인증 2026-C1-0040호)</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
+  <si>
+    <t xml:space="preserve"> 예비
+ 발전설비</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve"> 태양광
+ 발전설비</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
@@ -602,7 +603,7 @@
     <numFmt numFmtId="178" formatCode="0&quot;회&quot;"/>
     <numFmt numFmtId="179" formatCode="yyyy&quot;년&quot;\ m&quot;월&quot;\ d&quot;일&quot;;@"/>
   </numFmts>
-  <fonts count="26">
+  <fonts count="31">
     <font>
       <sz val="11"/>
       <name val="굴림체"/>
@@ -753,24 +754,6 @@
     </font>
     <font>
       <b/>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="맑은 고딕"/>
-      <family val="3"/>
-      <charset val="129"/>
-      <scheme val="major"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="0"/>
-      <name val="맑은 고딕"/>
-      <family val="3"/>
-      <charset val="129"/>
-      <scheme val="major"/>
-    </font>
-    <font>
-      <b/>
       <sz val="15"/>
       <color indexed="8"/>
       <name val="맑은 고딕"/>
@@ -815,6 +798,67 @@
     <font>
       <sz val="10"/>
       <color indexed="8"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
+      <scheme val="major"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color indexed="8"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
+      <scheme val="major"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="1"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
+      <scheme val="major"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color rgb="FF0070C0"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
+      <scheme val="major"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color rgb="FFFF0000"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
+      <scheme val="major"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color indexed="8"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
+      <scheme val="major"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <color indexed="8"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
+      <scheme val="major"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color theme="0"/>
       <name val="맑은 고딕"/>
       <family val="3"/>
       <charset val="129"/>
@@ -1472,7 +1516,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="261">
+  <cellXfs count="260">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1611,18 +1655,6 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1656,13 +1688,13 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1689,20 +1721,200 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="5" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="39" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="10" fillId="3" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="10" fillId="3" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="41" fontId="14" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
@@ -1731,23 +1943,8 @@
     <xf numFmtId="41" fontId="14" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="41" fontId="14" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="41" fontId="14" fillId="0" borderId="29" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
@@ -1758,23 +1955,29 @@
     <xf numFmtId="41" fontId="14" fillId="0" borderId="30" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="29" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="31" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="30" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    <xf numFmtId="41" fontId="14" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="14" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="14" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="14" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="14" fillId="0" borderId="24" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="14" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="14" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="14" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="176" fontId="8" fillId="0" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
@@ -1803,457 +2006,295 @@
     <xf numFmtId="176" fontId="8" fillId="0" borderId="26" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="24" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="24" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="24" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="28" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="28" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="28" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="24" fillId="0" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="24" fillId="0" borderId="27" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="24" fillId="0" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="28" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="28" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="28" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="24" fillId="0" borderId="23" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="24" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="24" fillId="0" borderId="24" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="28" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="28" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="28" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="24" fillId="0" borderId="25" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="24" fillId="0" borderId="28" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="24" fillId="0" borderId="26" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="28" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="28" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="28" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="24" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="24" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="24" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="24" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="24" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="24" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="24" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="24" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="24" fillId="0" borderId="29" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="24" fillId="0" borderId="31" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="24" fillId="0" borderId="30" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="24" fillId="0" borderId="35" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="24" fillId="0" borderId="40" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="24" fillId="0" borderId="41" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="4" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="4" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="27" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="23" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="24" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="25" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="28" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="26" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="14" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="14" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="14" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="14" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="14" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="14" fillId="0" borderId="24" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="14" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="14" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="14" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="5" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="5" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="5" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="35" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="40" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="41" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="7" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="7" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="7" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="9" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="20" fillId="5" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="10" fillId="3" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="10" fillId="3" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="5" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="39" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="30" fillId="6" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="6" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="10" fillId="5" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2884,41 +2925,41 @@
     <col min="24" max="24" width="9.625" style="7" customWidth="1"/>
     <col min="25" max="25" width="8.5" style="7" customWidth="1"/>
     <col min="26" max="27" width="9" style="7"/>
-    <col min="28" max="28" width="9" style="76"/>
-    <col min="29" max="29" width="29.25" style="76" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="8.125" style="76" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="9" style="76"/>
+    <col min="28" max="28" width="9" style="72"/>
+    <col min="29" max="29" width="29.25" style="72" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="8.125" style="72" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="9" style="72"/>
     <col min="32" max="16384" width="9" style="7"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:40" s="1" customFormat="1" ht="54">
-      <c r="A1" s="241" t="s">
-        <v>129</v>
-      </c>
-      <c r="B1" s="241"/>
-      <c r="C1" s="241"/>
-      <c r="D1" s="241"/>
-      <c r="E1" s="241"/>
-      <c r="F1" s="241"/>
-      <c r="G1" s="241"/>
-      <c r="H1" s="241"/>
-      <c r="I1" s="241"/>
-      <c r="J1" s="241"/>
-      <c r="K1" s="241"/>
-      <c r="L1" s="241"/>
-      <c r="M1" s="241"/>
-      <c r="N1" s="241"/>
-      <c r="O1" s="241"/>
-      <c r="P1" s="241"/>
-      <c r="Q1" s="241"/>
-      <c r="R1" s="241"/>
-      <c r="S1" s="241"/>
-      <c r="T1" s="241"/>
-      <c r="U1" s="241"/>
-      <c r="V1" s="241"/>
-      <c r="W1" s="241"/>
-      <c r="X1" s="241"/>
-      <c r="Y1" s="241"/>
+      <c r="A1" s="89" t="s">
+        <v>127</v>
+      </c>
+      <c r="B1" s="89"/>
+      <c r="C1" s="89"/>
+      <c r="D1" s="89"/>
+      <c r="E1" s="89"/>
+      <c r="F1" s="89"/>
+      <c r="G1" s="89"/>
+      <c r="H1" s="89"/>
+      <c r="I1" s="89"/>
+      <c r="J1" s="89"/>
+      <c r="K1" s="89"/>
+      <c r="L1" s="89"/>
+      <c r="M1" s="89"/>
+      <c r="N1" s="89"/>
+      <c r="O1" s="89"/>
+      <c r="P1" s="89"/>
+      <c r="Q1" s="89"/>
+      <c r="R1" s="89"/>
+      <c r="S1" s="89"/>
+      <c r="T1" s="89"/>
+      <c r="U1" s="89"/>
+      <c r="V1" s="89"/>
+      <c r="W1" s="89"/>
+      <c r="X1" s="89"/>
+      <c r="Y1" s="89"/>
       <c r="AB1" s="2"/>
       <c r="AC1" s="3"/>
       <c r="AD1" s="3"/>
@@ -2973,33 +3014,33 @@
       <c r="AN2" s="3"/>
     </row>
     <row r="3" spans="1:40" s="1" customFormat="1" ht="26.25">
-      <c r="A3" s="242" t="s">
-        <v>134</v>
-      </c>
-      <c r="B3" s="242"/>
-      <c r="C3" s="242"/>
-      <c r="D3" s="242"/>
-      <c r="E3" s="242"/>
-      <c r="F3" s="242"/>
-      <c r="G3" s="242"/>
-      <c r="H3" s="242"/>
-      <c r="I3" s="242"/>
-      <c r="J3" s="242"/>
-      <c r="K3" s="242"/>
-      <c r="L3" s="242"/>
-      <c r="M3" s="242"/>
-      <c r="N3" s="242"/>
-      <c r="O3" s="242"/>
-      <c r="P3" s="242"/>
-      <c r="Q3" s="242"/>
-      <c r="R3" s="242"/>
-      <c r="S3" s="242"/>
-      <c r="T3" s="242"/>
-      <c r="U3" s="242"/>
-      <c r="V3" s="242"/>
-      <c r="W3" s="242"/>
-      <c r="X3" s="242"/>
-      <c r="Y3" s="242"/>
+      <c r="A3" s="90" t="s">
+        <v>132</v>
+      </c>
+      <c r="B3" s="90"/>
+      <c r="C3" s="90"/>
+      <c r="D3" s="90"/>
+      <c r="E3" s="90"/>
+      <c r="F3" s="90"/>
+      <c r="G3" s="90"/>
+      <c r="H3" s="90"/>
+      <c r="I3" s="90"/>
+      <c r="J3" s="90"/>
+      <c r="K3" s="90"/>
+      <c r="L3" s="90"/>
+      <c r="M3" s="90"/>
+      <c r="N3" s="90"/>
+      <c r="O3" s="90"/>
+      <c r="P3" s="90"/>
+      <c r="Q3" s="90"/>
+      <c r="R3" s="90"/>
+      <c r="S3" s="90"/>
+      <c r="T3" s="90"/>
+      <c r="U3" s="90"/>
+      <c r="V3" s="90"/>
+      <c r="W3" s="90"/>
+      <c r="X3" s="90"/>
+      <c r="Y3" s="90"/>
       <c r="AB3" s="2"/>
       <c r="AC3" s="3"/>
       <c r="AD3" s="3"/>
@@ -3096,41 +3137,41 @@
     </row>
     <row r="6" spans="1:40" s="1" customFormat="1" ht="20.100000000000001" customHeight="1">
       <c r="A6" s="8" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B6" s="8"/>
-      <c r="C6" s="243">
+      <c r="C6" s="91">
         <f ca="1">TODAY()</f>
-        <v>46148</v>
-      </c>
-      <c r="D6" s="243"/>
-      <c r="E6" s="243"/>
-      <c r="F6" s="243"/>
+        <v>46150</v>
+      </c>
+      <c r="D6" s="91"/>
+      <c r="E6" s="91"/>
+      <c r="F6" s="91"/>
       <c r="G6" s="8"/>
       <c r="H6" s="8"/>
       <c r="I6" s="8"/>
       <c r="J6" s="9"/>
-      <c r="K6" s="230" t="s">
+      <c r="K6" s="114" t="s">
         <v>1</v>
       </c>
-      <c r="L6" s="222" t="s">
+      <c r="L6" s="107" t="s">
         <v>2</v>
       </c>
-      <c r="M6" s="223"/>
-      <c r="N6" s="224"/>
-      <c r="O6" s="249" t="s">
+      <c r="M6" s="108"/>
+      <c r="N6" s="109"/>
+      <c r="O6" s="101" t="s">
         <v>18</v>
       </c>
-      <c r="P6" s="250"/>
-      <c r="Q6" s="250"/>
-      <c r="R6" s="250"/>
-      <c r="S6" s="250"/>
-      <c r="T6" s="250"/>
-      <c r="U6" s="250"/>
-      <c r="V6" s="250"/>
-      <c r="W6" s="250"/>
-      <c r="X6" s="250"/>
-      <c r="Y6" s="251"/>
+      <c r="P6" s="102"/>
+      <c r="Q6" s="102"/>
+      <c r="R6" s="102"/>
+      <c r="S6" s="102"/>
+      <c r="T6" s="102"/>
+      <c r="U6" s="102"/>
+      <c r="V6" s="102"/>
+      <c r="W6" s="102"/>
+      <c r="X6" s="102"/>
+      <c r="Y6" s="103"/>
       <c r="AB6" s="2"/>
       <c r="AC6" s="3"/>
       <c r="AD6" s="3"/>
@@ -3147,11 +3188,11 @@
     </row>
     <row r="7" spans="1:40" s="1" customFormat="1" ht="20.100000000000001" customHeight="1">
       <c r="A7" s="10" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B7" s="8"/>
       <c r="C7" s="8" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="D7" s="8"/>
       <c r="E7" s="8"/>
@@ -3160,29 +3201,29 @@
       <c r="H7" s="8"/>
       <c r="I7" s="8"/>
       <c r="J7" s="9"/>
-      <c r="K7" s="231"/>
-      <c r="L7" s="229" t="s">
+      <c r="K7" s="115"/>
+      <c r="L7" s="93" t="s">
         <v>22</v>
       </c>
-      <c r="M7" s="192"/>
-      <c r="N7" s="193"/>
-      <c r="O7" s="197" t="s">
+      <c r="M7" s="94"/>
+      <c r="N7" s="95"/>
+      <c r="O7" s="104" t="s">
         <v>17</v>
       </c>
-      <c r="P7" s="198"/>
-      <c r="Q7" s="198"/>
-      <c r="R7" s="198"/>
-      <c r="S7" s="228" t="s">
+      <c r="P7" s="105"/>
+      <c r="Q7" s="105"/>
+      <c r="R7" s="105"/>
+      <c r="S7" s="113" t="s">
         <v>25</v>
       </c>
-      <c r="T7" s="192"/>
-      <c r="U7" s="193"/>
-      <c r="V7" s="197" t="s">
+      <c r="T7" s="94"/>
+      <c r="U7" s="95"/>
+      <c r="V7" s="104" t="s">
         <v>20</v>
       </c>
-      <c r="W7" s="198"/>
-      <c r="X7" s="198"/>
-      <c r="Y7" s="221"/>
+      <c r="W7" s="105"/>
+      <c r="X7" s="105"/>
+      <c r="Y7" s="106"/>
       <c r="AB7" s="2"/>
       <c r="AC7" s="2"/>
       <c r="AD7" s="2"/>
@@ -3199,25 +3240,25 @@
       <c r="H8" s="11"/>
       <c r="I8" s="11"/>
       <c r="J8" s="12"/>
-      <c r="K8" s="231"/>
-      <c r="L8" s="229" t="s">
+      <c r="K8" s="115"/>
+      <c r="L8" s="93" t="s">
         <v>21</v>
       </c>
-      <c r="M8" s="192"/>
-      <c r="N8" s="193"/>
-      <c r="O8" s="197" t="s">
-        <v>128</v>
-      </c>
-      <c r="P8" s="198"/>
-      <c r="Q8" s="198"/>
-      <c r="R8" s="198"/>
-      <c r="S8" s="198"/>
-      <c r="T8" s="198"/>
-      <c r="U8" s="198"/>
-      <c r="V8" s="198"/>
-      <c r="W8" s="198"/>
-      <c r="X8" s="198"/>
-      <c r="Y8" s="221"/>
+      <c r="M8" s="94"/>
+      <c r="N8" s="95"/>
+      <c r="O8" s="104" t="s">
+        <v>126</v>
+      </c>
+      <c r="P8" s="105"/>
+      <c r="Q8" s="105"/>
+      <c r="R8" s="105"/>
+      <c r="S8" s="105"/>
+      <c r="T8" s="105"/>
+      <c r="U8" s="105"/>
+      <c r="V8" s="105"/>
+      <c r="W8" s="105"/>
+      <c r="X8" s="105"/>
+      <c r="Y8" s="106"/>
       <c r="AA8" s="2"/>
       <c r="AB8" s="2"/>
       <c r="AC8" s="2"/>
@@ -3237,29 +3278,29 @@
       <c r="H9" s="10"/>
       <c r="I9" s="8"/>
       <c r="J9" s="10"/>
-      <c r="K9" s="231"/>
-      <c r="L9" s="229" t="s">
+      <c r="K9" s="115"/>
+      <c r="L9" s="93" t="s">
         <v>23</v>
       </c>
-      <c r="M9" s="192"/>
-      <c r="N9" s="193"/>
-      <c r="O9" s="197" t="s">
+      <c r="M9" s="94"/>
+      <c r="N9" s="95"/>
+      <c r="O9" s="104" t="s">
         <v>9</v>
       </c>
-      <c r="P9" s="198"/>
-      <c r="Q9" s="198"/>
-      <c r="R9" s="198"/>
-      <c r="S9" s="191" t="s">
+      <c r="P9" s="105"/>
+      <c r="Q9" s="105"/>
+      <c r="R9" s="105"/>
+      <c r="S9" s="120" t="s">
         <v>26</v>
       </c>
-      <c r="T9" s="192"/>
-      <c r="U9" s="193"/>
-      <c r="V9" s="201" t="s">
+      <c r="T9" s="94"/>
+      <c r="U9" s="95"/>
+      <c r="V9" s="126" t="s">
         <v>31</v>
       </c>
-      <c r="W9" s="202"/>
-      <c r="X9" s="202"/>
-      <c r="Y9" s="203"/>
+      <c r="W9" s="127"/>
+      <c r="X9" s="127"/>
+      <c r="Y9" s="128"/>
       <c r="AB9" s="2"/>
       <c r="AC9" s="2"/>
       <c r="AD9" s="2"/>
@@ -3278,29 +3319,29 @@
       <c r="H10" s="10"/>
       <c r="I10" s="8"/>
       <c r="J10" s="9"/>
-      <c r="K10" s="232"/>
-      <c r="L10" s="246" t="s">
+      <c r="K10" s="116"/>
+      <c r="L10" s="98" t="s">
         <v>24</v>
       </c>
-      <c r="M10" s="247"/>
-      <c r="N10" s="248"/>
-      <c r="O10" s="199" t="s">
-        <v>76</v>
-      </c>
-      <c r="P10" s="200"/>
-      <c r="Q10" s="200"/>
-      <c r="R10" s="200"/>
-      <c r="S10" s="194" t="s">
-        <v>63</v>
-      </c>
-      <c r="T10" s="195"/>
-      <c r="U10" s="196"/>
-      <c r="V10" s="199" t="s">
-        <v>77</v>
-      </c>
-      <c r="W10" s="200"/>
-      <c r="X10" s="200"/>
-      <c r="Y10" s="204"/>
+      <c r="M10" s="99"/>
+      <c r="N10" s="100"/>
+      <c r="O10" s="124" t="s">
+        <v>74</v>
+      </c>
+      <c r="P10" s="125"/>
+      <c r="Q10" s="125"/>
+      <c r="R10" s="125"/>
+      <c r="S10" s="121" t="s">
+        <v>61</v>
+      </c>
+      <c r="T10" s="122"/>
+      <c r="U10" s="123"/>
+      <c r="V10" s="124" t="s">
+        <v>75</v>
+      </c>
+      <c r="W10" s="125"/>
+      <c r="X10" s="125"/>
+      <c r="Y10" s="129"/>
       <c r="AB10" s="2"/>
       <c r="AC10" s="2"/>
       <c r="AD10" s="2"/>
@@ -3333,17 +3374,17 @@
       <c r="X11" s="2"/>
       <c r="Y11" s="2"/>
       <c r="AB11" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="AC11" s="2" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="AD11" s="2"/>
       <c r="AE11" s="2"/>
     </row>
     <row r="12" spans="1:40" s="1" customFormat="1" ht="20.100000000000001" customHeight="1">
       <c r="A12" s="14" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B12" s="15"/>
       <c r="C12" s="15"/>
@@ -3351,14 +3392,14 @@
       <c r="E12" s="15"/>
       <c r="F12" s="15"/>
       <c r="G12" s="15"/>
-      <c r="H12" s="135"/>
-      <c r="I12" s="135"/>
-      <c r="J12" s="135"/>
-      <c r="K12" s="135"/>
+      <c r="H12" s="92"/>
+      <c r="I12" s="92"/>
+      <c r="J12" s="92"/>
+      <c r="K12" s="92"/>
       <c r="L12" s="15"/>
       <c r="M12" s="16"/>
       <c r="N12" s="14" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="O12" s="17"/>
       <c r="P12" s="17"/>
@@ -3372,29 +3413,29 @@
       <c r="X12" s="17"/>
       <c r="Y12" s="18"/>
       <c r="AB12" s="19" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="AC12" s="20" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="AD12" s="20" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="AE12" s="21" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="13" spans="1:40" s="30" customFormat="1" ht="20.100000000000001" customHeight="1">
       <c r="A13" s="22"/>
       <c r="B13" s="23" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D13" s="24"/>
       <c r="E13" s="10" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="F13" s="10"/>
       <c r="G13" s="10"/>
@@ -3406,37 +3447,37 @@
       <c r="M13" s="28"/>
       <c r="N13" s="22"/>
       <c r="O13" s="3" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="P13" s="10" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="Q13" s="3"/>
-      <c r="R13" s="245" t="s">
+      <c r="R13" s="97" t="s">
+        <v>117</v>
+      </c>
+      <c r="S13" s="97"/>
+      <c r="T13" s="23" t="s">
+        <v>118</v>
+      </c>
+      <c r="U13" s="10" t="s">
         <v>119</v>
-      </c>
-      <c r="S13" s="245"/>
-      <c r="T13" s="23" t="s">
-        <v>120</v>
-      </c>
-      <c r="U13" s="10" t="s">
-        <v>121</v>
       </c>
       <c r="V13" s="3"/>
       <c r="W13" s="3"/>
       <c r="X13" s="3"/>
       <c r="Y13" s="29"/>
       <c r="AB13" s="31" t="s">
+        <v>77</v>
+      </c>
+      <c r="AC13" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="AD13" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="AC13" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="AD13" s="2" t="s">
-        <v>81</v>
-      </c>
       <c r="AE13" s="32" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="14" spans="1:40" s="30" customFormat="1" ht="20.100000000000001" customHeight="1">
@@ -3445,11 +3486,11 @@
         <v>29</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="D14" s="24"/>
       <c r="E14" s="10" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="F14" s="10"/>
       <c r="G14" s="10"/>
@@ -3464,18 +3505,18 @@
         <v>29</v>
       </c>
       <c r="P14" s="10" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="Q14" s="10"/>
-      <c r="R14" s="244" t="s">
-        <v>122</v>
-      </c>
-      <c r="S14" s="244"/>
+      <c r="R14" s="96" t="s">
+        <v>120</v>
+      </c>
+      <c r="S14" s="96"/>
       <c r="T14" s="23" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="U14" s="10" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="V14" s="10"/>
       <c r="W14" s="10"/>
@@ -3489,14 +3530,14 @@
     <row r="15" spans="1:40" s="1" customFormat="1" ht="20.100000000000001" customHeight="1">
       <c r="A15" s="35"/>
       <c r="B15" s="23" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C15" s="36" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="D15" s="10"/>
       <c r="E15" s="37" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="F15" s="37"/>
       <c r="G15" s="10"/>
@@ -3508,50 +3549,50 @@
       <c r="M15" s="38"/>
       <c r="N15" s="33"/>
       <c r="O15" s="10" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="P15" s="10" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="Q15" s="10"/>
-      <c r="R15" s="244" t="s">
-        <v>122</v>
-      </c>
-      <c r="S15" s="244"/>
+      <c r="R15" s="96" t="s">
+        <v>120</v>
+      </c>
+      <c r="S15" s="96"/>
       <c r="T15" s="23" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="U15" s="10" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="V15" s="10"/>
       <c r="W15" s="10"/>
       <c r="X15" s="10"/>
       <c r="Y15" s="34"/>
       <c r="AB15" s="31" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="AC15" s="2" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="AD15" s="2" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="AE15" s="39" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="16" spans="1:40" s="1" customFormat="1" ht="20.100000000000001" customHeight="1">
       <c r="A16" s="35"/>
       <c r="B16" s="23" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C16" s="36" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D16" s="10"/>
       <c r="E16" s="10" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="F16" s="37"/>
       <c r="G16" s="10"/>
@@ -3563,21 +3604,21 @@
       <c r="M16" s="38"/>
       <c r="N16" s="33"/>
       <c r="O16" s="10" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="P16" s="10" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="Q16" s="10"/>
-      <c r="R16" s="244" t="s">
-        <v>122</v>
-      </c>
-      <c r="S16" s="244"/>
+      <c r="R16" s="96" t="s">
+        <v>120</v>
+      </c>
+      <c r="S16" s="96"/>
       <c r="T16" s="23" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="U16" s="10" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="V16" s="10"/>
       <c r="W16" s="10"/>
@@ -3589,27 +3630,27 @@
       <c r="AE16" s="39"/>
     </row>
     <row r="17" spans="1:34" s="1" customFormat="1" ht="20.100000000000001" customHeight="1" thickBot="1">
-      <c r="A17" s="225" t="s">
-        <v>78</v>
-      </c>
-      <c r="B17" s="226"/>
-      <c r="C17" s="226"/>
-      <c r="D17" s="226"/>
-      <c r="E17" s="226"/>
-      <c r="F17" s="226"/>
-      <c r="G17" s="226"/>
-      <c r="H17" s="226"/>
-      <c r="I17" s="226"/>
-      <c r="J17" s="226"/>
-      <c r="K17" s="226"/>
-      <c r="L17" s="226"/>
-      <c r="M17" s="227"/>
+      <c r="A17" s="110" t="s">
+        <v>76</v>
+      </c>
+      <c r="B17" s="111"/>
+      <c r="C17" s="111"/>
+      <c r="D17" s="111"/>
+      <c r="E17" s="111"/>
+      <c r="F17" s="111"/>
+      <c r="G17" s="111"/>
+      <c r="H17" s="111"/>
+      <c r="I17" s="111"/>
+      <c r="J17" s="111"/>
+      <c r="K17" s="111"/>
+      <c r="L17" s="111"/>
+      <c r="M17" s="112"/>
       <c r="N17" s="40"/>
       <c r="O17" s="41" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="P17" s="41" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="Q17" s="41"/>
       <c r="R17" s="41"/>
@@ -3621,1386 +3662,1386 @@
       <c r="X17" s="41"/>
       <c r="Y17" s="42"/>
       <c r="AB17" s="31" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="AC17" s="2" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="AD17" s="2" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="AE17" s="39" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="18" spans="1:34" s="45" customFormat="1" ht="39.950000000000003" customHeight="1">
-      <c r="A18" s="205" t="s">
-        <v>68</v>
-      </c>
-      <c r="B18" s="206"/>
-      <c r="C18" s="206"/>
-      <c r="D18" s="206"/>
-      <c r="E18" s="206"/>
-      <c r="F18" s="206"/>
-      <c r="G18" s="206"/>
-      <c r="H18" s="206"/>
-      <c r="I18" s="207"/>
-      <c r="J18" s="238" t="s">
+      <c r="A18" s="130" t="s">
+        <v>66</v>
+      </c>
+      <c r="B18" s="131"/>
+      <c r="C18" s="131"/>
+      <c r="D18" s="131"/>
+      <c r="E18" s="131"/>
+      <c r="F18" s="131"/>
+      <c r="G18" s="131"/>
+      <c r="H18" s="131"/>
+      <c r="I18" s="132"/>
+      <c r="J18" s="86" t="s">
         <v>0</v>
       </c>
-      <c r="K18" s="239"/>
-      <c r="L18" s="239"/>
-      <c r="M18" s="240">
+      <c r="K18" s="87"/>
+      <c r="L18" s="87"/>
+      <c r="M18" s="88">
         <f>U41</f>
         <v>1600000</v>
       </c>
-      <c r="N18" s="240"/>
-      <c r="O18" s="240"/>
-      <c r="P18" s="240"/>
-      <c r="Q18" s="240"/>
+      <c r="N18" s="88"/>
+      <c r="O18" s="88"/>
+      <c r="P18" s="88"/>
+      <c r="Q18" s="88"/>
       <c r="R18" s="43" t="s">
         <v>28</v>
       </c>
       <c r="S18" s="43" t="s">
-        <v>55</v>
-      </c>
-      <c r="T18" s="237">
+        <v>54</v>
+      </c>
+      <c r="T18" s="85">
         <f>U41</f>
         <v>1600000</v>
       </c>
-      <c r="U18" s="237"/>
-      <c r="V18" s="237"/>
-      <c r="W18" s="237"/>
-      <c r="X18" s="237"/>
+      <c r="U18" s="85"/>
+      <c r="V18" s="85"/>
+      <c r="W18" s="85"/>
+      <c r="X18" s="85"/>
       <c r="Y18" s="44" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="AB18" s="19" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="AC18" s="20" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="AD18" s="20" t="s">
+        <v>78</v>
+      </c>
+      <c r="AE18" s="21" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="19" spans="1:34" s="1" customFormat="1" ht="20.100000000000001" customHeight="1">
+      <c r="A19" s="166" t="s">
+        <v>16</v>
+      </c>
+      <c r="B19" s="167"/>
+      <c r="C19" s="167"/>
+      <c r="D19" s="167"/>
+      <c r="E19" s="167"/>
+      <c r="F19" s="167"/>
+      <c r="G19" s="167"/>
+      <c r="H19" s="167"/>
+      <c r="I19" s="168"/>
+      <c r="J19" s="169" t="s">
+        <v>58</v>
+      </c>
+      <c r="K19" s="170"/>
+      <c r="L19" s="170"/>
+      <c r="M19" s="170"/>
+      <c r="N19" s="171"/>
+      <c r="O19" s="172" t="s">
+        <v>60</v>
+      </c>
+      <c r="P19" s="173"/>
+      <c r="Q19" s="174"/>
+      <c r="R19" s="166" t="s">
+        <v>43</v>
+      </c>
+      <c r="S19" s="167"/>
+      <c r="T19" s="167"/>
+      <c r="U19" s="167"/>
+      <c r="V19" s="168"/>
+      <c r="W19" s="166" t="s">
+        <v>42</v>
+      </c>
+      <c r="X19" s="167"/>
+      <c r="Y19" s="168"/>
+      <c r="AB19" s="31" t="s">
+        <v>82</v>
+      </c>
+      <c r="AC19" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="AD19" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="AE19" s="32" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="20" spans="1:34" s="1" customFormat="1" ht="20.100000000000001" customHeight="1">
+      <c r="A20" s="175"/>
+      <c r="B20" s="176"/>
+      <c r="C20" s="176"/>
+      <c r="D20" s="176"/>
+      <c r="E20" s="176"/>
+      <c r="F20" s="176"/>
+      <c r="G20" s="176"/>
+      <c r="H20" s="176"/>
+      <c r="I20" s="177"/>
+      <c r="J20" s="178" t="s">
+        <v>27</v>
+      </c>
+      <c r="K20" s="179" t="s">
+        <v>55</v>
+      </c>
+      <c r="L20" s="180" t="s">
+        <v>56</v>
+      </c>
+      <c r="M20" s="178" t="s">
+        <v>55</v>
+      </c>
+      <c r="N20" s="181" t="s">
+        <v>57</v>
+      </c>
+      <c r="O20" s="182"/>
+      <c r="P20" s="183"/>
+      <c r="Q20" s="184"/>
+      <c r="R20" s="175"/>
+      <c r="S20" s="176"/>
+      <c r="T20" s="176"/>
+      <c r="U20" s="176"/>
+      <c r="V20" s="177"/>
+      <c r="W20" s="175"/>
+      <c r="X20" s="176"/>
+      <c r="Y20" s="177"/>
+      <c r="AB20" s="31" t="s">
+        <v>82</v>
+      </c>
+      <c r="AC20" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="AD20" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="AE18" s="21" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="19" spans="1:34" s="1" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A19" s="134" t="s">
-        <v>16</v>
-      </c>
-      <c r="B19" s="135"/>
-      <c r="C19" s="135"/>
-      <c r="D19" s="135"/>
-      <c r="E19" s="135"/>
-      <c r="F19" s="135"/>
-      <c r="G19" s="135"/>
-      <c r="H19" s="135"/>
-      <c r="I19" s="136"/>
-      <c r="J19" s="113" t="s">
+      <c r="AE20" s="39" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="21" spans="1:34" s="1" customFormat="1" ht="31.5" customHeight="1" thickBot="1">
+      <c r="A21" s="229" t="s">
         <v>59</v>
       </c>
-      <c r="K19" s="114"/>
-      <c r="L19" s="114"/>
-      <c r="M19" s="114"/>
-      <c r="N19" s="115"/>
-      <c r="O19" s="128" t="s">
-        <v>61</v>
-      </c>
-      <c r="P19" s="129"/>
-      <c r="Q19" s="130"/>
-      <c r="R19" s="134" t="s">
-        <v>43</v>
-      </c>
-      <c r="S19" s="135"/>
-      <c r="T19" s="135"/>
-      <c r="U19" s="135"/>
-      <c r="V19" s="136"/>
-      <c r="W19" s="134" t="s">
-        <v>42</v>
-      </c>
-      <c r="X19" s="135"/>
-      <c r="Y19" s="136"/>
-      <c r="AB19" s="31" t="s">
-        <v>84</v>
-      </c>
-      <c r="AC19" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="AD19" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="AE19" s="32" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="20" spans="1:34" s="1" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A20" s="137"/>
-      <c r="B20" s="138"/>
-      <c r="C20" s="138"/>
-      <c r="D20" s="138"/>
-      <c r="E20" s="138"/>
-      <c r="F20" s="138"/>
-      <c r="G20" s="138"/>
-      <c r="H20" s="138"/>
-      <c r="I20" s="139"/>
-      <c r="J20" s="46" t="s">
-        <v>27</v>
-      </c>
-      <c r="K20" s="47" t="s">
-        <v>56</v>
-      </c>
-      <c r="L20" s="48" t="s">
-        <v>57</v>
-      </c>
-      <c r="M20" s="46" t="s">
-        <v>56</v>
-      </c>
-      <c r="N20" s="49" t="s">
-        <v>58</v>
-      </c>
-      <c r="O20" s="131"/>
-      <c r="P20" s="132"/>
-      <c r="Q20" s="133"/>
-      <c r="R20" s="137"/>
-      <c r="S20" s="138"/>
-      <c r="T20" s="138"/>
-      <c r="U20" s="138"/>
-      <c r="V20" s="139"/>
-      <c r="W20" s="137"/>
-      <c r="X20" s="138"/>
-      <c r="Y20" s="139"/>
-      <c r="AB20" s="31" t="s">
-        <v>84</v>
-      </c>
-      <c r="AC20" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="AD20" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="AE20" s="39" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="21" spans="1:34" s="1" customFormat="1" ht="31.5" customHeight="1" thickBot="1">
-      <c r="A21" s="95" t="s">
-        <v>60</v>
-      </c>
-      <c r="B21" s="96"/>
-      <c r="C21" s="96"/>
-      <c r="D21" s="96"/>
-      <c r="E21" s="96"/>
-      <c r="F21" s="96"/>
-      <c r="G21" s="96"/>
-      <c r="H21" s="96"/>
-      <c r="I21" s="97"/>
-      <c r="J21" s="110" t="s">
+      <c r="B21" s="230"/>
+      <c r="C21" s="230"/>
+      <c r="D21" s="230"/>
+      <c r="E21" s="230"/>
+      <c r="F21" s="230"/>
+      <c r="G21" s="230"/>
+      <c r="H21" s="230"/>
+      <c r="I21" s="231"/>
+      <c r="J21" s="232" t="s">
         <v>33</v>
       </c>
-      <c r="K21" s="111"/>
-      <c r="L21" s="111"/>
-      <c r="M21" s="111"/>
-      <c r="N21" s="112"/>
-      <c r="O21" s="116" t="s">
+      <c r="K21" s="233"/>
+      <c r="L21" s="233"/>
+      <c r="M21" s="233"/>
+      <c r="N21" s="234"/>
+      <c r="O21" s="185" t="s">
         <v>30</v>
       </c>
-      <c r="P21" s="117"/>
-      <c r="Q21" s="118"/>
-      <c r="R21" s="159">
+      <c r="P21" s="186"/>
+      <c r="Q21" s="187"/>
+      <c r="R21" s="188">
         <f>150000*8</f>
         <v>1200000</v>
       </c>
-      <c r="S21" s="160"/>
-      <c r="T21" s="160"/>
-      <c r="U21" s="160"/>
-      <c r="V21" s="161"/>
-      <c r="W21" s="92" t="s">
-        <v>125</v>
-      </c>
-      <c r="X21" s="93"/>
-      <c r="Y21" s="94"/>
-      <c r="AB21" s="50" t="s">
-        <v>84</v>
-      </c>
-      <c r="AC21" s="51" t="s">
+      <c r="S21" s="189"/>
+      <c r="T21" s="189"/>
+      <c r="U21" s="189"/>
+      <c r="V21" s="190"/>
+      <c r="W21" s="143" t="s">
+        <v>123</v>
+      </c>
+      <c r="X21" s="144"/>
+      <c r="Y21" s="145"/>
+      <c r="AB21" s="46" t="s">
+        <v>82</v>
+      </c>
+      <c r="AC21" s="47" t="s">
+        <v>86</v>
+      </c>
+      <c r="AD21" s="47" t="s">
+        <v>81</v>
+      </c>
+      <c r="AE21" s="48" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="22" spans="1:34" s="1" customFormat="1" ht="31.5" customHeight="1">
+      <c r="A22" s="229" t="s">
+        <v>45</v>
+      </c>
+      <c r="B22" s="230"/>
+      <c r="C22" s="230"/>
+      <c r="D22" s="230"/>
+      <c r="E22" s="230"/>
+      <c r="F22" s="230"/>
+      <c r="G22" s="230"/>
+      <c r="H22" s="230"/>
+      <c r="I22" s="231"/>
+      <c r="J22" s="232"/>
+      <c r="K22" s="233"/>
+      <c r="L22" s="233"/>
+      <c r="M22" s="233"/>
+      <c r="N22" s="234"/>
+      <c r="O22" s="191" t="s">
+        <v>10</v>
+      </c>
+      <c r="P22" s="192"/>
+      <c r="Q22" s="193"/>
+      <c r="R22" s="194">
+        <v>200000</v>
+      </c>
+      <c r="S22" s="195"/>
+      <c r="T22" s="195"/>
+      <c r="U22" s="195"/>
+      <c r="V22" s="196"/>
+      <c r="W22" s="133"/>
+      <c r="X22" s="146"/>
+      <c r="Y22" s="147"/>
+      <c r="AB22" s="19" t="s">
+        <v>77</v>
+      </c>
+      <c r="AC22" s="20" t="s">
+        <v>87</v>
+      </c>
+      <c r="AD22" s="20" t="s">
+        <v>78</v>
+      </c>
+      <c r="AE22" s="21" t="s">
+        <v>55</v>
+      </c>
+      <c r="AF22" s="133" t="s">
+        <v>92</v>
+      </c>
+      <c r="AG22" s="134"/>
+      <c r="AH22" s="135"/>
+    </row>
+    <row r="23" spans="1:34" s="1" customFormat="1" ht="31.5" customHeight="1">
+      <c r="A23" s="49"/>
+      <c r="B23" s="252" t="s">
+        <v>91</v>
+      </c>
+      <c r="C23" s="252"/>
+      <c r="D23" s="252"/>
+      <c r="E23" s="252"/>
+      <c r="F23" s="252"/>
+      <c r="G23" s="252"/>
+      <c r="H23" s="252"/>
+      <c r="I23" s="253"/>
+      <c r="J23" s="50"/>
+      <c r="K23" s="50" t="s">
+        <v>40</v>
+      </c>
+      <c r="L23" s="50" t="s">
+        <v>40</v>
+      </c>
+      <c r="M23" s="50" t="s">
+        <v>40</v>
+      </c>
+      <c r="N23" s="50" t="s">
+        <v>40</v>
+      </c>
+      <c r="O23" s="199"/>
+      <c r="P23" s="200"/>
+      <c r="Q23" s="201"/>
+      <c r="R23" s="202"/>
+      <c r="S23" s="203"/>
+      <c r="T23" s="203"/>
+      <c r="U23" s="203"/>
+      <c r="V23" s="204"/>
+      <c r="W23" s="148"/>
+      <c r="X23" s="149"/>
+      <c r="Y23" s="150"/>
+      <c r="AB23" s="31" t="s">
+        <v>77</v>
+      </c>
+      <c r="AC23" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="AD23" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="AE23" s="32" t="s">
+        <v>56</v>
+      </c>
+      <c r="AF23" s="136"/>
+      <c r="AG23" s="137"/>
+      <c r="AH23" s="138"/>
+    </row>
+    <row r="24" spans="1:34" s="1" customFormat="1" ht="31.5" customHeight="1">
+      <c r="A24" s="49"/>
+      <c r="B24" s="197" t="s">
+        <v>44</v>
+      </c>
+      <c r="C24" s="197"/>
+      <c r="D24" s="197"/>
+      <c r="E24" s="197"/>
+      <c r="F24" s="197"/>
+      <c r="G24" s="197"/>
+      <c r="H24" s="197"/>
+      <c r="I24" s="198"/>
+      <c r="J24" s="50"/>
+      <c r="K24" s="50"/>
+      <c r="L24" s="50"/>
+      <c r="M24" s="50"/>
+      <c r="N24" s="50" t="s">
+        <v>40</v>
+      </c>
+      <c r="O24" s="199"/>
+      <c r="P24" s="200"/>
+      <c r="Q24" s="201"/>
+      <c r="R24" s="202"/>
+      <c r="S24" s="203"/>
+      <c r="T24" s="203"/>
+      <c r="U24" s="203"/>
+      <c r="V24" s="204"/>
+      <c r="W24" s="148"/>
+      <c r="X24" s="149"/>
+      <c r="Y24" s="150"/>
+      <c r="AB24" s="31" t="s">
+        <v>77</v>
+      </c>
+      <c r="AC24" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="AD24" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="AE24" s="39" t="s">
+        <v>55</v>
+      </c>
+      <c r="AF24" s="136"/>
+      <c r="AG24" s="137"/>
+      <c r="AH24" s="138"/>
+    </row>
+    <row r="25" spans="1:34" s="1" customFormat="1" ht="31.5" customHeight="1" thickBot="1">
+      <c r="A25" s="49"/>
+      <c r="B25" s="197" t="s">
+        <v>3</v>
+      </c>
+      <c r="C25" s="197"/>
+      <c r="D25" s="197"/>
+      <c r="E25" s="197"/>
+      <c r="F25" s="197"/>
+      <c r="G25" s="197"/>
+      <c r="H25" s="197"/>
+      <c r="I25" s="198"/>
+      <c r="J25" s="50"/>
+      <c r="K25" s="50"/>
+      <c r="L25" s="50" t="s">
+        <v>40</v>
+      </c>
+      <c r="M25" s="50"/>
+      <c r="N25" s="50" t="s">
+        <v>40</v>
+      </c>
+      <c r="O25" s="205"/>
+      <c r="P25" s="206"/>
+      <c r="Q25" s="207"/>
+      <c r="R25" s="208"/>
+      <c r="S25" s="209"/>
+      <c r="T25" s="209"/>
+      <c r="U25" s="209"/>
+      <c r="V25" s="210"/>
+      <c r="W25" s="151"/>
+      <c r="X25" s="152"/>
+      <c r="Y25" s="153"/>
+      <c r="AB25" s="46" t="s">
+        <v>77</v>
+      </c>
+      <c r="AC25" s="47" t="s">
+        <v>87</v>
+      </c>
+      <c r="AD25" s="47" t="s">
+        <v>81</v>
+      </c>
+      <c r="AE25" s="48" t="s">
+        <v>57</v>
+      </c>
+      <c r="AF25" s="139"/>
+      <c r="AG25" s="140"/>
+      <c r="AH25" s="141"/>
+    </row>
+    <row r="26" spans="1:34" s="1" customFormat="1" ht="31.5" customHeight="1">
+      <c r="A26" s="229" t="s">
+        <v>46</v>
+      </c>
+      <c r="B26" s="230"/>
+      <c r="C26" s="230"/>
+      <c r="D26" s="230"/>
+      <c r="E26" s="230"/>
+      <c r="F26" s="230"/>
+      <c r="G26" s="230"/>
+      <c r="H26" s="230"/>
+      <c r="I26" s="231"/>
+      <c r="J26" s="51"/>
+      <c r="K26" s="52"/>
+      <c r="L26" s="52"/>
+      <c r="M26" s="52"/>
+      <c r="N26" s="53"/>
+      <c r="O26" s="191" t="s">
+        <v>11</v>
+      </c>
+      <c r="P26" s="192"/>
+      <c r="Q26" s="193"/>
+      <c r="R26" s="194">
+        <v>200000</v>
+      </c>
+      <c r="S26" s="195"/>
+      <c r="T26" s="195"/>
+      <c r="U26" s="195"/>
+      <c r="V26" s="196"/>
+      <c r="W26" s="133" t="s">
+        <v>72</v>
+      </c>
+      <c r="X26" s="134"/>
+      <c r="Y26" s="135"/>
+      <c r="AB26" s="19" t="s">
+        <v>82</v>
+      </c>
+      <c r="AC26" s="20" t="s">
+        <v>87</v>
+      </c>
+      <c r="AD26" s="20" t="s">
+        <v>78</v>
+      </c>
+      <c r="AE26" s="21" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="27" spans="1:34" s="1" customFormat="1" ht="31.5" customHeight="1">
+      <c r="A27" s="49"/>
+      <c r="B27" s="197" t="s">
+        <v>73</v>
+      </c>
+      <c r="C27" s="197"/>
+      <c r="D27" s="197"/>
+      <c r="E27" s="197"/>
+      <c r="F27" s="197"/>
+      <c r="G27" s="197"/>
+      <c r="H27" s="197"/>
+      <c r="I27" s="198"/>
+      <c r="J27" s="50"/>
+      <c r="K27" s="50"/>
+      <c r="L27" s="50"/>
+      <c r="M27" s="50"/>
+      <c r="N27" s="50" t="s">
+        <v>40</v>
+      </c>
+      <c r="O27" s="199"/>
+      <c r="P27" s="200"/>
+      <c r="Q27" s="201"/>
+      <c r="R27" s="202"/>
+      <c r="S27" s="203"/>
+      <c r="T27" s="203"/>
+      <c r="U27" s="203"/>
+      <c r="V27" s="204"/>
+      <c r="W27" s="136"/>
+      <c r="X27" s="137"/>
+      <c r="Y27" s="138"/>
+      <c r="AB27" s="31" t="s">
+        <v>82</v>
+      </c>
+      <c r="AC27" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="AD27" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="AE27" s="32" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="28" spans="1:34" s="1" customFormat="1" ht="31.5" customHeight="1">
+      <c r="A28" s="49"/>
+      <c r="B28" s="197" t="s">
+        <v>3</v>
+      </c>
+      <c r="C28" s="197"/>
+      <c r="D28" s="197"/>
+      <c r="E28" s="197"/>
+      <c r="F28" s="197"/>
+      <c r="G28" s="197"/>
+      <c r="H28" s="197"/>
+      <c r="I28" s="198"/>
+      <c r="J28" s="50"/>
+      <c r="K28" s="50"/>
+      <c r="L28" s="50"/>
+      <c r="M28" s="50"/>
+      <c r="N28" s="50" t="s">
+        <v>40</v>
+      </c>
+      <c r="O28" s="199"/>
+      <c r="P28" s="200"/>
+      <c r="Q28" s="201"/>
+      <c r="R28" s="202"/>
+      <c r="S28" s="203"/>
+      <c r="T28" s="203"/>
+      <c r="U28" s="203"/>
+      <c r="V28" s="204"/>
+      <c r="W28" s="136"/>
+      <c r="X28" s="137"/>
+      <c r="Y28" s="138"/>
+      <c r="AB28" s="31" t="s">
+        <v>82</v>
+      </c>
+      <c r="AC28" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="AD28" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="AE28" s="39" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="29" spans="1:34" s="1" customFormat="1" ht="31.5" customHeight="1" thickBot="1">
+      <c r="A29" s="229" t="s">
+        <v>47</v>
+      </c>
+      <c r="B29" s="230"/>
+      <c r="C29" s="230"/>
+      <c r="D29" s="230"/>
+      <c r="E29" s="230"/>
+      <c r="F29" s="230"/>
+      <c r="G29" s="230"/>
+      <c r="H29" s="230"/>
+      <c r="I29" s="231"/>
+      <c r="J29" s="51"/>
+      <c r="K29" s="52"/>
+      <c r="L29" s="52"/>
+      <c r="M29" s="52"/>
+      <c r="N29" s="53"/>
+      <c r="O29" s="191" t="s">
+        <v>12</v>
+      </c>
+      <c r="P29" s="192"/>
+      <c r="Q29" s="193"/>
+      <c r="R29" s="202"/>
+      <c r="S29" s="203"/>
+      <c r="T29" s="203"/>
+      <c r="U29" s="203"/>
+      <c r="V29" s="204"/>
+      <c r="W29" s="136"/>
+      <c r="X29" s="137"/>
+      <c r="Y29" s="138"/>
+      <c r="AB29" s="46" t="s">
+        <v>82</v>
+      </c>
+      <c r="AC29" s="47" t="s">
+        <v>87</v>
+      </c>
+      <c r="AD29" s="47" t="s">
+        <v>81</v>
+      </c>
+      <c r="AE29" s="48" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="30" spans="1:34" s="1" customFormat="1" ht="31.5" customHeight="1">
+      <c r="A30" s="54"/>
+      <c r="B30" s="197" t="s">
+        <v>73</v>
+      </c>
+      <c r="C30" s="197"/>
+      <c r="D30" s="197"/>
+      <c r="E30" s="197"/>
+      <c r="F30" s="197"/>
+      <c r="G30" s="197"/>
+      <c r="H30" s="197"/>
+      <c r="I30" s="198"/>
+      <c r="J30" s="55"/>
+      <c r="K30" s="55"/>
+      <c r="L30" s="55"/>
+      <c r="M30" s="55"/>
+      <c r="N30" s="50" t="s">
+        <v>40</v>
+      </c>
+      <c r="O30" s="199"/>
+      <c r="P30" s="200"/>
+      <c r="Q30" s="201"/>
+      <c r="R30" s="202"/>
+      <c r="S30" s="203"/>
+      <c r="T30" s="203"/>
+      <c r="U30" s="203"/>
+      <c r="V30" s="204"/>
+      <c r="W30" s="136"/>
+      <c r="X30" s="137"/>
+      <c r="Y30" s="138"/>
+      <c r="AB30" s="2" t="s">
         <v>88</v>
-      </c>
-      <c r="AD21" s="51" t="s">
-        <v>83</v>
-      </c>
-      <c r="AE21" s="52" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="22" spans="1:34" s="1" customFormat="1" ht="31.5" customHeight="1">
-      <c r="A22" s="95" t="s">
-        <v>45</v>
-      </c>
-      <c r="B22" s="96"/>
-      <c r="C22" s="96"/>
-      <c r="D22" s="96"/>
-      <c r="E22" s="96"/>
-      <c r="F22" s="96"/>
-      <c r="G22" s="96"/>
-      <c r="H22" s="96"/>
-      <c r="I22" s="97"/>
-      <c r="J22" s="110"/>
-      <c r="K22" s="111"/>
-      <c r="L22" s="111"/>
-      <c r="M22" s="111"/>
-      <c r="N22" s="112"/>
-      <c r="O22" s="119" t="s">
-        <v>10</v>
-      </c>
-      <c r="P22" s="120"/>
-      <c r="Q22" s="121"/>
-      <c r="R22" s="140">
-        <v>200000</v>
-      </c>
-      <c r="S22" s="141"/>
-      <c r="T22" s="141"/>
-      <c r="U22" s="141"/>
-      <c r="V22" s="142"/>
-      <c r="W22" s="77"/>
-      <c r="X22" s="162"/>
-      <c r="Y22" s="163"/>
-      <c r="AB22" s="19" t="s">
-        <v>79</v>
-      </c>
-      <c r="AC22" s="20" t="s">
-        <v>89</v>
-      </c>
-      <c r="AD22" s="20" t="s">
-        <v>80</v>
-      </c>
-      <c r="AE22" s="21" t="s">
-        <v>56</v>
-      </c>
-      <c r="AF22" s="77" t="s">
-        <v>94</v>
-      </c>
-      <c r="AG22" s="78"/>
-      <c r="AH22" s="79"/>
-    </row>
-    <row r="23" spans="1:34" s="1" customFormat="1" ht="31.5" customHeight="1">
-      <c r="A23" s="53"/>
-      <c r="B23" s="254" t="s">
-        <v>93</v>
-      </c>
-      <c r="C23" s="254"/>
-      <c r="D23" s="254"/>
-      <c r="E23" s="254"/>
-      <c r="F23" s="254"/>
-      <c r="G23" s="254"/>
-      <c r="H23" s="254"/>
-      <c r="I23" s="255"/>
-      <c r="J23" s="54"/>
-      <c r="K23" s="54" t="s">
-        <v>40</v>
-      </c>
-      <c r="L23" s="54" t="s">
-        <v>40</v>
-      </c>
-      <c r="M23" s="54" t="s">
-        <v>40</v>
-      </c>
-      <c r="N23" s="54" t="s">
-        <v>40</v>
-      </c>
-      <c r="O23" s="122"/>
-      <c r="P23" s="123"/>
-      <c r="Q23" s="124"/>
-      <c r="R23" s="143"/>
-      <c r="S23" s="144"/>
-      <c r="T23" s="144"/>
-      <c r="U23" s="144"/>
-      <c r="V23" s="145"/>
-      <c r="W23" s="164"/>
-      <c r="X23" s="165"/>
-      <c r="Y23" s="166"/>
-      <c r="AB23" s="31" t="s">
-        <v>79</v>
-      </c>
-      <c r="AC23" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="AD23" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="AE23" s="32" t="s">
-        <v>57</v>
-      </c>
-      <c r="AF23" s="80"/>
-      <c r="AG23" s="81"/>
-      <c r="AH23" s="82"/>
-    </row>
-    <row r="24" spans="1:34" s="1" customFormat="1" ht="31.5" customHeight="1">
-      <c r="A24" s="53"/>
-      <c r="B24" s="254" t="s">
-        <v>44</v>
-      </c>
-      <c r="C24" s="254"/>
-      <c r="D24" s="254"/>
-      <c r="E24" s="254"/>
-      <c r="F24" s="254"/>
-      <c r="G24" s="254"/>
-      <c r="H24" s="254"/>
-      <c r="I24" s="255"/>
-      <c r="J24" s="54"/>
-      <c r="K24" s="54"/>
-      <c r="L24" s="54"/>
-      <c r="M24" s="54"/>
-      <c r="N24" s="54" t="s">
-        <v>40</v>
-      </c>
-      <c r="O24" s="122"/>
-      <c r="P24" s="123"/>
-      <c r="Q24" s="124"/>
-      <c r="R24" s="143"/>
-      <c r="S24" s="144"/>
-      <c r="T24" s="144"/>
-      <c r="U24" s="144"/>
-      <c r="V24" s="145"/>
-      <c r="W24" s="164"/>
-      <c r="X24" s="165"/>
-      <c r="Y24" s="166"/>
-      <c r="AB24" s="31" t="s">
-        <v>79</v>
-      </c>
-      <c r="AC24" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="AD24" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="AE24" s="39" t="s">
-        <v>56</v>
-      </c>
-      <c r="AF24" s="80"/>
-      <c r="AG24" s="81"/>
-      <c r="AH24" s="82"/>
-    </row>
-    <row r="25" spans="1:34" s="1" customFormat="1" ht="31.5" customHeight="1" thickBot="1">
-      <c r="A25" s="53"/>
-      <c r="B25" s="254" t="s">
-        <v>3</v>
-      </c>
-      <c r="C25" s="254"/>
-      <c r="D25" s="254"/>
-      <c r="E25" s="254"/>
-      <c r="F25" s="254"/>
-      <c r="G25" s="254"/>
-      <c r="H25" s="254"/>
-      <c r="I25" s="255"/>
-      <c r="J25" s="54"/>
-      <c r="K25" s="54"/>
-      <c r="L25" s="54" t="s">
-        <v>40</v>
-      </c>
-      <c r="M25" s="54"/>
-      <c r="N25" s="54" t="s">
-        <v>40</v>
-      </c>
-      <c r="O25" s="125"/>
-      <c r="P25" s="126"/>
-      <c r="Q25" s="127"/>
-      <c r="R25" s="146"/>
-      <c r="S25" s="147"/>
-      <c r="T25" s="147"/>
-      <c r="U25" s="147"/>
-      <c r="V25" s="148"/>
-      <c r="W25" s="167"/>
-      <c r="X25" s="168"/>
-      <c r="Y25" s="169"/>
-      <c r="AB25" s="50" t="s">
-        <v>79</v>
-      </c>
-      <c r="AC25" s="51" t="s">
-        <v>89</v>
-      </c>
-      <c r="AD25" s="51" t="s">
-        <v>83</v>
-      </c>
-      <c r="AE25" s="52" t="s">
-        <v>58</v>
-      </c>
-      <c r="AF25" s="83"/>
-      <c r="AG25" s="84"/>
-      <c r="AH25" s="85"/>
-    </row>
-    <row r="26" spans="1:34" s="1" customFormat="1" ht="31.5" customHeight="1">
-      <c r="A26" s="95" t="s">
-        <v>46</v>
-      </c>
-      <c r="B26" s="96"/>
-      <c r="C26" s="96"/>
-      <c r="D26" s="96"/>
-      <c r="E26" s="96"/>
-      <c r="F26" s="96"/>
-      <c r="G26" s="96"/>
-      <c r="H26" s="96"/>
-      <c r="I26" s="97"/>
-      <c r="J26" s="55"/>
-      <c r="K26" s="56"/>
-      <c r="L26" s="56"/>
-      <c r="M26" s="56"/>
-      <c r="N26" s="57"/>
-      <c r="O26" s="119" t="s">
-        <v>11</v>
-      </c>
-      <c r="P26" s="120"/>
-      <c r="Q26" s="121"/>
-      <c r="R26" s="140">
-        <v>200000</v>
-      </c>
-      <c r="S26" s="141"/>
-      <c r="T26" s="141"/>
-      <c r="U26" s="141"/>
-      <c r="V26" s="142"/>
-      <c r="W26" s="77" t="s">
-        <v>74</v>
-      </c>
-      <c r="X26" s="78"/>
-      <c r="Y26" s="79"/>
-      <c r="AB26" s="19" t="s">
-        <v>84</v>
-      </c>
-      <c r="AC26" s="20" t="s">
-        <v>89</v>
-      </c>
-      <c r="AD26" s="20" t="s">
-        <v>80</v>
-      </c>
-      <c r="AE26" s="21" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="27" spans="1:34" s="1" customFormat="1" ht="31.5" customHeight="1">
-      <c r="A27" s="53"/>
-      <c r="B27" s="254" t="s">
-        <v>75</v>
-      </c>
-      <c r="C27" s="254"/>
-      <c r="D27" s="254"/>
-      <c r="E27" s="254"/>
-      <c r="F27" s="254"/>
-      <c r="G27" s="254"/>
-      <c r="H27" s="254"/>
-      <c r="I27" s="255"/>
-      <c r="J27" s="54"/>
-      <c r="K27" s="54"/>
-      <c r="L27" s="54"/>
-      <c r="M27" s="54"/>
-      <c r="N27" s="54" t="s">
-        <v>40</v>
-      </c>
-      <c r="O27" s="122"/>
-      <c r="P27" s="123"/>
-      <c r="Q27" s="124"/>
-      <c r="R27" s="143"/>
-      <c r="S27" s="144"/>
-      <c r="T27" s="144"/>
-      <c r="U27" s="144"/>
-      <c r="V27" s="145"/>
-      <c r="W27" s="80"/>
-      <c r="X27" s="81"/>
-      <c r="Y27" s="82"/>
-      <c r="AB27" s="31" t="s">
-        <v>84</v>
-      </c>
-      <c r="AC27" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="AD27" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="AE27" s="32" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="28" spans="1:34" s="1" customFormat="1" ht="31.5" customHeight="1">
-      <c r="A28" s="53"/>
-      <c r="B28" s="254" t="s">
-        <v>3</v>
-      </c>
-      <c r="C28" s="254"/>
-      <c r="D28" s="254"/>
-      <c r="E28" s="254"/>
-      <c r="F28" s="254"/>
-      <c r="G28" s="254"/>
-      <c r="H28" s="254"/>
-      <c r="I28" s="255"/>
-      <c r="J28" s="54"/>
-      <c r="K28" s="54"/>
-      <c r="L28" s="54"/>
-      <c r="M28" s="54"/>
-      <c r="N28" s="54" t="s">
-        <v>40</v>
-      </c>
-      <c r="O28" s="122"/>
-      <c r="P28" s="123"/>
-      <c r="Q28" s="124"/>
-      <c r="R28" s="143"/>
-      <c r="S28" s="144"/>
-      <c r="T28" s="144"/>
-      <c r="U28" s="144"/>
-      <c r="V28" s="145"/>
-      <c r="W28" s="80"/>
-      <c r="X28" s="81"/>
-      <c r="Y28" s="82"/>
-      <c r="AB28" s="31" t="s">
-        <v>84</v>
-      </c>
-      <c r="AC28" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="AD28" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="AE28" s="39" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="29" spans="1:34" s="1" customFormat="1" ht="31.5" customHeight="1" thickBot="1">
-      <c r="A29" s="95" t="s">
-        <v>47</v>
-      </c>
-      <c r="B29" s="96"/>
-      <c r="C29" s="96"/>
-      <c r="D29" s="96"/>
-      <c r="E29" s="96"/>
-      <c r="F29" s="96"/>
-      <c r="G29" s="96"/>
-      <c r="H29" s="96"/>
-      <c r="I29" s="97"/>
-      <c r="J29" s="55"/>
-      <c r="K29" s="56"/>
-      <c r="L29" s="56"/>
-      <c r="M29" s="56"/>
-      <c r="N29" s="57"/>
-      <c r="O29" s="119" t="s">
-        <v>12</v>
-      </c>
-      <c r="P29" s="120"/>
-      <c r="Q29" s="121"/>
-      <c r="R29" s="143"/>
-      <c r="S29" s="144"/>
-      <c r="T29" s="144"/>
-      <c r="U29" s="144"/>
-      <c r="V29" s="145"/>
-      <c r="W29" s="80"/>
-      <c r="X29" s="81"/>
-      <c r="Y29" s="82"/>
-      <c r="AB29" s="50" t="s">
-        <v>84</v>
-      </c>
-      <c r="AC29" s="51" t="s">
-        <v>89</v>
-      </c>
-      <c r="AD29" s="51" t="s">
-        <v>83</v>
-      </c>
-      <c r="AE29" s="52" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="30" spans="1:34" s="1" customFormat="1" ht="31.5" customHeight="1">
-      <c r="A30" s="58"/>
-      <c r="B30" s="254" t="s">
-        <v>75</v>
-      </c>
-      <c r="C30" s="254"/>
-      <c r="D30" s="254"/>
-      <c r="E30" s="254"/>
-      <c r="F30" s="254"/>
-      <c r="G30" s="254"/>
-      <c r="H30" s="254"/>
-      <c r="I30" s="255"/>
-      <c r="J30" s="59"/>
-      <c r="K30" s="59"/>
-      <c r="L30" s="59"/>
-      <c r="M30" s="59"/>
-      <c r="N30" s="54" t="s">
-        <v>40</v>
-      </c>
-      <c r="O30" s="122"/>
-      <c r="P30" s="123"/>
-      <c r="Q30" s="124"/>
-      <c r="R30" s="143"/>
-      <c r="S30" s="144"/>
-      <c r="T30" s="144"/>
-      <c r="U30" s="144"/>
-      <c r="V30" s="145"/>
-      <c r="W30" s="80"/>
-      <c r="X30" s="81"/>
-      <c r="Y30" s="82"/>
-      <c r="AB30" s="2" t="s">
-        <v>90</v>
       </c>
       <c r="AC30" s="2"/>
       <c r="AD30" s="2"/>
       <c r="AE30" s="2"/>
     </row>
     <row r="31" spans="1:34" s="1" customFormat="1" ht="31.5" customHeight="1">
-      <c r="A31" s="95" t="s">
+      <c r="A31" s="229" t="s">
         <v>48</v>
       </c>
-      <c r="B31" s="96"/>
-      <c r="C31" s="96"/>
-      <c r="D31" s="96"/>
-      <c r="E31" s="96"/>
-      <c r="F31" s="96"/>
-      <c r="G31" s="96"/>
-      <c r="H31" s="96"/>
-      <c r="I31" s="97"/>
-      <c r="J31" s="55"/>
-      <c r="K31" s="56"/>
-      <c r="L31" s="56"/>
-      <c r="M31" s="56"/>
-      <c r="N31" s="57"/>
-      <c r="O31" s="89" t="s">
+      <c r="B31" s="230"/>
+      <c r="C31" s="230"/>
+      <c r="D31" s="230"/>
+      <c r="E31" s="230"/>
+      <c r="F31" s="230"/>
+      <c r="G31" s="230"/>
+      <c r="H31" s="230"/>
+      <c r="I31" s="231"/>
+      <c r="J31" s="51"/>
+      <c r="K31" s="52"/>
+      <c r="L31" s="52"/>
+      <c r="M31" s="52"/>
+      <c r="N31" s="53"/>
+      <c r="O31" s="211" t="s">
         <v>13</v>
       </c>
-      <c r="P31" s="90"/>
-      <c r="Q31" s="91"/>
-      <c r="R31" s="146"/>
-      <c r="S31" s="147"/>
-      <c r="T31" s="147"/>
-      <c r="U31" s="147"/>
-      <c r="V31" s="148"/>
-      <c r="W31" s="83"/>
-      <c r="X31" s="84"/>
-      <c r="Y31" s="85"/>
+      <c r="P31" s="212"/>
+      <c r="Q31" s="213"/>
+      <c r="R31" s="208"/>
+      <c r="S31" s="209"/>
+      <c r="T31" s="209"/>
+      <c r="U31" s="209"/>
+      <c r="V31" s="210"/>
+      <c r="W31" s="139"/>
+      <c r="X31" s="140"/>
+      <c r="Y31" s="141"/>
       <c r="AB31" s="2" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="AC31" s="2" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="AD31" s="2"/>
       <c r="AE31" s="2"/>
     </row>
     <row r="32" spans="1:34" s="1" customFormat="1" ht="31.5" customHeight="1">
-      <c r="A32" s="212" t="s">
-        <v>49</v>
-      </c>
-      <c r="B32" s="213"/>
-      <c r="C32" s="214"/>
-      <c r="D32" s="86" t="s">
+      <c r="A32" s="235" t="s">
+        <v>133</v>
+      </c>
+      <c r="B32" s="236"/>
+      <c r="C32" s="237"/>
+      <c r="D32" s="163" t="s">
         <v>4</v>
       </c>
-      <c r="E32" s="87"/>
-      <c r="F32" s="87"/>
-      <c r="G32" s="87"/>
-      <c r="H32" s="87"/>
-      <c r="I32" s="88"/>
-      <c r="J32" s="60"/>
-      <c r="K32" s="54"/>
-      <c r="L32" s="54"/>
-      <c r="M32" s="54"/>
-      <c r="N32" s="54" t="s">
+      <c r="E32" s="164"/>
+      <c r="F32" s="164"/>
+      <c r="G32" s="164"/>
+      <c r="H32" s="164"/>
+      <c r="I32" s="165"/>
+      <c r="J32" s="56"/>
+      <c r="K32" s="50"/>
+      <c r="L32" s="50"/>
+      <c r="M32" s="50"/>
+      <c r="N32" s="50" t="s">
         <v>40</v>
       </c>
-      <c r="O32" s="119" t="s">
+      <c r="O32" s="191" t="s">
         <v>19</v>
       </c>
-      <c r="P32" s="120"/>
-      <c r="Q32" s="121"/>
-      <c r="R32" s="149">
+      <c r="P32" s="192"/>
+      <c r="Q32" s="193"/>
+      <c r="R32" s="214">
         <v>200000</v>
       </c>
-      <c r="S32" s="150"/>
-      <c r="T32" s="150"/>
-      <c r="U32" s="150"/>
-      <c r="V32" s="151"/>
-      <c r="W32" s="158"/>
-      <c r="X32" s="78"/>
-      <c r="Y32" s="79"/>
+      <c r="S32" s="215"/>
+      <c r="T32" s="215"/>
+      <c r="U32" s="215"/>
+      <c r="V32" s="216"/>
+      <c r="W32" s="142"/>
+      <c r="X32" s="134"/>
+      <c r="Y32" s="135"/>
       <c r="AB32" s="2"/>
       <c r="AC32" s="2"/>
       <c r="AD32" s="2"/>
       <c r="AE32" s="2"/>
     </row>
     <row r="33" spans="1:31" s="1" customFormat="1" ht="31.5" customHeight="1">
-      <c r="A33" s="215"/>
-      <c r="B33" s="216"/>
-      <c r="C33" s="217"/>
-      <c r="D33" s="86" t="s">
+      <c r="A33" s="238"/>
+      <c r="B33" s="239"/>
+      <c r="C33" s="240"/>
+      <c r="D33" s="163" t="s">
         <v>5</v>
       </c>
-      <c r="E33" s="87"/>
-      <c r="F33" s="87"/>
-      <c r="G33" s="87"/>
-      <c r="H33" s="87"/>
-      <c r="I33" s="88"/>
-      <c r="J33" s="60"/>
-      <c r="K33" s="54"/>
-      <c r="L33" s="54"/>
-      <c r="M33" s="54"/>
-      <c r="N33" s="54" t="s">
+      <c r="E33" s="164"/>
+      <c r="F33" s="164"/>
+      <c r="G33" s="164"/>
+      <c r="H33" s="164"/>
+      <c r="I33" s="165"/>
+      <c r="J33" s="56"/>
+      <c r="K33" s="50"/>
+      <c r="L33" s="50"/>
+      <c r="M33" s="50"/>
+      <c r="N33" s="50" t="s">
         <v>40</v>
       </c>
-      <c r="O33" s="122"/>
-      <c r="P33" s="123"/>
-      <c r="Q33" s="124"/>
-      <c r="R33" s="152"/>
-      <c r="S33" s="153"/>
-      <c r="T33" s="153"/>
-      <c r="U33" s="153"/>
-      <c r="V33" s="154"/>
-      <c r="W33" s="80"/>
-      <c r="X33" s="81"/>
-      <c r="Y33" s="82"/>
+      <c r="O33" s="199"/>
+      <c r="P33" s="200"/>
+      <c r="Q33" s="201"/>
+      <c r="R33" s="217"/>
+      <c r="S33" s="218"/>
+      <c r="T33" s="218"/>
+      <c r="U33" s="218"/>
+      <c r="V33" s="219"/>
+      <c r="W33" s="136"/>
+      <c r="X33" s="137"/>
+      <c r="Y33" s="138"/>
       <c r="AB33" s="2"/>
       <c r="AC33" s="2"/>
       <c r="AD33" s="2"/>
       <c r="AE33" s="2"/>
     </row>
     <row r="34" spans="1:31" s="1" customFormat="1" ht="31.5" customHeight="1">
-      <c r="A34" s="218"/>
-      <c r="B34" s="219"/>
-      <c r="C34" s="220"/>
-      <c r="D34" s="86" t="s">
+      <c r="A34" s="241"/>
+      <c r="B34" s="242"/>
+      <c r="C34" s="243"/>
+      <c r="D34" s="163" t="s">
         <v>6</v>
       </c>
-      <c r="E34" s="87"/>
-      <c r="F34" s="87"/>
-      <c r="G34" s="87"/>
-      <c r="H34" s="87"/>
-      <c r="I34" s="88"/>
-      <c r="J34" s="60"/>
-      <c r="K34" s="54" t="s">
+      <c r="E34" s="164"/>
+      <c r="F34" s="164"/>
+      <c r="G34" s="164"/>
+      <c r="H34" s="164"/>
+      <c r="I34" s="165"/>
+      <c r="J34" s="56"/>
+      <c r="K34" s="50" t="s">
         <v>40</v>
       </c>
-      <c r="L34" s="54" t="s">
+      <c r="L34" s="50" t="s">
         <v>40</v>
       </c>
-      <c r="M34" s="54" t="s">
+      <c r="M34" s="50" t="s">
         <v>40</v>
       </c>
-      <c r="N34" s="54" t="s">
+      <c r="N34" s="50" t="s">
         <v>40</v>
       </c>
-      <c r="O34" s="125"/>
-      <c r="P34" s="126"/>
-      <c r="Q34" s="127"/>
-      <c r="R34" s="155"/>
-      <c r="S34" s="156"/>
-      <c r="T34" s="156"/>
-      <c r="U34" s="156"/>
-      <c r="V34" s="157"/>
-      <c r="W34" s="83"/>
-      <c r="X34" s="84"/>
-      <c r="Y34" s="85"/>
+      <c r="O34" s="205"/>
+      <c r="P34" s="206"/>
+      <c r="Q34" s="207"/>
+      <c r="R34" s="220"/>
+      <c r="S34" s="221"/>
+      <c r="T34" s="221"/>
+      <c r="U34" s="221"/>
+      <c r="V34" s="222"/>
+      <c r="W34" s="139"/>
+      <c r="X34" s="140"/>
+      <c r="Y34" s="141"/>
       <c r="AB34" s="2"/>
       <c r="AC34" s="2"/>
       <c r="AD34" s="2"/>
       <c r="AE34" s="2"/>
     </row>
     <row r="35" spans="1:31" s="1" customFormat="1" ht="31.5" customHeight="1">
-      <c r="A35" s="95" t="s">
-        <v>50</v>
-      </c>
-      <c r="B35" s="96"/>
-      <c r="C35" s="96"/>
-      <c r="D35" s="96"/>
-      <c r="E35" s="96"/>
-      <c r="F35" s="96"/>
-      <c r="G35" s="96"/>
-      <c r="H35" s="96"/>
-      <c r="I35" s="97"/>
-      <c r="J35" s="54"/>
-      <c r="K35" s="54" t="s">
+      <c r="A35" s="229" t="s">
+        <v>49</v>
+      </c>
+      <c r="B35" s="230"/>
+      <c r="C35" s="230"/>
+      <c r="D35" s="230"/>
+      <c r="E35" s="230"/>
+      <c r="F35" s="230"/>
+      <c r="G35" s="230"/>
+      <c r="H35" s="230"/>
+      <c r="I35" s="231"/>
+      <c r="J35" s="50"/>
+      <c r="K35" s="50" t="s">
         <v>40</v>
       </c>
-      <c r="L35" s="54" t="s">
+      <c r="L35" s="50" t="s">
         <v>40</v>
       </c>
-      <c r="M35" s="54" t="s">
+      <c r="M35" s="50" t="s">
         <v>40</v>
       </c>
-      <c r="N35" s="54" t="s">
+      <c r="N35" s="50" t="s">
         <v>40</v>
       </c>
-      <c r="O35" s="89" t="s">
+      <c r="O35" s="211" t="s">
         <v>41</v>
       </c>
-      <c r="P35" s="90"/>
-      <c r="Q35" s="91"/>
-      <c r="R35" s="98">
+      <c r="P35" s="212"/>
+      <c r="Q35" s="213"/>
+      <c r="R35" s="223">
         <v>600000</v>
       </c>
-      <c r="S35" s="99"/>
-      <c r="T35" s="99"/>
-      <c r="U35" s="99"/>
-      <c r="V35" s="100"/>
-      <c r="W35" s="92"/>
-      <c r="X35" s="93"/>
-      <c r="Y35" s="94"/>
+      <c r="S35" s="224"/>
+      <c r="T35" s="224"/>
+      <c r="U35" s="224"/>
+      <c r="V35" s="225"/>
+      <c r="W35" s="143"/>
+      <c r="X35" s="144"/>
+      <c r="Y35" s="145"/>
       <c r="AB35" s="2"/>
       <c r="AC35" s="2"/>
       <c r="AD35" s="2"/>
       <c r="AE35" s="2"/>
     </row>
     <row r="36" spans="1:31" s="1" customFormat="1" ht="31.5" customHeight="1">
-      <c r="A36" s="95" t="s">
-        <v>51</v>
-      </c>
-      <c r="B36" s="96"/>
-      <c r="C36" s="96"/>
-      <c r="D36" s="96"/>
-      <c r="E36" s="96"/>
-      <c r="F36" s="96"/>
-      <c r="G36" s="96"/>
-      <c r="H36" s="96"/>
-      <c r="I36" s="97"/>
-      <c r="J36" s="54"/>
-      <c r="K36" s="54"/>
-      <c r="L36" s="54"/>
-      <c r="M36" s="54"/>
-      <c r="N36" s="54" t="s">
+      <c r="A36" s="229" t="s">
+        <v>50</v>
+      </c>
+      <c r="B36" s="230"/>
+      <c r="C36" s="230"/>
+      <c r="D36" s="230"/>
+      <c r="E36" s="230"/>
+      <c r="F36" s="230"/>
+      <c r="G36" s="230"/>
+      <c r="H36" s="230"/>
+      <c r="I36" s="231"/>
+      <c r="J36" s="50"/>
+      <c r="K36" s="50"/>
+      <c r="L36" s="50"/>
+      <c r="M36" s="50"/>
+      <c r="N36" s="50" t="s">
         <v>40</v>
       </c>
-      <c r="O36" s="89" t="s">
+      <c r="O36" s="211" t="s">
         <v>14</v>
       </c>
-      <c r="P36" s="90"/>
-      <c r="Q36" s="91"/>
-      <c r="R36" s="98">
+      <c r="P36" s="212"/>
+      <c r="Q36" s="213"/>
+      <c r="R36" s="223">
         <v>300000</v>
       </c>
-      <c r="S36" s="99"/>
-      <c r="T36" s="99"/>
-      <c r="U36" s="99"/>
-      <c r="V36" s="100"/>
-      <c r="W36" s="92"/>
-      <c r="X36" s="93"/>
-      <c r="Y36" s="94"/>
+      <c r="S36" s="224"/>
+      <c r="T36" s="224"/>
+      <c r="U36" s="224"/>
+      <c r="V36" s="225"/>
+      <c r="W36" s="143"/>
+      <c r="X36" s="144"/>
+      <c r="Y36" s="145"/>
       <c r="AB36" s="2"/>
       <c r="AC36" s="2"/>
       <c r="AD36" s="2"/>
       <c r="AE36" s="2"/>
     </row>
     <row r="37" spans="1:31" s="1" customFormat="1" ht="31.5" customHeight="1">
-      <c r="A37" s="173" t="s">
-        <v>52</v>
-      </c>
-      <c r="B37" s="174"/>
-      <c r="C37" s="174"/>
-      <c r="D37" s="174"/>
-      <c r="E37" s="174"/>
-      <c r="F37" s="174"/>
-      <c r="G37" s="174"/>
-      <c r="H37" s="174"/>
-      <c r="I37" s="175"/>
-      <c r="J37" s="60"/>
-      <c r="K37" s="54" t="s">
+      <c r="A37" s="229" t="s">
+        <v>51</v>
+      </c>
+      <c r="B37" s="230"/>
+      <c r="C37" s="230"/>
+      <c r="D37" s="230"/>
+      <c r="E37" s="230"/>
+      <c r="F37" s="230"/>
+      <c r="G37" s="230"/>
+      <c r="H37" s="230"/>
+      <c r="I37" s="231"/>
+      <c r="J37" s="56"/>
+      <c r="K37" s="50" t="s">
         <v>40</v>
       </c>
-      <c r="L37" s="54" t="s">
+      <c r="L37" s="50" t="s">
         <v>40</v>
       </c>
-      <c r="M37" s="54" t="s">
+      <c r="M37" s="50" t="s">
         <v>40</v>
       </c>
-      <c r="N37" s="54" t="s">
+      <c r="N37" s="50" t="s">
         <v>40</v>
       </c>
-      <c r="O37" s="116"/>
-      <c r="P37" s="117"/>
-      <c r="Q37" s="118"/>
-      <c r="R37" s="98">
+      <c r="O37" s="185"/>
+      <c r="P37" s="186"/>
+      <c r="Q37" s="187"/>
+      <c r="R37" s="223">
         <v>100000</v>
       </c>
-      <c r="S37" s="99"/>
-      <c r="T37" s="99"/>
-      <c r="U37" s="99"/>
-      <c r="V37" s="100"/>
-      <c r="W37" s="92"/>
-      <c r="X37" s="93"/>
-      <c r="Y37" s="94"/>
+      <c r="S37" s="224"/>
+      <c r="T37" s="224"/>
+      <c r="U37" s="224"/>
+      <c r="V37" s="225"/>
+      <c r="W37" s="143"/>
+      <c r="X37" s="144"/>
+      <c r="Y37" s="145"/>
       <c r="AB37" s="2"/>
       <c r="AC37" s="2"/>
       <c r="AD37" s="2"/>
       <c r="AE37" s="2"/>
     </row>
     <row r="38" spans="1:31" s="1" customFormat="1" ht="31.5" customHeight="1">
-      <c r="A38" s="176" t="s">
-        <v>62</v>
-      </c>
-      <c r="B38" s="177"/>
-      <c r="C38" s="178"/>
-      <c r="D38" s="86" t="s">
-        <v>71</v>
-      </c>
-      <c r="E38" s="87"/>
-      <c r="F38" s="87"/>
-      <c r="G38" s="87"/>
-      <c r="H38" s="87"/>
-      <c r="I38" s="88"/>
-      <c r="J38" s="60"/>
-      <c r="K38" s="54"/>
-      <c r="L38" s="54"/>
-      <c r="M38" s="54"/>
-      <c r="N38" s="54" t="s">
+      <c r="A38" s="235" t="s">
+        <v>134</v>
+      </c>
+      <c r="B38" s="244"/>
+      <c r="C38" s="245"/>
+      <c r="D38" s="163" t="s">
+        <v>69</v>
+      </c>
+      <c r="E38" s="164"/>
+      <c r="F38" s="164"/>
+      <c r="G38" s="164"/>
+      <c r="H38" s="164"/>
+      <c r="I38" s="165"/>
+      <c r="J38" s="56"/>
+      <c r="K38" s="50"/>
+      <c r="L38" s="50"/>
+      <c r="M38" s="50"/>
+      <c r="N38" s="50" t="s">
         <v>40</v>
       </c>
-      <c r="O38" s="119" t="s">
+      <c r="O38" s="191" t="s">
         <v>15</v>
       </c>
-      <c r="P38" s="120"/>
-      <c r="Q38" s="121"/>
-      <c r="R38" s="185"/>
-      <c r="S38" s="185"/>
-      <c r="T38" s="185"/>
-      <c r="U38" s="185"/>
-      <c r="V38" s="185"/>
-      <c r="W38" s="101"/>
-      <c r="X38" s="102"/>
-      <c r="Y38" s="103"/>
+      <c r="P38" s="192"/>
+      <c r="Q38" s="193"/>
+      <c r="R38" s="226"/>
+      <c r="S38" s="226"/>
+      <c r="T38" s="226"/>
+      <c r="U38" s="226"/>
+      <c r="V38" s="226"/>
+      <c r="W38" s="154"/>
+      <c r="X38" s="155"/>
+      <c r="Y38" s="156"/>
       <c r="AB38" s="2"/>
       <c r="AC38" s="2"/>
       <c r="AD38" s="2"/>
       <c r="AE38" s="2"/>
     </row>
     <row r="39" spans="1:31" s="1" customFormat="1" ht="31.5" customHeight="1">
-      <c r="A39" s="179"/>
-      <c r="B39" s="180"/>
-      <c r="C39" s="181"/>
-      <c r="D39" s="86" t="s">
-        <v>72</v>
-      </c>
-      <c r="E39" s="87"/>
-      <c r="F39" s="87"/>
-      <c r="G39" s="87"/>
-      <c r="H39" s="87"/>
-      <c r="I39" s="88"/>
-      <c r="J39" s="60"/>
-      <c r="K39" s="54"/>
-      <c r="L39" s="54"/>
-      <c r="M39" s="54"/>
-      <c r="N39" s="54"/>
-      <c r="O39" s="122"/>
-      <c r="P39" s="123"/>
-      <c r="Q39" s="124"/>
-      <c r="R39" s="186"/>
-      <c r="S39" s="186"/>
-      <c r="T39" s="186"/>
-      <c r="U39" s="186"/>
-      <c r="V39" s="186"/>
-      <c r="W39" s="104"/>
-      <c r="X39" s="105"/>
-      <c r="Y39" s="106"/>
+      <c r="A39" s="246"/>
+      <c r="B39" s="247"/>
+      <c r="C39" s="248"/>
+      <c r="D39" s="163" t="s">
+        <v>70</v>
+      </c>
+      <c r="E39" s="164"/>
+      <c r="F39" s="164"/>
+      <c r="G39" s="164"/>
+      <c r="H39" s="164"/>
+      <c r="I39" s="165"/>
+      <c r="J39" s="56"/>
+      <c r="K39" s="50"/>
+      <c r="L39" s="50"/>
+      <c r="M39" s="50"/>
+      <c r="N39" s="50"/>
+      <c r="O39" s="199"/>
+      <c r="P39" s="200"/>
+      <c r="Q39" s="201"/>
+      <c r="R39" s="227"/>
+      <c r="S39" s="227"/>
+      <c r="T39" s="227"/>
+      <c r="U39" s="227"/>
+      <c r="V39" s="227"/>
+      <c r="W39" s="157"/>
+      <c r="X39" s="158"/>
+      <c r="Y39" s="159"/>
       <c r="AB39" s="2"/>
       <c r="AC39" s="2"/>
       <c r="AD39" s="2"/>
       <c r="AE39" s="2"/>
     </row>
     <row r="40" spans="1:31" s="1" customFormat="1" ht="31.5" customHeight="1">
-      <c r="A40" s="182"/>
-      <c r="B40" s="183"/>
-      <c r="C40" s="184"/>
-      <c r="D40" s="86" t="s">
+      <c r="A40" s="249"/>
+      <c r="B40" s="250"/>
+      <c r="C40" s="251"/>
+      <c r="D40" s="163" t="s">
         <v>3</v>
       </c>
-      <c r="E40" s="87"/>
-      <c r="F40" s="87"/>
-      <c r="G40" s="87"/>
-      <c r="H40" s="87"/>
-      <c r="I40" s="88"/>
-      <c r="J40" s="60"/>
-      <c r="K40" s="54"/>
-      <c r="L40" s="54"/>
-      <c r="M40" s="54"/>
-      <c r="N40" s="54" t="s">
+      <c r="E40" s="164"/>
+      <c r="F40" s="164"/>
+      <c r="G40" s="164"/>
+      <c r="H40" s="164"/>
+      <c r="I40" s="165"/>
+      <c r="J40" s="56"/>
+      <c r="K40" s="50"/>
+      <c r="L40" s="50"/>
+      <c r="M40" s="50"/>
+      <c r="N40" s="50" t="s">
         <v>40</v>
       </c>
-      <c r="O40" s="125"/>
-      <c r="P40" s="126"/>
-      <c r="Q40" s="127"/>
-      <c r="R40" s="187"/>
-      <c r="S40" s="187"/>
-      <c r="T40" s="187"/>
-      <c r="U40" s="187"/>
-      <c r="V40" s="187"/>
-      <c r="W40" s="107"/>
-      <c r="X40" s="108"/>
-      <c r="Y40" s="109"/>
+      <c r="O40" s="205"/>
+      <c r="P40" s="206"/>
+      <c r="Q40" s="207"/>
+      <c r="R40" s="228"/>
+      <c r="S40" s="228"/>
+      <c r="T40" s="228"/>
+      <c r="U40" s="228"/>
+      <c r="V40" s="228"/>
+      <c r="W40" s="160"/>
+      <c r="X40" s="161"/>
+      <c r="Y40" s="162"/>
       <c r="AB40" s="2"/>
       <c r="AC40" s="2"/>
       <c r="AD40" s="2"/>
       <c r="AE40" s="2"/>
     </row>
     <row r="41" spans="1:31" s="1" customFormat="1" ht="30" customHeight="1">
-      <c r="A41" s="259" t="s">
+      <c r="A41" s="254" t="s">
         <v>39</v>
       </c>
-      <c r="B41" s="260"/>
-      <c r="C41" s="260"/>
-      <c r="D41" s="260"/>
-      <c r="E41" s="260"/>
-      <c r="F41" s="260"/>
-      <c r="G41" s="260"/>
-      <c r="H41" s="260"/>
-      <c r="I41" s="260"/>
-      <c r="J41" s="260"/>
-      <c r="K41" s="260"/>
-      <c r="L41" s="260"/>
-      <c r="M41" s="260"/>
-      <c r="N41" s="170" t="s">
-        <v>53</v>
-      </c>
-      <c r="O41" s="171"/>
-      <c r="P41" s="171"/>
-      <c r="Q41" s="171"/>
-      <c r="R41" s="171"/>
-      <c r="S41" s="171"/>
-      <c r="T41" s="172"/>
-      <c r="U41" s="211">
+      <c r="B41" s="255"/>
+      <c r="C41" s="255"/>
+      <c r="D41" s="255"/>
+      <c r="E41" s="255"/>
+      <c r="F41" s="255"/>
+      <c r="G41" s="255"/>
+      <c r="H41" s="255"/>
+      <c r="I41" s="255"/>
+      <c r="J41" s="255"/>
+      <c r="K41" s="255"/>
+      <c r="L41" s="255"/>
+      <c r="M41" s="255"/>
+      <c r="N41" s="256" t="s">
+        <v>52</v>
+      </c>
+      <c r="O41" s="257"/>
+      <c r="P41" s="257"/>
+      <c r="Q41" s="257"/>
+      <c r="R41" s="257"/>
+      <c r="S41" s="257"/>
+      <c r="T41" s="258"/>
+      <c r="U41" s="259">
         <f>SUM(R22:V40)</f>
         <v>1600000</v>
       </c>
-      <c r="V41" s="171"/>
-      <c r="W41" s="171"/>
-      <c r="X41" s="171"/>
-      <c r="Y41" s="172"/>
+      <c r="V41" s="257"/>
+      <c r="W41" s="257"/>
+      <c r="X41" s="257"/>
+      <c r="Y41" s="258"/>
       <c r="AB41" s="2"/>
       <c r="AC41" s="2"/>
       <c r="AD41" s="2"/>
       <c r="AE41" s="2"/>
     </row>
     <row r="42" spans="1:31" s="13" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A42" s="256" t="s">
+      <c r="A42" s="77" t="s">
         <v>34</v>
       </c>
-      <c r="B42" s="257"/>
-      <c r="C42" s="257"/>
-      <c r="D42" s="257"/>
-      <c r="E42" s="257"/>
-      <c r="F42" s="257"/>
-      <c r="G42" s="257"/>
-      <c r="H42" s="257"/>
-      <c r="I42" s="257"/>
-      <c r="J42" s="257"/>
-      <c r="K42" s="257"/>
-      <c r="L42" s="258"/>
-      <c r="M42" s="61" t="s">
+      <c r="B42" s="78"/>
+      <c r="C42" s="78"/>
+      <c r="D42" s="78"/>
+      <c r="E42" s="78"/>
+      <c r="F42" s="78"/>
+      <c r="G42" s="78"/>
+      <c r="H42" s="78"/>
+      <c r="I42" s="78"/>
+      <c r="J42" s="78"/>
+      <c r="K42" s="78"/>
+      <c r="L42" s="79"/>
+      <c r="M42" s="57" t="s">
         <v>35</v>
       </c>
-      <c r="N42" s="62"/>
-      <c r="O42" s="62"/>
-      <c r="P42" s="62"/>
-      <c r="Q42" s="62"/>
-      <c r="R42" s="62"/>
-      <c r="S42" s="62"/>
-      <c r="T42" s="62"/>
-      <c r="U42" s="62"/>
-      <c r="V42" s="62"/>
-      <c r="W42" s="62"/>
-      <c r="X42" s="62"/>
-      <c r="Y42" s="63"/>
-      <c r="AB42" s="64"/>
-      <c r="AC42" s="64"/>
-      <c r="AD42" s="64"/>
-      <c r="AE42" s="64"/>
+      <c r="N42" s="58"/>
+      <c r="O42" s="58"/>
+      <c r="P42" s="58"/>
+      <c r="Q42" s="58"/>
+      <c r="R42" s="58"/>
+      <c r="S42" s="58"/>
+      <c r="T42" s="58"/>
+      <c r="U42" s="58"/>
+      <c r="V42" s="58"/>
+      <c r="W42" s="58"/>
+      <c r="X42" s="58"/>
+      <c r="Y42" s="59"/>
+      <c r="AB42" s="60"/>
+      <c r="AC42" s="60"/>
+      <c r="AD42" s="60"/>
+      <c r="AE42" s="60"/>
     </row>
     <row r="43" spans="1:31" s="13" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A43" s="208" t="s">
+      <c r="A43" s="80" t="s">
         <v>36</v>
       </c>
-      <c r="B43" s="209"/>
-      <c r="C43" s="209"/>
-      <c r="D43" s="209"/>
-      <c r="E43" s="209"/>
-      <c r="F43" s="209"/>
-      <c r="G43" s="209"/>
-      <c r="H43" s="209"/>
-      <c r="I43" s="209"/>
-      <c r="J43" s="209"/>
-      <c r="K43" s="209"/>
-      <c r="L43" s="210"/>
-      <c r="M43" s="65" t="s">
+      <c r="B43" s="75"/>
+      <c r="C43" s="75"/>
+      <c r="D43" s="75"/>
+      <c r="E43" s="75"/>
+      <c r="F43" s="75"/>
+      <c r="G43" s="75"/>
+      <c r="H43" s="75"/>
+      <c r="I43" s="75"/>
+      <c r="J43" s="75"/>
+      <c r="K43" s="75"/>
+      <c r="L43" s="76"/>
+      <c r="M43" s="61" t="s">
+        <v>62</v>
+      </c>
+      <c r="Y43" s="38"/>
+      <c r="AB43" s="60"/>
+      <c r="AC43" s="60"/>
+      <c r="AD43" s="60"/>
+      <c r="AE43" s="60"/>
+    </row>
+    <row r="44" spans="1:31" s="13" customFormat="1" ht="20.100000000000001" customHeight="1">
+      <c r="A44" s="80" t="s">
+        <v>37</v>
+      </c>
+      <c r="B44" s="75"/>
+      <c r="C44" s="75"/>
+      <c r="D44" s="75"/>
+      <c r="E44" s="75"/>
+      <c r="F44" s="75"/>
+      <c r="G44" s="75"/>
+      <c r="H44" s="75"/>
+      <c r="I44" s="75"/>
+      <c r="J44" s="75"/>
+      <c r="K44" s="75"/>
+      <c r="L44" s="76"/>
+      <c r="M44" s="62" t="s">
+        <v>115</v>
+      </c>
+      <c r="N44" s="63"/>
+      <c r="O44" s="63"/>
+      <c r="P44" s="63"/>
+      <c r="Q44" s="63"/>
+      <c r="R44" s="63"/>
+      <c r="S44" s="63"/>
+      <c r="T44" s="63"/>
+      <c r="U44" s="63"/>
+      <c r="V44" s="63"/>
+      <c r="W44" s="63"/>
+      <c r="X44" s="63"/>
+      <c r="Y44" s="64"/>
+      <c r="AB44" s="60"/>
+      <c r="AC44" s="60"/>
+      <c r="AD44" s="60"/>
+      <c r="AE44" s="60"/>
+    </row>
+    <row r="45" spans="1:31" s="13" customFormat="1" ht="20.100000000000001" customHeight="1">
+      <c r="A45" s="80" t="s">
+        <v>32</v>
+      </c>
+      <c r="B45" s="75"/>
+      <c r="C45" s="75"/>
+      <c r="D45" s="75"/>
+      <c r="E45" s="75"/>
+      <c r="F45" s="75"/>
+      <c r="G45" s="75"/>
+      <c r="H45" s="75"/>
+      <c r="I45" s="75"/>
+      <c r="J45" s="75"/>
+      <c r="K45" s="75"/>
+      <c r="L45" s="76"/>
+      <c r="M45" s="65" t="s">
+        <v>114</v>
+      </c>
+      <c r="N45" s="66"/>
+      <c r="O45" s="66"/>
+      <c r="P45" s="66"/>
+      <c r="Q45" s="66"/>
+      <c r="R45" s="66"/>
+      <c r="S45" s="66"/>
+      <c r="T45" s="66"/>
+      <c r="U45" s="66"/>
+      <c r="V45" s="66"/>
+      <c r="W45" s="66"/>
+      <c r="X45" s="66"/>
+      <c r="Y45" s="67"/>
+      <c r="AB45" s="60"/>
+      <c r="AC45" s="60"/>
+      <c r="AD45" s="60"/>
+      <c r="AE45" s="60"/>
+    </row>
+    <row r="46" spans="1:31" s="13" customFormat="1" ht="20.100000000000001" customHeight="1">
+      <c r="A46" s="68" t="s">
+        <v>38</v>
+      </c>
+      <c r="B46" s="69"/>
+      <c r="C46" s="69"/>
+      <c r="D46" s="69"/>
+      <c r="E46" s="69"/>
+      <c r="F46" s="69"/>
+      <c r="G46" s="69"/>
+      <c r="H46" s="69"/>
+      <c r="I46" s="69"/>
+      <c r="J46" s="69"/>
+      <c r="K46" s="69"/>
+      <c r="L46" s="69"/>
+      <c r="M46" s="61" t="s">
+        <v>63</v>
+      </c>
+      <c r="Y46" s="38"/>
+      <c r="AB46" s="60"/>
+      <c r="AC46" s="60"/>
+      <c r="AD46" s="60"/>
+      <c r="AE46" s="60"/>
+    </row>
+    <row r="47" spans="1:31" s="13" customFormat="1" ht="20.100000000000001" customHeight="1">
+      <c r="A47" s="70" t="s">
+        <v>108</v>
+      </c>
+      <c r="D47" s="75" t="s">
+        <v>111</v>
+      </c>
+      <c r="E47" s="75"/>
+      <c r="F47" s="75"/>
+      <c r="G47" s="75"/>
+      <c r="H47" s="75"/>
+      <c r="I47" s="75"/>
+      <c r="J47" s="75"/>
+      <c r="K47" s="75"/>
+      <c r="L47" s="76"/>
+      <c r="M47" s="61" t="s">
+        <v>71</v>
+      </c>
+      <c r="Y47" s="38"/>
+      <c r="AB47" s="60"/>
+      <c r="AC47" s="60"/>
+      <c r="AD47" s="60"/>
+      <c r="AE47" s="60"/>
+    </row>
+    <row r="48" spans="1:31" s="13" customFormat="1" ht="20.100000000000001" customHeight="1">
+      <c r="A48" s="70" t="s">
+        <v>107</v>
+      </c>
+      <c r="D48" s="75" t="s">
+        <v>75</v>
+      </c>
+      <c r="E48" s="75"/>
+      <c r="F48" s="75"/>
+      <c r="G48" s="75"/>
+      <c r="H48" s="75"/>
+      <c r="I48" s="75"/>
+      <c r="J48" s="75"/>
+      <c r="K48" s="75"/>
+      <c r="L48" s="76"/>
+      <c r="M48" s="61" t="s">
         <v>64</v>
       </c>
-      <c r="Y43" s="38"/>
-      <c r="AB43" s="64"/>
-      <c r="AC43" s="64"/>
-      <c r="AD43" s="64"/>
-      <c r="AE43" s="64"/>
-    </row>
-    <row r="44" spans="1:31" s="13" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A44" s="208" t="s">
-        <v>37</v>
-      </c>
-      <c r="B44" s="209"/>
-      <c r="C44" s="209"/>
-      <c r="D44" s="209"/>
-      <c r="E44" s="209"/>
-      <c r="F44" s="209"/>
-      <c r="G44" s="209"/>
-      <c r="H44" s="209"/>
-      <c r="I44" s="209"/>
-      <c r="J44" s="209"/>
-      <c r="K44" s="209"/>
-      <c r="L44" s="210"/>
-      <c r="M44" s="66" t="s">
-        <v>117</v>
-      </c>
-      <c r="N44" s="67"/>
-      <c r="O44" s="67"/>
-      <c r="P44" s="67"/>
-      <c r="Q44" s="67"/>
-      <c r="R44" s="67"/>
-      <c r="S44" s="67"/>
-      <c r="T44" s="67"/>
-      <c r="U44" s="67"/>
-      <c r="V44" s="67"/>
-      <c r="W44" s="67"/>
-      <c r="X44" s="67"/>
-      <c r="Y44" s="68"/>
-      <c r="AB44" s="64"/>
-      <c r="AC44" s="64"/>
-      <c r="AD44" s="64"/>
-      <c r="AE44" s="64"/>
-    </row>
-    <row r="45" spans="1:31" s="13" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A45" s="208" t="s">
-        <v>32</v>
-      </c>
-      <c r="B45" s="209"/>
-      <c r="C45" s="209"/>
-      <c r="D45" s="209"/>
-      <c r="E45" s="209"/>
-      <c r="F45" s="209"/>
-      <c r="G45" s="209"/>
-      <c r="H45" s="209"/>
-      <c r="I45" s="209"/>
-      <c r="J45" s="209"/>
-      <c r="K45" s="209"/>
-      <c r="L45" s="210"/>
-      <c r="M45" s="69" t="s">
+      <c r="Y48" s="38"/>
+      <c r="AB48" s="60"/>
+      <c r="AC48" s="60"/>
+      <c r="AD48" s="60"/>
+      <c r="AE48" s="60"/>
+    </row>
+    <row r="49" spans="1:31" s="13" customFormat="1" ht="20.100000000000001" customHeight="1">
+      <c r="A49" s="70" t="s">
+        <v>109</v>
+      </c>
+      <c r="D49" s="73" t="s">
+        <v>112</v>
+      </c>
+      <c r="E49" s="73"/>
+      <c r="F49" s="73"/>
+      <c r="G49" s="73"/>
+      <c r="H49" s="73"/>
+      <c r="I49" s="73"/>
+      <c r="J49" s="73"/>
+      <c r="K49" s="73"/>
+      <c r="L49" s="74"/>
+      <c r="M49" s="61" t="s">
+        <v>65</v>
+      </c>
+      <c r="Y49" s="38"/>
+      <c r="AB49" s="60"/>
+      <c r="AC49" s="60"/>
+      <c r="AD49" s="60"/>
+      <c r="AE49" s="60"/>
+    </row>
+    <row r="50" spans="1:31" s="13" customFormat="1" ht="20.100000000000001" customHeight="1">
+      <c r="A50" s="70" t="s">
+        <v>110</v>
+      </c>
+      <c r="D50" s="81" t="s">
+        <v>113</v>
+      </c>
+      <c r="E50" s="81"/>
+      <c r="F50" s="81"/>
+      <c r="G50" s="81"/>
+      <c r="H50" s="81"/>
+      <c r="I50" s="81"/>
+      <c r="J50" s="81"/>
+      <c r="K50" s="81"/>
+      <c r="L50" s="82"/>
+      <c r="M50" s="61" t="s">
         <v>116</v>
       </c>
-      <c r="N45" s="70"/>
-      <c r="O45" s="70"/>
-      <c r="P45" s="70"/>
-      <c r="Q45" s="70"/>
-      <c r="R45" s="70"/>
-      <c r="S45" s="70"/>
-      <c r="T45" s="70"/>
-      <c r="U45" s="70"/>
-      <c r="V45" s="70"/>
-      <c r="W45" s="70"/>
-      <c r="X45" s="70"/>
-      <c r="Y45" s="71"/>
-      <c r="AB45" s="64"/>
-      <c r="AC45" s="64"/>
-      <c r="AD45" s="64"/>
-      <c r="AE45" s="64"/>
-    </row>
-    <row r="46" spans="1:31" s="13" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A46" s="72" t="s">
-        <v>38</v>
-      </c>
-      <c r="B46" s="73"/>
-      <c r="C46" s="73"/>
-      <c r="D46" s="73"/>
-      <c r="E46" s="73"/>
-      <c r="F46" s="73"/>
-      <c r="G46" s="73"/>
-      <c r="H46" s="73"/>
-      <c r="I46" s="73"/>
-      <c r="J46" s="73"/>
-      <c r="K46" s="73"/>
-      <c r="L46" s="73"/>
-      <c r="M46" s="65" t="s">
-        <v>65</v>
-      </c>
-      <c r="Y46" s="38"/>
-      <c r="AB46" s="64"/>
-      <c r="AC46" s="64"/>
-      <c r="AD46" s="64"/>
-      <c r="AE46" s="64"/>
-    </row>
-    <row r="47" spans="1:31" s="13" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A47" s="74" t="s">
-        <v>110</v>
-      </c>
-      <c r="D47" s="209" t="s">
-        <v>113</v>
-      </c>
-      <c r="E47" s="209"/>
-      <c r="F47" s="209"/>
-      <c r="G47" s="209"/>
-      <c r="H47" s="209"/>
-      <c r="I47" s="209"/>
-      <c r="J47" s="209"/>
-      <c r="K47" s="209"/>
-      <c r="L47" s="210"/>
-      <c r="M47" s="65" t="s">
-        <v>73</v>
-      </c>
-      <c r="Y47" s="38"/>
-      <c r="AB47" s="64"/>
-      <c r="AC47" s="64"/>
-      <c r="AD47" s="64"/>
-      <c r="AE47" s="64"/>
-    </row>
-    <row r="48" spans="1:31" s="13" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A48" s="74" t="s">
-        <v>109</v>
-      </c>
-      <c r="D48" s="209" t="s">
-        <v>77</v>
-      </c>
-      <c r="E48" s="209"/>
-      <c r="F48" s="209"/>
-      <c r="G48" s="209"/>
-      <c r="H48" s="209"/>
-      <c r="I48" s="209"/>
-      <c r="J48" s="209"/>
-      <c r="K48" s="209"/>
-      <c r="L48" s="210"/>
-      <c r="M48" s="65" t="s">
-        <v>66</v>
-      </c>
-      <c r="Y48" s="38"/>
-      <c r="AB48" s="64"/>
-      <c r="AC48" s="64"/>
-      <c r="AD48" s="64"/>
-      <c r="AE48" s="64"/>
-    </row>
-    <row r="49" spans="1:31" s="13" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A49" s="74" t="s">
-        <v>111</v>
-      </c>
-      <c r="D49" s="252" t="s">
-        <v>114</v>
-      </c>
-      <c r="E49" s="252"/>
-      <c r="F49" s="252"/>
-      <c r="G49" s="252"/>
-      <c r="H49" s="252"/>
-      <c r="I49" s="252"/>
-      <c r="J49" s="252"/>
-      <c r="K49" s="252"/>
-      <c r="L49" s="253"/>
-      <c r="M49" s="65" t="s">
+      <c r="Y50" s="38"/>
+      <c r="AB50" s="60"/>
+      <c r="AC50" s="60"/>
+      <c r="AD50" s="60"/>
+      <c r="AE50" s="60"/>
+    </row>
+    <row r="51" spans="1:31" s="13" customFormat="1" ht="20.100000000000001" customHeight="1">
+      <c r="A51" s="70"/>
+      <c r="D51" s="83"/>
+      <c r="E51" s="83"/>
+      <c r="F51" s="83"/>
+      <c r="G51" s="83"/>
+      <c r="H51" s="83"/>
+      <c r="I51" s="83"/>
+      <c r="J51" s="83"/>
+      <c r="K51" s="83"/>
+      <c r="L51" s="84"/>
+      <c r="M51" s="61" t="s">
+        <v>121</v>
+      </c>
+      <c r="Y51" s="38"/>
+      <c r="AB51" s="60"/>
+      <c r="AC51" s="60"/>
+      <c r="AD51" s="60"/>
+      <c r="AE51" s="60"/>
+    </row>
+    <row r="52" spans="1:31" s="1" customFormat="1" ht="35.25" customHeight="1">
+      <c r="A52" s="117" t="s">
         <v>67</v>
       </c>
-      <c r="Y49" s="38"/>
-      <c r="AB49" s="64"/>
-      <c r="AC49" s="64"/>
-      <c r="AD49" s="64"/>
-      <c r="AE49" s="64"/>
-    </row>
-    <row r="50" spans="1:31" s="13" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A50" s="74" t="s">
-        <v>112</v>
-      </c>
-      <c r="D50" s="233" t="s">
-        <v>115</v>
-      </c>
-      <c r="E50" s="233"/>
-      <c r="F50" s="233"/>
-      <c r="G50" s="233"/>
-      <c r="H50" s="233"/>
-      <c r="I50" s="233"/>
-      <c r="J50" s="233"/>
-      <c r="K50" s="233"/>
-      <c r="L50" s="234"/>
-      <c r="M50" s="65" t="s">
-        <v>118</v>
-      </c>
-      <c r="Y50" s="38"/>
-      <c r="AB50" s="64"/>
-      <c r="AC50" s="64"/>
-      <c r="AD50" s="64"/>
-      <c r="AE50" s="64"/>
-    </row>
-    <row r="51" spans="1:31" s="13" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A51" s="74"/>
-      <c r="D51" s="235"/>
-      <c r="E51" s="235"/>
-      <c r="F51" s="235"/>
-      <c r="G51" s="235"/>
-      <c r="H51" s="235"/>
-      <c r="I51" s="235"/>
-      <c r="J51" s="235"/>
-      <c r="K51" s="235"/>
-      <c r="L51" s="236"/>
-      <c r="M51" s="65" t="s">
-        <v>123</v>
-      </c>
-      <c r="Y51" s="38"/>
-      <c r="AB51" s="64"/>
-      <c r="AC51" s="64"/>
-      <c r="AD51" s="64"/>
-      <c r="AE51" s="64"/>
-    </row>
-    <row r="52" spans="1:31" s="1" customFormat="1" ht="35.25" customHeight="1">
-      <c r="A52" s="188" t="s">
-        <v>69</v>
-      </c>
-      <c r="B52" s="189"/>
-      <c r="C52" s="189"/>
-      <c r="D52" s="189"/>
-      <c r="E52" s="189"/>
-      <c r="F52" s="189"/>
-      <c r="G52" s="189"/>
-      <c r="H52" s="189"/>
-      <c r="I52" s="189"/>
-      <c r="J52" s="189"/>
-      <c r="K52" s="189"/>
-      <c r="L52" s="189"/>
-      <c r="M52" s="189"/>
-      <c r="N52" s="189"/>
-      <c r="O52" s="189"/>
-      <c r="P52" s="189"/>
-      <c r="Q52" s="189"/>
-      <c r="R52" s="189"/>
-      <c r="S52" s="189"/>
-      <c r="T52" s="189"/>
-      <c r="U52" s="189"/>
-      <c r="V52" s="189"/>
-      <c r="W52" s="189"/>
-      <c r="X52" s="189"/>
-      <c r="Y52" s="190"/>
+      <c r="B52" s="118"/>
+      <c r="C52" s="118"/>
+      <c r="D52" s="118"/>
+      <c r="E52" s="118"/>
+      <c r="F52" s="118"/>
+      <c r="G52" s="118"/>
+      <c r="H52" s="118"/>
+      <c r="I52" s="118"/>
+      <c r="J52" s="118"/>
+      <c r="K52" s="118"/>
+      <c r="L52" s="118"/>
+      <c r="M52" s="118"/>
+      <c r="N52" s="118"/>
+      <c r="O52" s="118"/>
+      <c r="P52" s="118"/>
+      <c r="Q52" s="118"/>
+      <c r="R52" s="118"/>
+      <c r="S52" s="118"/>
+      <c r="T52" s="118"/>
+      <c r="U52" s="118"/>
+      <c r="V52" s="118"/>
+      <c r="W52" s="118"/>
+      <c r="X52" s="118"/>
+      <c r="Y52" s="119"/>
       <c r="AB52" s="2"/>
       <c r="AC52" s="2"/>
       <c r="AD52" s="2"/>
       <c r="AE52" s="2"/>
     </row>
     <row r="53" spans="1:31" s="1" customFormat="1" ht="6" customHeight="1">
-      <c r="A53" s="75"/>
-      <c r="B53" s="75"/>
-      <c r="C53" s="75"/>
-      <c r="D53" s="75"/>
-      <c r="E53" s="75"/>
-      <c r="F53" s="75"/>
-      <c r="G53" s="75"/>
-      <c r="H53" s="75"/>
-      <c r="I53" s="75"/>
-      <c r="J53" s="75"/>
-      <c r="K53" s="75"/>
-      <c r="L53" s="75"/>
-      <c r="M53" s="75"/>
-      <c r="N53" s="75"/>
-      <c r="O53" s="75"/>
-      <c r="P53" s="75"/>
-      <c r="Q53" s="75"/>
-      <c r="R53" s="75"/>
-      <c r="S53" s="75"/>
-      <c r="T53" s="75"/>
-      <c r="U53" s="75"/>
-      <c r="V53" s="75"/>
-      <c r="W53" s="75"/>
-      <c r="X53" s="75"/>
-      <c r="Y53" s="75"/>
+      <c r="A53" s="71"/>
+      <c r="B53" s="71"/>
+      <c r="C53" s="71"/>
+      <c r="D53" s="71"/>
+      <c r="E53" s="71"/>
+      <c r="F53" s="71"/>
+      <c r="G53" s="71"/>
+      <c r="H53" s="71"/>
+      <c r="I53" s="71"/>
+      <c r="J53" s="71"/>
+      <c r="K53" s="71"/>
+      <c r="L53" s="71"/>
+      <c r="M53" s="71"/>
+      <c r="N53" s="71"/>
+      <c r="O53" s="71"/>
+      <c r="P53" s="71"/>
+      <c r="Q53" s="71"/>
+      <c r="R53" s="71"/>
+      <c r="S53" s="71"/>
+      <c r="T53" s="71"/>
+      <c r="U53" s="71"/>
+      <c r="V53" s="71"/>
+      <c r="W53" s="71"/>
+      <c r="X53" s="71"/>
+      <c r="Y53" s="71"/>
       <c r="AB53" s="2"/>
       <c r="AC53" s="2"/>
       <c r="AD53" s="2"/>
@@ -5008,20 +5049,75 @@
     </row>
   </sheetData>
   <mergeCells count="99">
-    <mergeCell ref="D49:L49"/>
-    <mergeCell ref="D48:L48"/>
-    <mergeCell ref="D47:L47"/>
-    <mergeCell ref="B23:I23"/>
-    <mergeCell ref="B24:I24"/>
-    <mergeCell ref="B25:I25"/>
-    <mergeCell ref="B27:I27"/>
-    <mergeCell ref="B28:I28"/>
-    <mergeCell ref="B30:I30"/>
-    <mergeCell ref="A42:L42"/>
-    <mergeCell ref="A43:L43"/>
-    <mergeCell ref="A44:L44"/>
-    <mergeCell ref="A41:M41"/>
-    <mergeCell ref="A29:I29"/>
+    <mergeCell ref="AF22:AH25"/>
+    <mergeCell ref="D39:I39"/>
+    <mergeCell ref="D40:I40"/>
+    <mergeCell ref="O35:Q35"/>
+    <mergeCell ref="W35:Y35"/>
+    <mergeCell ref="A35:I35"/>
+    <mergeCell ref="R35:V35"/>
+    <mergeCell ref="D32:I32"/>
+    <mergeCell ref="D33:I33"/>
+    <mergeCell ref="D34:I34"/>
+    <mergeCell ref="W36:Y36"/>
+    <mergeCell ref="W37:Y37"/>
+    <mergeCell ref="W38:Y40"/>
+    <mergeCell ref="J21:N21"/>
+    <mergeCell ref="J22:N22"/>
+    <mergeCell ref="J19:N19"/>
+    <mergeCell ref="O36:Q36"/>
+    <mergeCell ref="O37:Q37"/>
+    <mergeCell ref="O32:Q34"/>
+    <mergeCell ref="O26:Q28"/>
+    <mergeCell ref="O29:Q30"/>
+    <mergeCell ref="O31:Q31"/>
+    <mergeCell ref="O19:Q20"/>
+    <mergeCell ref="O21:Q21"/>
+    <mergeCell ref="O22:Q25"/>
+    <mergeCell ref="W19:Y20"/>
+    <mergeCell ref="R26:V31"/>
+    <mergeCell ref="W26:Y31"/>
+    <mergeCell ref="R32:V34"/>
+    <mergeCell ref="W32:Y34"/>
+    <mergeCell ref="R19:V20"/>
+    <mergeCell ref="R21:V21"/>
+    <mergeCell ref="W21:Y21"/>
+    <mergeCell ref="R22:V25"/>
+    <mergeCell ref="W22:Y25"/>
+    <mergeCell ref="N41:T41"/>
+    <mergeCell ref="A36:I36"/>
+    <mergeCell ref="O38:Q40"/>
+    <mergeCell ref="A37:I37"/>
+    <mergeCell ref="A38:C40"/>
+    <mergeCell ref="R36:V36"/>
+    <mergeCell ref="R37:V37"/>
+    <mergeCell ref="D38:I38"/>
+    <mergeCell ref="R38:V40"/>
+    <mergeCell ref="A19:I20"/>
+    <mergeCell ref="A52:Y52"/>
+    <mergeCell ref="S9:U9"/>
+    <mergeCell ref="S10:U10"/>
+    <mergeCell ref="O9:R9"/>
+    <mergeCell ref="O10:R10"/>
+    <mergeCell ref="V9:Y9"/>
+    <mergeCell ref="V10:Y10"/>
+    <mergeCell ref="A21:I21"/>
+    <mergeCell ref="A22:I22"/>
+    <mergeCell ref="A18:I18"/>
+    <mergeCell ref="A26:I26"/>
+    <mergeCell ref="A45:L45"/>
+    <mergeCell ref="U41:Y41"/>
+    <mergeCell ref="A31:I31"/>
+    <mergeCell ref="A32:C34"/>
+    <mergeCell ref="V7:Y7"/>
+    <mergeCell ref="L6:N6"/>
+    <mergeCell ref="A17:M17"/>
+    <mergeCell ref="O8:Y8"/>
+    <mergeCell ref="O7:R7"/>
+    <mergeCell ref="S7:U7"/>
+    <mergeCell ref="L7:N7"/>
+    <mergeCell ref="L8:N8"/>
+    <mergeCell ref="K6:K10"/>
     <mergeCell ref="D50:L51"/>
     <mergeCell ref="T18:X18"/>
     <mergeCell ref="J18:L18"/>
@@ -5038,75 +5134,20 @@
     <mergeCell ref="R15:S15"/>
     <mergeCell ref="L10:N10"/>
     <mergeCell ref="O6:Y6"/>
-    <mergeCell ref="V7:Y7"/>
-    <mergeCell ref="L6:N6"/>
-    <mergeCell ref="A17:M17"/>
-    <mergeCell ref="O8:Y8"/>
-    <mergeCell ref="O7:R7"/>
-    <mergeCell ref="S7:U7"/>
-    <mergeCell ref="L7:N7"/>
-    <mergeCell ref="L8:N8"/>
-    <mergeCell ref="K6:K10"/>
-    <mergeCell ref="A19:I20"/>
-    <mergeCell ref="A52:Y52"/>
-    <mergeCell ref="S9:U9"/>
-    <mergeCell ref="S10:U10"/>
-    <mergeCell ref="O9:R9"/>
-    <mergeCell ref="O10:R10"/>
-    <mergeCell ref="V9:Y9"/>
-    <mergeCell ref="V10:Y10"/>
-    <mergeCell ref="A21:I21"/>
-    <mergeCell ref="A22:I22"/>
-    <mergeCell ref="A18:I18"/>
-    <mergeCell ref="A26:I26"/>
-    <mergeCell ref="A45:L45"/>
-    <mergeCell ref="U41:Y41"/>
-    <mergeCell ref="A31:I31"/>
-    <mergeCell ref="A32:C34"/>
-    <mergeCell ref="N41:T41"/>
-    <mergeCell ref="A36:I36"/>
-    <mergeCell ref="O38:Q40"/>
-    <mergeCell ref="A37:I37"/>
-    <mergeCell ref="A38:C40"/>
-    <mergeCell ref="R36:V36"/>
-    <mergeCell ref="R37:V37"/>
-    <mergeCell ref="D38:I38"/>
-    <mergeCell ref="R38:V40"/>
-    <mergeCell ref="W19:Y20"/>
-    <mergeCell ref="R26:V31"/>
-    <mergeCell ref="W26:Y31"/>
-    <mergeCell ref="R32:V34"/>
-    <mergeCell ref="W32:Y34"/>
-    <mergeCell ref="R19:V20"/>
-    <mergeCell ref="R21:V21"/>
-    <mergeCell ref="W21:Y21"/>
-    <mergeCell ref="R22:V25"/>
-    <mergeCell ref="W22:Y25"/>
-    <mergeCell ref="J21:N21"/>
-    <mergeCell ref="J22:N22"/>
-    <mergeCell ref="J19:N19"/>
-    <mergeCell ref="O36:Q36"/>
-    <mergeCell ref="O37:Q37"/>
-    <mergeCell ref="O32:Q34"/>
-    <mergeCell ref="O26:Q28"/>
-    <mergeCell ref="O29:Q30"/>
-    <mergeCell ref="O31:Q31"/>
-    <mergeCell ref="O19:Q20"/>
-    <mergeCell ref="O21:Q21"/>
-    <mergeCell ref="O22:Q25"/>
-    <mergeCell ref="AF22:AH25"/>
-    <mergeCell ref="D39:I39"/>
-    <mergeCell ref="D40:I40"/>
-    <mergeCell ref="O35:Q35"/>
-    <mergeCell ref="W35:Y35"/>
-    <mergeCell ref="A35:I35"/>
-    <mergeCell ref="R35:V35"/>
-    <mergeCell ref="D32:I32"/>
-    <mergeCell ref="D33:I33"/>
-    <mergeCell ref="D34:I34"/>
-    <mergeCell ref="W36:Y36"/>
-    <mergeCell ref="W37:Y37"/>
-    <mergeCell ref="W38:Y40"/>
+    <mergeCell ref="D49:L49"/>
+    <mergeCell ref="D48:L48"/>
+    <mergeCell ref="D47:L47"/>
+    <mergeCell ref="B23:I23"/>
+    <mergeCell ref="B24:I24"/>
+    <mergeCell ref="B25:I25"/>
+    <mergeCell ref="B27:I27"/>
+    <mergeCell ref="B28:I28"/>
+    <mergeCell ref="B30:I30"/>
+    <mergeCell ref="A42:L42"/>
+    <mergeCell ref="A43:L43"/>
+    <mergeCell ref="A44:L44"/>
+    <mergeCell ref="A41:M41"/>
+    <mergeCell ref="A29:I29"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <hyperlinks>

</xml_diff>